<commit_message>
perf(cpp): reuse bounded large message storage
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rbe8e809860b040a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R3ac8e77ade874242"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R1170dfca6f57475a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R1bf24953ca764982"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R62d40d21952b4479"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R9eccf4ccc3c14320"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R81bafb0439e44844"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R3dd561753f324f72"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>Not started</x:v>
+        <x:v>PAIR/tcp 미달 — candidate A retained; candidate B rejected</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -540,7 +540,7 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="B12" s="18" t="n">
-        <x:f>COUNTIF('Paired Results'!U5:U400,"통과")</x:f>
+        <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
@@ -555,11 +555,11 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="B13" s="18" t="n">
-        <x:f>COUNTIF('Paired Results'!U5:U400,"미달")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
-        <x:v>Paired aggregate misses a gate; improvement evidence required</x:v>
+        <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
       </x:c>
       <x:c r="D13" s="17" t="str">
         <x:v>No unresolved fail</x:v>
@@ -570,7 +570,7 @@
         <x:v>Unmeasured</x:v>
       </x:c>
       <x:c r="B14" s="18" t="n">
-        <x:f>COUNTIF('Paired Results'!U5:U400,"미측정")</x:f>
+        <x:f>COUNTIFS('Paired Results'!U4:U400,"미측정",'Paired Results'!F4:F400,64)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C14" s="17" t="str">
@@ -691,24 +691,46 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="28" t="str"/>
+      <x:c r="A4" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
       <x:c r="B4" s="10" t="str">
         <x:v>C++</x:v>
       </x:c>
       <x:c r="C4" s="10" t="str">
         <x:v>Single</x:v>
       </x:c>
-      <x:c r="D4" s="10" t="str"/>
-      <x:c r="E4" s="10" t="str"/>
-      <x:c r="F4" s="10"/>
-      <x:c r="G4" s="26"/>
-      <x:c r="H4" s="26"/>
-      <x:c r="I4" s="22"/>
-      <x:c r="J4" s="24"/>
-      <x:c r="K4" s="24"/>
-      <x:c r="L4" s="24"/>
+      <x:c r="D4" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E4" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F4" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G4" s="26" t="n">
+        <x:v>2064848.4</x:v>
+      </x:c>
+      <x:c r="H4" s="26" t="n">
+        <x:v>1922350.2</x:v>
+      </x:c>
+      <x:c r="I4" s="22" t="n">
+        <x:f>H4/G4</x:f>
+        <x:v>0.9309885413379501</x:v>
+      </x:c>
+      <x:c r="J4" s="24" t="n">
+        <x:v>0.32</x:v>
+      </x:c>
+      <x:c r="K4" s="24" t="n">
+        <x:v>0.352</x:v>
+      </x:c>
+      <x:c r="L4" s="24" t="n">
+        <x:f>K4/J4</x:f>
+        <x:v>1.0999999999999999</x:v>
+      </x:c>
       <x:c r="M4" s="10" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N4" s="10" t="n">
         <x:v>5</x:v>
@@ -723,115 +745,790 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R4" s="10" t="str">
-        <x:v>0d12a1e8f5</x:v>
-      </x:c>
-      <x:c r="S4" s="10" t="str"/>
-      <x:c r="T4" s="10" t="str"/>
+        <x:v>dd4b246e8a</x:v>
+      </x:c>
+      <x:c r="S4" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_145312_cpp-pair-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T4" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_145550_cpp-pair-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
       <x:c r="U4" s="10" t="str">
-        <x:v>미측정</x:v>
+        <x:v>미달</x:v>
       </x:c>
       <x:c r="V4" s="10" t="str">
-        <x:v>Fresh ledger: do not carry 0.13.0 values.</x:v>
+        <x:v>Baseline: throughput aggregate mean 91.0%; latency median ratio 1.12x (pass).</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="29"/>
-      <x:c r="G5" s="27"/>
-      <x:c r="H5" s="27"/>
-      <x:c r="I5" s="23"/>
-      <x:c r="J5" s="25"/>
-      <x:c r="K5" s="25"/>
-      <x:c r="L5" s="25"/>
+      <x:c r="A5" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B5" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C5" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D5" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E5" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F5" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G5" s="26" t="n">
+        <x:v>1403138.4</x:v>
+      </x:c>
+      <x:c r="H5" s="26" t="n">
+        <x:v>1263976</x:v>
+      </x:c>
+      <x:c r="I5" s="22" t="n">
+        <x:f>H5/G5</x:f>
+        <x:v>0.9008206175527661</x:v>
+      </x:c>
+      <x:c r="J5" s="24" t="n">
+        <x:v>1.216</x:v>
+      </x:c>
+      <x:c r="K5" s="24" t="n">
+        <x:v>1.378</x:v>
+      </x:c>
+      <x:c r="L5" s="24" t="n">
+        <x:f>K5/J5</x:f>
+        <x:v>1.1332236842105263</x:v>
+      </x:c>
+      <x:c r="M5" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N5" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O5" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P5" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q5" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R5" s="10" t="str">
+        <x:v>dd4b246e8a</x:v>
+      </x:c>
+      <x:c r="S5" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_145312_cpp-pair-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T5" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_145550_cpp-pair-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U5" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V5" s="10" t="str">
+        <x:v>Baseline: throughput aggregate mean 91.0%; latency median ratio 1.12x (pass).</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="29"/>
-      <x:c r="G6" s="27"/>
-      <x:c r="H6" s="27"/>
-      <x:c r="I6" s="23"/>
-      <x:c r="J6" s="25"/>
-      <x:c r="K6" s="25"/>
-      <x:c r="L6" s="25"/>
+      <x:c r="A6" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B6" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C6" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D6" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F6" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G6" s="26" t="n">
+        <x:v>581576.2</x:v>
+      </x:c>
+      <x:c r="H6" s="26" t="n">
+        <x:v>553331</x:v>
+      </x:c>
+      <x:c r="I6" s="22" t="n">
+        <x:f>H6/G6</x:f>
+        <x:v>0.9514333633322685</x:v>
+      </x:c>
+      <x:c r="J6" s="24" t="n">
+        <x:v>0.829</x:v>
+      </x:c>
+      <x:c r="K6" s="24" t="n">
+        <x:v>0.872</x:v>
+      </x:c>
+      <x:c r="L6" s="24" t="n">
+        <x:f>K6/J6</x:f>
+        <x:v>1.051869722557298</x:v>
+      </x:c>
+      <x:c r="M6" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N6" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O6" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P6" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q6" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R6" s="10" t="str">
+        <x:v>dd4b246e8a</x:v>
+      </x:c>
+      <x:c r="S6" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_145312_cpp-pair-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T6" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_145550_cpp-pair-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U6" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V6" s="10" t="str">
+        <x:v>Baseline: throughput aggregate mean 91.0%; latency median ratio 1.12x (pass).</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="29"/>
-      <x:c r="G7" s="27"/>
-      <x:c r="H7" s="27"/>
-      <x:c r="I7" s="23"/>
-      <x:c r="J7" s="25"/>
-      <x:c r="K7" s="25"/>
-      <x:c r="L7" s="25"/>
+      <x:c r="A7" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B7" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C7" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D7" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E7" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F7" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G7" s="26" t="n">
+        <x:v>33079</x:v>
+      </x:c>
+      <x:c r="H7" s="26" t="n">
+        <x:v>26469.8</x:v>
+      </x:c>
+      <x:c r="I7" s="22" t="n">
+        <x:f>H7/G7</x:f>
+        <x:v>0.800199522355573</x:v>
+      </x:c>
+      <x:c r="J7" s="24" t="n">
+        <x:v>0.297</x:v>
+      </x:c>
+      <x:c r="K7" s="24" t="n">
+        <x:v>0.388</x:v>
+      </x:c>
+      <x:c r="L7" s="24" t="n">
+        <x:f>K7/J7</x:f>
+        <x:v>1.3063973063973064</x:v>
+      </x:c>
+      <x:c r="M7" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N7" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O7" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P7" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q7" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R7" s="10" t="str">
+        <x:v>dd4b246e8a</x:v>
+      </x:c>
+      <x:c r="S7" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_145312_cpp-pair-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T7" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_145550_cpp-pair-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U7" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V7" s="10" t="str">
+        <x:v>Baseline: throughput aggregate mean 91.0%; latency median ratio 1.12x (pass).</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="29"/>
-      <x:c r="G8" s="27"/>
-      <x:c r="H8" s="27"/>
-      <x:c r="I8" s="23"/>
-      <x:c r="J8" s="25"/>
-      <x:c r="K8" s="25"/>
-      <x:c r="L8" s="25"/>
+      <x:c r="A8" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B8" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D8" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F8" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G8" s="26" t="n">
+        <x:v>22856.6</x:v>
+      </x:c>
+      <x:c r="H8" s="26" t="n">
+        <x:v>20687.2</x:v>
+      </x:c>
+      <x:c r="I8" s="22" t="n">
+        <x:f>H8/G8</x:f>
+        <x:v>0.9050864958042755</x:v>
+      </x:c>
+      <x:c r="J8" s="24" t="n">
+        <x:v>0.27</x:v>
+      </x:c>
+      <x:c r="K8" s="24" t="n">
+        <x:v>0.305</x:v>
+      </x:c>
+      <x:c r="L8" s="24" t="n">
+        <x:f>K8/J8</x:f>
+        <x:v>1.1296296296296295</x:v>
+      </x:c>
+      <x:c r="M8" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N8" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O8" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P8" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q8" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R8" s="10" t="str">
+        <x:v>dd4b246e8a</x:v>
+      </x:c>
+      <x:c r="S8" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_145312_cpp-pair-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T8" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_145550_cpp-pair-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U8" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V8" s="10" t="str">
+        <x:v>Baseline: throughput aggregate mean 91.0%; latency median ratio 1.12x (pass).</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="29"/>
-      <x:c r="G9" s="27"/>
-      <x:c r="H9" s="27"/>
-      <x:c r="I9" s="23"/>
-      <x:c r="J9" s="25"/>
-      <x:c r="K9" s="25"/>
-      <x:c r="L9" s="25"/>
+      <x:c r="A9" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B9" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C9" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D9" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E9" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F9" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G9" s="26" t="n">
+        <x:v>13821</x:v>
+      </x:c>
+      <x:c r="H9" s="26" t="n">
+        <x:v>13420.4</x:v>
+      </x:c>
+      <x:c r="I9" s="22" t="n">
+        <x:f>H9/G9</x:f>
+        <x:v>0.971015121915925</x:v>
+      </x:c>
+      <x:c r="J9" s="24" t="n">
+        <x:v>0.297</x:v>
+      </x:c>
+      <x:c r="K9" s="24" t="n">
+        <x:v>0.303</x:v>
+      </x:c>
+      <x:c r="L9" s="24" t="n">
+        <x:f>K9/J9</x:f>
+        <x:v>1.02020202020202</x:v>
+      </x:c>
+      <x:c r="M9" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N9" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O9" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P9" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q9" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R9" s="10" t="str">
+        <x:v>dd4b246e8a</x:v>
+      </x:c>
+      <x:c r="S9" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_145312_cpp-pair-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T9" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_145550_cpp-pair-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U9" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V9" s="10" t="str">
+        <x:v>Baseline: throughput aggregate mean 91.0%; latency median ratio 1.12x (pass).</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="29"/>
-      <x:c r="G10" s="27"/>
-      <x:c r="H10" s="27"/>
-      <x:c r="I10" s="23"/>
-      <x:c r="J10" s="25"/>
-      <x:c r="K10" s="25"/>
-      <x:c r="L10" s="25"/>
+      <x:c r="A10" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B10" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C10" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D10" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E10" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F10" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G10" s="26" t="n">
+        <x:v>2060741.4</x:v>
+      </x:c>
+      <x:c r="H10" s="26" t="n">
+        <x:v>1955948.4</x:v>
+      </x:c>
+      <x:c r="I10" s="22" t="n">
+        <x:f>H10/G10</x:f>
+        <x:v>0.9491479134645424</x:v>
+      </x:c>
+      <x:c r="J10" s="24" t="n">
+        <x:v>0.514</x:v>
+      </x:c>
+      <x:c r="K10" s="24" t="n">
+        <x:v>0.294</x:v>
+      </x:c>
+      <x:c r="L10" s="24" t="n">
+        <x:f>K10/J10</x:f>
+        <x:v>0.5719844357976653</x:v>
+      </x:c>
+      <x:c r="M10" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N10" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O10" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P10" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q10" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R10" s="10" t="str">
+        <x:v>dd4b246e8a</x:v>
+      </x:c>
+      <x:c r="S10" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_151518_cpp-pair-tcp-local0132-candidate-a-teardown-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T10" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_151758_cpp-pair-tcp-local0132-candidate-a-teardown-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U10" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V10" s="10" t="str">
+        <x:v>Candidate A final: throughput aggregate mean 94.37%; latency median ratio 1.04x (pass); strict 95% gate missed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="29"/>
-      <x:c r="G11" s="27"/>
-      <x:c r="H11" s="27"/>
-      <x:c r="I11" s="23"/>
-      <x:c r="J11" s="25"/>
-      <x:c r="K11" s="25"/>
-      <x:c r="L11" s="25"/>
+      <x:c r="A11" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B11" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C11" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D11" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E11" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F11" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G11" s="26" t="n">
+        <x:v>1296799.6</x:v>
+      </x:c>
+      <x:c r="H11" s="26" t="n">
+        <x:v>1302445</x:v>
+      </x:c>
+      <x:c r="I11" s="22" t="n">
+        <x:f>H11/G11</x:f>
+        <x:v>1.0043533326197818</x:v>
+      </x:c>
+      <x:c r="J11" s="24" t="n">
+        <x:v>1.327</x:v>
+      </x:c>
+      <x:c r="K11" s="24" t="n">
+        <x:v>1.351</x:v>
+      </x:c>
+      <x:c r="L11" s="24" t="n">
+        <x:f>K11/J11</x:f>
+        <x:v>1.0180859080633007</x:v>
+      </x:c>
+      <x:c r="M11" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N11" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O11" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P11" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q11" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R11" s="10" t="str">
+        <x:v>dd4b246e8a</x:v>
+      </x:c>
+      <x:c r="S11" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_151518_cpp-pair-tcp-local0132-candidate-a-teardown-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T11" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_151758_cpp-pair-tcp-local0132-candidate-a-teardown-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U11" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V11" s="10" t="str">
+        <x:v>Candidate A final: throughput aggregate mean 94.37%; latency median ratio 1.04x (pass); strict 95% gate missed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="29"/>
-      <x:c r="G12" s="27"/>
-      <x:c r="H12" s="27"/>
-      <x:c r="I12" s="23"/>
-      <x:c r="J12" s="25"/>
-      <x:c r="K12" s="25"/>
-      <x:c r="L12" s="25"/>
+      <x:c r="A12" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C12" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D12" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F12" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G12" s="26" t="n">
+        <x:v>554947</x:v>
+      </x:c>
+      <x:c r="H12" s="26" t="n">
+        <x:v>542962.4</x:v>
+      </x:c>
+      <x:c r="I12" s="22" t="n">
+        <x:f>H12/G12</x:f>
+        <x:v>0.9784040638114991</x:v>
+      </x:c>
+      <x:c r="J12" s="24" t="n">
+        <x:v>0.87</x:v>
+      </x:c>
+      <x:c r="K12" s="24" t="n">
+        <x:v>0.895</x:v>
+      </x:c>
+      <x:c r="L12" s="24" t="n">
+        <x:f>K12/J12</x:f>
+        <x:v>1.028735632183908</x:v>
+      </x:c>
+      <x:c r="M12" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N12" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O12" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P12" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q12" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R12" s="10" t="str">
+        <x:v>dd4b246e8a</x:v>
+      </x:c>
+      <x:c r="S12" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_151518_cpp-pair-tcp-local0132-candidate-a-teardown-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T12" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_151758_cpp-pair-tcp-local0132-candidate-a-teardown-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U12" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V12" s="10" t="str">
+        <x:v>Candidate A final: throughput aggregate mean 94.37%; latency median ratio 1.04x (pass); strict 95% gate missed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="29"/>
-      <x:c r="G13" s="27"/>
-      <x:c r="H13" s="27"/>
-      <x:c r="I13" s="23"/>
-      <x:c r="J13" s="25"/>
-      <x:c r="K13" s="25"/>
-      <x:c r="L13" s="25"/>
+      <x:c r="A13" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B13" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C13" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D13" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E13" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F13" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G13" s="26" t="n">
+        <x:v>31060.4</x:v>
+      </x:c>
+      <x:c r="H13" s="26" t="n">
+        <x:v>26669.8</x:v>
+      </x:c>
+      <x:c r="I13" s="22" t="n">
+        <x:f>H13/G13</x:f>
+        <x:v>0.8586431597790112</x:v>
+      </x:c>
+      <x:c r="J13" s="24" t="n">
+        <x:v>0.317</x:v>
+      </x:c>
+      <x:c r="K13" s="24" t="n">
+        <x:v>0.392</x:v>
+      </x:c>
+      <x:c r="L13" s="24" t="n">
+        <x:f>K13/J13</x:f>
+        <x:v>1.2365930599369086</x:v>
+      </x:c>
+      <x:c r="M13" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N13" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O13" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P13" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q13" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R13" s="10" t="str">
+        <x:v>dd4b246e8a</x:v>
+      </x:c>
+      <x:c r="S13" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_151518_cpp-pair-tcp-local0132-candidate-a-teardown-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T13" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_151758_cpp-pair-tcp-local0132-candidate-a-teardown-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U13" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V13" s="10" t="str">
+        <x:v>Candidate A final: throughput aggregate mean 94.37%; latency median ratio 1.04x (pass); strict 95% gate missed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="29"/>
-      <x:c r="G14" s="27"/>
-      <x:c r="H14" s="27"/>
-      <x:c r="I14" s="23"/>
-      <x:c r="J14" s="25"/>
-      <x:c r="K14" s="25"/>
-      <x:c r="L14" s="25"/>
+      <x:c r="A14" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B14" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C14" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D14" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E14" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F14" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G14" s="26" t="n">
+        <x:v>21682.2</x:v>
+      </x:c>
+      <x:c r="H14" s="26" t="n">
+        <x:v>20719</x:v>
+      </x:c>
+      <x:c r="I14" s="22" t="n">
+        <x:f>H14/G14</x:f>
+        <x:v>0.9555764636429882</x:v>
+      </x:c>
+      <x:c r="J14" s="24" t="n">
+        <x:v>0.284</x:v>
+      </x:c>
+      <x:c r="K14" s="24" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="L14" s="24" t="n">
+        <x:f>K14/J14</x:f>
+        <x:v>1.0563380281690142</x:v>
+      </x:c>
+      <x:c r="M14" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N14" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O14" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P14" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q14" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R14" s="10" t="str">
+        <x:v>dd4b246e8a</x:v>
+      </x:c>
+      <x:c r="S14" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_151518_cpp-pair-tcp-local0132-candidate-a-teardown-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T14" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_151758_cpp-pair-tcp-local0132-candidate-a-teardown-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U14" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V14" s="10" t="str">
+        <x:v>Candidate A final: throughput aggregate mean 94.37%; latency median ratio 1.04x (pass); strict 95% gate missed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="29"/>
-      <x:c r="G15" s="27"/>
-      <x:c r="H15" s="27"/>
-      <x:c r="I15" s="23"/>
-      <x:c r="J15" s="25"/>
-      <x:c r="K15" s="25"/>
-      <x:c r="L15" s="25"/>
+      <x:c r="A15" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B15" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C15" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D15" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E15" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F15" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G15" s="26" t="n">
+        <x:v>13573</x:v>
+      </x:c>
+      <x:c r="H15" s="26" t="n">
+        <x:v>12435.2</x:v>
+      </x:c>
+      <x:c r="I15" s="22" t="n">
+        <x:f>H15/G15</x:f>
+        <x:v>0.9161718116849629</x:v>
+      </x:c>
+      <x:c r="J15" s="24" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="K15" s="24" t="n">
+        <x:v>0.326</x:v>
+      </x:c>
+      <x:c r="L15" s="24" t="n">
+        <x:f>K15/J15</x:f>
+        <x:v>1.0866666666666667</x:v>
+      </x:c>
+      <x:c r="M15" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N15" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O15" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P15" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q15" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R15" s="10" t="str">
+        <x:v>dd4b246e8a</x:v>
+      </x:c>
+      <x:c r="S15" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_151518_cpp-pair-tcp-local0132-candidate-a-teardown-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T15" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_151758_cpp-pair-tcp-local0132-candidate-a-teardown-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U15" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V15" s="10" t="str">
+        <x:v>Candidate A final: throughput aggregate mean 94.37%; latency median ratio 1.04x (pass); strict 95% gate missed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="29"/>
@@ -4386,28 +5083,90 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="10" t="str"/>
-      <x:c r="B4" s="10" t="str"/>
-      <x:c r="C4" s="10" t="str"/>
-      <x:c r="D4" s="10" t="str"/>
-      <x:c r="E4" s="10" t="str"/>
-      <x:c r="F4" s="10" t="str"/>
+      <x:c r="A4" s="10" t="str">
+        <x:v>2026-08-25 15:18</x:v>
+      </x:c>
+      <x:c r="B4" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C4" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D4" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E4" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F4" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 95%</x:v>
+      </x:c>
       <x:c r="G4" s="10" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="H4" s="10" t="str"/>
+      <x:c r="H4" s="10" t="str">
+        <x:v>Enable existing bounded 8MiB large-message pool for 128KiB–1MiB; keep singleton alive through process teardown.</x:v>
+      </x:c>
       <x:c r="I4" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
-      <x:c r="J4" s="10" t="str"/>
-      <x:c r="K4" s="10" t="str"/>
-      <x:c r="L4" s="22"/>
-      <x:c r="M4" s="22"/>
-      <x:c r="N4" s="10" t="str"/>
+      <x:c r="J4" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_145550_cpp-pair-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K4" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_151758_cpp-pair-tcp-local0132-candidate-a-teardown-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L4" s="22" t="n">
+        <x:v>0.91</x:v>
+      </x:c>
+      <x:c r="M4" s="22" t="n">
+        <x:v>0.944</x:v>
+      </x:c>
+      <x:c r="N4" s="10" t="str">
+        <x:v>Keep candidate A. Sol review required immortal lifetime to avoid teardown UAF; contract tests passed. Strict gate remains 미달.</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="L5" s="23"/>
-      <x:c r="M5" s="23"/>
+      <x:c r="A5" s="10" t="str">
+        <x:v>2026-08-25 15:06</x:v>
+      </x:c>
+      <x:c r="B5" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C5" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D5" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E5" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F5" s="10" t="str">
+        <x:v>64KiB throughput gap</x:v>
+      </x:c>
+      <x:c r="G5" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H5" s="10" t="str">
+        <x:v>Lower the same pool threshold to 64KiB; same 8MiB cap and release callback.</x:v>
+      </x:c>
+      <x:c r="I5" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J5" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_151758_cpp-pair-tcp-local0132-candidate-a-teardown-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K5" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_150618_cpp-pair-tcp-local0132-candidate-b-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L5" s="22" t="n">
+        <x:v>0.944</x:v>
+      </x:c>
+      <x:c r="M5" s="22"/>
+      <x:c r="N5" s="10" t="str">
+        <x:v>REJECT: 64KiB run timed out; partial report (25/30 result lines). Reverted threshold to 128KiB.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="L6" s="23"/>

</xml_diff>

<commit_message>
perf(cpp): record core 0.13.2 pubsub baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R62d40d21952b4479"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R9eccf4ccc3c14320"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R81bafb0439e44844"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R3dd561753f324f72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R071dfbe321aa400c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R6e0f77fa593f4825"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rdd21f9878edf4e2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Ra38e4e056bd64795"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -1531,58 +1531,424 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="29"/>
-      <x:c r="G16" s="27"/>
-      <x:c r="H16" s="27"/>
-      <x:c r="I16" s="23"/>
-      <x:c r="J16" s="25"/>
-      <x:c r="K16" s="25"/>
-      <x:c r="L16" s="25"/>
+      <x:c r="A16" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B16" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C16" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D16" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F16" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G16" s="26" t="n">
+        <x:v>1122126.4</x:v>
+      </x:c>
+      <x:c r="H16" s="26" t="n">
+        <x:v>1054066.2</x:v>
+      </x:c>
+      <x:c r="I16" s="22" t="n">
+        <x:f>H16/G16</x:f>
+        <x:v>0.939347118114323</x:v>
+      </x:c>
+      <x:c r="J16" s="24" t="n">
+        <x:v>0.122</x:v>
+      </x:c>
+      <x:c r="K16" s="24" t="n">
+        <x:v>0.14</x:v>
+      </x:c>
+      <x:c r="L16" s="24" t="n">
+        <x:f>K16/J16</x:f>
+        <x:v>1.1475409836065575</x:v>
+      </x:c>
+      <x:c r="M16" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N16" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O16" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P16" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q16" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R16" s="10" t="str">
+        <x:v>438f281aa1</x:v>
+      </x:c>
+      <x:c r="S16" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_152813_cpp-pubsub-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T16" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_153122_cpp-pubsub-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U16" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V16" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.60%; latency median ratio 1.07x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="29"/>
-      <x:c r="G17" s="27"/>
-      <x:c r="H17" s="27"/>
-      <x:c r="I17" s="23"/>
-      <x:c r="J17" s="25"/>
-      <x:c r="K17" s="25"/>
-      <x:c r="L17" s="25"/>
+      <x:c r="A17" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B17" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C17" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D17" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E17" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F17" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G17" s="26" t="n">
+        <x:v>898586.8</x:v>
+      </x:c>
+      <x:c r="H17" s="26" t="n">
+        <x:v>874541.6</x:v>
+      </x:c>
+      <x:c r="I17" s="22" t="n">
+        <x:f>H17/G17</x:f>
+        <x:v>0.9732410936817678</x:v>
+      </x:c>
+      <x:c r="J17" s="24" t="n">
+        <x:v>1.663</x:v>
+      </x:c>
+      <x:c r="K17" s="24" t="n">
+        <x:v>1.743</x:v>
+      </x:c>
+      <x:c r="L17" s="24" t="n">
+        <x:f>K17/J17</x:f>
+        <x:v>1.048105832832231</x:v>
+      </x:c>
+      <x:c r="M17" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N17" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O17" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P17" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q17" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R17" s="10" t="str">
+        <x:v>438f281aa1</x:v>
+      </x:c>
+      <x:c r="S17" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_152813_cpp-pubsub-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T17" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_153122_cpp-pubsub-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U17" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V17" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.60%; latency median ratio 1.07x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="29"/>
-      <x:c r="G18" s="27"/>
-      <x:c r="H18" s="27"/>
-      <x:c r="I18" s="23"/>
-      <x:c r="J18" s="25"/>
-      <x:c r="K18" s="25"/>
-      <x:c r="L18" s="25"/>
+      <x:c r="A18" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B18" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C18" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D18" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E18" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F18" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G18" s="26" t="n">
+        <x:v>527062.6</x:v>
+      </x:c>
+      <x:c r="H18" s="26" t="n">
+        <x:v>519073.8</x:v>
+      </x:c>
+      <x:c r="I18" s="22" t="n">
+        <x:f>H18/G18</x:f>
+        <x:v>0.9848427871755652</x:v>
+      </x:c>
+      <x:c r="J18" s="24" t="n">
+        <x:v>0.877</x:v>
+      </x:c>
+      <x:c r="K18" s="24" t="n">
+        <x:v>0.892</x:v>
+      </x:c>
+      <x:c r="L18" s="24" t="n">
+        <x:f>K18/J18</x:f>
+        <x:v>1.017103762827822</x:v>
+      </x:c>
+      <x:c r="M18" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N18" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O18" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P18" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q18" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R18" s="10" t="str">
+        <x:v>438f281aa1</x:v>
+      </x:c>
+      <x:c r="S18" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_152813_cpp-pubsub-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T18" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_153122_cpp-pubsub-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U18" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V18" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.60%; latency median ratio 1.07x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="29"/>
-      <x:c r="G19" s="27"/>
-      <x:c r="H19" s="27"/>
-      <x:c r="I19" s="23"/>
-      <x:c r="J19" s="25"/>
-      <x:c r="K19" s="25"/>
-      <x:c r="L19" s="25"/>
+      <x:c r="A19" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B19" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C19" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D19" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E19" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F19" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G19" s="26" t="n">
+        <x:v>32355.2</x:v>
+      </x:c>
+      <x:c r="H19" s="26" t="n">
+        <x:v>29939.6</x:v>
+      </x:c>
+      <x:c r="I19" s="22" t="n">
+        <x:f>H19/G19</x:f>
+        <x:v>0.925341212540797</x:v>
+      </x:c>
+      <x:c r="J19" s="24" t="n">
+        <x:v>0.283</x:v>
+      </x:c>
+      <x:c r="K19" s="24" t="n">
+        <x:v>0.313</x:v>
+      </x:c>
+      <x:c r="L19" s="24" t="n">
+        <x:f>K19/J19</x:f>
+        <x:v>1.1060070671378093</x:v>
+      </x:c>
+      <x:c r="M19" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N19" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O19" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P19" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q19" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R19" s="10" t="str">
+        <x:v>438f281aa1</x:v>
+      </x:c>
+      <x:c r="S19" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_152813_cpp-pubsub-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T19" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_153122_cpp-pubsub-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U19" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V19" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.60%; latency median ratio 1.07x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="29"/>
-      <x:c r="G20" s="27"/>
-      <x:c r="H20" s="27"/>
-      <x:c r="I20" s="23"/>
-      <x:c r="J20" s="25"/>
-      <x:c r="K20" s="25"/>
-      <x:c r="L20" s="25"/>
+      <x:c r="A20" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B20" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C20" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D20" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E20" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F20" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G20" s="26" t="n">
+        <x:v>20237.8</x:v>
+      </x:c>
+      <x:c r="H20" s="26" t="n">
+        <x:v>20248.6</x:v>
+      </x:c>
+      <x:c r="I20" s="22" t="n">
+        <x:f>H20/G20</x:f>
+        <x:v>1.0005336548439059</x:v>
+      </x:c>
+      <x:c r="J20" s="24" t="n">
+        <x:v>0.287</x:v>
+      </x:c>
+      <x:c r="K20" s="24" t="n">
+        <x:v>0.288</x:v>
+      </x:c>
+      <x:c r="L20" s="24" t="n">
+        <x:f>K20/J20</x:f>
+        <x:v>1.0034843205574913</x:v>
+      </x:c>
+      <x:c r="M20" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N20" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O20" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P20" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q20" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R20" s="10" t="str">
+        <x:v>438f281aa1</x:v>
+      </x:c>
+      <x:c r="S20" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_152813_cpp-pubsub-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T20" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_153122_cpp-pubsub-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U20" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V20" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.60%; latency median ratio 1.07x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="29"/>
-      <x:c r="G21" s="27"/>
-      <x:c r="H21" s="27"/>
-      <x:c r="I21" s="23"/>
-      <x:c r="J21" s="25"/>
-      <x:c r="K21" s="25"/>
-      <x:c r="L21" s="25"/>
+      <x:c r="A21" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B21" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C21" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D21" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E21" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F21" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G21" s="26" t="n">
+        <x:v>12946.2</x:v>
+      </x:c>
+      <x:c r="H21" s="26" t="n">
+        <x:v>11812.8</x:v>
+      </x:c>
+      <x:c r="I21" s="22" t="n">
+        <x:f>H21/G21</x:f>
+        <x:v>0.9124530750336005</x:v>
+      </x:c>
+      <x:c r="J21" s="24" t="n">
+        <x:v>0.302</x:v>
+      </x:c>
+      <x:c r="K21" s="24" t="n">
+        <x:v>0.332</x:v>
+      </x:c>
+      <x:c r="L21" s="24" t="n">
+        <x:f>K21/J21</x:f>
+        <x:v>1.099337748344371</x:v>
+      </x:c>
+      <x:c r="M21" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N21" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O21" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P21" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q21" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R21" s="10" t="str">
+        <x:v>438f281aa1</x:v>
+      </x:c>
+      <x:c r="S21" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_152813_cpp-pubsub-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T21" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_153122_cpp-pubsub-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U21" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V21" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.60%; latency median ratio 1.07x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="29"/>

</xml_diff>

<commit_message>
perf(cpp): record core 0.13.2 dealer baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R071dfbe321aa400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R6e0f77fa593f4825"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rdd21f9878edf4e2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Ra38e4e056bd64795"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R959246f3aad44eb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rfbd97069c90648c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rb646ddb837854f0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R197759f40dee4fad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>PAIR/tcp 미달 — candidate A retained; candidate B rejected</x:v>
+        <x:v>PAIR/tcp 미달 기록 완료; PUBSUB·DEALER_DEALER/tcp 통과</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -1951,58 +1951,424 @@
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="29"/>
-      <x:c r="G22" s="27"/>
-      <x:c r="H22" s="27"/>
-      <x:c r="I22" s="23"/>
-      <x:c r="J22" s="25"/>
-      <x:c r="K22" s="25"/>
-      <x:c r="L22" s="25"/>
+      <x:c r="A22" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B22" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C22" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D22" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E22" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F22" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G22" s="26" t="n">
+        <x:v>2484124.6</x:v>
+      </x:c>
+      <x:c r="H22" s="26" t="n">
+        <x:v>1977984.4</x:v>
+      </x:c>
+      <x:c r="I22" s="22" t="n">
+        <x:f>H22/G22</x:f>
+        <x:v>0.7962500753786665</x:v>
+      </x:c>
+      <x:c r="J22" s="24" t="n">
+        <x:v>0.215</x:v>
+      </x:c>
+      <x:c r="K22" s="24" t="n">
+        <x:v>0.169</x:v>
+      </x:c>
+      <x:c r="L22" s="24" t="n">
+        <x:f>K22/J22</x:f>
+        <x:v>0.7860465116279071</x:v>
+      </x:c>
+      <x:c r="M22" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N22" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O22" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P22" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q22" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R22" s="10" t="str">
+        <x:v>7321518d22</x:v>
+      </x:c>
+      <x:c r="S22" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_160956_cpp-dealer-dealer-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T22" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_161237_cpp-dealer-dealer-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U22" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V22" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 86.25%; latency median ratio 1.20x; pass. 64B and 64KiB are individual outliers below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="29"/>
-      <x:c r="G23" s="27"/>
-      <x:c r="H23" s="27"/>
-      <x:c r="I23" s="23"/>
-      <x:c r="J23" s="25"/>
-      <x:c r="K23" s="25"/>
-      <x:c r="L23" s="25"/>
+      <x:c r="A23" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B23" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C23" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D23" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E23" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F23" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G23" s="26" t="n">
+        <x:v>1382673.2</x:v>
+      </x:c>
+      <x:c r="H23" s="26" t="n">
+        <x:v>1339006.4</x:v>
+      </x:c>
+      <x:c r="I23" s="22" t="n">
+        <x:f>H23/G23</x:f>
+        <x:v>0.9684185677425439</x:v>
+      </x:c>
+      <x:c r="J23" s="24" t="n">
+        <x:v>1.211</x:v>
+      </x:c>
+      <x:c r="K23" s="24" t="n">
+        <x:v>1.269</x:v>
+      </x:c>
+      <x:c r="L23" s="24" t="n">
+        <x:f>K23/J23</x:f>
+        <x:v>1.0478943022295621</x:v>
+      </x:c>
+      <x:c r="M23" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N23" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O23" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P23" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q23" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R23" s="10" t="str">
+        <x:v>7321518d22</x:v>
+      </x:c>
+      <x:c r="S23" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_160956_cpp-dealer-dealer-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T23" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_161237_cpp-dealer-dealer-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U23" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V23" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 86.25%; latency median ratio 1.20x; pass. 64B and 64KiB are individual outliers below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="29"/>
-      <x:c r="G24" s="27"/>
-      <x:c r="H24" s="27"/>
-      <x:c r="I24" s="23"/>
-      <x:c r="J24" s="25"/>
-      <x:c r="K24" s="25"/>
-      <x:c r="L24" s="25"/>
+      <x:c r="A24" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B24" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C24" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D24" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E24" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F24" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G24" s="26" t="n">
+        <x:v>585600</x:v>
+      </x:c>
+      <x:c r="H24" s="26" t="n">
+        <x:v>543508.8</x:v>
+      </x:c>
+      <x:c r="I24" s="22" t="n">
+        <x:f>H24/G24</x:f>
+        <x:v>0.9281229508196722</x:v>
+      </x:c>
+      <x:c r="J24" s="24" t="n">
+        <x:v>0.827</x:v>
+      </x:c>
+      <x:c r="K24" s="24" t="n">
+        <x:v>0.885</x:v>
+      </x:c>
+      <x:c r="L24" s="24" t="n">
+        <x:f>K24/J24</x:f>
+        <x:v>1.0701330108827087</x:v>
+      </x:c>
+      <x:c r="M24" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N24" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O24" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P24" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q24" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R24" s="10" t="str">
+        <x:v>7321518d22</x:v>
+      </x:c>
+      <x:c r="S24" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_160956_cpp-dealer-dealer-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T24" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_161237_cpp-dealer-dealer-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U24" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V24" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 86.25%; latency median ratio 1.20x; pass. 64B and 64KiB are individual outliers below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="29"/>
-      <x:c r="G25" s="27"/>
-      <x:c r="H25" s="27"/>
-      <x:c r="I25" s="23"/>
-      <x:c r="J25" s="25"/>
-      <x:c r="K25" s="25"/>
-      <x:c r="L25" s="25"/>
+      <x:c r="A25" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B25" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C25" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D25" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E25" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F25" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G25" s="26" t="n">
+        <x:v>33875.8</x:v>
+      </x:c>
+      <x:c r="H25" s="26" t="n">
+        <x:v>26739.4</x:v>
+      </x:c>
+      <x:c r="I25" s="22" t="n">
+        <x:f>H25/G25</x:f>
+        <x:v>0.7893363403963891</x:v>
+      </x:c>
+      <x:c r="J25" s="24" t="n">
+        <x:v>0.29</x:v>
+      </x:c>
+      <x:c r="K25" s="24" t="n">
+        <x:v>0.387</x:v>
+      </x:c>
+      <x:c r="L25" s="24" t="n">
+        <x:f>K25/J25</x:f>
+        <x:v>1.3344827586206898</x:v>
+      </x:c>
+      <x:c r="M25" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N25" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O25" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P25" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q25" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R25" s="10" t="str">
+        <x:v>7321518d22</x:v>
+      </x:c>
+      <x:c r="S25" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_160956_cpp-dealer-dealer-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T25" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_161237_cpp-dealer-dealer-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U25" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V25" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 86.25%; latency median ratio 1.20x; pass. 64B and 64KiB are individual outliers below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="29"/>
-      <x:c r="G26" s="27"/>
-      <x:c r="H26" s="27"/>
-      <x:c r="I26" s="23"/>
-      <x:c r="J26" s="25"/>
-      <x:c r="K26" s="25"/>
-      <x:c r="L26" s="25"/>
+      <x:c r="A26" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B26" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C26" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D26" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E26" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F26" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G26" s="26" t="n">
+        <x:v>22519.8</x:v>
+      </x:c>
+      <x:c r="H26" s="26" t="n">
+        <x:v>18562.4</x:v>
+      </x:c>
+      <x:c r="I26" s="22" t="n">
+        <x:f>H26/G26</x:f>
+        <x:v>0.8242701977815079</x:v>
+      </x:c>
+      <x:c r="J26" s="24" t="n">
+        <x:v>0.292</x:v>
+      </x:c>
+      <x:c r="K26" s="24" t="n">
+        <x:v>0.368</x:v>
+      </x:c>
+      <x:c r="L26" s="24" t="n">
+        <x:f>K26/J26</x:f>
+        <x:v>1.2602739726027399</x:v>
+      </x:c>
+      <x:c r="M26" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N26" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O26" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P26" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q26" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R26" s="10" t="str">
+        <x:v>7321518d22</x:v>
+      </x:c>
+      <x:c r="S26" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_160956_cpp-dealer-dealer-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T26" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_161237_cpp-dealer-dealer-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U26" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V26" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 86.25%; latency median ratio 1.20x; pass. 64B and 64KiB are individual outliers below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="29"/>
-      <x:c r="G27" s="27"/>
-      <x:c r="H27" s="27"/>
-      <x:c r="I27" s="23"/>
-      <x:c r="J27" s="25"/>
-      <x:c r="K27" s="25"/>
-      <x:c r="L27" s="25"/>
+      <x:c r="A27" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B27" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C27" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D27" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E27" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F27" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G27" s="26" t="n">
+        <x:v>13147</x:v>
+      </x:c>
+      <x:c r="H27" s="26" t="n">
+        <x:v>11420.6</x:v>
+      </x:c>
+      <x:c r="I27" s="22" t="n">
+        <x:f>H27/G27</x:f>
+        <x:v>0.8686848710732487</x:v>
+      </x:c>
+      <x:c r="J27" s="24" t="n">
+        <x:v>0.311</x:v>
+      </x:c>
+      <x:c r="K27" s="24" t="n">
+        <x:v>0.356</x:v>
+      </x:c>
+      <x:c r="L27" s="24" t="n">
+        <x:f>K27/J27</x:f>
+        <x:v>1.1446945337620578</x:v>
+      </x:c>
+      <x:c r="M27" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N27" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O27" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P27" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q27" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R27" s="10" t="str">
+        <x:v>7321518d22</x:v>
+      </x:c>
+      <x:c r="S27" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_160956_cpp-dealer-dealer-tcp-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T27" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_161237_cpp-dealer-dealer-tcp-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U27" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V27" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 86.25%; latency median ratio 1.20x; pass. 64B and 64KiB are individual outliers below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="29"/>

</xml_diff>

<commit_message>
perf(cpp): record core 0.13.2 dealer router baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R959246f3aad44eb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rfbd97069c90648c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rb646ddb837854f0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R197759f40dee4fad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7437273c10c24b9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R6ecdc0f4db674e2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R8d45f850a8fc4f72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Ra71173b38b3d44ea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>PAIR/tcp 미달 기록 완료; PUBSUB·DEALER_DEALER/tcp 통과</x:v>
+        <x:v>PAIR/tcp 미달 기록 완료; PUBSUB·DEALER_DEALER·DEALER_ROUTER/tcp 통과</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -2371,58 +2371,424 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="29"/>
-      <x:c r="G28" s="27"/>
-      <x:c r="H28" s="27"/>
-      <x:c r="I28" s="23"/>
-      <x:c r="J28" s="25"/>
-      <x:c r="K28" s="25"/>
-      <x:c r="L28" s="25"/>
+      <x:c r="A28" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B28" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C28" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D28" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E28" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F28" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G28" s="26" t="n">
+        <x:v>2513011.4</x:v>
+      </x:c>
+      <x:c r="H28" s="26" t="n">
+        <x:v>1957767.6</x:v>
+      </x:c>
+      <x:c r="I28" s="22" t="n">
+        <x:f>H28/G28</x:f>
+        <x:v>0.7790524149631793</x:v>
+      </x:c>
+      <x:c r="J28" s="24" t="n">
+        <x:v>0.272</x:v>
+      </x:c>
+      <x:c r="K28" s="24" t="n">
+        <x:v>0.246</x:v>
+      </x:c>
+      <x:c r="L28" s="24" t="n">
+        <x:f>K28/J28</x:f>
+        <x:v>0.9044117647058822</x:v>
+      </x:c>
+      <x:c r="M28" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N28" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O28" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P28" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q28" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R28" s="10" t="str">
+        <x:v>1b55529575</x:v>
+      </x:c>
+      <x:c r="S28" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_161948_cpp-dealer-router-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T28" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_162125_cpp-dealer-router-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U28" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V28" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 89.38%; latency median ratio 1.05x; pass. 64B and 64KiB are individual outliers below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="29"/>
-      <x:c r="G29" s="27"/>
-      <x:c r="H29" s="27"/>
-      <x:c r="I29" s="23"/>
-      <x:c r="J29" s="25"/>
-      <x:c r="K29" s="25"/>
-      <x:c r="L29" s="25"/>
+      <x:c r="A29" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B29" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C29" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D29" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E29" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F29" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G29" s="26" t="n">
+        <x:v>1374500</x:v>
+      </x:c>
+      <x:c r="H29" s="26" t="n">
+        <x:v>1376774.2</x:v>
+      </x:c>
+      <x:c r="I29" s="22" t="n">
+        <x:f>H29/G29</x:f>
+        <x:v>1.0016545652964715</x:v>
+      </x:c>
+      <x:c r="J29" s="24" t="n">
+        <x:v>1.233</x:v>
+      </x:c>
+      <x:c r="K29" s="24" t="n">
+        <x:v>1.265</x:v>
+      </x:c>
+      <x:c r="L29" s="24" t="n">
+        <x:f>K29/J29</x:f>
+        <x:v>1.0259529602595294</x:v>
+      </x:c>
+      <x:c r="M29" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N29" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O29" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P29" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q29" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R29" s="10" t="str">
+        <x:v>1b55529575</x:v>
+      </x:c>
+      <x:c r="S29" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_161948_cpp-dealer-router-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T29" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_162125_cpp-dealer-router-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U29" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V29" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 89.38%; latency median ratio 1.05x; pass. 64B and 64KiB are individual outliers below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="29"/>
-      <x:c r="G30" s="27"/>
-      <x:c r="H30" s="27"/>
-      <x:c r="I30" s="23"/>
-      <x:c r="J30" s="25"/>
-      <x:c r="K30" s="25"/>
-      <x:c r="L30" s="25"/>
+      <x:c r="A30" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B30" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C30" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D30" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E30" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F30" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G30" s="26" t="n">
+        <x:v>599229.2</x:v>
+      </x:c>
+      <x:c r="H30" s="26" t="n">
+        <x:v>595717.4</x:v>
+      </x:c>
+      <x:c r="I30" s="22" t="n">
+        <x:f>H30/G30</x:f>
+        <x:v>0.9941394711739683</x:v>
+      </x:c>
+      <x:c r="J30" s="24" t="n">
+        <x:v>0.807</x:v>
+      </x:c>
+      <x:c r="K30" s="24" t="n">
+        <x:v>0.811</x:v>
+      </x:c>
+      <x:c r="L30" s="24" t="n">
+        <x:f>K30/J30</x:f>
+        <x:v>1.0049566294919454</x:v>
+      </x:c>
+      <x:c r="M30" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N30" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O30" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P30" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q30" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R30" s="10" t="str">
+        <x:v>1b55529575</x:v>
+      </x:c>
+      <x:c r="S30" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_161948_cpp-dealer-router-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T30" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_162125_cpp-dealer-router-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U30" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V30" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 89.38%; latency median ratio 1.05x; pass. 64B and 64KiB are individual outliers below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="29"/>
-      <x:c r="G31" s="27"/>
-      <x:c r="H31" s="27"/>
-      <x:c r="I31" s="23"/>
-      <x:c r="J31" s="25"/>
-      <x:c r="K31" s="25"/>
-      <x:c r="L31" s="25"/>
+      <x:c r="A31" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B31" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C31" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D31" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E31" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F31" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G31" s="26" t="n">
+        <x:v>31311.2</x:v>
+      </x:c>
+      <x:c r="H31" s="26" t="n">
+        <x:v>24195.2</x:v>
+      </x:c>
+      <x:c r="I31" s="22" t="n">
+        <x:f>H31/G31</x:f>
+        <x:v>0.7727330795370346</x:v>
+      </x:c>
+      <x:c r="J31" s="24" t="n">
+        <x:v>0.343</x:v>
+      </x:c>
+      <x:c r="K31" s="24" t="n">
+        <x:v>0.459</x:v>
+      </x:c>
+      <x:c r="L31" s="24" t="n">
+        <x:f>K31/J31</x:f>
+        <x:v>1.3381924198250728</x:v>
+      </x:c>
+      <x:c r="M31" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N31" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O31" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P31" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q31" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R31" s="10" t="str">
+        <x:v>1b55529575</x:v>
+      </x:c>
+      <x:c r="S31" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_161948_cpp-dealer-router-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T31" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_162125_cpp-dealer-router-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U31" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V31" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 89.38%; latency median ratio 1.05x; pass. 64B and 64KiB are individual outliers below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="29"/>
-      <x:c r="G32" s="27"/>
-      <x:c r="H32" s="27"/>
-      <x:c r="I32" s="23"/>
-      <x:c r="J32" s="25"/>
-      <x:c r="K32" s="25"/>
-      <x:c r="L32" s="25"/>
+      <x:c r="A32" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B32" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C32" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D32" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E32" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F32" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G32" s="26" t="n">
+        <x:v>22168.4</x:v>
+      </x:c>
+      <x:c r="H32" s="26" t="n">
+        <x:v>19714.6</x:v>
+      </x:c>
+      <x:c r="I32" s="22" t="n">
+        <x:f>H32/G32</x:f>
+        <x:v>0.8893109110265061</x:v>
+      </x:c>
+      <x:c r="J32" s="24" t="n">
+        <x:v>0.28</x:v>
+      </x:c>
+      <x:c r="K32" s="24" t="n">
+        <x:v>0.317</x:v>
+      </x:c>
+      <x:c r="L32" s="24" t="n">
+        <x:f>K32/J32</x:f>
+        <x:v>1.1321428571428571</x:v>
+      </x:c>
+      <x:c r="M32" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N32" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O32" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P32" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q32" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R32" s="10" t="str">
+        <x:v>1b55529575</x:v>
+      </x:c>
+      <x:c r="S32" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_161948_cpp-dealer-router-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T32" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_162125_cpp-dealer-router-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U32" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V32" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 89.38%; latency median ratio 1.05x; pass. 64B and 64KiB are individual outliers below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="29"/>
-      <x:c r="G33" s="27"/>
-      <x:c r="H33" s="27"/>
-      <x:c r="I33" s="23"/>
-      <x:c r="J33" s="25"/>
-      <x:c r="K33" s="25"/>
-      <x:c r="L33" s="25"/>
+      <x:c r="A33" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B33" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C33" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D33" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E33" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F33" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G33" s="26" t="n">
+        <x:v>13869.8</x:v>
+      </x:c>
+      <x:c r="H33" s="26" t="n">
+        <x:v>12846.2</x:v>
+      </x:c>
+      <x:c r="I33" s="22" t="n">
+        <x:f>H33/G33</x:f>
+        <x:v>0.9261993684119455</x:v>
+      </x:c>
+      <x:c r="J33" s="24" t="n">
+        <x:v>0.295</x:v>
+      </x:c>
+      <x:c r="K33" s="24" t="n">
+        <x:v>0.317</x:v>
+      </x:c>
+      <x:c r="L33" s="24" t="n">
+        <x:f>K33/J33</x:f>
+        <x:v>1.0745762711864408</x:v>
+      </x:c>
+      <x:c r="M33" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N33" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O33" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P33" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q33" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R33" s="10" t="str">
+        <x:v>1b55529575</x:v>
+      </x:c>
+      <x:c r="S33" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_161948_cpp-dealer-router-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T33" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_162125_cpp-dealer-router-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U33" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V33" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 89.38%; latency median ratio 1.05x; pass. 64B and 64KiB are individual outliers below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="29"/>

</xml_diff>

<commit_message>
perf(cpp): streamline single part requests
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7437273c10c24b9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R6ecdc0f4db674e2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R8d45f850a8fc4f72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Ra71173b38b3d44ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb69a5c06fd824a81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R3cfa15dd51234ce6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rc137408284834776"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R42117525f7df450c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>PAIR/tcp 미달 기록 완료; PUBSUB·DEALER_DEALER·DEALER_ROUTER/tcp 통과</x:v>
+        <x:v>PAIR·DEALER_ROUTER_REQREP/tcp 미달 기록 완료; 3개 tcp 패턴 통과</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -2791,166 +2791,1264 @@
       </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="29"/>
-      <x:c r="G34" s="27"/>
-      <x:c r="H34" s="27"/>
-      <x:c r="I34" s="23"/>
-      <x:c r="J34" s="25"/>
-      <x:c r="K34" s="25"/>
-      <x:c r="L34" s="25"/>
+      <x:c r="A34" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B34" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C34" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D34" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E34" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F34" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G34" s="26" t="n">
+        <x:v>162087</x:v>
+      </x:c>
+      <x:c r="H34" s="26" t="n">
+        <x:v>88846</x:v>
+      </x:c>
+      <x:c r="I34" s="22" t="n">
+        <x:f>H34/G34</x:f>
+        <x:v>0.5481377285038281</x:v>
+      </x:c>
+      <x:c r="J34" s="24" t="n">
+        <x:v>0.275</x:v>
+      </x:c>
+      <x:c r="K34" s="24" t="n">
+        <x:v>0.567</x:v>
+      </x:c>
+      <x:c r="L34" s="24" t="n">
+        <x:f>K34/J34</x:f>
+        <x:v>2.0618181818181816</x:v>
+      </x:c>
+      <x:c r="M34" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N34" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O34" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P34" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q34" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R34" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S34" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T34" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_162635_cpp-dealer-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U34" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V34" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 66.57%; latency median ratio 1.70x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="29"/>
-      <x:c r="G35" s="27"/>
-      <x:c r="H35" s="27"/>
-      <x:c r="I35" s="23"/>
-      <x:c r="J35" s="25"/>
-      <x:c r="K35" s="25"/>
-      <x:c r="L35" s="25"/>
+      <x:c r="A35" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B35" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C35" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D35" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E35" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F35" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G35" s="26" t="n">
+        <x:v>156086.8</x:v>
+      </x:c>
+      <x:c r="H35" s="26" t="n">
+        <x:v>87923.2</x:v>
+      </x:c>
+      <x:c r="I35" s="22" t="n">
+        <x:f>H35/G35</x:f>
+        <x:v>0.563296832275375</x:v>
+      </x:c>
+      <x:c r="J35" s="24" t="n">
+        <x:v>0.281</x:v>
+      </x:c>
+      <x:c r="K35" s="24" t="n">
+        <x:v>0.583</x:v>
+      </x:c>
+      <x:c r="L35" s="24" t="n">
+        <x:f>K35/J35</x:f>
+        <x:v>2.074733096085409</x:v>
+      </x:c>
+      <x:c r="M35" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N35" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O35" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P35" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q35" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R35" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S35" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T35" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_162635_cpp-dealer-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U35" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V35" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 66.57%; latency median ratio 1.70x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="29"/>
-      <x:c r="G36" s="27"/>
-      <x:c r="H36" s="27"/>
-      <x:c r="I36" s="23"/>
-      <x:c r="J36" s="25"/>
-      <x:c r="K36" s="25"/>
-      <x:c r="L36" s="25"/>
+      <x:c r="A36" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B36" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C36" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D36" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E36" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F36" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G36" s="26" t="n">
+        <x:v>144801.8</x:v>
+      </x:c>
+      <x:c r="H36" s="26" t="n">
+        <x:v>56953.2</x:v>
+      </x:c>
+      <x:c r="I36" s="22" t="n">
+        <x:f>H36/G36</x:f>
+        <x:v>0.39331831510381776</x:v>
+      </x:c>
+      <x:c r="J36" s="24" t="n">
+        <x:v>0.373</x:v>
+      </x:c>
+      <x:c r="K36" s="24" t="n">
+        <x:v>1.041</x:v>
+      </x:c>
+      <x:c r="L36" s="24" t="n">
+        <x:f>K36/J36</x:f>
+        <x:v>2.7908847184986594</x:v>
+      </x:c>
+      <x:c r="M36" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N36" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O36" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P36" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q36" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R36" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S36" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T36" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_162635_cpp-dealer-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U36" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V36" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 66.57%; latency median ratio 1.70x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="29"/>
-      <x:c r="G37" s="27"/>
-      <x:c r="H37" s="27"/>
-      <x:c r="I37" s="23"/>
-      <x:c r="J37" s="25"/>
-      <x:c r="K37" s="25"/>
-      <x:c r="L37" s="25"/>
+      <x:c r="A37" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B37" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C37" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D37" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E37" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F37" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G37" s="26" t="n">
+        <x:v>15954</x:v>
+      </x:c>
+      <x:c r="H37" s="26" t="n">
+        <x:v>11757.4</x:v>
+      </x:c>
+      <x:c r="I37" s="22" t="n">
+        <x:f>H37/G37</x:f>
+        <x:v>0.7369562492164974</x:v>
+      </x:c>
+      <x:c r="J37" s="24" t="n">
+        <x:v>0.749</x:v>
+      </x:c>
+      <x:c r="K37" s="24" t="n">
+        <x:v>0.997</x:v>
+      </x:c>
+      <x:c r="L37" s="24" t="n">
+        <x:f>K37/J37</x:f>
+        <x:v>1.3311081441922563</x:v>
+      </x:c>
+      <x:c r="M37" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N37" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O37" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P37" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q37" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R37" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S37" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T37" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_162635_cpp-dealer-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U37" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V37" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 66.57%; latency median ratio 1.70x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="29"/>
-      <x:c r="G38" s="27"/>
-      <x:c r="H38" s="27"/>
-      <x:c r="I38" s="23"/>
-      <x:c r="J38" s="25"/>
-      <x:c r="K38" s="25"/>
-      <x:c r="L38" s="25"/>
+      <x:c r="A38" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B38" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C38" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D38" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E38" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F38" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G38" s="26" t="n">
+        <x:v>10823.2</x:v>
+      </x:c>
+      <x:c r="H38" s="26" t="n">
+        <x:v>9072.2</x:v>
+      </x:c>
+      <x:c r="I38" s="22" t="n">
+        <x:f>H38/G38</x:f>
+        <x:v>0.8382179022839825</x:v>
+      </x:c>
+      <x:c r="J38" s="24" t="n">
+        <x:v>0.548</x:v>
+      </x:c>
+      <x:c r="K38" s="24" t="n">
+        <x:v>0.638</x:v>
+      </x:c>
+      <x:c r="L38" s="24" t="n">
+        <x:f>K38/J38</x:f>
+        <x:v>1.1642335766423357</x:v>
+      </x:c>
+      <x:c r="M38" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N38" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O38" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P38" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q38" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R38" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S38" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T38" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_162635_cpp-dealer-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U38" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V38" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 66.57%; latency median ratio 1.70x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="29"/>
-      <x:c r="G39" s="27"/>
-      <x:c r="H39" s="27"/>
-      <x:c r="I39" s="23"/>
-      <x:c r="J39" s="25"/>
-      <x:c r="K39" s="25"/>
-      <x:c r="L39" s="25"/>
+      <x:c r="A39" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B39" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C39" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D39" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E39" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F39" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G39" s="26" t="n">
+        <x:v>6466</x:v>
+      </x:c>
+      <x:c r="H39" s="26" t="n">
+        <x:v>5912.4</x:v>
+      </x:c>
+      <x:c r="I39" s="22" t="n">
+        <x:f>H39/G39</x:f>
+        <x:v>0.914382926074853</x:v>
+      </x:c>
+      <x:c r="J39" s="24" t="n">
+        <x:v>0.459</x:v>
+      </x:c>
+      <x:c r="K39" s="24" t="n">
+        <x:v>0.482</x:v>
+      </x:c>
+      <x:c r="L39" s="24" t="n">
+        <x:f>K39/J39</x:f>
+        <x:v>1.0501089324618735</x:v>
+      </x:c>
+      <x:c r="M39" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N39" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O39" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P39" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q39" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R39" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S39" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T39" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_162635_cpp-dealer-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U39" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V39" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 66.57%; latency median ratio 1.70x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="29"/>
-      <x:c r="G40" s="27"/>
-      <x:c r="H40" s="27"/>
-      <x:c r="I40" s="23"/>
-      <x:c r="J40" s="25"/>
-      <x:c r="K40" s="25"/>
-      <x:c r="L40" s="25"/>
+      <x:c r="A40" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B40" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C40" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D40" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E40" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F40" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G40" s="26" t="n">
+        <x:v>162087</x:v>
+      </x:c>
+      <x:c r="H40" s="26" t="n">
+        <x:v>107145.2</x:v>
+      </x:c>
+      <x:c r="I40" s="22" t="n">
+        <x:f>H40/G40</x:f>
+        <x:v>0.6610351231128961</x:v>
+      </x:c>
+      <x:c r="J40" s="24" t="n">
+        <x:v>0.275</x:v>
+      </x:c>
+      <x:c r="K40" s="24" t="n">
+        <x:v>0.47</x:v>
+      </x:c>
+      <x:c r="L40" s="24" t="n">
+        <x:f>K40/J40</x:f>
+        <x:v>1.7090909090909088</x:v>
+      </x:c>
+      <x:c r="M40" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N40" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O40" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P40" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q40" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R40" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S40" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T40" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_163735_cpp-dealer-router-reqrep-tcp-local0132-candidate-a-safe-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U40" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V40" s="10" t="str">
+        <x:v>Candidate A final: throughput aggregate mean 67.53%; latency median ratio 1.53x; fail. Keep the safe single-part borrowed-view fast path.</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="29"/>
-      <x:c r="G41" s="27"/>
-      <x:c r="H41" s="27"/>
-      <x:c r="I41" s="23"/>
-      <x:c r="J41" s="25"/>
-      <x:c r="K41" s="25"/>
-      <x:c r="L41" s="25"/>
+      <x:c r="A41" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B41" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C41" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D41" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E41" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F41" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G41" s="26" t="n">
+        <x:v>156086.8</x:v>
+      </x:c>
+      <x:c r="H41" s="26" t="n">
+        <x:v>89164.4</x:v>
+      </x:c>
+      <x:c r="I41" s="22" t="n">
+        <x:f>H41/G41</x:f>
+        <x:v>0.5712488179653885</x:v>
+      </x:c>
+      <x:c r="J41" s="24" t="n">
+        <x:v>0.281</x:v>
+      </x:c>
+      <x:c r="K41" s="24" t="n">
+        <x:v>0.578</x:v>
+      </x:c>
+      <x:c r="L41" s="24" t="n">
+        <x:f>K41/J41</x:f>
+        <x:v>2.0569395017793592</x:v>
+      </x:c>
+      <x:c r="M41" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N41" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O41" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P41" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q41" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R41" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S41" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T41" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_163735_cpp-dealer-router-reqrep-tcp-local0132-candidate-a-safe-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U41" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V41" s="10" t="str">
+        <x:v>Candidate A final: throughput aggregate mean 67.53%; latency median ratio 1.53x; fail. Keep the safe single-part borrowed-view fast path.</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="29"/>
-      <x:c r="G42" s="27"/>
-      <x:c r="H42" s="27"/>
-      <x:c r="I42" s="23"/>
-      <x:c r="J42" s="25"/>
-      <x:c r="K42" s="25"/>
-      <x:c r="L42" s="25"/>
+      <x:c r="A42" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B42" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C42" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D42" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E42" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F42" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G42" s="26" t="n">
+        <x:v>144801.8</x:v>
+      </x:c>
+      <x:c r="H42" s="26" t="n">
+        <x:v>56149.4</x:v>
+      </x:c>
+      <x:c r="I42" s="22" t="n">
+        <x:f>H42/G42</x:f>
+        <x:v>0.38776727913603287</x:v>
+      </x:c>
+      <x:c r="J42" s="24" t="n">
+        <x:v>0.373</x:v>
+      </x:c>
+      <x:c r="K42" s="24" t="n">
+        <x:v>1.065</x:v>
+      </x:c>
+      <x:c r="L42" s="24" t="n">
+        <x:f>K42/J42</x:f>
+        <x:v>2.8552278820375334</x:v>
+      </x:c>
+      <x:c r="M42" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N42" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O42" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P42" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q42" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R42" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S42" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T42" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_163735_cpp-dealer-router-reqrep-tcp-local0132-candidate-a-safe-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U42" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V42" s="10" t="str">
+        <x:v>Candidate A final: throughput aggregate mean 67.53%; latency median ratio 1.53x; fail. Keep the safe single-part borrowed-view fast path.</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="29"/>
-      <x:c r="G43" s="27"/>
-      <x:c r="H43" s="27"/>
-      <x:c r="I43" s="23"/>
-      <x:c r="J43" s="25"/>
-      <x:c r="K43" s="25"/>
-      <x:c r="L43" s="25"/>
+      <x:c r="A43" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B43" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C43" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D43" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E43" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F43" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G43" s="26" t="n">
+        <x:v>15954</x:v>
+      </x:c>
+      <x:c r="H43" s="26" t="n">
+        <x:v>11532.4</x:v>
+      </x:c>
+      <x:c r="I43" s="22" t="n">
+        <x:f>H43/G43</x:f>
+        <x:v>0.7228532029585056</x:v>
+      </x:c>
+      <x:c r="J43" s="24" t="n">
+        <x:v>0.749</x:v>
+      </x:c>
+      <x:c r="K43" s="24" t="n">
+        <x:v>1.016</x:v>
+      </x:c>
+      <x:c r="L43" s="24" t="n">
+        <x:f>K43/J43</x:f>
+        <x:v>1.356475300400534</x:v>
+      </x:c>
+      <x:c r="M43" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N43" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O43" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P43" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q43" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R43" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S43" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T43" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_163735_cpp-dealer-router-reqrep-tcp-local0132-candidate-a-safe-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U43" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V43" s="10" t="str">
+        <x:v>Candidate A final: throughput aggregate mean 67.53%; latency median ratio 1.53x; fail. Keep the safe single-part borrowed-view fast path.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="29"/>
-      <x:c r="G44" s="27"/>
-      <x:c r="H44" s="27"/>
-      <x:c r="I44" s="23"/>
-      <x:c r="J44" s="25"/>
-      <x:c r="K44" s="25"/>
-      <x:c r="L44" s="25"/>
+      <x:c r="A44" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B44" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C44" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D44" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E44" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F44" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G44" s="26" t="n">
+        <x:v>10823.2</x:v>
+      </x:c>
+      <x:c r="H44" s="26" t="n">
+        <x:v>8697</x:v>
+      </x:c>
+      <x:c r="I44" s="22" t="n">
+        <x:f>H44/G44</x:f>
+        <x:v>0.8035516298322122</x:v>
+      </x:c>
+      <x:c r="J44" s="24" t="n">
+        <x:v>0.548</x:v>
+      </x:c>
+      <x:c r="K44" s="24" t="n">
+        <x:v>0.664</x:v>
+      </x:c>
+      <x:c r="L44" s="24" t="n">
+        <x:f>K44/J44</x:f>
+        <x:v>1.2116788321167884</x:v>
+      </x:c>
+      <x:c r="M44" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N44" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O44" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P44" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q44" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R44" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S44" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T44" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_163735_cpp-dealer-router-reqrep-tcp-local0132-candidate-a-safe-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U44" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V44" s="10" t="str">
+        <x:v>Candidate A final: throughput aggregate mean 67.53%; latency median ratio 1.53x; fail. Keep the safe single-part borrowed-view fast path.</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="29"/>
-      <x:c r="G45" s="27"/>
-      <x:c r="H45" s="27"/>
-      <x:c r="I45" s="23"/>
-      <x:c r="J45" s="25"/>
-      <x:c r="K45" s="25"/>
-      <x:c r="L45" s="25"/>
+      <x:c r="A45" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B45" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C45" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D45" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E45" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F45" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G45" s="26" t="n">
+        <x:v>6466</x:v>
+      </x:c>
+      <x:c r="H45" s="26" t="n">
+        <x:v>5854.4</x:v>
+      </x:c>
+      <x:c r="I45" s="22" t="n">
+        <x:f>H45/G45</x:f>
+        <x:v>0.9054129291679553</x:v>
+      </x:c>
+      <x:c r="J45" s="24" t="n">
+        <x:v>0.459</x:v>
+      </x:c>
+      <x:c r="K45" s="24" t="n">
+        <x:v>0.488</x:v>
+      </x:c>
+      <x:c r="L45" s="24" t="n">
+        <x:f>K45/J45</x:f>
+        <x:v>1.06318082788671</x:v>
+      </x:c>
+      <x:c r="M45" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N45" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O45" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P45" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q45" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R45" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S45" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T45" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_163735_cpp-dealer-router-reqrep-tcp-local0132-candidate-a-safe-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U45" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V45" s="10" t="str">
+        <x:v>Candidate A final: throughput aggregate mean 67.53%; latency median ratio 1.53x; fail. Keep the safe single-part borrowed-view fast path.</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="29"/>
-      <x:c r="G46" s="27"/>
-      <x:c r="H46" s="27"/>
-      <x:c r="I46" s="23"/>
-      <x:c r="J46" s="25"/>
-      <x:c r="K46" s="25"/>
-      <x:c r="L46" s="25"/>
+      <x:c r="A46" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B46" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C46" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D46" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E46" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F46" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G46" s="26" t="n">
+        <x:v>162087</x:v>
+      </x:c>
+      <x:c r="H46" s="26" t="n">
+        <x:v>107039.8</x:v>
+      </x:c>
+      <x:c r="I46" s="22" t="n">
+        <x:f>H46/G46</x:f>
+        <x:v>0.660384855046981</x:v>
+      </x:c>
+      <x:c r="J46" s="24" t="n">
+        <x:v>0.275</x:v>
+      </x:c>
+      <x:c r="K46" s="24" t="n">
+        <x:v>0.468</x:v>
+      </x:c>
+      <x:c r="L46" s="24" t="n">
+        <x:f>K46/J46</x:f>
+        <x:v>1.7018181818181817</x:v>
+      </x:c>
+      <x:c r="M46" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N46" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O46" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P46" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q46" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R46" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S46" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T46" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_164045_cpp-dealer-router-reqrep-tcp-local0132-candidate-b-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U46" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V46" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 63.87%; latency median ratio 1.70x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" s="29"/>
-      <x:c r="G47" s="27"/>
-      <x:c r="H47" s="27"/>
-      <x:c r="I47" s="23"/>
-      <x:c r="J47" s="25"/>
-      <x:c r="K47" s="25"/>
-      <x:c r="L47" s="25"/>
+      <x:c r="A47" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B47" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C47" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D47" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E47" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F47" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G47" s="26" t="n">
+        <x:v>156086.8</x:v>
+      </x:c>
+      <x:c r="H47" s="26" t="n">
+        <x:v>83863.8</x:v>
+      </x:c>
+      <x:c r="I47" s="22" t="n">
+        <x:f>H47/G47</x:f>
+        <x:v>0.5372895081454678</x:v>
+      </x:c>
+      <x:c r="J47" s="24" t="n">
+        <x:v>0.281</x:v>
+      </x:c>
+      <x:c r="K47" s="24" t="n">
+        <x:v>0.606</x:v>
+      </x:c>
+      <x:c r="L47" s="24" t="n">
+        <x:f>K47/J47</x:f>
+        <x:v>2.1565836298932384</x:v>
+      </x:c>
+      <x:c r="M47" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N47" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O47" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P47" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q47" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R47" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S47" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T47" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_164045_cpp-dealer-router-reqrep-tcp-local0132-candidate-b-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U47" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V47" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 63.87%; latency median ratio 1.70x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="29"/>
-      <x:c r="G48" s="27"/>
-      <x:c r="H48" s="27"/>
-      <x:c r="I48" s="23"/>
-      <x:c r="J48" s="25"/>
-      <x:c r="K48" s="25"/>
-      <x:c r="L48" s="25"/>
+      <x:c r="A48" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B48" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C48" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D48" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E48" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F48" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G48" s="26" t="n">
+        <x:v>144801.8</x:v>
+      </x:c>
+      <x:c r="H48" s="26" t="n">
+        <x:v>55502.4</x:v>
+      </x:c>
+      <x:c r="I48" s="22" t="n">
+        <x:f>H48/G48</x:f>
+        <x:v>0.3832991026354645</x:v>
+      </x:c>
+      <x:c r="J48" s="24" t="n">
+        <x:v>0.373</x:v>
+      </x:c>
+      <x:c r="K48" s="24" t="n">
+        <x:v>1.071</x:v>
+      </x:c>
+      <x:c r="L48" s="24" t="n">
+        <x:f>K48/J48</x:f>
+        <x:v>2.871313672922252</x:v>
+      </x:c>
+      <x:c r="M48" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N48" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O48" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P48" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q48" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R48" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S48" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T48" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_164045_cpp-dealer-router-reqrep-tcp-local0132-candidate-b-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U48" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V48" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 63.87%; latency median ratio 1.70x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="29"/>
-      <x:c r="G49" s="27"/>
-      <x:c r="H49" s="27"/>
-      <x:c r="I49" s="23"/>
-      <x:c r="J49" s="25"/>
-      <x:c r="K49" s="25"/>
-      <x:c r="L49" s="25"/>
+      <x:c r="A49" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B49" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C49" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D49" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E49" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F49" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G49" s="26" t="n">
+        <x:v>15954</x:v>
+      </x:c>
+      <x:c r="H49" s="26" t="n">
+        <x:v>11425.2</x:v>
+      </x:c>
+      <x:c r="I49" s="22" t="n">
+        <x:f>H49/G49</x:f>
+        <x:v>0.7161338849191425</x:v>
+      </x:c>
+      <x:c r="J49" s="24" t="n">
+        <x:v>0.749</x:v>
+      </x:c>
+      <x:c r="K49" s="24" t="n">
+        <x:v>1.025</x:v>
+      </x:c>
+      <x:c r="L49" s="24" t="n">
+        <x:f>K49/J49</x:f>
+        <x:v>1.3684913217623498</x:v>
+      </x:c>
+      <x:c r="M49" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N49" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O49" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P49" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q49" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R49" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S49" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T49" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_164045_cpp-dealer-router-reqrep-tcp-local0132-candidate-b-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U49" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V49" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 63.87%; latency median ratio 1.70x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="29"/>
-      <x:c r="G50" s="27"/>
-      <x:c r="H50" s="27"/>
-      <x:c r="I50" s="23"/>
-      <x:c r="J50" s="25"/>
-      <x:c r="K50" s="25"/>
-      <x:c r="L50" s="25"/>
+      <x:c r="A50" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B50" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C50" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D50" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E50" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F50" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G50" s="26" t="n">
+        <x:v>10823.2</x:v>
+      </x:c>
+      <x:c r="H50" s="26" t="n">
+        <x:v>8045.6</x:v>
+      </x:c>
+      <x:c r="I50" s="22" t="n">
+        <x:f>H50/G50</x:f>
+        <x:v>0.7433661024465962</x:v>
+      </x:c>
+      <x:c r="J50" s="24" t="n">
+        <x:v>0.548</x:v>
+      </x:c>
+      <x:c r="K50" s="24" t="n">
+        <x:v>0.717</x:v>
+      </x:c>
+      <x:c r="L50" s="24" t="n">
+        <x:f>K50/J50</x:f>
+        <x:v>1.3083941605839415</x:v>
+      </x:c>
+      <x:c r="M50" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N50" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O50" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P50" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q50" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R50" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S50" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T50" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_164045_cpp-dealer-router-reqrep-tcp-local0132-candidate-b-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U50" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V50" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 63.87%; latency median ratio 1.70x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="29"/>
-      <x:c r="G51" s="27"/>
-      <x:c r="H51" s="27"/>
-      <x:c r="I51" s="23"/>
-      <x:c r="J51" s="25"/>
-      <x:c r="K51" s="25"/>
-      <x:c r="L51" s="25"/>
+      <x:c r="A51" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B51" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C51" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D51" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E51" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F51" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G51" s="26" t="n">
+        <x:v>6466</x:v>
+      </x:c>
+      <x:c r="H51" s="26" t="n">
+        <x:v>5118.4</x:v>
+      </x:c>
+      <x:c r="I51" s="22" t="n">
+        <x:f>H51/G51</x:f>
+        <x:v>0.7915867615218063</x:v>
+      </x:c>
+      <x:c r="J51" s="24" t="n">
+        <x:v>0.459</x:v>
+      </x:c>
+      <x:c r="K51" s="24" t="n">
+        <x:v>0.556</x:v>
+      </x:c>
+      <x:c r="L51" s="24" t="n">
+        <x:f>K51/J51</x:f>
+        <x:v>1.2113289760348585</x:v>
+      </x:c>
+      <x:c r="M51" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N51" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O51" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P51" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q51" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R51" s="10" t="str">
+        <x:v>d1184f7d0a</x:v>
+      </x:c>
+      <x:c r="S51" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_162455_cpp-dealer-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T51" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_164045_cpp-dealer-router-reqrep-tcp-local0132-candidate-b-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U51" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V51" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 63.87%; latency median ratio 1.70x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="29"/>
@@ -6267,12 +7365,92 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="L6" s="23"/>
-      <x:c r="M6" s="23"/>
+      <x:c r="A6" s="10" t="str">
+        <x:v>2026-08-25 16:37</x:v>
+      </x:c>
+      <x:c r="B6" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C6" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D6" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F6" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G6" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H6" s="10" t="str">
+        <x:v>Submit one shallow borrowed native view for the public single-part request; retain generic multipart path.</x:v>
+      </x:c>
+      <x:c r="I6" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J6" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_162635_cpp-dealer-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K6" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_163735_cpp-dealer-router-reqrep-tcp-local0132-candidate-a-safe-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L6" s="22" t="n">
+        <x:v>0.666</x:v>
+      </x:c>
+      <x:c r="M6" s="22" t="n">
+        <x:v>0.675</x:v>
+      </x:c>
+      <x:c r="N6" s="10" t="str">
+        <x:v>Keep: aggregate +0.96%p; failure keeps lvalue ownership and success closes the original shared reference. POSDDD: separates single/multipart responsibility; target remains 미달.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="L7" s="23"/>
-      <x:c r="M7" s="23"/>
+      <x:c r="A7" s="10" t="str">
+        <x:v>2026-08-25 16:40</x:v>
+      </x:c>
+      <x:c r="B7" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C7" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D7" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E7" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F7" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G7" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H7" s="10" t="str">
+        <x:v>Direct async completion sink; remove bridge allocation, mutex and staging only from async().</x:v>
+      </x:c>
+      <x:c r="I7" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J7" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_163735_cpp-dealer-router-reqrep-tcp-local0132-candidate-a-safe-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K7" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_164045_cpp-dealer-router-reqrep-tcp-local0132-candidate-b-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L7" s="22" t="n">
+        <x:v>0.675</x:v>
+      </x:c>
+      <x:c r="M7" s="22" t="n">
+        <x:v>0.639</x:v>
+      </x:c>
+      <x:c r="N7" s="10" t="str">
+        <x:v>REJECT: aggregate regressed. Removed to avoid new complexity; callback and blocking APIs were never changed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="L8" s="23"/>

</xml_diff>

<commit_message>
perf(cpp): record core 0.13.2 router baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb69a5c06fd824a81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R3cfa15dd51234ce6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rc137408284834776"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R42117525f7df450c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R571fd9b91f3d44ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R5e18b7c8246e40c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rbd7ca3a637214a77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R0ed1f7d0b48149b0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>PAIR·DEALER_ROUTER_REQREP/tcp 미달 기록 완료; 3개 tcp 패턴 통과</x:v>
+        <x:v>PAIR·DEALER_ROUTER_REQREP/tcp 미달 기록 완료; 4개 tcp 패턴 통과</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -4051,58 +4051,424 @@
       </x:c>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="29"/>
-      <x:c r="G52" s="27"/>
-      <x:c r="H52" s="27"/>
-      <x:c r="I52" s="23"/>
-      <x:c r="J52" s="25"/>
-      <x:c r="K52" s="25"/>
-      <x:c r="L52" s="25"/>
+      <x:c r="A52" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B52" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C52" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D52" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E52" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F52" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G52" s="26" t="n">
+        <x:v>2415454</x:v>
+      </x:c>
+      <x:c r="H52" s="26" t="n">
+        <x:v>1993132.8</x:v>
+      </x:c>
+      <x:c r="I52" s="22" t="n">
+        <x:f>H52/G52</x:f>
+        <x:v>0.825158665824313</x:v>
+      </x:c>
+      <x:c r="J52" s="24" t="n">
+        <x:v>0.613</x:v>
+      </x:c>
+      <x:c r="K52" s="24" t="n">
+        <x:v>0.243</x:v>
+      </x:c>
+      <x:c r="L52" s="24" t="n">
+        <x:f>K52/J52</x:f>
+        <x:v>0.3964110929853181</x:v>
+      </x:c>
+      <x:c r="M52" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N52" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O52" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P52" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q52" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R52" s="10" t="str">
+        <x:v>542641b839</x:v>
+      </x:c>
+      <x:c r="S52" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_164903_cpp-router-router-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T52" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_165042_cpp-router-router-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U52" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V52" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 86.97%; latency median ratio 1.10x; pass. 64KiB is an individual outlier below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="29"/>
-      <x:c r="G53" s="27"/>
-      <x:c r="H53" s="27"/>
-      <x:c r="I53" s="23"/>
-      <x:c r="J53" s="25"/>
-      <x:c r="K53" s="25"/>
-      <x:c r="L53" s="25"/>
+      <x:c r="A53" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B53" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C53" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D53" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E53" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F53" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G53" s="26" t="n">
+        <x:v>1400736.4</x:v>
+      </x:c>
+      <x:c r="H53" s="26" t="n">
+        <x:v>1241371.6</x:v>
+      </x:c>
+      <x:c r="I53" s="22" t="n">
+        <x:f>H53/G53</x:f>
+        <x:v>0.8862278441539752</x:v>
+      </x:c>
+      <x:c r="J53" s="24" t="n">
+        <x:v>27.851</x:v>
+      </x:c>
+      <x:c r="K53" s="24" t="n">
+        <x:v>28.058</x:v>
+      </x:c>
+      <x:c r="L53" s="24" t="n">
+        <x:f>K53/J53</x:f>
+        <x:v>1.0074324081720585</x:v>
+      </x:c>
+      <x:c r="M53" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N53" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O53" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P53" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q53" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R53" s="10" t="str">
+        <x:v>542641b839</x:v>
+      </x:c>
+      <x:c r="S53" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_164903_cpp-router-router-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T53" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_165042_cpp-router-router-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U53" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V53" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 86.97%; latency median ratio 1.10x; pass. 64KiB is an individual outlier below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="29"/>
-      <x:c r="G54" s="27"/>
-      <x:c r="H54" s="27"/>
-      <x:c r="I54" s="23"/>
-      <x:c r="J54" s="25"/>
-      <x:c r="K54" s="25"/>
-      <x:c r="L54" s="25"/>
+      <x:c r="A54" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B54" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C54" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D54" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E54" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F54" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G54" s="26" t="n">
+        <x:v>646290.4</x:v>
+      </x:c>
+      <x:c r="H54" s="26" t="n">
+        <x:v>611191.8</x:v>
+      </x:c>
+      <x:c r="I54" s="22" t="n">
+        <x:f>H54/G54</x:f>
+        <x:v>0.9456922151404384</x:v>
+      </x:c>
+      <x:c r="J54" s="24" t="n">
+        <x:v>12.312</x:v>
+      </x:c>
+      <x:c r="K54" s="24" t="n">
+        <x:v>13.81</x:v>
+      </x:c>
+      <x:c r="L54" s="24" t="n">
+        <x:f>K54/J54</x:f>
+        <x:v>1.1216699155295649</x:v>
+      </x:c>
+      <x:c r="M54" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N54" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O54" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P54" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q54" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R54" s="10" t="str">
+        <x:v>542641b839</x:v>
+      </x:c>
+      <x:c r="S54" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_164903_cpp-router-router-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T54" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_165042_cpp-router-router-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U54" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V54" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 86.97%; latency median ratio 1.10x; pass. 64KiB is an individual outlier below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="29"/>
-      <x:c r="G55" s="27"/>
-      <x:c r="H55" s="27"/>
-      <x:c r="I55" s="23"/>
-      <x:c r="J55" s="25"/>
-      <x:c r="K55" s="25"/>
-      <x:c r="L55" s="25"/>
+      <x:c r="A55" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B55" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C55" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D55" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E55" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F55" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G55" s="26" t="n">
+        <x:v>34343</x:v>
+      </x:c>
+      <x:c r="H55" s="26" t="n">
+        <x:v>26648.2</x:v>
+      </x:c>
+      <x:c r="I55" s="22" t="n">
+        <x:f>H55/G55</x:f>
+        <x:v>0.775942695745858</x:v>
+      </x:c>
+      <x:c r="J55" s="24" t="n">
+        <x:v>0.29</x:v>
+      </x:c>
+      <x:c r="K55" s="24" t="n">
+        <x:v>0.383</x:v>
+      </x:c>
+      <x:c r="L55" s="24" t="n">
+        <x:f>K55/J55</x:f>
+        <x:v>1.3206896551724139</x:v>
+      </x:c>
+      <x:c r="M55" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N55" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O55" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P55" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q55" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R55" s="10" t="str">
+        <x:v>542641b839</x:v>
+      </x:c>
+      <x:c r="S55" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_164903_cpp-router-router-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T55" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_165042_cpp-router-router-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U55" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V55" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 86.97%; latency median ratio 1.10x; pass. 64KiB is an individual outlier below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="29"/>
-      <x:c r="G56" s="27"/>
-      <x:c r="H56" s="27"/>
-      <x:c r="I56" s="23"/>
-      <x:c r="J56" s="25"/>
-      <x:c r="K56" s="25"/>
-      <x:c r="L56" s="25"/>
+      <x:c r="A56" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B56" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C56" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D56" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E56" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F56" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G56" s="26" t="n">
+        <x:v>21945.6</x:v>
+      </x:c>
+      <x:c r="H56" s="26" t="n">
+        <x:v>18794.6</x:v>
+      </x:c>
+      <x:c r="I56" s="22" t="n">
+        <x:f>H56/G56</x:f>
+        <x:v>0.8564176873724118</x:v>
+      </x:c>
+      <x:c r="J56" s="24" t="n">
+        <x:v>0.278</x:v>
+      </x:c>
+      <x:c r="K56" s="24" t="n">
+        <x:v>0.326</x:v>
+      </x:c>
+      <x:c r="L56" s="24" t="n">
+        <x:f>K56/J56</x:f>
+        <x:v>1.1726618705035972</x:v>
+      </x:c>
+      <x:c r="M56" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N56" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O56" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P56" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q56" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R56" s="10" t="str">
+        <x:v>542641b839</x:v>
+      </x:c>
+      <x:c r="S56" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_164903_cpp-router-router-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T56" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_165042_cpp-router-router-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U56" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V56" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 86.97%; latency median ratio 1.10x; pass. 64KiB is an individual outlier below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="29"/>
-      <x:c r="G57" s="27"/>
-      <x:c r="H57" s="27"/>
-      <x:c r="I57" s="23"/>
-      <x:c r="J57" s="25"/>
-      <x:c r="K57" s="25"/>
-      <x:c r="L57" s="25"/>
+      <x:c r="A57" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B57" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C57" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D57" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E57" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F57" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G57" s="26" t="n">
+        <x:v>13586.4</x:v>
+      </x:c>
+      <x:c r="H57" s="26" t="n">
+        <x:v>12619.6</x:v>
+      </x:c>
+      <x:c r="I57" s="22" t="n">
+        <x:f>H57/G57</x:f>
+        <x:v>0.9288406053111936</x:v>
+      </x:c>
+      <x:c r="J57" s="24" t="n">
+        <x:v>0.301</x:v>
+      </x:c>
+      <x:c r="K57" s="24" t="n">
+        <x:v>0.323</x:v>
+      </x:c>
+      <x:c r="L57" s="24" t="n">
+        <x:f>K57/J57</x:f>
+        <x:v>1.0730897009966778</x:v>
+      </x:c>
+      <x:c r="M57" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N57" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O57" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P57" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q57" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R57" s="10" t="str">
+        <x:v>542641b839</x:v>
+      </x:c>
+      <x:c r="S57" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_164903_cpp-router-router-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T57" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_165042_cpp-router-router-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U57" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V57" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 86.97%; latency median ratio 1.10x; pass. 64KiB is an individual outlier below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="29"/>

</xml_diff>

<commit_message>
perf(cpp): record router request reply baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R571fd9b91f3d44ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R5e18b7c8246e40c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rbd7ca3a637214a77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R0ed1f7d0b48149b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2e4469da094d4230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R3ad0f13563bc4c5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R5adafa5bb0ba40cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R889f24357e484814"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>PAIR·DEALER_ROUTER_REQREP/tcp 미달 기록 완료; 4개 tcp 패턴 통과</x:v>
+        <x:v>PAIR·두 request/reply/tcp 미달 기록 완료; 4개 tcp 패턴 통과</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -4471,166 +4471,1264 @@
       </x:c>
     </x:row>
     <x:row r="58">
-      <x:c r="A58" s="29"/>
-      <x:c r="G58" s="27"/>
-      <x:c r="H58" s="27"/>
-      <x:c r="I58" s="23"/>
-      <x:c r="J58" s="25"/>
-      <x:c r="K58" s="25"/>
-      <x:c r="L58" s="25"/>
+      <x:c r="A58" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B58" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C58" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D58" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E58" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F58" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G58" s="26" t="n">
+        <x:v>172112.8</x:v>
+      </x:c>
+      <x:c r="H58" s="26" t="n">
+        <x:v>115355</x:v>
+      </x:c>
+      <x:c r="I58" s="22" t="n">
+        <x:f>H58/G58</x:f>
+        <x:v>0.6702290590821833</x:v>
+      </x:c>
+      <x:c r="J58" s="24" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="K58" s="24" t="n">
+        <x:v>0.431</x:v>
+      </x:c>
+      <x:c r="L58" s="24" t="n">
+        <x:f>K58/J58</x:f>
+        <x:v>1.724</x:v>
+      </x:c>
+      <x:c r="M58" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N58" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O58" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P58" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q58" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R58" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S58" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T58" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_165702_cpp-router-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U58" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V58" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 68.66%; latency median ratio 1.58x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
-      <x:c r="A59" s="29"/>
-      <x:c r="G59" s="27"/>
-      <x:c r="H59" s="27"/>
-      <x:c r="I59" s="23"/>
-      <x:c r="J59" s="25"/>
-      <x:c r="K59" s="25"/>
-      <x:c r="L59" s="25"/>
+      <x:c r="A59" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B59" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C59" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D59" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E59" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F59" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G59" s="26" t="n">
+        <x:v>157814.4</x:v>
+      </x:c>
+      <x:c r="H59" s="26" t="n">
+        <x:v>89988.8</x:v>
+      </x:c>
+      <x:c r="I59" s="22" t="n">
+        <x:f>H59/G59</x:f>
+        <x:v>0.570219194192672</x:v>
+      </x:c>
+      <x:c r="J59" s="24" t="n">
+        <x:v>0.279</x:v>
+      </x:c>
+      <x:c r="K59" s="24" t="n">
+        <x:v>0.57</x:v>
+      </x:c>
+      <x:c r="L59" s="24" t="n">
+        <x:f>K59/J59</x:f>
+        <x:v>2.0430107526881716</x:v>
+      </x:c>
+      <x:c r="M59" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N59" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O59" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P59" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q59" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R59" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S59" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T59" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_165702_cpp-router-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U59" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V59" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 68.66%; latency median ratio 1.58x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
-      <x:c r="A60" s="29"/>
-      <x:c r="G60" s="27"/>
-      <x:c r="H60" s="27"/>
-      <x:c r="I60" s="23"/>
-      <x:c r="J60" s="25"/>
-      <x:c r="K60" s="25"/>
-      <x:c r="L60" s="25"/>
+      <x:c r="A60" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B60" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C60" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D60" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E60" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F60" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G60" s="26" t="n">
+        <x:v>144750.4</x:v>
+      </x:c>
+      <x:c r="H60" s="26" t="n">
+        <x:v>57291.8</x:v>
+      </x:c>
+      <x:c r="I60" s="22" t="n">
+        <x:f>H60/G60</x:f>
+        <x:v>0.3957971791442373</x:v>
+      </x:c>
+      <x:c r="J60" s="24" t="n">
+        <x:v>0.362</x:v>
+      </x:c>
+      <x:c r="K60" s="24" t="n">
+        <x:v>1.037</x:v>
+      </x:c>
+      <x:c r="L60" s="24" t="n">
+        <x:f>K60/J60</x:f>
+        <x:v>2.8646408839779003</x:v>
+      </x:c>
+      <x:c r="M60" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N60" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O60" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P60" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q60" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R60" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S60" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T60" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_165702_cpp-router-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U60" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V60" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 68.66%; latency median ratio 1.58x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="61">
-      <x:c r="A61" s="29"/>
-      <x:c r="G61" s="27"/>
-      <x:c r="H61" s="27"/>
-      <x:c r="I61" s="23"/>
-      <x:c r="J61" s="25"/>
-      <x:c r="K61" s="25"/>
-      <x:c r="L61" s="25"/>
+      <x:c r="A61" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B61" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C61" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D61" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E61" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F61" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G61" s="26" t="n">
+        <x:v>15830.6</x:v>
+      </x:c>
+      <x:c r="H61" s="26" t="n">
+        <x:v>10979.6</x:v>
+      </x:c>
+      <x:c r="I61" s="22" t="n">
+        <x:f>H61/G61</x:f>
+        <x:v>0.6935681528179601</x:v>
+      </x:c>
+      <x:c r="J61" s="24" t="n">
+        <x:v>0.749</x:v>
+      </x:c>
+      <x:c r="K61" s="24" t="n">
+        <x:v>1.082</x:v>
+      </x:c>
+      <x:c r="L61" s="24" t="n">
+        <x:f>K61/J61</x:f>
+        <x:v>1.444592790387183</x:v>
+      </x:c>
+      <x:c r="M61" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N61" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O61" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P61" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q61" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R61" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S61" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T61" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_165702_cpp-router-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U61" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V61" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 68.66%; latency median ratio 1.58x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
-      <x:c r="A62" s="29"/>
-      <x:c r="G62" s="27"/>
-      <x:c r="H62" s="27"/>
-      <x:c r="I62" s="23"/>
-      <x:c r="J62" s="25"/>
-      <x:c r="K62" s="25"/>
-      <x:c r="L62" s="25"/>
+      <x:c r="A62" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B62" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C62" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D62" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E62" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F62" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G62" s="26" t="n">
+        <x:v>10914.6</x:v>
+      </x:c>
+      <x:c r="H62" s="26" t="n">
+        <x:v>8704.4</x:v>
+      </x:c>
+      <x:c r="I62" s="22" t="n">
+        <x:f>H62/G62</x:f>
+        <x:v>0.7975005955325893</x:v>
+      </x:c>
+      <x:c r="J62" s="24" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="K62" s="24" t="n">
+        <x:v>0.664</x:v>
+      </x:c>
+      <x:c r="L62" s="24" t="n">
+        <x:f>K62/J62</x:f>
+        <x:v>1.1066666666666667</x:v>
+      </x:c>
+      <x:c r="M62" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N62" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O62" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P62" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q62" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R62" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S62" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T62" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_165702_cpp-router-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U62" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V62" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 68.66%; latency median ratio 1.58x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
-      <x:c r="A63" s="29"/>
-      <x:c r="G63" s="27"/>
-      <x:c r="H63" s="27"/>
-      <x:c r="I63" s="23"/>
-      <x:c r="J63" s="25"/>
-      <x:c r="K63" s="25"/>
-      <x:c r="L63" s="25"/>
+      <x:c r="A63" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B63" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C63" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D63" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E63" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F63" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G63" s="26" t="n">
+        <x:v>5891.2</x:v>
+      </x:c>
+      <x:c r="H63" s="26" t="n">
+        <x:v>5844.6</x:v>
+      </x:c>
+      <x:c r="I63" s="22" t="n">
+        <x:f>H63/G63</x:f>
+        <x:v>0.9920898967952201</x:v>
+      </x:c>
+      <x:c r="J63" s="24" t="n">
+        <x:v>0.502</x:v>
+      </x:c>
+      <x:c r="K63" s="24" t="n">
+        <x:v>0.489</x:v>
+      </x:c>
+      <x:c r="L63" s="24" t="n">
+        <x:f>K63/J63</x:f>
+        <x:v>0.9741035856573705</x:v>
+      </x:c>
+      <x:c r="M63" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N63" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O63" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P63" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q63" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R63" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S63" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T63" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_165702_cpp-router-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U63" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V63" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 68.66%; latency median ratio 1.58x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="64">
-      <x:c r="A64" s="29"/>
-      <x:c r="G64" s="27"/>
-      <x:c r="H64" s="27"/>
-      <x:c r="I64" s="23"/>
-      <x:c r="J64" s="25"/>
-      <x:c r="K64" s="25"/>
-      <x:c r="L64" s="25"/>
+      <x:c r="A64" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B64" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C64" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D64" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E64" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F64" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G64" s="26" t="n">
+        <x:v>172112.8</x:v>
+      </x:c>
+      <x:c r="H64" s="26" t="n">
+        <x:v>105201.4</x:v>
+      </x:c>
+      <x:c r="I64" s="22" t="n">
+        <x:f>H64/G64</x:f>
+        <x:v>0.6112351899451988</x:v>
+      </x:c>
+      <x:c r="J64" s="24" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="K64" s="24" t="n">
+        <x:v>0.472</x:v>
+      </x:c>
+      <x:c r="L64" s="24" t="n">
+        <x:f>K64/J64</x:f>
+        <x:v>1.888</x:v>
+      </x:c>
+      <x:c r="M64" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N64" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O64" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P64" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q64" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R64" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S64" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T64" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_170021_cpp-router-router-reqrep-tcp-local0132-candidate-a-bridge-owner-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U64" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V64" s="10" t="str">
+        <x:v>Candidate A: throughput aggregate mean 66.61%; latency median ratio 1.64x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="65">
-      <x:c r="A65" s="29"/>
-      <x:c r="G65" s="27"/>
-      <x:c r="H65" s="27"/>
-      <x:c r="I65" s="23"/>
-      <x:c r="J65" s="25"/>
-      <x:c r="K65" s="25"/>
-      <x:c r="L65" s="25"/>
+      <x:c r="A65" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B65" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C65" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D65" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E65" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F65" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G65" s="26" t="n">
+        <x:v>157814.4</x:v>
+      </x:c>
+      <x:c r="H65" s="26" t="n">
+        <x:v>87524.6</x:v>
+      </x:c>
+      <x:c r="I65" s="22" t="n">
+        <x:f>H65/G65</x:f>
+        <x:v>0.5546046495123386</x:v>
+      </x:c>
+      <x:c r="J65" s="24" t="n">
+        <x:v>0.279</x:v>
+      </x:c>
+      <x:c r="K65" s="24" t="n">
+        <x:v>0.589</x:v>
+      </x:c>
+      <x:c r="L65" s="24" t="n">
+        <x:f>K65/J65</x:f>
+        <x:v>2.1111111111111107</x:v>
+      </x:c>
+      <x:c r="M65" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N65" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O65" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P65" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q65" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R65" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S65" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T65" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_170021_cpp-router-router-reqrep-tcp-local0132-candidate-a-bridge-owner-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U65" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V65" s="10" t="str">
+        <x:v>Candidate A: throughput aggregate mean 66.61%; latency median ratio 1.64x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="66">
-      <x:c r="A66" s="29"/>
-      <x:c r="G66" s="27"/>
-      <x:c r="H66" s="27"/>
-      <x:c r="I66" s="23"/>
-      <x:c r="J66" s="25"/>
-      <x:c r="K66" s="25"/>
-      <x:c r="L66" s="25"/>
+      <x:c r="A66" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B66" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C66" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D66" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E66" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F66" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G66" s="26" t="n">
+        <x:v>144750.4</x:v>
+      </x:c>
+      <x:c r="H66" s="26" t="n">
+        <x:v>54115.2</x:v>
+      </x:c>
+      <x:c r="I66" s="22" t="n">
+        <x:f>H66/G66</x:f>
+        <x:v>0.3738518166443754</x:v>
+      </x:c>
+      <x:c r="J66" s="24" t="n">
+        <x:v>0.362</x:v>
+      </x:c>
+      <x:c r="K66" s="24" t="n">
+        <x:v>1.073</x:v>
+      </x:c>
+      <x:c r="L66" s="24" t="n">
+        <x:f>K66/J66</x:f>
+        <x:v>2.9640883977900554</x:v>
+      </x:c>
+      <x:c r="M66" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N66" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O66" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P66" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q66" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R66" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S66" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T66" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_170021_cpp-router-router-reqrep-tcp-local0132-candidate-a-bridge-owner-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U66" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V66" s="10" t="str">
+        <x:v>Candidate A: throughput aggregate mean 66.61%; latency median ratio 1.64x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
-      <x:c r="A67" s="29"/>
-      <x:c r="G67" s="27"/>
-      <x:c r="H67" s="27"/>
-      <x:c r="I67" s="23"/>
-      <x:c r="J67" s="25"/>
-      <x:c r="K67" s="25"/>
-      <x:c r="L67" s="25"/>
+      <x:c r="A67" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B67" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C67" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D67" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E67" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F67" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G67" s="26" t="n">
+        <x:v>15830.6</x:v>
+      </x:c>
+      <x:c r="H67" s="26" t="n">
+        <x:v>11273.8</x:v>
+      </x:c>
+      <x:c r="I67" s="22" t="n">
+        <x:f>H67/G67</x:f>
+        <x:v>0.7121524136798352</x:v>
+      </x:c>
+      <x:c r="J67" s="24" t="n">
+        <x:v>0.749</x:v>
+      </x:c>
+      <x:c r="K67" s="24" t="n">
+        <x:v>1.04</x:v>
+      </x:c>
+      <x:c r="L67" s="24" t="n">
+        <x:f>K67/J67</x:f>
+        <x:v>1.3885180240320427</x:v>
+      </x:c>
+      <x:c r="M67" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N67" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O67" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P67" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q67" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R67" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S67" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T67" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_170021_cpp-router-router-reqrep-tcp-local0132-candidate-a-bridge-owner-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U67" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V67" s="10" t="str">
+        <x:v>Candidate A: throughput aggregate mean 66.61%; latency median ratio 1.64x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
-      <x:c r="A68" s="29"/>
-      <x:c r="G68" s="27"/>
-      <x:c r="H68" s="27"/>
-      <x:c r="I68" s="23"/>
-      <x:c r="J68" s="25"/>
-      <x:c r="K68" s="25"/>
-      <x:c r="L68" s="25"/>
+      <x:c r="A68" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B68" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C68" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D68" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E68" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F68" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G68" s="26" t="n">
+        <x:v>10914.6</x:v>
+      </x:c>
+      <x:c r="H68" s="26" t="n">
+        <x:v>8820</x:v>
+      </x:c>
+      <x:c r="I68" s="22" t="n">
+        <x:f>H68/G68</x:f>
+        <x:v>0.8080919135836402</x:v>
+      </x:c>
+      <x:c r="J68" s="24" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="K68" s="24" t="n">
+        <x:v>0.656</x:v>
+      </x:c>
+      <x:c r="L68" s="24" t="n">
+        <x:f>K68/J68</x:f>
+        <x:v>1.0933333333333335</x:v>
+      </x:c>
+      <x:c r="M68" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N68" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O68" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P68" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q68" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R68" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S68" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T68" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_170021_cpp-router-router-reqrep-tcp-local0132-candidate-a-bridge-owner-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U68" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V68" s="10" t="str">
+        <x:v>Candidate A: throughput aggregate mean 66.61%; latency median ratio 1.64x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
-      <x:c r="A69" s="29"/>
-      <x:c r="G69" s="27"/>
-      <x:c r="H69" s="27"/>
-      <x:c r="I69" s="23"/>
-      <x:c r="J69" s="25"/>
-      <x:c r="K69" s="25"/>
-      <x:c r="L69" s="25"/>
+      <x:c r="A69" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B69" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C69" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D69" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E69" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F69" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G69" s="26" t="n">
+        <x:v>5891.2</x:v>
+      </x:c>
+      <x:c r="H69" s="26" t="n">
+        <x:v>5520.2</x:v>
+      </x:c>
+      <x:c r="I69" s="22" t="n">
+        <x:f>H69/G69</x:f>
+        <x:v>0.9370247148288974</x:v>
+      </x:c>
+      <x:c r="J69" s="24" t="n">
+        <x:v>0.502</x:v>
+      </x:c>
+      <x:c r="K69" s="24" t="n">
+        <x:v>0.517</x:v>
+      </x:c>
+      <x:c r="L69" s="24" t="n">
+        <x:f>K69/J69</x:f>
+        <x:v>1.0298804780876494</x:v>
+      </x:c>
+      <x:c r="M69" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N69" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O69" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P69" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q69" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R69" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S69" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T69" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_170021_cpp-router-router-reqrep-tcp-local0132-candidate-a-bridge-owner-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U69" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V69" s="10" t="str">
+        <x:v>Candidate A: throughput aggregate mean 66.61%; latency median ratio 1.64x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
-      <x:c r="A70" s="29"/>
-      <x:c r="G70" s="27"/>
-      <x:c r="H70" s="27"/>
-      <x:c r="I70" s="23"/>
-      <x:c r="J70" s="25"/>
-      <x:c r="K70" s="25"/>
-      <x:c r="L70" s="25"/>
+      <x:c r="A70" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B70" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C70" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D70" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E70" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F70" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G70" s="26" t="n">
+        <x:v>172112.8</x:v>
+      </x:c>
+      <x:c r="H70" s="26" t="n">
+        <x:v>94586.4</x:v>
+      </x:c>
+      <x:c r="I70" s="22" t="n">
+        <x:f>H70/G70</x:f>
+        <x:v>0.5495605207747477</x:v>
+      </x:c>
+      <x:c r="J70" s="24" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="K70" s="24" t="n">
+        <x:v>0.498</x:v>
+      </x:c>
+      <x:c r="L70" s="24" t="n">
+        <x:f>K70/J70</x:f>
+        <x:v>1.992</x:v>
+      </x:c>
+      <x:c r="M70" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N70" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O70" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P70" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q70" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R70" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S70" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T70" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_170349_cpp-router-router-reqrep-tcp-local0132-candidate-b-async-bridge-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U70" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V70" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 68.66%; latency median ratio 1.74x; reject: no aggregate gain and worse latency.</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
-      <x:c r="A71" s="29"/>
-      <x:c r="G71" s="27"/>
-      <x:c r="H71" s="27"/>
-      <x:c r="I71" s="23"/>
-      <x:c r="J71" s="25"/>
-      <x:c r="K71" s="25"/>
-      <x:c r="L71" s="25"/>
+      <x:c r="A71" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B71" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C71" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D71" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E71" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F71" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G71" s="26" t="n">
+        <x:v>157814.4</x:v>
+      </x:c>
+      <x:c r="H71" s="26" t="n">
+        <x:v>91143.8</x:v>
+      </x:c>
+      <x:c r="I71" s="22" t="n">
+        <x:f>H71/G71</x:f>
+        <x:v>0.5775379179593244</x:v>
+      </x:c>
+      <x:c r="J71" s="24" t="n">
+        <x:v>0.279</x:v>
+      </x:c>
+      <x:c r="K71" s="24" t="n">
+        <x:v>0.567</x:v>
+      </x:c>
+      <x:c r="L71" s="24" t="n">
+        <x:f>K71/J71</x:f>
+        <x:v>2.0322580645161286</x:v>
+      </x:c>
+      <x:c r="M71" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N71" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O71" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P71" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q71" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R71" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S71" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T71" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_170349_cpp-router-router-reqrep-tcp-local0132-candidate-b-async-bridge-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U71" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V71" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 68.66%; latency median ratio 1.74x; reject: no aggregate gain and worse latency.</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
-      <x:c r="A72" s="29"/>
-      <x:c r="G72" s="27"/>
-      <x:c r="H72" s="27"/>
-      <x:c r="I72" s="23"/>
-      <x:c r="J72" s="25"/>
-      <x:c r="K72" s="25"/>
-      <x:c r="L72" s="25"/>
+      <x:c r="A72" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B72" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C72" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D72" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E72" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F72" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G72" s="26" t="n">
+        <x:v>144750.4</x:v>
+      </x:c>
+      <x:c r="H72" s="26" t="n">
+        <x:v>59097.8</x:v>
+      </x:c>
+      <x:c r="I72" s="22" t="n">
+        <x:f>H72/G72</x:f>
+        <x:v>0.4082738286042733</x:v>
+      </x:c>
+      <x:c r="J72" s="24" t="n">
+        <x:v>0.362</x:v>
+      </x:c>
+      <x:c r="K72" s="24" t="n">
+        <x:v>1.007</x:v>
+      </x:c>
+      <x:c r="L72" s="24" t="n">
+        <x:f>K72/J72</x:f>
+        <x:v>2.781767955801105</x:v>
+      </x:c>
+      <x:c r="M72" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N72" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O72" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P72" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q72" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R72" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S72" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T72" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_170349_cpp-router-router-reqrep-tcp-local0132-candidate-b-async-bridge-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U72" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V72" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 68.66%; latency median ratio 1.74x; reject: no aggregate gain and worse latency.</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
-      <x:c r="A73" s="29"/>
-      <x:c r="G73" s="27"/>
-      <x:c r="H73" s="27"/>
-      <x:c r="I73" s="23"/>
-      <x:c r="J73" s="25"/>
-      <x:c r="K73" s="25"/>
-      <x:c r="L73" s="25"/>
+      <x:c r="A73" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B73" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C73" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D73" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E73" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F73" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G73" s="26" t="n">
+        <x:v>15830.6</x:v>
+      </x:c>
+      <x:c r="H73" s="26" t="n">
+        <x:v>11892.2</x:v>
+      </x:c>
+      <x:c r="I73" s="22" t="n">
+        <x:f>H73/G73</x:f>
+        <x:v>0.7512159993935795</x:v>
+      </x:c>
+      <x:c r="J73" s="24" t="n">
+        <x:v>0.749</x:v>
+      </x:c>
+      <x:c r="K73" s="24" t="n">
+        <x:v>1.11</x:v>
+      </x:c>
+      <x:c r="L73" s="24" t="n">
+        <x:f>K73/J73</x:f>
+        <x:v>1.4819759679572766</x:v>
+      </x:c>
+      <x:c r="M73" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N73" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O73" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P73" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q73" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R73" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S73" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T73" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_170349_cpp-router-router-reqrep-tcp-local0132-candidate-b-async-bridge-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U73" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V73" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 68.66%; latency median ratio 1.74x; reject: no aggregate gain and worse latency.</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
-      <x:c r="A74" s="29"/>
-      <x:c r="G74" s="27"/>
-      <x:c r="H74" s="27"/>
-      <x:c r="I74" s="23"/>
-      <x:c r="J74" s="25"/>
-      <x:c r="K74" s="25"/>
-      <x:c r="L74" s="25"/>
+      <x:c r="A74" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B74" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C74" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D74" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E74" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F74" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G74" s="26" t="n">
+        <x:v>10914.6</x:v>
+      </x:c>
+      <x:c r="H74" s="26" t="n">
+        <x:v>8993.8</x:v>
+      </x:c>
+      <x:c r="I74" s="22" t="n">
+        <x:f>H74/G74</x:f>
+        <x:v>0.8240155388195627</x:v>
+      </x:c>
+      <x:c r="J74" s="24" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="K74" s="24" t="n">
+        <x:v>0.644</x:v>
+      </x:c>
+      <x:c r="L74" s="24" t="n">
+        <x:f>K74/J74</x:f>
+        <x:v>1.0733333333333335</x:v>
+      </x:c>
+      <x:c r="M74" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N74" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O74" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P74" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q74" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R74" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S74" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T74" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_170349_cpp-router-router-reqrep-tcp-local0132-candidate-b-async-bridge-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U74" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V74" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 68.66%; latency median ratio 1.74x; reject: no aggregate gain and worse latency.</x:v>
+      </x:c>
     </x:row>
     <x:row r="75">
-      <x:c r="A75" s="29"/>
-      <x:c r="G75" s="27"/>
-      <x:c r="H75" s="27"/>
-      <x:c r="I75" s="23"/>
-      <x:c r="J75" s="25"/>
-      <x:c r="K75" s="25"/>
-      <x:c r="L75" s="25"/>
+      <x:c r="A75" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B75" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C75" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D75" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E75" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F75" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G75" s="26" t="n">
+        <x:v>5891.2</x:v>
+      </x:c>
+      <x:c r="H75" s="26" t="n">
+        <x:v>5942.6</x:v>
+      </x:c>
+      <x:c r="I75" s="22" t="n">
+        <x:f>H75/G75</x:f>
+        <x:v>1.0087248777838131</x:v>
+      </x:c>
+      <x:c r="J75" s="24" t="n">
+        <x:v>0.502</x:v>
+      </x:c>
+      <x:c r="K75" s="24" t="n">
+        <x:v>0.48</x:v>
+      </x:c>
+      <x:c r="L75" s="24" t="n">
+        <x:f>K75/J75</x:f>
+        <x:v>0.9561752988047808</x:v>
+      </x:c>
+      <x:c r="M75" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N75" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O75" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P75" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q75" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R75" s="10" t="str">
+        <x:v>c3fd621065</x:v>
+      </x:c>
+      <x:c r="S75" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_165412_cpp-router-router-reqrep-tcp-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T75" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_170349_cpp-router-router-reqrep-tcp-local0132-candidate-b-async-bridge-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U75" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V75" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 68.66%; latency median ratio 1.74x; reject: no aggregate gain and worse latency.</x:v>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="29"/>
@@ -7819,12 +8917,92 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="L8" s="23"/>
-      <x:c r="M8" s="23"/>
+      <x:c r="A8" s="10" t="str">
+        <x:v>2026-08-25 17:00</x:v>
+      </x:c>
+      <x:c r="B8" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D8" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F8" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G8" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H8" s="10" t="str">
+        <x:v>Make accepted request completion bridge callback-owned to remove shared_ptr control-block and userdata allocation.</x:v>
+      </x:c>
+      <x:c r="I8" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J8" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_165702_cpp-router-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K8" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_170021_cpp-router-router-reqrep-tcp-local0132-candidate-a-bridge-owner-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L8" s="22" t="n">
+        <x:v>0.687</x:v>
+      </x:c>
+      <x:c r="M8" s="22" t="n">
+        <x:v>0.666</x:v>
+      </x:c>
+      <x:c r="N8" s="10" t="str">
+        <x:v>REJECT: aggregate regressed. Contract tests passed; change removed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="L9" s="23"/>
-      <x:c r="M9" s="23"/>
+      <x:c r="A9" s="10" t="str">
+        <x:v>2026-08-25 17:03</x:v>
+      </x:c>
+      <x:c r="B9" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C9" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D9" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E9" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F9" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G9" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H9" s="10" t="str">
+        <x:v>Use an async-only completion bridge and delegate terminal synchronization to async_operation_state_t.</x:v>
+      </x:c>
+      <x:c r="I9" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J9" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_165702_cpp-router-router-reqrep-tcp-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K9" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_170349_cpp-router-router-reqrep-tcp-local0132-candidate-b-async-bridge-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L9" s="22" t="n">
+        <x:v>0.687</x:v>
+      </x:c>
+      <x:c r="M9" s="22" t="n">
+        <x:v>0.687</x:v>
+      </x:c>
+      <x:c r="N9" s="10" t="str">
+        <x:v>REJECT: no aggregate gain and latency worsened. POSDDD boundary was clear, but new complexity has no performance benefit; removed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="L10" s="23"/>

</xml_diff>

<commit_message>
perf(cpp): record websocket pair baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2e4469da094d4230"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R3ad0f13563bc4c5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R5adafa5bb0ba40cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R889f24357e484814"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R979cc231ef3d4d03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rca2e5c85fddc440f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rf87ed430253c42df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R8097dd9d900d49e8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>PAIR·두 request/reply/tcp 미달 기록 완료; 4개 tcp 패턴 통과</x:v>
+        <x:v>tcp 4개 통과·3개 미달, PAIR/ws strict 목표 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -5731,58 +5731,424 @@
       </x:c>
     </x:row>
     <x:row r="76">
-      <x:c r="A76" s="29"/>
-      <x:c r="G76" s="27"/>
-      <x:c r="H76" s="27"/>
-      <x:c r="I76" s="23"/>
-      <x:c r="J76" s="25"/>
-      <x:c r="K76" s="25"/>
-      <x:c r="L76" s="25"/>
+      <x:c r="A76" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B76" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C76" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D76" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E76" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F76" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G76" s="26" t="n">
+        <x:v>2192995.8</x:v>
+      </x:c>
+      <x:c r="H76" s="26" t="n">
+        <x:v>1734785.4</x:v>
+      </x:c>
+      <x:c r="I76" s="22" t="n">
+        <x:f>H76/G76</x:f>
+        <x:v>0.7910573289743646</x:v>
+      </x:c>
+      <x:c r="J76" s="24" t="n">
+        <x:v>41.572</x:v>
+      </x:c>
+      <x:c r="K76" s="24" t="n">
+        <x:v>50.686</x:v>
+      </x:c>
+      <x:c r="L76" s="24" t="n">
+        <x:f>K76/J76</x:f>
+        <x:v>1.2192340998749158</x:v>
+      </x:c>
+      <x:c r="M76" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N76" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O76" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P76" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q76" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R76" s="10" t="str">
+        <x:v>30ee3845f5</x:v>
+      </x:c>
+      <x:c r="S76" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_170906_cpp-pair-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T76" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_171045_cpp-pair-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U76" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V76" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 93.46%; latency median ratio 1.03x; strict 95% gate missed. No safe distinct candidate: 64KiB pool lowering previously timed out; mutex/weak removal and pool expansion are forbidden.</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
-      <x:c r="A77" s="29"/>
-      <x:c r="G77" s="27"/>
-      <x:c r="H77" s="27"/>
-      <x:c r="I77" s="23"/>
-      <x:c r="J77" s="25"/>
-      <x:c r="K77" s="25"/>
-      <x:c r="L77" s="25"/>
+      <x:c r="A77" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B77" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C77" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D77" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E77" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F77" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G77" s="26" t="n">
+        <x:v>1029540.6</x:v>
+      </x:c>
+      <x:c r="H77" s="26" t="n">
+        <x:v>1012645.6</x:v>
+      </x:c>
+      <x:c r="I77" s="22" t="n">
+        <x:f>H77/G77</x:f>
+        <x:v>0.9835897680965666</x:v>
+      </x:c>
+      <x:c r="J77" s="24" t="n">
+        <x:v>35.064</x:v>
+      </x:c>
+      <x:c r="K77" s="24" t="n">
+        <x:v>32.357</x:v>
+      </x:c>
+      <x:c r="L77" s="24" t="n">
+        <x:f>K77/J77</x:f>
+        <x:v>0.9227983116586812</x:v>
+      </x:c>
+      <x:c r="M77" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N77" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O77" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P77" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q77" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R77" s="10" t="str">
+        <x:v>30ee3845f5</x:v>
+      </x:c>
+      <x:c r="S77" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_170906_cpp-pair-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T77" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_171045_cpp-pair-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U77" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V77" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 93.46%; latency median ratio 1.03x; strict 95% gate missed. No safe distinct candidate: 64KiB pool lowering previously timed out; mutex/weak removal and pool expansion are forbidden.</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
-      <x:c r="A78" s="29"/>
-      <x:c r="G78" s="27"/>
-      <x:c r="H78" s="27"/>
-      <x:c r="I78" s="23"/>
-      <x:c r="J78" s="25"/>
-      <x:c r="K78" s="25"/>
-      <x:c r="L78" s="25"/>
+      <x:c r="A78" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B78" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C78" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D78" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E78" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F78" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G78" s="26" t="n">
+        <x:v>408427.2</x:v>
+      </x:c>
+      <x:c r="H78" s="26" t="n">
+        <x:v>390855.8</x:v>
+      </x:c>
+      <x:c r="I78" s="22" t="n">
+        <x:f>H78/G78</x:f>
+        <x:v>0.9569778898173285</x:v>
+      </x:c>
+      <x:c r="J78" s="24" t="n">
+        <x:v>21.973</x:v>
+      </x:c>
+      <x:c r="K78" s="24" t="n">
+        <x:v>20.428</x:v>
+      </x:c>
+      <x:c r="L78" s="24" t="n">
+        <x:f>K78/J78</x:f>
+        <x:v>0.9296864333500205</x:v>
+      </x:c>
+      <x:c r="M78" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N78" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O78" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P78" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q78" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R78" s="10" t="str">
+        <x:v>30ee3845f5</x:v>
+      </x:c>
+      <x:c r="S78" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_170906_cpp-pair-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T78" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_171045_cpp-pair-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U78" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V78" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 93.46%; latency median ratio 1.03x; strict 95% gate missed. No safe distinct candidate: 64KiB pool lowering previously timed out; mutex/weak removal and pool expansion are forbidden.</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
-      <x:c r="A79" s="29"/>
-      <x:c r="G79" s="27"/>
-      <x:c r="H79" s="27"/>
-      <x:c r="I79" s="23"/>
-      <x:c r="J79" s="25"/>
-      <x:c r="K79" s="25"/>
-      <x:c r="L79" s="25"/>
+      <x:c r="A79" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B79" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C79" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D79" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E79" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F79" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G79" s="26" t="n">
+        <x:v>18940.4</x:v>
+      </x:c>
+      <x:c r="H79" s="26" t="n">
+        <x:v>17313</x:v>
+      </x:c>
+      <x:c r="I79" s="22" t="n">
+        <x:f>H79/G79</x:f>
+        <x:v>0.9140778441849168</x:v>
+      </x:c>
+      <x:c r="J79" s="24" t="n">
+        <x:v>6.194</x:v>
+      </x:c>
+      <x:c r="K79" s="24" t="n">
+        <x:v>6.834</x:v>
+      </x:c>
+      <x:c r="L79" s="24" t="n">
+        <x:f>K79/J79</x:f>
+        <x:v>1.103325799160478</x:v>
+      </x:c>
+      <x:c r="M79" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N79" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O79" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P79" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q79" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R79" s="10" t="str">
+        <x:v>30ee3845f5</x:v>
+      </x:c>
+      <x:c r="S79" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_170906_cpp-pair-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T79" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_171045_cpp-pair-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U79" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V79" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 93.46%; latency median ratio 1.03x; strict 95% gate missed. No safe distinct candidate: 64KiB pool lowering previously timed out; mutex/weak removal and pool expansion are forbidden.</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
-      <x:c r="A80" s="29"/>
-      <x:c r="G80" s="27"/>
-      <x:c r="H80" s="27"/>
-      <x:c r="I80" s="23"/>
-      <x:c r="J80" s="25"/>
-      <x:c r="K80" s="25"/>
-      <x:c r="L80" s="25"/>
+      <x:c r="A80" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B80" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C80" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D80" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E80" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F80" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G80" s="26" t="n">
+        <x:v>13343.2</x:v>
+      </x:c>
+      <x:c r="H80" s="26" t="n">
+        <x:v>12451</x:v>
+      </x:c>
+      <x:c r="I80" s="22" t="n">
+        <x:f>H80/G80</x:f>
+        <x:v>0.9331344804844415</x:v>
+      </x:c>
+      <x:c r="J80" s="24" t="n">
+        <x:v>0.44</x:v>
+      </x:c>
+      <x:c r="K80" s="24" t="n">
+        <x:v>0.48</x:v>
+      </x:c>
+      <x:c r="L80" s="24" t="n">
+        <x:f>K80/J80</x:f>
+        <x:v>1.0909090909090908</x:v>
+      </x:c>
+      <x:c r="M80" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N80" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O80" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P80" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q80" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R80" s="10" t="str">
+        <x:v>30ee3845f5</x:v>
+      </x:c>
+      <x:c r="S80" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_170906_cpp-pair-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T80" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_171045_cpp-pair-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U80" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V80" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 93.46%; latency median ratio 1.03x; strict 95% gate missed. No safe distinct candidate: 64KiB pool lowering previously timed out; mutex/weak removal and pool expansion are forbidden.</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
-      <x:c r="A81" s="29"/>
-      <x:c r="G81" s="27"/>
-      <x:c r="H81" s="27"/>
-      <x:c r="I81" s="23"/>
-      <x:c r="J81" s="25"/>
-      <x:c r="K81" s="25"/>
-      <x:c r="L81" s="25"/>
+      <x:c r="A81" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B81" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C81" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D81" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E81" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F81" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G81" s="26" t="n">
+        <x:v>8003.4</x:v>
+      </x:c>
+      <x:c r="H81" s="26" t="n">
+        <x:v>8231.8</x:v>
+      </x:c>
+      <x:c r="I81" s="22" t="n">
+        <x:f>H81/G81</x:f>
+        <x:v>1.028537871404653</x:v>
+      </x:c>
+      <x:c r="J81" s="24" t="n">
+        <x:v>0.512</x:v>
+      </x:c>
+      <x:c r="K81" s="24" t="n">
+        <x:v>0.499</x:v>
+      </x:c>
+      <x:c r="L81" s="24" t="n">
+        <x:f>K81/J81</x:f>
+        <x:v>0.974609375</x:v>
+      </x:c>
+      <x:c r="M81" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N81" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O81" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P81" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q81" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R81" s="10" t="str">
+        <x:v>30ee3845f5</x:v>
+      </x:c>
+      <x:c r="S81" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_170906_cpp-pair-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T81" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_171045_cpp-pair-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U81" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V81" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 93.46%; latency median ratio 1.03x; strict 95% gate missed. No safe distinct candidate: 64KiB pool lowering previously timed out; mutex/weak removal and pool expansion are forbidden.</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="29"/>
@@ -9005,12 +9371,88 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="L10" s="23"/>
-      <x:c r="M10" s="23"/>
+      <x:c r="A10" s="10" t="str">
+        <x:v>2026-08-25 17:10</x:v>
+      </x:c>
+      <x:c r="B10" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C10" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D10" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E10" s="10" t="str">
+        <x:v>ws</x:v>
+      </x:c>
+      <x:c r="F10" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%</x:v>
+      </x:c>
+      <x:c r="G10" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H10" s="10" t="str">
+        <x:v>Re-evaluate current direct single-part send, bounded pool and state reuse as candidate inputs.</x:v>
+      </x:c>
+      <x:c r="I10" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J10" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_171045_cpp-pair-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K10" s="10" t="str">
+        <x:v>N/A — already applied</x:v>
+      </x:c>
+      <x:c r="L10" s="22" t="n">
+        <x:v>0.935</x:v>
+      </x:c>
+      <x:c r="M10" s="22"/>
+      <x:c r="N10" s="10" t="str">
+        <x:v>NO-GO: these are already in the baseline, so repeating them is not an A/B candidate.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="L11" s="23"/>
-      <x:c r="M11" s="23"/>
+      <x:c r="A11" s="10" t="str">
+        <x:v>2026-08-25 17:10</x:v>
+      </x:c>
+      <x:c r="B11" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C11" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D11" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E11" s="10" t="str">
+        <x:v>ws</x:v>
+      </x:c>
+      <x:c r="F11" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%</x:v>
+      </x:c>
+      <x:c r="G11" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H11" s="10" t="str">
+        <x:v>Lower large-message pool threshold, remove attempt mutex/weak lifetime guard, or expand pool cap.</x:v>
+      </x:c>
+      <x:c r="I11" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J11" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_171045_cpp-pair-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K11" s="10" t="str">
+        <x:v>N/A — contract/known-timeout no-go</x:v>
+      </x:c>
+      <x:c r="L11" s="22" t="n">
+        <x:v>0.935</x:v>
+      </x:c>
+      <x:c r="M11" s="22"/>
+      <x:c r="N11" s="10" t="str">
+        <x:v>NO-GO: 64KiB pool lowering previously timed out; mutex/weak removal and pool expansion violate documented contract/memory boundaries.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="L12" s="23"/>

</xml_diff>

<commit_message>
perf(cpp): record websocket pubsub baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R979cc231ef3d4d03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rca2e5c85fddc440f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rf87ed430253c42df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R8097dd9d900d49e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf8d606384803472f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R4319910a07614dc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R7a14e4aeb6fd4c53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R85cc3c4c20f2414c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, PAIR/ws strict 목표 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws PUBSUB 통과·PAIR strict 목표 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -6151,58 +6151,424 @@
       </x:c>
     </x:row>
     <x:row r="82">
-      <x:c r="A82" s="29"/>
-      <x:c r="G82" s="27"/>
-      <x:c r="H82" s="27"/>
-      <x:c r="I82" s="23"/>
-      <x:c r="J82" s="25"/>
-      <x:c r="K82" s="25"/>
-      <x:c r="L82" s="25"/>
+      <x:c r="A82" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B82" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C82" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D82" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E82" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F82" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G82" s="26" t="n">
+        <x:v>1212066.6</x:v>
+      </x:c>
+      <x:c r="H82" s="26" t="n">
+        <x:v>1139438.4</x:v>
+      </x:c>
+      <x:c r="I82" s="22" t="n">
+        <x:f>H82/G82</x:f>
+        <x:v>0.9400790352609335</x:v>
+      </x:c>
+      <x:c r="J82" s="24" t="n">
+        <x:v>61.612</x:v>
+      </x:c>
+      <x:c r="K82" s="24" t="n">
+        <x:v>70.699</x:v>
+      </x:c>
+      <x:c r="L82" s="24" t="n">
+        <x:f>K82/J82</x:f>
+        <x:v>1.1474875024345905</x:v>
+      </x:c>
+      <x:c r="M82" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N82" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O82" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P82" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q82" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R82" s="10" t="str">
+        <x:v>2d801160aa</x:v>
+      </x:c>
+      <x:c r="S82" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_171534_cpp-pubsub-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T82" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_171731_cpp-pubsub-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U82" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V82" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 98.15%; latency median ratio 1.06x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="83">
-      <x:c r="A83" s="29"/>
-      <x:c r="G83" s="27"/>
-      <x:c r="H83" s="27"/>
-      <x:c r="I83" s="23"/>
-      <x:c r="J83" s="25"/>
-      <x:c r="K83" s="25"/>
-      <x:c r="L83" s="25"/>
+      <x:c r="A83" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B83" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C83" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D83" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E83" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F83" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G83" s="26" t="n">
+        <x:v>929416.6</x:v>
+      </x:c>
+      <x:c r="H83" s="26" t="n">
+        <x:v>939247.4</x:v>
+      </x:c>
+      <x:c r="I83" s="22" t="n">
+        <x:f>H83/G83</x:f>
+        <x:v>1.010577388008779</x:v>
+      </x:c>
+      <x:c r="J83" s="24" t="n">
+        <x:v>30.762</x:v>
+      </x:c>
+      <x:c r="K83" s="24" t="n">
+        <x:v>36.933</x:v>
+      </x:c>
+      <x:c r="L83" s="24" t="n">
+        <x:f>K83/J83</x:f>
+        <x:v>1.2006046420908913</x:v>
+      </x:c>
+      <x:c r="M83" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N83" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O83" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P83" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q83" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R83" s="10" t="str">
+        <x:v>2d801160aa</x:v>
+      </x:c>
+      <x:c r="S83" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_171534_cpp-pubsub-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T83" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_171731_cpp-pubsub-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U83" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V83" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 98.15%; latency median ratio 1.06x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="84">
-      <x:c r="A84" s="29"/>
-      <x:c r="G84" s="27"/>
-      <x:c r="H84" s="27"/>
-      <x:c r="I84" s="23"/>
-      <x:c r="J84" s="25"/>
-      <x:c r="K84" s="25"/>
-      <x:c r="L84" s="25"/>
+      <x:c r="A84" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B84" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C84" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D84" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E84" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F84" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G84" s="26" t="n">
+        <x:v>439019.8</x:v>
+      </x:c>
+      <x:c r="H84" s="26" t="n">
+        <x:v>449508.8</x:v>
+      </x:c>
+      <x:c r="I84" s="22" t="n">
+        <x:f>H84/G84</x:f>
+        <x:v>1.0238918609137901</x:v>
+      </x:c>
+      <x:c r="J84" s="24" t="n">
+        <x:v>19.806</x:v>
+      </x:c>
+      <x:c r="K84" s="24" t="n">
+        <x:v>20.707</x:v>
+      </x:c>
+      <x:c r="L84" s="24" t="n">
+        <x:f>K84/J84</x:f>
+        <x:v>1.0454912652731496</x:v>
+      </x:c>
+      <x:c r="M84" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N84" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O84" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P84" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q84" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R84" s="10" t="str">
+        <x:v>2d801160aa</x:v>
+      </x:c>
+      <x:c r="S84" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_171534_cpp-pubsub-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T84" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_171731_cpp-pubsub-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U84" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V84" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 98.15%; latency median ratio 1.06x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="85">
-      <x:c r="A85" s="29"/>
-      <x:c r="G85" s="27"/>
-      <x:c r="H85" s="27"/>
-      <x:c r="I85" s="23"/>
-      <x:c r="J85" s="25"/>
-      <x:c r="K85" s="25"/>
-      <x:c r="L85" s="25"/>
+      <x:c r="A85" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B85" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C85" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D85" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E85" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F85" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G85" s="26" t="n">
+        <x:v>26401</x:v>
+      </x:c>
+      <x:c r="H85" s="26" t="n">
+        <x:v>24892.2</x:v>
+      </x:c>
+      <x:c r="I85" s="22" t="n">
+        <x:f>H85/G85</x:f>
+        <x:v>0.9428506495966062</x:v>
+      </x:c>
+      <x:c r="J85" s="24" t="n">
+        <x:v>4.927</x:v>
+      </x:c>
+      <x:c r="K85" s="24" t="n">
+        <x:v>5.011</x:v>
+      </x:c>
+      <x:c r="L85" s="24" t="n">
+        <x:f>K85/J85</x:f>
+        <x:v>1.0170489141465395</x:v>
+      </x:c>
+      <x:c r="M85" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N85" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O85" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P85" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q85" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R85" s="10" t="str">
+        <x:v>2d801160aa</x:v>
+      </x:c>
+      <x:c r="S85" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_171534_cpp-pubsub-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T85" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_171731_cpp-pubsub-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U85" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V85" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 98.15%; latency median ratio 1.06x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="86">
-      <x:c r="A86" s="29"/>
-      <x:c r="G86" s="27"/>
-      <x:c r="H86" s="27"/>
-      <x:c r="I86" s="23"/>
-      <x:c r="J86" s="25"/>
-      <x:c r="K86" s="25"/>
-      <x:c r="L86" s="25"/>
+      <x:c r="A86" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B86" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C86" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D86" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E86" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F86" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G86" s="26" t="n">
+        <x:v>17165</x:v>
+      </x:c>
+      <x:c r="H86" s="26" t="n">
+        <x:v>17058.8</x:v>
+      </x:c>
+      <x:c r="I86" s="22" t="n">
+        <x:f>H86/G86</x:f>
+        <x:v>0.9938129915525779</x:v>
+      </x:c>
+      <x:c r="J86" s="24" t="n">
+        <x:v>4.268</x:v>
+      </x:c>
+      <x:c r="K86" s="24" t="n">
+        <x:v>4.561</x:v>
+      </x:c>
+      <x:c r="L86" s="24" t="n">
+        <x:f>K86/J86</x:f>
+        <x:v>1.0686504217432053</x:v>
+      </x:c>
+      <x:c r="M86" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N86" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O86" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P86" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q86" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R86" s="10" t="str">
+        <x:v>2d801160aa</x:v>
+      </x:c>
+      <x:c r="S86" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_171534_cpp-pubsub-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T86" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_171731_cpp-pubsub-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U86" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V86" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 98.15%; latency median ratio 1.06x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
-      <x:c r="A87" s="29"/>
-      <x:c r="G87" s="27"/>
-      <x:c r="H87" s="27"/>
-      <x:c r="I87" s="23"/>
-      <x:c r="J87" s="25"/>
-      <x:c r="K87" s="25"/>
-      <x:c r="L87" s="25"/>
+      <x:c r="A87" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B87" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C87" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D87" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E87" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F87" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G87" s="26" t="n">
+        <x:v>12246.6</x:v>
+      </x:c>
+      <x:c r="H87" s="26" t="n">
+        <x:v>11973.8</x:v>
+      </x:c>
+      <x:c r="I87" s="22" t="n">
+        <x:f>H87/G87</x:f>
+        <x:v>0.9777244296376136</x:v>
+      </x:c>
+      <x:c r="J87" s="24" t="n">
+        <x:v>0.34</x:v>
+      </x:c>
+      <x:c r="K87" s="24" t="n">
+        <x:v>0.349</x:v>
+      </x:c>
+      <x:c r="L87" s="24" t="n">
+        <x:f>K87/J87</x:f>
+        <x:v>1.026470588235294</x:v>
+      </x:c>
+      <x:c r="M87" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N87" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O87" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P87" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q87" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R87" s="10" t="str">
+        <x:v>2d801160aa</x:v>
+      </x:c>
+      <x:c r="S87" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_171534_cpp-pubsub-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T87" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_171731_cpp-pubsub-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U87" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V87" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 98.15%; latency median ratio 1.06x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="29"/>

</xml_diff>

<commit_message>
perf(cpp): record websocket dealer baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf8d606384803472f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R4319910a07614dc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R7a14e4aeb6fd4c53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R85cc3c4c20f2414c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf177656489f84831"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R8dd910bbfbeb44bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R714043588dd1446b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R9f5101185ada44fd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws PUBSUB 통과·PAIR strict 목표 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws PUBSUB·DEALER_DEALER 통과·PAIR strict 목표 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -6571,58 +6571,424 @@
       </x:c>
     </x:row>
     <x:row r="88">
-      <x:c r="A88" s="29"/>
-      <x:c r="G88" s="27"/>
-      <x:c r="H88" s="27"/>
-      <x:c r="I88" s="23"/>
-      <x:c r="J88" s="25"/>
-      <x:c r="K88" s="25"/>
-      <x:c r="L88" s="25"/>
+      <x:c r="A88" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B88" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C88" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D88" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E88" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F88" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G88" s="26" t="n">
+        <x:v>2675430</x:v>
+      </x:c>
+      <x:c r="H88" s="26" t="n">
+        <x:v>2195279</x:v>
+      </x:c>
+      <x:c r="I88" s="22" t="n">
+        <x:f>H88/G88</x:f>
+        <x:v>0.8205331479425737</x:v>
+      </x:c>
+      <x:c r="J88" s="24" t="n">
+        <x:v>35.663</x:v>
+      </x:c>
+      <x:c r="K88" s="24" t="n">
+        <x:v>38.792</x:v>
+      </x:c>
+      <x:c r="L88" s="24" t="n">
+        <x:f>K88/J88</x:f>
+        <x:v>1.087737991756162</x:v>
+      </x:c>
+      <x:c r="M88" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N88" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O88" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P88" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q88" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R88" s="10" t="str">
+        <x:v>fd9e53057b</x:v>
+      </x:c>
+      <x:c r="S88" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_172115_cpp-dealer-dealer-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T88" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_172252_cpp-dealer-dealer-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U88" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V88" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 94.78%; latency median ratio 1.03x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="89">
-      <x:c r="A89" s="29"/>
-      <x:c r="G89" s="27"/>
-      <x:c r="H89" s="27"/>
-      <x:c r="I89" s="23"/>
-      <x:c r="J89" s="25"/>
-      <x:c r="K89" s="25"/>
-      <x:c r="L89" s="25"/>
+      <x:c r="A89" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B89" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C89" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D89" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E89" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F89" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G89" s="26" t="n">
+        <x:v>1246048.2</x:v>
+      </x:c>
+      <x:c r="H89" s="26" t="n">
+        <x:v>1206152</x:v>
+      </x:c>
+      <x:c r="I89" s="22" t="n">
+        <x:f>H89/G89</x:f>
+        <x:v>0.9679818164337464</x:v>
+      </x:c>
+      <x:c r="J89" s="24" t="n">
+        <x:v>26.737</x:v>
+      </x:c>
+      <x:c r="K89" s="24" t="n">
+        <x:v>25.906</x:v>
+      </x:c>
+      <x:c r="L89" s="24" t="n">
+        <x:f>K89/J89</x:f>
+        <x:v>0.9689194748849909</x:v>
+      </x:c>
+      <x:c r="M89" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N89" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O89" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P89" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q89" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R89" s="10" t="str">
+        <x:v>fd9e53057b</x:v>
+      </x:c>
+      <x:c r="S89" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_172115_cpp-dealer-dealer-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T89" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_172252_cpp-dealer-dealer-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U89" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V89" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 94.78%; latency median ratio 1.03x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="90">
-      <x:c r="A90" s="29"/>
-      <x:c r="G90" s="27"/>
-      <x:c r="H90" s="27"/>
-      <x:c r="I90" s="23"/>
-      <x:c r="J90" s="25"/>
-      <x:c r="K90" s="25"/>
-      <x:c r="L90" s="25"/>
+      <x:c r="A90" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B90" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C90" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D90" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E90" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F90" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G90" s="26" t="n">
+        <x:v>460396.8</x:v>
+      </x:c>
+      <x:c r="H90" s="26" t="n">
+        <x:v>442304.2</x:v>
+      </x:c>
+      <x:c r="I90" s="22" t="n">
+        <x:f>H90/G90</x:f>
+        <x:v>0.9607021595284764</x:v>
+      </x:c>
+      <x:c r="J90" s="24" t="n">
+        <x:v>17.027</x:v>
+      </x:c>
+      <x:c r="K90" s="24" t="n">
+        <x:v>17.685</x:v>
+      </x:c>
+      <x:c r="L90" s="24" t="n">
+        <x:f>K90/J90</x:f>
+        <x:v>1.0386445057849296</x:v>
+      </x:c>
+      <x:c r="M90" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N90" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O90" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P90" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q90" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R90" s="10" t="str">
+        <x:v>fd9e53057b</x:v>
+      </x:c>
+      <x:c r="S90" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_172115_cpp-dealer-dealer-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T90" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_172252_cpp-dealer-dealer-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U90" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V90" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 94.78%; latency median ratio 1.03x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="91">
-      <x:c r="A91" s="29"/>
-      <x:c r="G91" s="27"/>
-      <x:c r="H91" s="27"/>
-      <x:c r="I91" s="23"/>
-      <x:c r="J91" s="25"/>
-      <x:c r="K91" s="25"/>
-      <x:c r="L91" s="25"/>
+      <x:c r="A91" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B91" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C91" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D91" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E91" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F91" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G91" s="26" t="n">
+        <x:v>22996.6</x:v>
+      </x:c>
+      <x:c r="H91" s="26" t="n">
+        <x:v>21830.8</x:v>
+      </x:c>
+      <x:c r="I91" s="22" t="n">
+        <x:f>H91/G91</x:f>
+        <x:v>0.9493055495160154</x:v>
+      </x:c>
+      <x:c r="J91" s="24" t="n">
+        <x:v>6.221</x:v>
+      </x:c>
+      <x:c r="K91" s="24" t="n">
+        <x:v>6.394</x:v>
+      </x:c>
+      <x:c r="L91" s="24" t="n">
+        <x:f>K91/J91</x:f>
+        <x:v>1.0278090339173767</x:v>
+      </x:c>
+      <x:c r="M91" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N91" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O91" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P91" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q91" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R91" s="10" t="str">
+        <x:v>fd9e53057b</x:v>
+      </x:c>
+      <x:c r="S91" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_172115_cpp-dealer-dealer-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T91" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_172252_cpp-dealer-dealer-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U91" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V91" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 94.78%; latency median ratio 1.03x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="92">
-      <x:c r="A92" s="29"/>
-      <x:c r="G92" s="27"/>
-      <x:c r="H92" s="27"/>
-      <x:c r="I92" s="23"/>
-      <x:c r="J92" s="25"/>
-      <x:c r="K92" s="25"/>
-      <x:c r="L92" s="25"/>
+      <x:c r="A92" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B92" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C92" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D92" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E92" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F92" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G92" s="26" t="n">
+        <x:v>15332.6</x:v>
+      </x:c>
+      <x:c r="H92" s="26" t="n">
+        <x:v>15078</x:v>
+      </x:c>
+      <x:c r="I92" s="22" t="n">
+        <x:f>H92/G92</x:f>
+        <x:v>0.9833948580149485</x:v>
+      </x:c>
+      <x:c r="J92" s="24" t="n">
+        <x:v>0.386</x:v>
+      </x:c>
+      <x:c r="K92" s="24" t="n">
+        <x:v>0.403</x:v>
+      </x:c>
+      <x:c r="L92" s="24" t="n">
+        <x:f>K92/J92</x:f>
+        <x:v>1.044041450777202</x:v>
+      </x:c>
+      <x:c r="M92" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N92" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O92" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P92" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q92" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R92" s="10" t="str">
+        <x:v>fd9e53057b</x:v>
+      </x:c>
+      <x:c r="S92" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_172115_cpp-dealer-dealer-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T92" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_172252_cpp-dealer-dealer-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U92" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V92" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 94.78%; latency median ratio 1.03x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="93">
-      <x:c r="A93" s="29"/>
-      <x:c r="G93" s="27"/>
-      <x:c r="H93" s="27"/>
-      <x:c r="I93" s="23"/>
-      <x:c r="J93" s="25"/>
-      <x:c r="K93" s="25"/>
-      <x:c r="L93" s="25"/>
+      <x:c r="A93" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B93" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C93" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D93" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E93" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F93" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G93" s="26" t="n">
+        <x:v>9568</x:v>
+      </x:c>
+      <x:c r="H93" s="26" t="n">
+        <x:v>9617.2</x:v>
+      </x:c>
+      <x:c r="I93" s="22" t="n">
+        <x:f>H93/G93</x:f>
+        <x:v>1.0051421404682275</x:v>
+      </x:c>
+      <x:c r="J93" s="24" t="n">
+        <x:v>0.433</x:v>
+      </x:c>
+      <x:c r="K93" s="24" t="n">
+        <x:v>0.427</x:v>
+      </x:c>
+      <x:c r="L93" s="24" t="n">
+        <x:f>K93/J93</x:f>
+        <x:v>0.9861431870669746</x:v>
+      </x:c>
+      <x:c r="M93" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N93" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O93" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P93" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q93" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R93" s="10" t="str">
+        <x:v>fd9e53057b</x:v>
+      </x:c>
+      <x:c r="S93" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_172115_cpp-dealer-dealer-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T93" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_172252_cpp-dealer-dealer-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U93" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V93" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 94.78%; latency median ratio 1.03x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="29"/>

</xml_diff>

<commit_message>
perf(cpp): record websocket dealer router baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf177656489f84831"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R8dd910bbfbeb44bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R714043588dd1446b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R9f5101185ada44fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6ede1aedf2fb4efd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Re60bc0e3bffa400b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R364a643c53ae4928"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R63b977581e3443a8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws PUBSUB·DEALER_DEALER 통과·PAIR strict 목표 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws PUBSUB·DEALER_* 통과·PAIR strict 목표 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -6991,58 +6991,424 @@
       </x:c>
     </x:row>
     <x:row r="94">
-      <x:c r="A94" s="29"/>
-      <x:c r="G94" s="27"/>
-      <x:c r="H94" s="27"/>
-      <x:c r="I94" s="23"/>
-      <x:c r="J94" s="25"/>
-      <x:c r="K94" s="25"/>
-      <x:c r="L94" s="25"/>
+      <x:c r="A94" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B94" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C94" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D94" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E94" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F94" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G94" s="26" t="n">
+        <x:v>2760776.6</x:v>
+      </x:c>
+      <x:c r="H94" s="26" t="n">
+        <x:v>2176032.6</x:v>
+      </x:c>
+      <x:c r="I94" s="22" t="n">
+        <x:f>H94/G94</x:f>
+        <x:v>0.7881958286664702</x:v>
+      </x:c>
+      <x:c r="J94" s="24" t="n">
+        <x:v>33.687</x:v>
+      </x:c>
+      <x:c r="K94" s="24" t="n">
+        <x:v>40.434</x:v>
+      </x:c>
+      <x:c r="L94" s="24" t="n">
+        <x:f>K94/J94</x:f>
+        <x:v>1.2002849764003918</x:v>
+      </x:c>
+      <x:c r="M94" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N94" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O94" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P94" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q94" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R94" s="10" t="str">
+        <x:v>e230fdb9c2</x:v>
+      </x:c>
+      <x:c r="S94" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_172620_cpp-dealer-router-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T94" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_172759_cpp-dealer-router-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U94" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V94" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.94%; latency median ratio 1.07x; pass. 64B is an individual outlier below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="95">
-      <x:c r="A95" s="29"/>
-      <x:c r="G95" s="27"/>
-      <x:c r="H95" s="27"/>
-      <x:c r="I95" s="23"/>
-      <x:c r="J95" s="25"/>
-      <x:c r="K95" s="25"/>
-      <x:c r="L95" s="25"/>
+      <x:c r="A95" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B95" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C95" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D95" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E95" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F95" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G95" s="26" t="n">
+        <x:v>1312397.4</x:v>
+      </x:c>
+      <x:c r="H95" s="26" t="n">
+        <x:v>1257607.8</x:v>
+      </x:c>
+      <x:c r="I95" s="22" t="n">
+        <x:f>H95/G95</x:f>
+        <x:v>0.9582522793781824</x:v>
+      </x:c>
+      <x:c r="J95" s="24" t="n">
+        <x:v>24.212</x:v>
+      </x:c>
+      <x:c r="K95" s="24" t="n">
+        <x:v>27.502</x:v>
+      </x:c>
+      <x:c r="L95" s="24" t="n">
+        <x:f>K95/J95</x:f>
+        <x:v>1.1358830332066743</x:v>
+      </x:c>
+      <x:c r="M95" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N95" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O95" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P95" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q95" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R95" s="10" t="str">
+        <x:v>e230fdb9c2</x:v>
+      </x:c>
+      <x:c r="S95" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_172620_cpp-dealer-router-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T95" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_172759_cpp-dealer-router-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U95" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V95" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.94%; latency median ratio 1.07x; pass. 64B is an individual outlier below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="96">
-      <x:c r="A96" s="29"/>
-      <x:c r="G96" s="27"/>
-      <x:c r="H96" s="27"/>
-      <x:c r="I96" s="23"/>
-      <x:c r="J96" s="25"/>
-      <x:c r="K96" s="25"/>
-      <x:c r="L96" s="25"/>
+      <x:c r="A96" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B96" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C96" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D96" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E96" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F96" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G96" s="26" t="n">
+        <x:v>467308</x:v>
+      </x:c>
+      <x:c r="H96" s="26" t="n">
+        <x:v>470631.2</x:v>
+      </x:c>
+      <x:c r="I96" s="22" t="n">
+        <x:f>H96/G96</x:f>
+        <x:v>1.0071113698032133</x:v>
+      </x:c>
+      <x:c r="J96" s="24" t="n">
+        <x:v>17.349</x:v>
+      </x:c>
+      <x:c r="K96" s="24" t="n">
+        <x:v>17.31</x:v>
+      </x:c>
+      <x:c r="L96" s="24" t="n">
+        <x:f>K96/J96</x:f>
+        <x:v>0.9977520318173957</x:v>
+      </x:c>
+      <x:c r="M96" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N96" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O96" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P96" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q96" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R96" s="10" t="str">
+        <x:v>e230fdb9c2</x:v>
+      </x:c>
+      <x:c r="S96" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_172620_cpp-dealer-router-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T96" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_172759_cpp-dealer-router-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U96" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V96" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.94%; latency median ratio 1.07x; pass. 64B is an individual outlier below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="97">
-      <x:c r="A97" s="29"/>
-      <x:c r="G97" s="27"/>
-      <x:c r="H97" s="27"/>
-      <x:c r="I97" s="23"/>
-      <x:c r="J97" s="25"/>
-      <x:c r="K97" s="25"/>
-      <x:c r="L97" s="25"/>
+      <x:c r="A97" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B97" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C97" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D97" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E97" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F97" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G97" s="26" t="n">
+        <x:v>23448.2</x:v>
+      </x:c>
+      <x:c r="H97" s="26" t="n">
+        <x:v>23009.6</x:v>
+      </x:c>
+      <x:c r="I97" s="22" t="n">
+        <x:f>H97/G97</x:f>
+        <x:v>0.9812949394836277</x:v>
+      </x:c>
+      <x:c r="J97" s="24" t="n">
+        <x:v>5.311</x:v>
+      </x:c>
+      <x:c r="K97" s="24" t="n">
+        <x:v>6.343</x:v>
+      </x:c>
+      <x:c r="L97" s="24" t="n">
+        <x:f>K97/J97</x:f>
+        <x:v>1.1943136885708907</x:v>
+      </x:c>
+      <x:c r="M97" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N97" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O97" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P97" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q97" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R97" s="10" t="str">
+        <x:v>e230fdb9c2</x:v>
+      </x:c>
+      <x:c r="S97" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_172620_cpp-dealer-router-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T97" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_172759_cpp-dealer-router-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U97" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V97" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.94%; latency median ratio 1.07x; pass. 64B is an individual outlier below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="98">
-      <x:c r="A98" s="29"/>
-      <x:c r="G98" s="27"/>
-      <x:c r="H98" s="27"/>
-      <x:c r="I98" s="23"/>
-      <x:c r="J98" s="25"/>
-      <x:c r="K98" s="25"/>
-      <x:c r="L98" s="25"/>
+      <x:c r="A98" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B98" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C98" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D98" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E98" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F98" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G98" s="26" t="n">
+        <x:v>15187</x:v>
+      </x:c>
+      <x:c r="H98" s="26" t="n">
+        <x:v>15515</x:v>
+      </x:c>
+      <x:c r="I98" s="22" t="n">
+        <x:f>H98/G98</x:f>
+        <x:v>1.021597418845065</x:v>
+      </x:c>
+      <x:c r="J98" s="24" t="n">
+        <x:v>0.418</x:v>
+      </x:c>
+      <x:c r="K98" s="24" t="n">
+        <x:v>0.411</x:v>
+      </x:c>
+      <x:c r="L98" s="24" t="n">
+        <x:f>K98/J98</x:f>
+        <x:v>0.9832535885167464</x:v>
+      </x:c>
+      <x:c r="M98" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N98" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O98" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P98" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q98" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R98" s="10" t="str">
+        <x:v>e230fdb9c2</x:v>
+      </x:c>
+      <x:c r="S98" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_172620_cpp-dealer-router-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T98" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_172759_cpp-dealer-router-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U98" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V98" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.94%; latency median ratio 1.07x; pass. 64B is an individual outlier below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="99">
-      <x:c r="A99" s="29"/>
-      <x:c r="G99" s="27"/>
-      <x:c r="H99" s="27"/>
-      <x:c r="I99" s="23"/>
-      <x:c r="J99" s="25"/>
-      <x:c r="K99" s="25"/>
-      <x:c r="L99" s="25"/>
+      <x:c r="A99" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B99" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C99" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D99" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E99" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F99" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G99" s="26" t="n">
+        <x:v>9513.4</x:v>
+      </x:c>
+      <x:c r="H99" s="26" t="n">
+        <x:v>9514.6</x:v>
+      </x:c>
+      <x:c r="I99" s="22" t="n">
+        <x:f>H99/G99</x:f>
+        <x:v>1.0001261378686905</x:v>
+      </x:c>
+      <x:c r="J99" s="24" t="n">
+        <x:v>0.436</x:v>
+      </x:c>
+      <x:c r="K99" s="24" t="n">
+        <x:v>0.436</x:v>
+      </x:c>
+      <x:c r="L99" s="24" t="n">
+        <x:f>K99/J99</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M99" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N99" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O99" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P99" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q99" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R99" s="10" t="str">
+        <x:v>e230fdb9c2</x:v>
+      </x:c>
+      <x:c r="S99" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_172620_cpp-dealer-router-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T99" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_172759_cpp-dealer-router-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U99" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V99" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.94%; latency median ratio 1.07x; pass. 64B is an individual outlier below 80%.</x:v>
+      </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="29"/>

</xml_diff>

<commit_message>
perf(cpp): record websocket dealer request baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6ede1aedf2fb4efd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Re60bc0e3bffa400b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R364a643c53ae4928"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R63b977581e3443a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra813bc036b6e4844"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rdb77654c8f3f4445"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R047a740e71914b9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R09a7ce42ea7b4b91"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws PUBSUB·DEALER_* 통과·PAIR strict 목표 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws PUBSUB·DEALER one-way 통과·PAIR/REQREP 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -7411,112 +7411,844 @@
       </x:c>
     </x:row>
     <x:row r="100">
-      <x:c r="A100" s="29"/>
-      <x:c r="G100" s="27"/>
-      <x:c r="H100" s="27"/>
-      <x:c r="I100" s="23"/>
-      <x:c r="J100" s="25"/>
-      <x:c r="K100" s="25"/>
-      <x:c r="L100" s="25"/>
+      <x:c r="A100" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B100" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C100" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D100" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E100" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F100" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G100" s="26" t="n">
+        <x:v>189770.8</x:v>
+      </x:c>
+      <x:c r="H100" s="26" t="n">
+        <x:v>47598.4</x:v>
+      </x:c>
+      <x:c r="I100" s="22" t="n">
+        <x:f>H100/G100</x:f>
+        <x:v>0.25082046342219144</x:v>
+      </x:c>
+      <x:c r="J100" s="24" t="n">
+        <x:v>0.291</x:v>
+      </x:c>
+      <x:c r="K100" s="24" t="n">
+        <x:v>1.309</x:v>
+      </x:c>
+      <x:c r="L100" s="24" t="n">
+        <x:f>K100/J100</x:f>
+        <x:v>4.498281786941581</x:v>
+      </x:c>
+      <x:c r="M100" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N100" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O100" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P100" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q100" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R100" s="10" t="str">
+        <x:v>70b7606b4a</x:v>
+      </x:c>
+      <x:c r="S100" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_173116_cpp-dealer-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T100" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173254_cpp-dealer-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U100" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V100" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 58.34%; latency median ratio 2.19x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="101">
-      <x:c r="A101" s="29"/>
-      <x:c r="G101" s="27"/>
-      <x:c r="H101" s="27"/>
-      <x:c r="I101" s="23"/>
-      <x:c r="J101" s="25"/>
-      <x:c r="K101" s="25"/>
-      <x:c r="L101" s="25"/>
+      <x:c r="A101" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B101" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C101" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D101" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E101" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F101" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G101" s="26" t="n">
+        <x:v>137622.8</x:v>
+      </x:c>
+      <x:c r="H101" s="26" t="n">
+        <x:v>39663.2</x:v>
+      </x:c>
+      <x:c r="I101" s="22" t="n">
+        <x:f>H101/G101</x:f>
+        <x:v>0.2882022455581488</x:v>
+      </x:c>
+      <x:c r="J101" s="24" t="n">
+        <x:v>0.433</x:v>
+      </x:c>
+      <x:c r="K101" s="24" t="n">
+        <x:v>1.581</x:v>
+      </x:c>
+      <x:c r="L101" s="24" t="n">
+        <x:f>K101/J101</x:f>
+        <x:v>3.651270207852194</x:v>
+      </x:c>
+      <x:c r="M101" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N101" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O101" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P101" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q101" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R101" s="10" t="str">
+        <x:v>70b7606b4a</x:v>
+      </x:c>
+      <x:c r="S101" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_173116_cpp-dealer-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T101" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173254_cpp-dealer-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U101" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V101" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 58.34%; latency median ratio 2.19x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="102">
-      <x:c r="A102" s="29"/>
-      <x:c r="G102" s="27"/>
-      <x:c r="H102" s="27"/>
-      <x:c r="I102" s="23"/>
-      <x:c r="J102" s="25"/>
-      <x:c r="K102" s="25"/>
-      <x:c r="L102" s="25"/>
+      <x:c r="A102" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B102" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C102" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D102" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E102" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F102" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G102" s="26" t="n">
+        <x:v>79820.4</x:v>
+      </x:c>
+      <x:c r="H102" s="26" t="n">
+        <x:v>25328</x:v>
+      </x:c>
+      <x:c r="I102" s="22" t="n">
+        <x:f>H102/G102</x:f>
+        <x:v>0.3173123662622588</x:v>
+      </x:c>
+      <x:c r="J102" s="24" t="n">
+        <x:v>0.784</x:v>
+      </x:c>
+      <x:c r="K102" s="24" t="n">
+        <x:v>2.501</x:v>
+      </x:c>
+      <x:c r="L102" s="24" t="n">
+        <x:f>K102/J102</x:f>
+        <x:v>3.190051020408163</x:v>
+      </x:c>
+      <x:c r="M102" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N102" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O102" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P102" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q102" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R102" s="10" t="str">
+        <x:v>70b7606b4a</x:v>
+      </x:c>
+      <x:c r="S102" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_173116_cpp-dealer-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T102" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173254_cpp-dealer-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U102" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V102" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 58.34%; latency median ratio 2.19x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="103">
-      <x:c r="A103" s="29"/>
-      <x:c r="G103" s="27"/>
-      <x:c r="H103" s="27"/>
-      <x:c r="I103" s="23"/>
-      <x:c r="J103" s="25"/>
-      <x:c r="K103" s="25"/>
-      <x:c r="L103" s="25"/>
+      <x:c r="A103" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B103" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C103" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D103" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E103" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F103" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G103" s="26" t="n">
+        <x:v>11413.6</x:v>
+      </x:c>
+      <x:c r="H103" s="26" t="n">
+        <x:v>9745.6</x:v>
+      </x:c>
+      <x:c r="I103" s="22" t="n">
+        <x:f>H103/G103</x:f>
+        <x:v>0.8538585547066657</x:v>
+      </x:c>
+      <x:c r="J103" s="24" t="n">
+        <x:v>1.046</x:v>
+      </x:c>
+      <x:c r="K103" s="24" t="n">
+        <x:v>1.214</x:v>
+      </x:c>
+      <x:c r="L103" s="24" t="n">
+        <x:f>K103/J103</x:f>
+        <x:v>1.1606118546845123</x:v>
+      </x:c>
+      <x:c r="M103" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N103" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O103" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P103" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q103" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R103" s="10" t="str">
+        <x:v>70b7606b4a</x:v>
+      </x:c>
+      <x:c r="S103" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_173116_cpp-dealer-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T103" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173254_cpp-dealer-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U103" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V103" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 58.34%; latency median ratio 2.19x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="104">
-      <x:c r="A104" s="29"/>
-      <x:c r="G104" s="27"/>
-      <x:c r="H104" s="27"/>
-      <x:c r="I104" s="23"/>
-      <x:c r="J104" s="25"/>
-      <x:c r="K104" s="25"/>
-      <x:c r="L104" s="25"/>
+      <x:c r="A104" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B104" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C104" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D104" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E104" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F104" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G104" s="26" t="n">
+        <x:v>7906.6</x:v>
+      </x:c>
+      <x:c r="H104" s="26" t="n">
+        <x:v>7050.8</x:v>
+      </x:c>
+      <x:c r="I104" s="22" t="n">
+        <x:f>H104/G104</x:f>
+        <x:v>0.8917613133331647</x:v>
+      </x:c>
+      <x:c r="J104" s="24" t="n">
+        <x:v>0.769</x:v>
+      </x:c>
+      <x:c r="K104" s="24" t="n">
+        <x:v>0.919</x:v>
+      </x:c>
+      <x:c r="L104" s="24" t="n">
+        <x:f>K104/J104</x:f>
+        <x:v>1.1950585175552666</x:v>
+      </x:c>
+      <x:c r="M104" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N104" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O104" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P104" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q104" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R104" s="10" t="str">
+        <x:v>70b7606b4a</x:v>
+      </x:c>
+      <x:c r="S104" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_173116_cpp-dealer-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T104" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173254_cpp-dealer-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U104" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V104" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 58.34%; latency median ratio 2.19x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="105">
-      <x:c r="A105" s="29"/>
-      <x:c r="G105" s="27"/>
-      <x:c r="H105" s="27"/>
-      <x:c r="I105" s="23"/>
-      <x:c r="J105" s="25"/>
-      <x:c r="K105" s="25"/>
-      <x:c r="L105" s="25"/>
+      <x:c r="A105" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B105" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C105" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D105" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E105" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F105" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G105" s="26" t="n">
+        <x:v>5200</x:v>
+      </x:c>
+      <x:c r="H105" s="26" t="n">
+        <x:v>4672.6</x:v>
+      </x:c>
+      <x:c r="I105" s="22" t="n">
+        <x:f>H105/G105</x:f>
+        <x:v>0.8985769230769232</x:v>
+      </x:c>
+      <x:c r="J105" s="24" t="n">
+        <x:v>0.574</x:v>
+      </x:c>
+      <x:c r="K105" s="24" t="n">
+        <x:v>0.623</x:v>
+      </x:c>
+      <x:c r="L105" s="24" t="n">
+        <x:f>K105/J105</x:f>
+        <x:v>1.0853658536585367</x:v>
+      </x:c>
+      <x:c r="M105" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N105" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O105" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P105" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q105" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R105" s="10" t="str">
+        <x:v>70b7606b4a</x:v>
+      </x:c>
+      <x:c r="S105" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_173116_cpp-dealer-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T105" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173254_cpp-dealer-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U105" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V105" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 58.34%; latency median ratio 2.19x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="106">
-      <x:c r="A106" s="29"/>
-      <x:c r="G106" s="27"/>
-      <x:c r="H106" s="27"/>
-      <x:c r="I106" s="23"/>
-      <x:c r="J106" s="25"/>
-      <x:c r="K106" s="25"/>
-      <x:c r="L106" s="25"/>
+      <x:c r="A106" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B106" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C106" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D106" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E106" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F106" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G106" s="26" t="n">
+        <x:v>189770.8</x:v>
+      </x:c>
+      <x:c r="H106" s="26" t="n">
+        <x:v>45362.6</x:v>
+      </x:c>
+      <x:c r="I106" s="22" t="n">
+        <x:f>H106/G106</x:f>
+        <x:v>0.23903888269428175</x:v>
+      </x:c>
+      <x:c r="J106" s="24" t="n">
+        <x:v>0.291</x:v>
+      </x:c>
+      <x:c r="K106" s="24" t="n">
+        <x:v>1.334</x:v>
+      </x:c>
+      <x:c r="L106" s="24" t="n">
+        <x:f>K106/J106</x:f>
+        <x:v>4.5841924398625435</x:v>
+      </x:c>
+      <x:c r="M106" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N106" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O106" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P106" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q106" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R106" s="10" t="str">
+        <x:v>70b7606b4a</x:v>
+      </x:c>
+      <x:c r="S106" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_173116_cpp-dealer-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T106" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173741_cpp-dealer-router-reqrep-ws-local0132-candidate-b-async-bridge-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U106" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V106" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 54.58%; latency median ratio 2.38x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="107">
-      <x:c r="A107" s="29"/>
-      <x:c r="G107" s="27"/>
-      <x:c r="H107" s="27"/>
-      <x:c r="I107" s="23"/>
-      <x:c r="J107" s="25"/>
-      <x:c r="K107" s="25"/>
-      <x:c r="L107" s="25"/>
+      <x:c r="A107" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B107" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C107" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D107" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E107" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F107" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G107" s="26" t="n">
+        <x:v>137622.8</x:v>
+      </x:c>
+      <x:c r="H107" s="26" t="n">
+        <x:v>38713.6</x:v>
+      </x:c>
+      <x:c r="I107" s="22" t="n">
+        <x:f>H107/G107</x:f>
+        <x:v>0.28130222608463135</x:v>
+      </x:c>
+      <x:c r="J107" s="24" t="n">
+        <x:v>0.433</x:v>
+      </x:c>
+      <x:c r="K107" s="24" t="n">
+        <x:v>1.622</x:v>
+      </x:c>
+      <x:c r="L107" s="24" t="n">
+        <x:f>K107/J107</x:f>
+        <x:v>3.745958429561201</x:v>
+      </x:c>
+      <x:c r="M107" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N107" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O107" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P107" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q107" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R107" s="10" t="str">
+        <x:v>70b7606b4a</x:v>
+      </x:c>
+      <x:c r="S107" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_173116_cpp-dealer-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T107" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173741_cpp-dealer-router-reqrep-ws-local0132-candidate-b-async-bridge-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U107" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V107" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 54.58%; latency median ratio 2.38x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="108">
-      <x:c r="A108" s="29"/>
-      <x:c r="G108" s="27"/>
-      <x:c r="H108" s="27"/>
-      <x:c r="I108" s="23"/>
-      <x:c r="J108" s="25"/>
-      <x:c r="K108" s="25"/>
-      <x:c r="L108" s="25"/>
+      <x:c r="A108" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B108" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C108" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D108" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E108" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F108" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G108" s="26" t="n">
+        <x:v>79820.4</x:v>
+      </x:c>
+      <x:c r="H108" s="26" t="n">
+        <x:v>25503.6</x:v>
+      </x:c>
+      <x:c r="I108" s="22" t="n">
+        <x:f>H108/G108</x:f>
+        <x:v>0.31951230512500567</x:v>
+      </x:c>
+      <x:c r="J108" s="24" t="n">
+        <x:v>0.784</x:v>
+      </x:c>
+      <x:c r="K108" s="24" t="n">
+        <x:v>2.688</x:v>
+      </x:c>
+      <x:c r="L108" s="24" t="n">
+        <x:f>K108/J108</x:f>
+        <x:v>3.428571428571429</x:v>
+      </x:c>
+      <x:c r="M108" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N108" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O108" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P108" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q108" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R108" s="10" t="str">
+        <x:v>70b7606b4a</x:v>
+      </x:c>
+      <x:c r="S108" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_173116_cpp-dealer-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T108" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173741_cpp-dealer-router-reqrep-ws-local0132-candidate-b-async-bridge-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U108" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V108" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 54.58%; latency median ratio 2.38x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="109">
-      <x:c r="A109" s="29"/>
-      <x:c r="G109" s="27"/>
-      <x:c r="H109" s="27"/>
-      <x:c r="I109" s="23"/>
-      <x:c r="J109" s="25"/>
-      <x:c r="K109" s="25"/>
-      <x:c r="L109" s="25"/>
+      <x:c r="A109" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B109" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C109" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D109" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E109" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F109" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G109" s="26" t="n">
+        <x:v>11413.6</x:v>
+      </x:c>
+      <x:c r="H109" s="26" t="n">
+        <x:v>8491</x:v>
+      </x:c>
+      <x:c r="I109" s="22" t="n">
+        <x:f>H109/G109</x:f>
+        <x:v>0.7439370575453844</x:v>
+      </x:c>
+      <x:c r="J109" s="24" t="n">
+        <x:v>1.046</x:v>
+      </x:c>
+      <x:c r="K109" s="24" t="n">
+        <x:v>1.382</x:v>
+      </x:c>
+      <x:c r="L109" s="24" t="n">
+        <x:f>K109/J109</x:f>
+        <x:v>1.3212237093690247</x:v>
+      </x:c>
+      <x:c r="M109" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N109" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O109" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P109" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q109" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R109" s="10" t="str">
+        <x:v>70b7606b4a</x:v>
+      </x:c>
+      <x:c r="S109" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_173116_cpp-dealer-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T109" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173741_cpp-dealer-router-reqrep-ws-local0132-candidate-b-async-bridge-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U109" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V109" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 54.58%; latency median ratio 2.38x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="110">
-      <x:c r="A110" s="29"/>
-      <x:c r="G110" s="27"/>
-      <x:c r="H110" s="27"/>
-      <x:c r="I110" s="23"/>
-      <x:c r="J110" s="25"/>
-      <x:c r="K110" s="25"/>
-      <x:c r="L110" s="25"/>
+      <x:c r="A110" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B110" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C110" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D110" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E110" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F110" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G110" s="26" t="n">
+        <x:v>7906.6</x:v>
+      </x:c>
+      <x:c r="H110" s="26" t="n">
+        <x:v>6843</x:v>
+      </x:c>
+      <x:c r="I110" s="22" t="n">
+        <x:f>H110/G110</x:f>
+        <x:v>0.8654794728454709</x:v>
+      </x:c>
+      <x:c r="J110" s="24" t="n">
+        <x:v>0.769</x:v>
+      </x:c>
+      <x:c r="K110" s="24" t="n">
+        <x:v>0.857</x:v>
+      </x:c>
+      <x:c r="L110" s="24" t="n">
+        <x:f>K110/J110</x:f>
+        <x:v>1.1144343302990898</x:v>
+      </x:c>
+      <x:c r="M110" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N110" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O110" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P110" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q110" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R110" s="10" t="str">
+        <x:v>70b7606b4a</x:v>
+      </x:c>
+      <x:c r="S110" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_173116_cpp-dealer-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T110" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173741_cpp-dealer-router-reqrep-ws-local0132-candidate-b-async-bridge-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U110" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V110" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 54.58%; latency median ratio 2.38x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="111">
-      <x:c r="A111" s="29"/>
-      <x:c r="G111" s="27"/>
-      <x:c r="H111" s="27"/>
-      <x:c r="I111" s="23"/>
-      <x:c r="J111" s="25"/>
-      <x:c r="K111" s="25"/>
-      <x:c r="L111" s="25"/>
+      <x:c r="A111" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B111" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C111" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D111" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E111" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F111" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G111" s="26" t="n">
+        <x:v>5200</x:v>
+      </x:c>
+      <x:c r="H111" s="26" t="n">
+        <x:v>4294</x:v>
+      </x:c>
+      <x:c r="I111" s="22" t="n">
+        <x:f>H111/G111</x:f>
+        <x:v>0.8257692307692308</x:v>
+      </x:c>
+      <x:c r="J111" s="24" t="n">
+        <x:v>0.574</x:v>
+      </x:c>
+      <x:c r="K111" s="24" t="n">
+        <x:v>0.677</x:v>
+      </x:c>
+      <x:c r="L111" s="24" t="n">
+        <x:f>K111/J111</x:f>
+        <x:v>1.1794425087108016</x:v>
+      </x:c>
+      <x:c r="M111" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N111" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O111" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P111" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q111" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R111" s="10" t="str">
+        <x:v>70b7606b4a</x:v>
+      </x:c>
+      <x:c r="S111" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_173116_cpp-dealer-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T111" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173741_cpp-dealer-router-reqrep-ws-local0132-candidate-b-async-bridge-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U111" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V111" s="10" t="str">
+        <x:v>Candidate B: throughput aggregate mean 54.58%; latency median ratio 2.38x; reject for regression.</x:v>
+      </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="29"/>
@@ -10553,12 +11285,90 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="L12" s="23"/>
-      <x:c r="M12" s="23"/>
+      <x:c r="A12" s="10" t="str">
+        <x:v>2026-08-25 17:34</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C12" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D12" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="str">
+        <x:v>ws</x:v>
+      </x:c>
+      <x:c r="F12" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G12" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H12" s="10" t="str">
+        <x:v>Use Core default DEALER request selection for single-part shallow views, avoiding exact transport-pair selection.</x:v>
+      </x:c>
+      <x:c r="I12" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J12" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173254_cpp-dealer-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K12" s="10" t="str">
+        <x:v>N/A — contract failed</x:v>
+      </x:c>
+      <x:c r="L12" s="22" t="n">
+        <x:v>0.583</x:v>
+      </x:c>
+      <x:c r="M12" s="22"/>
+      <x:c r="N12" s="10" t="str">
+        <x:v>REJECT before benchmark: initial routed target absence no longer reports not_connected terminal; public contract test failed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="L13" s="23"/>
-      <x:c r="M13" s="23"/>
+      <x:c r="A13" s="10" t="str">
+        <x:v>2026-08-25 17:37</x:v>
+      </x:c>
+      <x:c r="B13" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C13" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D13" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E13" s="10" t="str">
+        <x:v>ws</x:v>
+      </x:c>
+      <x:c r="F13" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G13" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H13" s="10" t="str">
+        <x:v>Use async-only completion bridge and delegate terminal synchronization to async_operation_state_t.</x:v>
+      </x:c>
+      <x:c r="I13" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J13" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173254_cpp-dealer-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K13" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_173741_cpp-dealer-router-reqrep-ws-local0132-candidate-b-async-bridge-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L13" s="22" t="n">
+        <x:v>0.583</x:v>
+      </x:c>
+      <x:c r="M13" s="22" t="n">
+        <x:v>0.546</x:v>
+      </x:c>
+      <x:c r="N13" s="10" t="str">
+        <x:v>REJECT: aggregate and latency regressed. Contract tests passed; source removed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="L14" s="23"/>

</xml_diff>

<commit_message>
perf(cpp): record websocket router baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra813bc036b6e4844"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rdb77654c8f3f4445"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R047a740e71914b9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R09a7ce42ea7b4b91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rdd95f36d52674d17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rcfa2326f284947e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R0ed162c1b71f4477"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R0a7d0acd28e14eb1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws PUBSUB·DEALER one-way 통과·PAIR/REQREP 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 4개 one-way 통과·PAIR/DEALER_REQREP 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -8251,58 +8251,424 @@
       </x:c>
     </x:row>
     <x:row r="112">
-      <x:c r="A112" s="29"/>
-      <x:c r="G112" s="27"/>
-      <x:c r="H112" s="27"/>
-      <x:c r="I112" s="23"/>
-      <x:c r="J112" s="25"/>
-      <x:c r="K112" s="25"/>
-      <x:c r="L112" s="25"/>
+      <x:c r="A112" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B112" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C112" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D112" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E112" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F112" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G112" s="26" t="n">
+        <x:v>2138983</x:v>
+      </x:c>
+      <x:c r="H112" s="26" t="n">
+        <x:v>1836904.6</x:v>
+      </x:c>
+      <x:c r="I112" s="22" t="n">
+        <x:f>H112/G112</x:f>
+        <x:v>0.8587747541705568</x:v>
+      </x:c>
+      <x:c r="J112" s="24" t="n">
+        <x:v>46.836</x:v>
+      </x:c>
+      <x:c r="K112" s="24" t="n">
+        <x:v>49.54</x:v>
+      </x:c>
+      <x:c r="L112" s="24" t="n">
+        <x:f>K112/J112</x:f>
+        <x:v>1.0577333674950893</x:v>
+      </x:c>
+      <x:c r="M112" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N112" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O112" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P112" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q112" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R112" s="10" t="str">
+        <x:v>f3660efe6f</x:v>
+      </x:c>
+      <x:c r="S112" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174322_cpp-router-router-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T112" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_174501_cpp-router-router-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U112" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V112" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.09%; latency median ratio 1.08x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="113">
-      <x:c r="A113" s="29"/>
-      <x:c r="G113" s="27"/>
-      <x:c r="H113" s="27"/>
-      <x:c r="I113" s="23"/>
-      <x:c r="J113" s="25"/>
-      <x:c r="K113" s="25"/>
-      <x:c r="L113" s="25"/>
+      <x:c r="A113" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B113" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C113" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D113" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E113" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F113" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G113" s="26" t="n">
+        <x:v>1156319.2</x:v>
+      </x:c>
+      <x:c r="H113" s="26" t="n">
+        <x:v>1183093.2</x:v>
+      </x:c>
+      <x:c r="I113" s="22" t="n">
+        <x:f>H113/G113</x:f>
+        <x:v>1.0231545061259901</x:v>
+      </x:c>
+      <x:c r="J113" s="24" t="n">
+        <x:v>28.408</x:v>
+      </x:c>
+      <x:c r="K113" s="24" t="n">
+        <x:v>26.356</x:v>
+      </x:c>
+      <x:c r="L113" s="24" t="n">
+        <x:f>K113/J113</x:f>
+        <x:v>0.9277668262461278</x:v>
+      </x:c>
+      <x:c r="M113" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N113" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O113" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P113" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q113" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R113" s="10" t="str">
+        <x:v>f3660efe6f</x:v>
+      </x:c>
+      <x:c r="S113" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174322_cpp-router-router-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T113" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_174501_cpp-router-router-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U113" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V113" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.09%; latency median ratio 1.08x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="114">
-      <x:c r="A114" s="29"/>
-      <x:c r="G114" s="27"/>
-      <x:c r="H114" s="27"/>
-      <x:c r="I114" s="23"/>
-      <x:c r="J114" s="25"/>
-      <x:c r="K114" s="25"/>
-      <x:c r="L114" s="25"/>
+      <x:c r="A114" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B114" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C114" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D114" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E114" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F114" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G114" s="26" t="n">
+        <x:v>525365</x:v>
+      </x:c>
+      <x:c r="H114" s="26" t="n">
+        <x:v>515401.6</x:v>
+      </x:c>
+      <x:c r="I114" s="22" t="n">
+        <x:f>H114/G114</x:f>
+        <x:v>0.9810352802337422</x:v>
+      </x:c>
+      <x:c r="J114" s="24" t="n">
+        <x:v>18.312</x:v>
+      </x:c>
+      <x:c r="K114" s="24" t="n">
+        <x:v>18.686</x:v>
+      </x:c>
+      <x:c r="L114" s="24" t="n">
+        <x:f>K114/J114</x:f>
+        <x:v>1.0204237658366098</x:v>
+      </x:c>
+      <x:c r="M114" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N114" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O114" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P114" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q114" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R114" s="10" t="str">
+        <x:v>f3660efe6f</x:v>
+      </x:c>
+      <x:c r="S114" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174322_cpp-router-router-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T114" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_174501_cpp-router-router-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U114" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V114" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.09%; latency median ratio 1.08x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="115">
-      <x:c r="A115" s="29"/>
-      <x:c r="G115" s="27"/>
-      <x:c r="H115" s="27"/>
-      <x:c r="I115" s="23"/>
-      <x:c r="J115" s="25"/>
-      <x:c r="K115" s="25"/>
-      <x:c r="L115" s="25"/>
+      <x:c r="A115" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B115" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C115" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D115" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E115" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F115" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G115" s="26" t="n">
+        <x:v>19017.8</x:v>
+      </x:c>
+      <x:c r="H115" s="26" t="n">
+        <x:v>17456</x:v>
+      </x:c>
+      <x:c r="I115" s="22" t="n">
+        <x:f>H115/G115</x:f>
+        <x:v>0.9178769363438464</x:v>
+      </x:c>
+      <x:c r="J115" s="24" t="n">
+        <x:v>6.79</x:v>
+      </x:c>
+      <x:c r="K115" s="24" t="n">
+        <x:v>7.762</x:v>
+      </x:c>
+      <x:c r="L115" s="24" t="n">
+        <x:f>K115/J115</x:f>
+        <x:v>1.1431516936671575</x:v>
+      </x:c>
+      <x:c r="M115" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N115" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O115" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P115" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q115" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R115" s="10" t="str">
+        <x:v>f3660efe6f</x:v>
+      </x:c>
+      <x:c r="S115" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174322_cpp-router-router-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T115" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_174501_cpp-router-router-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U115" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V115" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.09%; latency median ratio 1.08x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="116">
-      <x:c r="A116" s="29"/>
-      <x:c r="G116" s="27"/>
-      <x:c r="H116" s="27"/>
-      <x:c r="I116" s="23"/>
-      <x:c r="J116" s="25"/>
-      <x:c r="K116" s="25"/>
-      <x:c r="L116" s="25"/>
+      <x:c r="A116" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B116" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C116" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D116" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E116" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F116" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G116" s="26" t="n">
+        <x:v>12052.8</x:v>
+      </x:c>
+      <x:c r="H116" s="26" t="n">
+        <x:v>11109.2</x:v>
+      </x:c>
+      <x:c r="I116" s="22" t="n">
+        <x:f>H116/G116</x:f>
+        <x:v>0.9217111376609586</x:v>
+      </x:c>
+      <x:c r="J116" s="24" t="n">
+        <x:v>5.586</x:v>
+      </x:c>
+      <x:c r="K116" s="24" t="n">
+        <x:v>6.428</x:v>
+      </x:c>
+      <x:c r="L116" s="24" t="n">
+        <x:f>K116/J116</x:f>
+        <x:v>1.150733977801647</x:v>
+      </x:c>
+      <x:c r="M116" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N116" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O116" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P116" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q116" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R116" s="10" t="str">
+        <x:v>f3660efe6f</x:v>
+      </x:c>
+      <x:c r="S116" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174322_cpp-router-router-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T116" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_174501_cpp-router-router-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U116" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V116" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.09%; latency median ratio 1.08x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="117">
-      <x:c r="A117" s="29"/>
-      <x:c r="G117" s="27"/>
-      <x:c r="H117" s="27"/>
-      <x:c r="I117" s="23"/>
-      <x:c r="J117" s="25"/>
-      <x:c r="K117" s="25"/>
-      <x:c r="L117" s="25"/>
+      <x:c r="A117" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B117" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C117" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D117" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E117" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F117" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G117" s="26" t="n">
+        <x:v>8005.8</x:v>
+      </x:c>
+      <x:c r="H117" s="26" t="n">
+        <x:v>8030</x:v>
+      </x:c>
+      <x:c r="I117" s="22" t="n">
+        <x:f>H117/G117</x:f>
+        <x:v>1.0030228084638637</x:v>
+      </x:c>
+      <x:c r="J117" s="24" t="n">
+        <x:v>0.517</x:v>
+      </x:c>
+      <x:c r="K117" s="24" t="n">
+        <x:v>0.566</x:v>
+      </x:c>
+      <x:c r="L117" s="24" t="n">
+        <x:f>K117/J117</x:f>
+        <x:v>1.094777562862669</x:v>
+      </x:c>
+      <x:c r="M117" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N117" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O117" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P117" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q117" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R117" s="10" t="str">
+        <x:v>f3660efe6f</x:v>
+      </x:c>
+      <x:c r="S117" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174322_cpp-router-router-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T117" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_174501_cpp-router-router-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U117" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V117" s="10" t="str">
+        <x:v>Final: throughput aggregate mean 95.09%; latency median ratio 1.08x; pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="29"/>

</xml_diff>

<commit_message>
perf(cpp): streamline websocket router request completion
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rdd95f36d52674d17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rcfa2326f284947e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R0ed162c1b71f4477"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R0a7d0acd28e14eb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rfaa08790e86b46bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R3b6ed54767664cef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rf8fa0204a7ba454f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Rb6a11a2c7796403a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 4개 one-way 통과·PAIR/DEALER_REQREP 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달(개선 pass 포함) 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -8671,112 +8671,844 @@
       </x:c>
     </x:row>
     <x:row r="118">
-      <x:c r="A118" s="29"/>
-      <x:c r="G118" s="27"/>
-      <x:c r="H118" s="27"/>
-      <x:c r="I118" s="23"/>
-      <x:c r="J118" s="25"/>
-      <x:c r="K118" s="25"/>
-      <x:c r="L118" s="25"/>
+      <x:c r="A118" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B118" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C118" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D118" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E118" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F118" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G118" s="26" t="n">
+        <x:v>165224</x:v>
+      </x:c>
+      <x:c r="H118" s="26" t="n">
+        <x:v>45714.6</x:v>
+      </x:c>
+      <x:c r="I118" s="22" t="n">
+        <x:f>H118/G118</x:f>
+        <x:v>0.27668256427637633</x:v>
+      </x:c>
+      <x:c r="J118" s="24" t="n">
+        <x:v>0.318</x:v>
+      </x:c>
+      <x:c r="K118" s="24" t="n">
+        <x:v>1.341</x:v>
+      </x:c>
+      <x:c r="L118" s="24" t="n">
+        <x:f>K118/J118</x:f>
+        <x:v>4.216981132075471</x:v>
+      </x:c>
+      <x:c r="M118" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N118" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O118" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P118" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q118" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R118" s="10" t="str">
+        <x:v>453dc26538</x:v>
+      </x:c>
+      <x:c r="S118" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174829_cpp-router-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T118" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_175007_cpp-router-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U118" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V118" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 56.86%; latency median ratio 2.41x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="119">
-      <x:c r="A119" s="29"/>
-      <x:c r="G119" s="27"/>
-      <x:c r="H119" s="27"/>
-      <x:c r="I119" s="23"/>
-      <x:c r="J119" s="25"/>
-      <x:c r="K119" s="25"/>
-      <x:c r="L119" s="25"/>
+      <x:c r="A119" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B119" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C119" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D119" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E119" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F119" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G119" s="26" t="n">
+        <x:v>122474.6</x:v>
+      </x:c>
+      <x:c r="H119" s="26" t="n">
+        <x:v>36544</x:v>
+      </x:c>
+      <x:c r="I119" s="22" t="n">
+        <x:f>H119/G119</x:f>
+        <x:v>0.2983802355753764</x:v>
+      </x:c>
+      <x:c r="J119" s="24" t="n">
+        <x:v>0.449</x:v>
+      </x:c>
+      <x:c r="K119" s="24" t="n">
+        <x:v>1.694</x:v>
+      </x:c>
+      <x:c r="L119" s="24" t="n">
+        <x:f>K119/J119</x:f>
+        <x:v>3.7728285077951</x:v>
+      </x:c>
+      <x:c r="M119" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N119" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O119" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P119" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q119" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R119" s="10" t="str">
+        <x:v>453dc26538</x:v>
+      </x:c>
+      <x:c r="S119" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174829_cpp-router-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T119" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_175007_cpp-router-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U119" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V119" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 56.86%; latency median ratio 2.41x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="120">
-      <x:c r="A120" s="29"/>
-      <x:c r="G120" s="27"/>
-      <x:c r="H120" s="27"/>
-      <x:c r="I120" s="23"/>
-      <x:c r="J120" s="25"/>
-      <x:c r="K120" s="25"/>
-      <x:c r="L120" s="25"/>
+      <x:c r="A120" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B120" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C120" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D120" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E120" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F120" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G120" s="26" t="n">
+        <x:v>80142</x:v>
+      </x:c>
+      <x:c r="H120" s="26" t="n">
+        <x:v>24131.6</x:v>
+      </x:c>
+      <x:c r="I120" s="22" t="n">
+        <x:f>H120/G120</x:f>
+        <x:v>0.3011105288113598</x:v>
+      </x:c>
+      <x:c r="J120" s="24" t="n">
+        <x:v>0.744</x:v>
+      </x:c>
+      <x:c r="K120" s="24" t="n">
+        <x:v>2.72</x:v>
+      </x:c>
+      <x:c r="L120" s="24" t="n">
+        <x:f>K120/J120</x:f>
+        <x:v>3.655913978494624</x:v>
+      </x:c>
+      <x:c r="M120" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N120" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O120" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P120" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q120" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R120" s="10" t="str">
+        <x:v>453dc26538</x:v>
+      </x:c>
+      <x:c r="S120" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174829_cpp-router-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T120" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_175007_cpp-router-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U120" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V120" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 56.86%; latency median ratio 2.41x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="121">
-      <x:c r="A121" s="29"/>
-      <x:c r="G121" s="27"/>
-      <x:c r="H121" s="27"/>
-      <x:c r="I121" s="23"/>
-      <x:c r="J121" s="25"/>
-      <x:c r="K121" s="25"/>
-      <x:c r="L121" s="25"/>
+      <x:c r="A121" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B121" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C121" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D121" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E121" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F121" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G121" s="26" t="n">
+        <x:v>9674</x:v>
+      </x:c>
+      <x:c r="H121" s="26" t="n">
+        <x:v>8236</x:v>
+      </x:c>
+      <x:c r="I121" s="22" t="n">
+        <x:f>H121/G121</x:f>
+        <x:v>0.8513541451312797</x:v>
+      </x:c>
+      <x:c r="J121" s="24" t="n">
+        <x:v>1.351</x:v>
+      </x:c>
+      <x:c r="K121" s="24" t="n">
+        <x:v>1.507</x:v>
+      </x:c>
+      <x:c r="L121" s="24" t="n">
+        <x:f>K121/J121</x:f>
+        <x:v>1.1154700222057734</x:v>
+      </x:c>
+      <x:c r="M121" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N121" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O121" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P121" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q121" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R121" s="10" t="str">
+        <x:v>453dc26538</x:v>
+      </x:c>
+      <x:c r="S121" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174829_cpp-router-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T121" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_175007_cpp-router-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U121" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V121" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 56.86%; latency median ratio 2.41x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="122">
-      <x:c r="A122" s="29"/>
-      <x:c r="G122" s="27"/>
-      <x:c r="H122" s="27"/>
-      <x:c r="I122" s="23"/>
-      <x:c r="J122" s="25"/>
-      <x:c r="K122" s="25"/>
-      <x:c r="L122" s="25"/>
+      <x:c r="A122" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B122" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C122" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D122" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E122" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F122" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G122" s="26" t="n">
+        <x:v>6421.8</x:v>
+      </x:c>
+      <x:c r="H122" s="26" t="n">
+        <x:v>5402.8</x:v>
+      </x:c>
+      <x:c r="I122" s="22" t="n">
+        <x:f>H122/G122</x:f>
+        <x:v>0.841321747796568</x:v>
+      </x:c>
+      <x:c r="J122" s="24" t="n">
+        <x:v>0.929</x:v>
+      </x:c>
+      <x:c r="K122" s="24" t="n">
+        <x:v>1.083</x:v>
+      </x:c>
+      <x:c r="L122" s="24" t="n">
+        <x:f>K122/J122</x:f>
+        <x:v>1.1657696447793324</x:v>
+      </x:c>
+      <x:c r="M122" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N122" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O122" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P122" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q122" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R122" s="10" t="str">
+        <x:v>453dc26538</x:v>
+      </x:c>
+      <x:c r="S122" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174829_cpp-router-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T122" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_175007_cpp-router-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U122" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V122" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 56.86%; latency median ratio 2.41x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="123">
-      <x:c r="A123" s="29"/>
-      <x:c r="G123" s="27"/>
-      <x:c r="H123" s="27"/>
-      <x:c r="I123" s="23"/>
-      <x:c r="J123" s="25"/>
-      <x:c r="K123" s="25"/>
-      <x:c r="L123" s="25"/>
+      <x:c r="A123" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B123" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C123" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D123" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E123" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F123" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G123" s="26" t="n">
+        <x:v>4645.2</x:v>
+      </x:c>
+      <x:c r="H123" s="26" t="n">
+        <x:v>3914.6</x:v>
+      </x:c>
+      <x:c r="I123" s="22" t="n">
+        <x:f>H123/G123</x:f>
+        <x:v>0.8427193662275037</x:v>
+      </x:c>
+      <x:c r="J123" s="24" t="n">
+        <x:v>0.642</x:v>
+      </x:c>
+      <x:c r="K123" s="24" t="n">
+        <x:v>0.739</x:v>
+      </x:c>
+      <x:c r="L123" s="24" t="n">
+        <x:f>K123/J123</x:f>
+        <x:v>1.1510903426791277</x:v>
+      </x:c>
+      <x:c r="M123" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N123" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O123" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P123" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q123" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R123" s="10" t="str">
+        <x:v>453dc26538</x:v>
+      </x:c>
+      <x:c r="S123" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174829_cpp-router-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T123" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_175007_cpp-router-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U123" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V123" s="10" t="str">
+        <x:v>Before: throughput aggregate mean 56.86%; latency median ratio 2.41x; fail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="124">
-      <x:c r="A124" s="29"/>
-      <x:c r="G124" s="27"/>
-      <x:c r="H124" s="27"/>
-      <x:c r="I124" s="23"/>
-      <x:c r="J124" s="25"/>
-      <x:c r="K124" s="25"/>
-      <x:c r="L124" s="25"/>
+      <x:c r="A124" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B124" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C124" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D124" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E124" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F124" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G124" s="26" t="n">
+        <x:v>165224</x:v>
+      </x:c>
+      <x:c r="H124" s="26" t="n">
+        <x:v>51220.2</x:v>
+      </x:c>
+      <x:c r="I124" s="22" t="n">
+        <x:f>H124/G124</x:f>
+        <x:v>0.31000459981600736</x:v>
+      </x:c>
+      <x:c r="J124" s="24" t="n">
+        <x:v>0.318</x:v>
+      </x:c>
+      <x:c r="K124" s="24" t="n">
+        <x:v>1.194</x:v>
+      </x:c>
+      <x:c r="L124" s="24" t="n">
+        <x:f>K124/J124</x:f>
+        <x:v>3.7547169811320753</x:v>
+      </x:c>
+      <x:c r="M124" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N124" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O124" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P124" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q124" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R124" s="10" t="str">
+        <x:v>453dc26538</x:v>
+      </x:c>
+      <x:c r="S124" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174829_cpp-router-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T124" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U124" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V124" s="10" t="str">
+        <x:v>Candidate B final: throughput aggregate mean 59.98%; latency median ratio 2.15x; improved but both request/reply gates remain fail. Keep the async-only completion bridge; callback/blocking behavior is unchanged.</x:v>
+      </x:c>
     </x:row>
     <x:row r="125">
-      <x:c r="A125" s="29"/>
-      <x:c r="G125" s="27"/>
-      <x:c r="H125" s="27"/>
-      <x:c r="I125" s="23"/>
-      <x:c r="J125" s="25"/>
-      <x:c r="K125" s="25"/>
-      <x:c r="L125" s="25"/>
+      <x:c r="A125" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B125" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C125" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D125" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E125" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F125" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G125" s="26" t="n">
+        <x:v>122474.6</x:v>
+      </x:c>
+      <x:c r="H125" s="26" t="n">
+        <x:v>39940.6</x:v>
+      </x:c>
+      <x:c r="I125" s="22" t="n">
+        <x:f>H125/G125</x:f>
+        <x:v>0.32611333288698224</x:v>
+      </x:c>
+      <x:c r="J125" s="24" t="n">
+        <x:v>0.449</x:v>
+      </x:c>
+      <x:c r="K125" s="24" t="n">
+        <x:v>1.525</x:v>
+      </x:c>
+      <x:c r="L125" s="24" t="n">
+        <x:f>K125/J125</x:f>
+        <x:v>3.396436525612472</x:v>
+      </x:c>
+      <x:c r="M125" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N125" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O125" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P125" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q125" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R125" s="10" t="str">
+        <x:v>453dc26538</x:v>
+      </x:c>
+      <x:c r="S125" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174829_cpp-router-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T125" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U125" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V125" s="10" t="str">
+        <x:v>Candidate B final: throughput aggregate mean 59.98%; latency median ratio 2.15x; improved but both request/reply gates remain fail. Keep the async-only completion bridge; callback/blocking behavior is unchanged.</x:v>
+      </x:c>
     </x:row>
     <x:row r="126">
-      <x:c r="A126" s="29"/>
-      <x:c r="G126" s="27"/>
-      <x:c r="H126" s="27"/>
-      <x:c r="I126" s="23"/>
-      <x:c r="J126" s="25"/>
-      <x:c r="K126" s="25"/>
-      <x:c r="L126" s="25"/>
+      <x:c r="A126" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B126" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C126" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D126" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E126" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F126" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G126" s="26" t="n">
+        <x:v>80142</x:v>
+      </x:c>
+      <x:c r="H126" s="26" t="n">
+        <x:v>26885.6</x:v>
+      </x:c>
+      <x:c r="I126" s="22" t="n">
+        <x:f>H126/G126</x:f>
+        <x:v>0.3354745327044496</x:v>
+      </x:c>
+      <x:c r="J126" s="24" t="n">
+        <x:v>0.744</x:v>
+      </x:c>
+      <x:c r="K126" s="24" t="n">
+        <x:v>2.343</x:v>
+      </x:c>
+      <x:c r="L126" s="24" t="n">
+        <x:f>K126/J126</x:f>
+        <x:v>3.149193548387097</x:v>
+      </x:c>
+      <x:c r="M126" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N126" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O126" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P126" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q126" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R126" s="10" t="str">
+        <x:v>453dc26538</x:v>
+      </x:c>
+      <x:c r="S126" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174829_cpp-router-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T126" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U126" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V126" s="10" t="str">
+        <x:v>Candidate B final: throughput aggregate mean 59.98%; latency median ratio 2.15x; improved but both request/reply gates remain fail. Keep the async-only completion bridge; callback/blocking behavior is unchanged.</x:v>
+      </x:c>
     </x:row>
     <x:row r="127">
-      <x:c r="A127" s="29"/>
-      <x:c r="G127" s="27"/>
-      <x:c r="H127" s="27"/>
-      <x:c r="I127" s="23"/>
-      <x:c r="J127" s="25"/>
-      <x:c r="K127" s="25"/>
-      <x:c r="L127" s="25"/>
+      <x:c r="A127" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B127" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C127" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D127" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E127" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F127" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G127" s="26" t="n">
+        <x:v>9674</x:v>
+      </x:c>
+      <x:c r="H127" s="26" t="n">
+        <x:v>8320.8</x:v>
+      </x:c>
+      <x:c r="I127" s="22" t="n">
+        <x:f>H127/G127</x:f>
+        <x:v>0.8601199090345255</x:v>
+      </x:c>
+      <x:c r="J127" s="24" t="n">
+        <x:v>1.351</x:v>
+      </x:c>
+      <x:c r="K127" s="24" t="n">
+        <x:v>1.419</x:v>
+      </x:c>
+      <x:c r="L127" s="24" t="n">
+        <x:f>K127/J127</x:f>
+        <x:v>1.0503330866025167</x:v>
+      </x:c>
+      <x:c r="M127" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N127" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O127" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P127" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q127" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R127" s="10" t="str">
+        <x:v>453dc26538</x:v>
+      </x:c>
+      <x:c r="S127" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174829_cpp-router-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T127" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U127" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V127" s="10" t="str">
+        <x:v>Candidate B final: throughput aggregate mean 59.98%; latency median ratio 2.15x; improved but both request/reply gates remain fail. Keep the async-only completion bridge; callback/blocking behavior is unchanged.</x:v>
+      </x:c>
     </x:row>
     <x:row r="128">
-      <x:c r="A128" s="29"/>
-      <x:c r="G128" s="27"/>
-      <x:c r="H128" s="27"/>
-      <x:c r="I128" s="23"/>
-      <x:c r="J128" s="25"/>
-      <x:c r="K128" s="25"/>
-      <x:c r="L128" s="25"/>
+      <x:c r="A128" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B128" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C128" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D128" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E128" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F128" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G128" s="26" t="n">
+        <x:v>6421.8</x:v>
+      </x:c>
+      <x:c r="H128" s="26" t="n">
+        <x:v>5846</x:v>
+      </x:c>
+      <x:c r="I128" s="22" t="n">
+        <x:f>H128/G128</x:f>
+        <x:v>0.9103366657323492</x:v>
+      </x:c>
+      <x:c r="J128" s="24" t="n">
+        <x:v>0.929</x:v>
+      </x:c>
+      <x:c r="K128" s="24" t="n">
+        <x:v>1.003</x:v>
+      </x:c>
+      <x:c r="L128" s="24" t="n">
+        <x:f>K128/J128</x:f>
+        <x:v>1.0796555435952635</x:v>
+      </x:c>
+      <x:c r="M128" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N128" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O128" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P128" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q128" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R128" s="10" t="str">
+        <x:v>453dc26538</x:v>
+      </x:c>
+      <x:c r="S128" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174829_cpp-router-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T128" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U128" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V128" s="10" t="str">
+        <x:v>Candidate B final: throughput aggregate mean 59.98%; latency median ratio 2.15x; improved but both request/reply gates remain fail. Keep the async-only completion bridge; callback/blocking behavior is unchanged.</x:v>
+      </x:c>
     </x:row>
     <x:row r="129">
-      <x:c r="A129" s="29"/>
-      <x:c r="G129" s="27"/>
-      <x:c r="H129" s="27"/>
-      <x:c r="I129" s="23"/>
-      <x:c r="J129" s="25"/>
-      <x:c r="K129" s="25"/>
-      <x:c r="L129" s="25"/>
+      <x:c r="A129" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B129" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C129" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D129" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E129" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F129" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G129" s="26" t="n">
+        <x:v>4645.2</x:v>
+      </x:c>
+      <x:c r="H129" s="26" t="n">
+        <x:v>3955</x:v>
+      </x:c>
+      <x:c r="I129" s="22" t="n">
+        <x:f>H129/G129</x:f>
+        <x:v>0.851416515973478</x:v>
+      </x:c>
+      <x:c r="J129" s="24" t="n">
+        <x:v>0.642</x:v>
+      </x:c>
+      <x:c r="K129" s="24" t="n">
+        <x:v>0.737</x:v>
+      </x:c>
+      <x:c r="L129" s="24" t="n">
+        <x:f>K129/J129</x:f>
+        <x:v>1.1479750778816198</x:v>
+      </x:c>
+      <x:c r="M129" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N129" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O129" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P129" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q129" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R129" s="10" t="str">
+        <x:v>453dc26538</x:v>
+      </x:c>
+      <x:c r="S129" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_174829_cpp-router-router-reqrep-ws-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T129" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U129" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V129" s="10" t="str">
+        <x:v>Candidate B final: throughput aggregate mean 59.98%; latency median ratio 2.15x; improved but both request/reply gates remain fail. Keep the async-only completion bridge; callback/blocking behavior is unchanged.</x:v>
+      </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="29"/>
@@ -11737,12 +12469,90 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="L14" s="23"/>
-      <x:c r="M14" s="23"/>
+      <x:c r="A14" s="10" t="str">
+        <x:v>2026-08-25 17:52</x:v>
+      </x:c>
+      <x:c r="B14" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C14" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D14" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E14" s="10" t="str">
+        <x:v>ws</x:v>
+      </x:c>
+      <x:c r="F14" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%; latency &gt; 2.0x</x:v>
+      </x:c>
+      <x:c r="G14" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H14" s="10" t="str">
+        <x:v>Use the Core normal-router request route for single-part shallow views, avoiding exact transport-pair selection.</x:v>
+      </x:c>
+      <x:c r="I14" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J14" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_175007_cpp-router-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K14" s="10" t="str">
+        <x:v>N/A — exact-target contract no-go</x:v>
+      </x:c>
+      <x:c r="L14" s="22" t="n">
+        <x:v>0.569</x:v>
+      </x:c>
+      <x:c r="M14" s="22"/>
+      <x:c r="N14" s="10" t="str">
+        <x:v>NO-GO: omitting transport pair id/generation allows failover and changes public target/terminal semantics.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="L15" s="23"/>
-      <x:c r="M15" s="23"/>
+      <x:c r="A15" s="10" t="str">
+        <x:v>2026-08-25 18:01</x:v>
+      </x:c>
+      <x:c r="B15" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C15" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D15" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E15" s="10" t="str">
+        <x:v>ws</x:v>
+      </x:c>
+      <x:c r="F15" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%; latency &gt; 2.0x</x:v>
+      </x:c>
+      <x:c r="G15" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H15" s="10" t="str">
+        <x:v>Use an async-only completion bridge and delegate terminal synchronization to async_operation_state_t; retain explicit failure-path userdata deletion.</x:v>
+      </x:c>
+      <x:c r="I15" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J15" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_175007_cpp-router-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K15" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L15" s="22" t="n">
+        <x:v>0.569</x:v>
+      </x:c>
+      <x:c r="M15" s="22" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="N15" s="10" t="str">
+        <x:v>KEEP: aggregate +3.12%p and latency 2.41x→2.15x. Contract tests 4/4 pass; synchronous completion ownership is safe and callback/blocking APIs are unchanged. Both performance gates remain 미달.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="L16" s="23"/>

</xml_diff>

<commit_message>
docs(perf): record secure pair baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rfaa08790e86b46bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R3b6ed54767664cef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rf8fa0204a7ba454f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Rb6a11a2c7796403a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R9c24df9581204555"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R2aeaed0cdec24cb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R0318b1facb0745b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Rf7f6032ed8d54b6b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달(개선 pass 포함) 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss PAIR 통과 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -5744,7 +5744,7 @@
         <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E76" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F76" s="10" t="n">
         <x:v>64</x:v>
@@ -5814,7 +5814,7 @@
         <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E77" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F77" s="10" t="n">
         <x:v>256</x:v>
@@ -5884,7 +5884,7 @@
         <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E78" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F78" s="10" t="n">
         <x:v>1024</x:v>
@@ -5954,7 +5954,7 @@
         <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E79" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F79" s="10" t="n">
         <x:v>65536</x:v>
@@ -6024,7 +6024,7 @@
         <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E80" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F80" s="10" t="n">
         <x:v>131072</x:v>
@@ -6094,7 +6094,7 @@
         <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E81" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F81" s="10" t="n">
         <x:v>262144</x:v>
@@ -6164,7 +6164,7 @@
         <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E82" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F82" s="10" t="n">
         <x:v>64</x:v>
@@ -6234,7 +6234,7 @@
         <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E83" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F83" s="10" t="n">
         <x:v>256</x:v>
@@ -6304,7 +6304,7 @@
         <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E84" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F84" s="10" t="n">
         <x:v>1024</x:v>
@@ -6374,7 +6374,7 @@
         <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E85" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F85" s="10" t="n">
         <x:v>65536</x:v>
@@ -6444,7 +6444,7 @@
         <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E86" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F86" s="10" t="n">
         <x:v>131072</x:v>
@@ -6514,7 +6514,7 @@
         <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E87" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F87" s="10" t="n">
         <x:v>262144</x:v>
@@ -6584,7 +6584,7 @@
         <x:v>DEALER_DEALER</x:v>
       </x:c>
       <x:c r="E88" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F88" s="10" t="n">
         <x:v>64</x:v>
@@ -6654,7 +6654,7 @@
         <x:v>DEALER_DEALER</x:v>
       </x:c>
       <x:c r="E89" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F89" s="10" t="n">
         <x:v>256</x:v>
@@ -6724,7 +6724,7 @@
         <x:v>DEALER_DEALER</x:v>
       </x:c>
       <x:c r="E90" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F90" s="10" t="n">
         <x:v>1024</x:v>
@@ -6794,7 +6794,7 @@
         <x:v>DEALER_DEALER</x:v>
       </x:c>
       <x:c r="E91" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F91" s="10" t="n">
         <x:v>65536</x:v>
@@ -6864,7 +6864,7 @@
         <x:v>DEALER_DEALER</x:v>
       </x:c>
       <x:c r="E92" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F92" s="10" t="n">
         <x:v>131072</x:v>
@@ -6934,7 +6934,7 @@
         <x:v>DEALER_DEALER</x:v>
       </x:c>
       <x:c r="E93" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F93" s="10" t="n">
         <x:v>262144</x:v>
@@ -7004,7 +7004,7 @@
         <x:v>DEALER_ROUTER</x:v>
       </x:c>
       <x:c r="E94" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F94" s="10" t="n">
         <x:v>64</x:v>
@@ -7074,7 +7074,7 @@
         <x:v>DEALER_ROUTER</x:v>
       </x:c>
       <x:c r="E95" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F95" s="10" t="n">
         <x:v>256</x:v>
@@ -7144,7 +7144,7 @@
         <x:v>DEALER_ROUTER</x:v>
       </x:c>
       <x:c r="E96" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F96" s="10" t="n">
         <x:v>1024</x:v>
@@ -7214,7 +7214,7 @@
         <x:v>DEALER_ROUTER</x:v>
       </x:c>
       <x:c r="E97" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F97" s="10" t="n">
         <x:v>65536</x:v>
@@ -7284,7 +7284,7 @@
         <x:v>DEALER_ROUTER</x:v>
       </x:c>
       <x:c r="E98" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F98" s="10" t="n">
         <x:v>131072</x:v>
@@ -7354,7 +7354,7 @@
         <x:v>DEALER_ROUTER</x:v>
       </x:c>
       <x:c r="E99" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F99" s="10" t="n">
         <x:v>262144</x:v>
@@ -7424,7 +7424,7 @@
         <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E100" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F100" s="10" t="n">
         <x:v>64</x:v>
@@ -7494,7 +7494,7 @@
         <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E101" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F101" s="10" t="n">
         <x:v>256</x:v>
@@ -7564,7 +7564,7 @@
         <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E102" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F102" s="10" t="n">
         <x:v>1024</x:v>
@@ -7634,7 +7634,7 @@
         <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E103" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F103" s="10" t="n">
         <x:v>65536</x:v>
@@ -7704,7 +7704,7 @@
         <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E104" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F104" s="10" t="n">
         <x:v>131072</x:v>
@@ -7774,7 +7774,7 @@
         <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E105" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F105" s="10" t="n">
         <x:v>262144</x:v>
@@ -7844,7 +7844,7 @@
         <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E106" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F106" s="10" t="n">
         <x:v>64</x:v>
@@ -7914,7 +7914,7 @@
         <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E107" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F107" s="10" t="n">
         <x:v>256</x:v>
@@ -7984,7 +7984,7 @@
         <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E108" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F108" s="10" t="n">
         <x:v>1024</x:v>
@@ -8054,7 +8054,7 @@
         <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E109" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F109" s="10" t="n">
         <x:v>65536</x:v>
@@ -8124,7 +8124,7 @@
         <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E110" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F110" s="10" t="n">
         <x:v>131072</x:v>
@@ -8194,7 +8194,7 @@
         <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E111" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F111" s="10" t="n">
         <x:v>262144</x:v>
@@ -8264,7 +8264,7 @@
         <x:v>ROUTER_ROUTER</x:v>
       </x:c>
       <x:c r="E112" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F112" s="10" t="n">
         <x:v>64</x:v>
@@ -8334,7 +8334,7 @@
         <x:v>ROUTER_ROUTER</x:v>
       </x:c>
       <x:c r="E113" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F113" s="10" t="n">
         <x:v>256</x:v>
@@ -8404,7 +8404,7 @@
         <x:v>ROUTER_ROUTER</x:v>
       </x:c>
       <x:c r="E114" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F114" s="10" t="n">
         <x:v>1024</x:v>
@@ -8474,7 +8474,7 @@
         <x:v>ROUTER_ROUTER</x:v>
       </x:c>
       <x:c r="E115" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F115" s="10" t="n">
         <x:v>65536</x:v>
@@ -8544,7 +8544,7 @@
         <x:v>ROUTER_ROUTER</x:v>
       </x:c>
       <x:c r="E116" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F116" s="10" t="n">
         <x:v>131072</x:v>
@@ -8614,7 +8614,7 @@
         <x:v>ROUTER_ROUTER</x:v>
       </x:c>
       <x:c r="E117" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F117" s="10" t="n">
         <x:v>262144</x:v>
@@ -8684,7 +8684,7 @@
         <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E118" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F118" s="10" t="n">
         <x:v>64</x:v>
@@ -8754,7 +8754,7 @@
         <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E119" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F119" s="10" t="n">
         <x:v>256</x:v>
@@ -8824,7 +8824,7 @@
         <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E120" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F120" s="10" t="n">
         <x:v>1024</x:v>
@@ -8894,7 +8894,7 @@
         <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E121" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F121" s="10" t="n">
         <x:v>65536</x:v>
@@ -8964,7 +8964,7 @@
         <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E122" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F122" s="10" t="n">
         <x:v>131072</x:v>
@@ -9034,7 +9034,7 @@
         <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E123" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F123" s="10" t="n">
         <x:v>262144</x:v>
@@ -9104,7 +9104,7 @@
         <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E124" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F124" s="10" t="n">
         <x:v>64</x:v>
@@ -9174,7 +9174,7 @@
         <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E125" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F125" s="10" t="n">
         <x:v>256</x:v>
@@ -9244,7 +9244,7 @@
         <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E126" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F126" s="10" t="n">
         <x:v>1024</x:v>
@@ -9314,7 +9314,7 @@
         <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E127" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F127" s="10" t="n">
         <x:v>65536</x:v>
@@ -9384,7 +9384,7 @@
         <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E128" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F128" s="10" t="n">
         <x:v>131072</x:v>
@@ -9454,7 +9454,7 @@
         <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E129" s="10" t="str">
-        <x:v>tcp</x:v>
+        <x:v>ws</x:v>
       </x:c>
       <x:c r="F129" s="10" t="n">
         <x:v>262144</x:v>
@@ -9511,58 +9511,424 @@
       </x:c>
     </x:row>
     <x:row r="130">
-      <x:c r="A130" s="29"/>
-      <x:c r="G130" s="27"/>
-      <x:c r="H130" s="27"/>
-      <x:c r="I130" s="23"/>
-      <x:c r="J130" s="25"/>
-      <x:c r="K130" s="25"/>
-      <x:c r="L130" s="25"/>
+      <x:c r="A130" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B130" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C130" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D130" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E130" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F130" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G130" s="26" t="n">
+        <x:v>2045013.2</x:v>
+      </x:c>
+      <x:c r="H130" s="26" t="n">
+        <x:v>1803329.8</x:v>
+      </x:c>
+      <x:c r="I130" s="22" t="n">
+        <x:f>H130/G130</x:f>
+        <x:v>0.8818181711492131</x:v>
+      </x:c>
+      <x:c r="J130" s="24" t="n">
+        <x:v>47.35</x:v>
+      </x:c>
+      <x:c r="K130" s="24" t="n">
+        <x:v>54.122</x:v>
+      </x:c>
+      <x:c r="L130" s="24" t="n">
+        <x:f>K130/J130</x:f>
+        <x:v>1.1430200633579726</x:v>
+      </x:c>
+      <x:c r="M130" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N130" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O130" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P130" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q130" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R130" s="10" t="str">
+        <x:v>eff6284a79</x:v>
+      </x:c>
+      <x:c r="S130" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_180556_cpp-pair-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T130" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180845_cpp-pair-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U130" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V130" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 95.77%; latency median ratio 1.07x; strict gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="131">
-      <x:c r="A131" s="29"/>
-      <x:c r="G131" s="27"/>
-      <x:c r="H131" s="27"/>
-      <x:c r="I131" s="23"/>
-      <x:c r="J131" s="25"/>
-      <x:c r="K131" s="25"/>
-      <x:c r="L131" s="25"/>
+      <x:c r="A131" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B131" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C131" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D131" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E131" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F131" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G131" s="26" t="n">
+        <x:v>682986.6</x:v>
+      </x:c>
+      <x:c r="H131" s="26" t="n">
+        <x:v>725062.2</x:v>
+      </x:c>
+      <x:c r="I131" s="22" t="n">
+        <x:f>H131/G131</x:f>
+        <x:v>1.0616053082154173</x:v>
+      </x:c>
+      <x:c r="J131" s="24" t="n">
+        <x:v>46.801</x:v>
+      </x:c>
+      <x:c r="K131" s="24" t="n">
+        <x:v>46.416</x:v>
+      </x:c>
+      <x:c r="L131" s="24" t="n">
+        <x:f>K131/J131</x:f>
+        <x:v>0.9917736800495714</x:v>
+      </x:c>
+      <x:c r="M131" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N131" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O131" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P131" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q131" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R131" s="10" t="str">
+        <x:v>eff6284a79</x:v>
+      </x:c>
+      <x:c r="S131" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_180556_cpp-pair-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T131" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180845_cpp-pair-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U131" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V131" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 95.77%; latency median ratio 1.07x; strict gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="132">
-      <x:c r="A132" s="29"/>
-      <x:c r="G132" s="27"/>
-      <x:c r="H132" s="27"/>
-      <x:c r="I132" s="23"/>
-      <x:c r="J132" s="25"/>
-      <x:c r="K132" s="25"/>
-      <x:c r="L132" s="25"/>
+      <x:c r="A132" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B132" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C132" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D132" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E132" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F132" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G132" s="26" t="n">
+        <x:v>230921.2</x:v>
+      </x:c>
+      <x:c r="H132" s="26" t="n">
+        <x:v>224608.2</x:v>
+      </x:c>
+      <x:c r="I132" s="22" t="n">
+        <x:f>H132/G132</x:f>
+        <x:v>0.972661669868336</x:v>
+      </x:c>
+      <x:c r="J132" s="24" t="n">
+        <x:v>30.415</x:v>
+      </x:c>
+      <x:c r="K132" s="24" t="n">
+        <x:v>32.491</x:v>
+      </x:c>
+      <x:c r="L132" s="24" t="n">
+        <x:f>K132/J132</x:f>
+        <x:v>1.0682557948380733</x:v>
+      </x:c>
+      <x:c r="M132" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N132" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O132" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P132" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q132" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R132" s="10" t="str">
+        <x:v>eff6284a79</x:v>
+      </x:c>
+      <x:c r="S132" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_180556_cpp-pair-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T132" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180845_cpp-pair-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U132" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V132" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 95.77%; latency median ratio 1.07x; strict gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="133">
-      <x:c r="A133" s="29"/>
-      <x:c r="G133" s="27"/>
-      <x:c r="H133" s="27"/>
-      <x:c r="I133" s="23"/>
-      <x:c r="J133" s="25"/>
-      <x:c r="K133" s="25"/>
-      <x:c r="L133" s="25"/>
+      <x:c r="A133" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B133" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C133" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D133" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E133" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F133" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G133" s="26" t="n">
+        <x:v>8643</x:v>
+      </x:c>
+      <x:c r="H133" s="26" t="n">
+        <x:v>8344</x:v>
+      </x:c>
+      <x:c r="I133" s="22" t="n">
+        <x:f>H133/G133</x:f>
+        <x:v>0.9654055304870994</x:v>
+      </x:c>
+      <x:c r="J133" s="24" t="n">
+        <x:v>13.078</x:v>
+      </x:c>
+      <x:c r="K133" s="24" t="n">
+        <x:v>14.106</x:v>
+      </x:c>
+      <x:c r="L133" s="24" t="n">
+        <x:f>K133/J133</x:f>
+        <x:v>1.0786052913289494</x:v>
+      </x:c>
+      <x:c r="M133" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N133" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O133" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P133" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q133" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R133" s="10" t="str">
+        <x:v>eff6284a79</x:v>
+      </x:c>
+      <x:c r="S133" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_180556_cpp-pair-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T133" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180845_cpp-pair-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U133" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V133" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 95.77%; latency median ratio 1.07x; strict gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="134">
-      <x:c r="A134" s="29"/>
-      <x:c r="G134" s="27"/>
-      <x:c r="H134" s="27"/>
-      <x:c r="I134" s="23"/>
-      <x:c r="J134" s="25"/>
-      <x:c r="K134" s="25"/>
-      <x:c r="L134" s="25"/>
+      <x:c r="A134" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B134" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C134" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D134" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E134" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F134" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G134" s="26" t="n">
+        <x:v>5108</x:v>
+      </x:c>
+      <x:c r="H134" s="26" t="n">
+        <x:v>5053</x:v>
+      </x:c>
+      <x:c r="I134" s="22" t="n">
+        <x:f>H134/G134</x:f>
+        <x:v>0.9892325763508223</x:v>
+      </x:c>
+      <x:c r="J134" s="24" t="n">
+        <x:v>11.22</x:v>
+      </x:c>
+      <x:c r="K134" s="24" t="n">
+        <x:v>11.681</x:v>
+      </x:c>
+      <x:c r="L134" s="24" t="n">
+        <x:f>K134/J134</x:f>
+        <x:v>1.0410873440285204</x:v>
+      </x:c>
+      <x:c r="M134" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N134" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O134" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P134" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q134" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R134" s="10" t="str">
+        <x:v>eff6284a79</x:v>
+      </x:c>
+      <x:c r="S134" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_180556_cpp-pair-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T134" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180845_cpp-pair-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U134" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V134" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 95.77%; latency median ratio 1.07x; strict gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="135">
-      <x:c r="A135" s="29"/>
-      <x:c r="G135" s="27"/>
-      <x:c r="H135" s="27"/>
-      <x:c r="I135" s="23"/>
-      <x:c r="J135" s="25"/>
-      <x:c r="K135" s="25"/>
-      <x:c r="L135" s="25"/>
+      <x:c r="A135" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B135" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C135" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D135" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E135" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F135" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G135" s="26" t="n">
+        <x:v>2770.8</x:v>
+      </x:c>
+      <x:c r="H135" s="26" t="n">
+        <x:v>2425.2</x:v>
+      </x:c>
+      <x:c r="I135" s="22" t="n">
+        <x:f>H135/G135</x:f>
+        <x:v>0.8752706799480293</x:v>
+      </x:c>
+      <x:c r="J135" s="24" t="n">
+        <x:v>11.024</x:v>
+      </x:c>
+      <x:c r="K135" s="24" t="n">
+        <x:v>12.904</x:v>
+      </x:c>
+      <x:c r="L135" s="24" t="n">
+        <x:f>K135/J135</x:f>
+        <x:v>1.1705370101596517</x:v>
+      </x:c>
+      <x:c r="M135" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N135" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O135" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P135" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q135" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R135" s="10" t="str">
+        <x:v>eff6284a79</x:v>
+      </x:c>
+      <x:c r="S135" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_180556_cpp-pair-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T135" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180845_cpp-pair-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U135" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V135" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 95.77%; latency median ratio 1.07x; strict gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="29"/>

</xml_diff>

<commit_message>
docs(perf): record secure pubsub baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R9c24df9581204555"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R2aeaed0cdec24cb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R0318b1facb0745b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Rf7f6032ed8d54b6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R00daaaa6fecd42bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R5bcf7b76a1bd4e63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rb9b3b48210f04fab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R5a337297c1144266"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss PAIR 통과 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss PAIR·PUBSUB 통과 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -9931,58 +9931,424 @@
       </x:c>
     </x:row>
     <x:row r="136">
-      <x:c r="A136" s="29"/>
-      <x:c r="G136" s="27"/>
-      <x:c r="H136" s="27"/>
-      <x:c r="I136" s="23"/>
-      <x:c r="J136" s="25"/>
-      <x:c r="K136" s="25"/>
-      <x:c r="L136" s="25"/>
+      <x:c r="A136" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B136" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C136" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D136" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E136" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F136" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G136" s="26" t="n">
+        <x:v>1121741.2</x:v>
+      </x:c>
+      <x:c r="H136" s="26" t="n">
+        <x:v>1066244.8</x:v>
+      </x:c>
+      <x:c r="I136" s="22" t="n">
+        <x:f>H136/G136</x:f>
+        <x:v>0.950526556392865</x:v>
+      </x:c>
+      <x:c r="J136" s="24" t="n">
+        <x:v>63.983</x:v>
+      </x:c>
+      <x:c r="K136" s="24" t="n">
+        <x:v>75.742</x:v>
+      </x:c>
+      <x:c r="L136" s="24" t="n">
+        <x:f>K136/J136</x:f>
+        <x:v>1.1837831924104842</x:v>
+      </x:c>
+      <x:c r="M136" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N136" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O136" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P136" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q136" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R136" s="10" t="str">
+        <x:v>b7688c325f</x:v>
+      </x:c>
+      <x:c r="S136" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_181435_cpp-pubsub-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T136" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_181820_cpp-pubsub-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U136" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V136" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 98.25%; latency median ratio 1.04x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="137">
-      <x:c r="A137" s="29"/>
-      <x:c r="G137" s="27"/>
-      <x:c r="H137" s="27"/>
-      <x:c r="I137" s="23"/>
-      <x:c r="J137" s="25"/>
-      <x:c r="K137" s="25"/>
-      <x:c r="L137" s="25"/>
+      <x:c r="A137" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B137" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C137" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D137" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E137" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F137" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G137" s="26" t="n">
+        <x:v>610082</x:v>
+      </x:c>
+      <x:c r="H137" s="26" t="n">
+        <x:v>590108.8</x:v>
+      </x:c>
+      <x:c r="I137" s="22" t="n">
+        <x:f>H137/G137</x:f>
+        <x:v>0.9672614501001505</x:v>
+      </x:c>
+      <x:c r="J137" s="24" t="n">
+        <x:v>43.663</x:v>
+      </x:c>
+      <x:c r="K137" s="24" t="n">
+        <x:v>44.331</x:v>
+      </x:c>
+      <x:c r="L137" s="24" t="n">
+        <x:f>K137/J137</x:f>
+        <x:v>1.0152989945720634</x:v>
+      </x:c>
+      <x:c r="M137" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N137" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O137" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P137" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q137" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R137" s="10" t="str">
+        <x:v>b7688c325f</x:v>
+      </x:c>
+      <x:c r="S137" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_181435_cpp-pubsub-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T137" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_181820_cpp-pubsub-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U137" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V137" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 98.25%; latency median ratio 1.04x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="138">
-      <x:c r="A138" s="29"/>
-      <x:c r="G138" s="27"/>
-      <x:c r="H138" s="27"/>
-      <x:c r="I138" s="23"/>
-      <x:c r="J138" s="25"/>
-      <x:c r="K138" s="25"/>
-      <x:c r="L138" s="25"/>
+      <x:c r="A138" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B138" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C138" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D138" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E138" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F138" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G138" s="26" t="n">
+        <x:v>214261</x:v>
+      </x:c>
+      <x:c r="H138" s="26" t="n">
+        <x:v>206526.6</x:v>
+      </x:c>
+      <x:c r="I138" s="22" t="n">
+        <x:f>H138/G138</x:f>
+        <x:v>0.9639019700272098</x:v>
+      </x:c>
+      <x:c r="J138" s="24" t="n">
+        <x:v>32.783</x:v>
+      </x:c>
+      <x:c r="K138" s="24" t="n">
+        <x:v>34.674</x:v>
+      </x:c>
+      <x:c r="L138" s="24" t="n">
+        <x:f>K138/J138</x:f>
+        <x:v>1.0576823353567397</x:v>
+      </x:c>
+      <x:c r="M138" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N138" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O138" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P138" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q138" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R138" s="10" t="str">
+        <x:v>b7688c325f</x:v>
+      </x:c>
+      <x:c r="S138" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_181435_cpp-pubsub-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T138" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_181820_cpp-pubsub-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U138" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V138" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 98.25%; latency median ratio 1.04x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="139">
-      <x:c r="A139" s="29"/>
-      <x:c r="G139" s="27"/>
-      <x:c r="H139" s="27"/>
-      <x:c r="I139" s="23"/>
-      <x:c r="J139" s="25"/>
-      <x:c r="K139" s="25"/>
-      <x:c r="L139" s="25"/>
+      <x:c r="A139" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B139" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C139" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D139" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E139" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F139" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G139" s="26" t="n">
+        <x:v>8827.2</x:v>
+      </x:c>
+      <x:c r="H139" s="26" t="n">
+        <x:v>8873.6</x:v>
+      </x:c>
+      <x:c r="I139" s="22" t="n">
+        <x:f>H139/G139</x:f>
+        <x:v>1.0052564799709987</x:v>
+      </x:c>
+      <x:c r="J139" s="24" t="n">
+        <x:v>14.695</x:v>
+      </x:c>
+      <x:c r="K139" s="24" t="n">
+        <x:v>14.628</x:v>
+      </x:c>
+      <x:c r="L139" s="24" t="n">
+        <x:f>K139/J139</x:f>
+        <x:v>0.9954406260632869</x:v>
+      </x:c>
+      <x:c r="M139" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N139" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O139" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P139" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q139" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R139" s="10" t="str">
+        <x:v>b7688c325f</x:v>
+      </x:c>
+      <x:c r="S139" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_181435_cpp-pubsub-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T139" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_181820_cpp-pubsub-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U139" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V139" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 98.25%; latency median ratio 1.04x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="140">
-      <x:c r="A140" s="29"/>
-      <x:c r="G140" s="27"/>
-      <x:c r="H140" s="27"/>
-      <x:c r="I140" s="23"/>
-      <x:c r="J140" s="25"/>
-      <x:c r="K140" s="25"/>
-      <x:c r="L140" s="25"/>
+      <x:c r="A140" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B140" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C140" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D140" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E140" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F140" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G140" s="26" t="n">
+        <x:v>5015.6</x:v>
+      </x:c>
+      <x:c r="H140" s="26" t="n">
+        <x:v>5112.4</x:v>
+      </x:c>
+      <x:c r="I140" s="22" t="n">
+        <x:f>H140/G140</x:f>
+        <x:v>1.0192997846718237</x:v>
+      </x:c>
+      <x:c r="J140" s="24" t="n">
+        <x:v>11.58</x:v>
+      </x:c>
+      <x:c r="K140" s="24" t="n">
+        <x:v>11.311</x:v>
+      </x:c>
+      <x:c r="L140" s="24" t="n">
+        <x:f>K140/J140</x:f>
+        <x:v>0.9767702936096718</x:v>
+      </x:c>
+      <x:c r="M140" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N140" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O140" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P140" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q140" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R140" s="10" t="str">
+        <x:v>b7688c325f</x:v>
+      </x:c>
+      <x:c r="S140" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_181435_cpp-pubsub-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T140" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_181820_cpp-pubsub-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U140" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V140" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 98.25%; latency median ratio 1.04x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="141">
-      <x:c r="A141" s="29"/>
-      <x:c r="G141" s="27"/>
-      <x:c r="H141" s="27"/>
-      <x:c r="I141" s="23"/>
-      <x:c r="J141" s="25"/>
-      <x:c r="K141" s="25"/>
-      <x:c r="L141" s="25"/>
+      <x:c r="A141" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B141" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C141" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D141" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E141" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F141" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G141" s="26" t="n">
+        <x:v>3006.4</x:v>
+      </x:c>
+      <x:c r="H141" s="26" t="n">
+        <x:v>2973.4</x:v>
+      </x:c>
+      <x:c r="I141" s="22" t="n">
+        <x:f>H141/G141</x:f>
+        <x:v>0.9890234167110165</x:v>
+      </x:c>
+      <x:c r="J141" s="24" t="n">
+        <x:v>10.261</x:v>
+      </x:c>
+      <x:c r="K141" s="24" t="n">
+        <x:v>11.482</x:v>
+      </x:c>
+      <x:c r="L141" s="24" t="n">
+        <x:f>K141/J141</x:f>
+        <x:v>1.1189942500730923</x:v>
+      </x:c>
+      <x:c r="M141" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N141" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O141" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P141" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q141" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R141" s="10" t="str">
+        <x:v>b7688c325f</x:v>
+      </x:c>
+      <x:c r="S141" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_181435_cpp-pubsub-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T141" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_181820_cpp-pubsub-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U141" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V141" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 98.25%; latency median ratio 1.04x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="29"/>

</xml_diff>

<commit_message>
docs(perf): record secure dealer baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R00daaaa6fecd42bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R5bcf7b76a1bd4e63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rb9b3b48210f04fab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R5a337297c1144266"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rffc24aca86e74216"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R762d71f092b94268"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R48397ea3fbe14360"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R56a5588f6b2b4bf3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss PAIR·PUBSUB 통과 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss PAIR·PUBSUB·DEALER_DEALER 통과 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -10351,58 +10351,424 @@
       </x:c>
     </x:row>
     <x:row r="142">
-      <x:c r="A142" s="29"/>
-      <x:c r="G142" s="27"/>
-      <x:c r="H142" s="27"/>
-      <x:c r="I142" s="23"/>
-      <x:c r="J142" s="25"/>
-      <x:c r="K142" s="25"/>
-      <x:c r="L142" s="25"/>
+      <x:c r="A142" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B142" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C142" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D142" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E142" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F142" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G142" s="26" t="n">
+        <x:v>1985873.6</x:v>
+      </x:c>
+      <x:c r="H142" s="26" t="n">
+        <x:v>1811222.8</x:v>
+      </x:c>
+      <x:c r="I142" s="22" t="n">
+        <x:f>H142/G142</x:f>
+        <x:v>0.912053415685671</x:v>
+      </x:c>
+      <x:c r="J142" s="24" t="n">
+        <x:v>50.892</x:v>
+      </x:c>
+      <x:c r="K142" s="24" t="n">
+        <x:v>58.014</x:v>
+      </x:c>
+      <x:c r="L142" s="24" t="n">
+        <x:f>K142/J142</x:f>
+        <x:v>1.139943409573214</x:v>
+      </x:c>
+      <x:c r="M142" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N142" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O142" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P142" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q142" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R142" s="10" t="str">
+        <x:v>e1eb9baef2</x:v>
+      </x:c>
+      <x:c r="S142" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_182334_cpp-dealer-dealer-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T142" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_182620_cpp-dealer-dealer-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U142" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V142" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 93.89%; latency median ratio 1.07x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="143">
-      <x:c r="A143" s="29"/>
-      <x:c r="G143" s="27"/>
-      <x:c r="H143" s="27"/>
-      <x:c r="I143" s="23"/>
-      <x:c r="J143" s="25"/>
-      <x:c r="K143" s="25"/>
-      <x:c r="L143" s="25"/>
+      <x:c r="A143" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B143" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C143" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D143" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E143" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F143" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G143" s="26" t="n">
+        <x:v>713581.4</x:v>
+      </x:c>
+      <x:c r="H143" s="26" t="n">
+        <x:v>694613.4</x:v>
+      </x:c>
+      <x:c r="I143" s="22" t="n">
+        <x:f>H143/G143</x:f>
+        <x:v>0.9734185896661545</x:v>
+      </x:c>
+      <x:c r="J143" s="24" t="n">
+        <x:v>49.795</x:v>
+      </x:c>
+      <x:c r="K143" s="24" t="n">
+        <x:v>39.34</x:v>
+      </x:c>
+      <x:c r="L143" s="24" t="n">
+        <x:f>K143/J143</x:f>
+        <x:v>0.790039160558289</x:v>
+      </x:c>
+      <x:c r="M143" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N143" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O143" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P143" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q143" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R143" s="10" t="str">
+        <x:v>e1eb9baef2</x:v>
+      </x:c>
+      <x:c r="S143" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_182334_cpp-dealer-dealer-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T143" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_182620_cpp-dealer-dealer-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U143" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V143" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 93.89%; latency median ratio 1.07x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="144">
-      <x:c r="A144" s="29"/>
-      <x:c r="G144" s="27"/>
-      <x:c r="H144" s="27"/>
-      <x:c r="I144" s="23"/>
-      <x:c r="J144" s="25"/>
-      <x:c r="K144" s="25"/>
-      <x:c r="L144" s="25"/>
+      <x:c r="A144" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B144" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C144" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D144" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E144" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F144" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G144" s="26" t="n">
+        <x:v>217510.4</x:v>
+      </x:c>
+      <x:c r="H144" s="26" t="n">
+        <x:v>197635.8</x:v>
+      </x:c>
+      <x:c r="I144" s="22" t="n">
+        <x:f>H144/G144</x:f>
+        <x:v>0.9086268978402872</x:v>
+      </x:c>
+      <x:c r="J144" s="24" t="n">
+        <x:v>32.627</x:v>
+      </x:c>
+      <x:c r="K144" s="24" t="n">
+        <x:v>36.349</x:v>
+      </x:c>
+      <x:c r="L144" s="24" t="n">
+        <x:f>K144/J144</x:f>
+        <x:v>1.1140772979434208</x:v>
+      </x:c>
+      <x:c r="M144" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N144" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O144" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P144" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q144" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R144" s="10" t="str">
+        <x:v>e1eb9baef2</x:v>
+      </x:c>
+      <x:c r="S144" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_182334_cpp-dealer-dealer-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T144" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_182620_cpp-dealer-dealer-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U144" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V144" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 93.89%; latency median ratio 1.07x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="145">
-      <x:c r="A145" s="29"/>
-      <x:c r="G145" s="27"/>
-      <x:c r="H145" s="27"/>
-      <x:c r="I145" s="23"/>
-      <x:c r="J145" s="25"/>
-      <x:c r="K145" s="25"/>
-      <x:c r="L145" s="25"/>
+      <x:c r="A145" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B145" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C145" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D145" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E145" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F145" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G145" s="26" t="n">
+        <x:v>7884.6</x:v>
+      </x:c>
+      <x:c r="H145" s="26" t="n">
+        <x:v>8194.4</x:v>
+      </x:c>
+      <x:c r="I145" s="22" t="n">
+        <x:f>H145/G145</x:f>
+        <x:v>1.0392917839839686</x:v>
+      </x:c>
+      <x:c r="J145" s="24" t="n">
+        <x:v>16.436</x:v>
+      </x:c>
+      <x:c r="K145" s="24" t="n">
+        <x:v>16.756</x:v>
+      </x:c>
+      <x:c r="L145" s="24" t="n">
+        <x:f>K145/J145</x:f>
+        <x:v>1.019469457288878</x:v>
+      </x:c>
+      <x:c r="M145" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N145" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O145" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P145" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q145" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R145" s="10" t="str">
+        <x:v>e1eb9baef2</x:v>
+      </x:c>
+      <x:c r="S145" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_182334_cpp-dealer-dealer-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T145" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_182620_cpp-dealer-dealer-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U145" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V145" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 93.89%; latency median ratio 1.07x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="146">
-      <x:c r="A146" s="29"/>
-      <x:c r="G146" s="27"/>
-      <x:c r="H146" s="27"/>
-      <x:c r="I146" s="23"/>
-      <x:c r="J146" s="25"/>
-      <x:c r="K146" s="25"/>
-      <x:c r="L146" s="25"/>
+      <x:c r="A146" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B146" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C146" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D146" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E146" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F146" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G146" s="26" t="n">
+        <x:v>5042.2</x:v>
+      </x:c>
+      <x:c r="H146" s="26" t="n">
+        <x:v>4846.4</x:v>
+      </x:c>
+      <x:c r="I146" s="22" t="n">
+        <x:f>H146/G146</x:f>
+        <x:v>0.9611677442386259</x:v>
+      </x:c>
+      <x:c r="J146" s="24" t="n">
+        <x:v>12.125</x:v>
+      </x:c>
+      <x:c r="K146" s="24" t="n">
+        <x:v>12.515</x:v>
+      </x:c>
+      <x:c r="L146" s="24" t="n">
+        <x:f>K146/J146</x:f>
+        <x:v>1.0321649484536084</x:v>
+      </x:c>
+      <x:c r="M146" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N146" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O146" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P146" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q146" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R146" s="10" t="str">
+        <x:v>e1eb9baef2</x:v>
+      </x:c>
+      <x:c r="S146" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_182334_cpp-dealer-dealer-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T146" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_182620_cpp-dealer-dealer-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U146" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V146" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 93.89%; latency median ratio 1.07x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="147">
-      <x:c r="A147" s="29"/>
-      <x:c r="G147" s="27"/>
-      <x:c r="H147" s="27"/>
-      <x:c r="I147" s="23"/>
-      <x:c r="J147" s="25"/>
-      <x:c r="K147" s="25"/>
-      <x:c r="L147" s="25"/>
+      <x:c r="A147" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B147" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C147" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D147" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E147" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F147" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G147" s="26" t="n">
+        <x:v>2782</x:v>
+      </x:c>
+      <x:c r="H147" s="26" t="n">
+        <x:v>2332</x:v>
+      </x:c>
+      <x:c r="I147" s="22" t="n">
+        <x:f>H147/G147</x:f>
+        <x:v>0.8382458662832495</x:v>
+      </x:c>
+      <x:c r="J147" s="24" t="n">
+        <x:v>11.658</x:v>
+      </x:c>
+      <x:c r="K147" s="24" t="n">
+        <x:v>13.949</x:v>
+      </x:c>
+      <x:c r="L147" s="24" t="n">
+        <x:f>K147/J147</x:f>
+        <x:v>1.1965174129353233</x:v>
+      </x:c>
+      <x:c r="M147" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N147" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O147" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P147" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q147" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R147" s="10" t="str">
+        <x:v>e1eb9baef2</x:v>
+      </x:c>
+      <x:c r="S147" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_182334_cpp-dealer-dealer-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T147" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_182620_cpp-dealer-dealer-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U147" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V147" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 93.89%; latency median ratio 1.07x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="29"/>

</xml_diff>

<commit_message>
docs(perf): record secure routed baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rffc24aca86e74216"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R762d71f092b94268"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R48397ea3fbe14360"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R56a5588f6b2b4bf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R495f22bd94bf4b8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Ra0aae48a88484ffe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rd8de070a003c40ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R7df4b879a7434002"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss PAIR·PUBSUB·DEALER_DEALER 통과 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss one-way 4개 통과 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -10771,58 +10771,424 @@
       </x:c>
     </x:row>
     <x:row r="148">
-      <x:c r="A148" s="29"/>
-      <x:c r="G148" s="27"/>
-      <x:c r="H148" s="27"/>
-      <x:c r="I148" s="23"/>
-      <x:c r="J148" s="25"/>
-      <x:c r="K148" s="25"/>
-      <x:c r="L148" s="25"/>
+      <x:c r="A148" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B148" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C148" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D148" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E148" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F148" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G148" s="26" t="n">
+        <x:v>2010431.4</x:v>
+      </x:c>
+      <x:c r="H148" s="26" t="n">
+        <x:v>1922976.2</x:v>
+      </x:c>
+      <x:c r="I148" s="22" t="n">
+        <x:f>H148/G148</x:f>
+        <x:v>0.9564992866705126</x:v>
+      </x:c>
+      <x:c r="J148" s="24" t="n">
+        <x:v>52.721</x:v>
+      </x:c>
+      <x:c r="K148" s="24" t="n">
+        <x:v>48.999</x:v>
+      </x:c>
+      <x:c r="L148" s="24" t="n">
+        <x:f>K148/J148</x:f>
+        <x:v>0.9294019460935871</x:v>
+      </x:c>
+      <x:c r="M148" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N148" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O148" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P148" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q148" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R148" s="10" t="str">
+        <x:v>6cfa7aad3e</x:v>
+      </x:c>
+      <x:c r="S148" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_183058_cpp-dealer-router-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T148" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_183422_cpp-dealer-router-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U148" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V148" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 99.49%; latency median ratio 0.99x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="149">
-      <x:c r="A149" s="29"/>
-      <x:c r="G149" s="27"/>
-      <x:c r="H149" s="27"/>
-      <x:c r="I149" s="23"/>
-      <x:c r="J149" s="25"/>
-      <x:c r="K149" s="25"/>
-      <x:c r="L149" s="25"/>
+      <x:c r="A149" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B149" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C149" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D149" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E149" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F149" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G149" s="26" t="n">
+        <x:v>709733.2</x:v>
+      </x:c>
+      <x:c r="H149" s="26" t="n">
+        <x:v>738630.8</x:v>
+      </x:c>
+      <x:c r="I149" s="22" t="n">
+        <x:f>H149/G149</x:f>
+        <x:v>1.0407161451655356</x:v>
+      </x:c>
+      <x:c r="J149" s="24" t="n">
+        <x:v>39.786</x:v>
+      </x:c>
+      <x:c r="K149" s="24" t="n">
+        <x:v>38.903</x:v>
+      </x:c>
+      <x:c r="L149" s="24" t="n">
+        <x:f>K149/J149</x:f>
+        <x:v>0.9778062635097773</x:v>
+      </x:c>
+      <x:c r="M149" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N149" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O149" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P149" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q149" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R149" s="10" t="str">
+        <x:v>6cfa7aad3e</x:v>
+      </x:c>
+      <x:c r="S149" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_183058_cpp-dealer-router-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T149" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_183422_cpp-dealer-router-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U149" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V149" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 99.49%; latency median ratio 0.99x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="150">
-      <x:c r="A150" s="29"/>
-      <x:c r="G150" s="27"/>
-      <x:c r="H150" s="27"/>
-      <x:c r="I150" s="23"/>
-      <x:c r="J150" s="25"/>
-      <x:c r="K150" s="25"/>
-      <x:c r="L150" s="25"/>
+      <x:c r="A150" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B150" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C150" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D150" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E150" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F150" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G150" s="26" t="n">
+        <x:v>219168.4</x:v>
+      </x:c>
+      <x:c r="H150" s="26" t="n">
+        <x:v>216957.6</x:v>
+      </x:c>
+      <x:c r="I150" s="22" t="n">
+        <x:f>H150/G150</x:f>
+        <x:v>0.9899127793970299</x:v>
+      </x:c>
+      <x:c r="J150" s="24" t="n">
+        <x:v>33.823</x:v>
+      </x:c>
+      <x:c r="K150" s="24" t="n">
+        <x:v>38.037</x:v>
+      </x:c>
+      <x:c r="L150" s="24" t="n">
+        <x:f>K150/J150</x:f>
+        <x:v>1.1245897761878012</x:v>
+      </x:c>
+      <x:c r="M150" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N150" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O150" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P150" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q150" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R150" s="10" t="str">
+        <x:v>6cfa7aad3e</x:v>
+      </x:c>
+      <x:c r="S150" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_183058_cpp-dealer-router-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T150" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_183422_cpp-dealer-router-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U150" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V150" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 99.49%; latency median ratio 0.99x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="151">
-      <x:c r="A151" s="29"/>
-      <x:c r="G151" s="27"/>
-      <x:c r="H151" s="27"/>
-      <x:c r="I151" s="23"/>
-      <x:c r="J151" s="25"/>
-      <x:c r="K151" s="25"/>
-      <x:c r="L151" s="25"/>
+      <x:c r="A151" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B151" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C151" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D151" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E151" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F151" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G151" s="26" t="n">
+        <x:v>8196.2</x:v>
+      </x:c>
+      <x:c r="H151" s="26" t="n">
+        <x:v>8146.2</x:v>
+      </x:c>
+      <x:c r="I151" s="22" t="n">
+        <x:f>H151/G151</x:f>
+        <x:v>0.9938996120153241</x:v>
+      </x:c>
+      <x:c r="J151" s="24" t="n">
+        <x:v>15.993</x:v>
+      </x:c>
+      <x:c r="K151" s="24" t="n">
+        <x:v>16.163</x:v>
+      </x:c>
+      <x:c r="L151" s="24" t="n">
+        <x:f>K151/J151</x:f>
+        <x:v>1.0106296504720815</x:v>
+      </x:c>
+      <x:c r="M151" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N151" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O151" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P151" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q151" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R151" s="10" t="str">
+        <x:v>6cfa7aad3e</x:v>
+      </x:c>
+      <x:c r="S151" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_183058_cpp-dealer-router-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T151" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_183422_cpp-dealer-router-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U151" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V151" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 99.49%; latency median ratio 0.99x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="152">
-      <x:c r="A152" s="29"/>
-      <x:c r="G152" s="27"/>
-      <x:c r="H152" s="27"/>
-      <x:c r="I152" s="23"/>
-      <x:c r="J152" s="25"/>
-      <x:c r="K152" s="25"/>
-      <x:c r="L152" s="25"/>
+      <x:c r="A152" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B152" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C152" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D152" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E152" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F152" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G152" s="26" t="n">
+        <x:v>4704</x:v>
+      </x:c>
+      <x:c r="H152" s="26" t="n">
+        <x:v>5066.6</x:v>
+      </x:c>
+      <x:c r="I152" s="22" t="n">
+        <x:f>H152/G152</x:f>
+        <x:v>1.0770833333333334</x:v>
+      </x:c>
+      <x:c r="J152" s="24" t="n">
+        <x:v>12.921</x:v>
+      </x:c>
+      <x:c r="K152" s="24" t="n">
+        <x:v>12.253</x:v>
+      </x:c>
+      <x:c r="L152" s="24" t="n">
+        <x:f>K152/J152</x:f>
+        <x:v>0.9483012150762326</x:v>
+      </x:c>
+      <x:c r="M152" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N152" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O152" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P152" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q152" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R152" s="10" t="str">
+        <x:v>6cfa7aad3e</x:v>
+      </x:c>
+      <x:c r="S152" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_183058_cpp-dealer-router-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T152" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_183422_cpp-dealer-router-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U152" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V152" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 99.49%; latency median ratio 0.99x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="153">
-      <x:c r="A153" s="29"/>
-      <x:c r="G153" s="27"/>
-      <x:c r="H153" s="27"/>
-      <x:c r="I153" s="23"/>
-      <x:c r="J153" s="25"/>
-      <x:c r="K153" s="25"/>
-      <x:c r="L153" s="25"/>
+      <x:c r="A153" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B153" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C153" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D153" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E153" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F153" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G153" s="26" t="n">
+        <x:v>2647.8</x:v>
+      </x:c>
+      <x:c r="H153" s="26" t="n">
+        <x:v>2413.2</x:v>
+      </x:c>
+      <x:c r="I153" s="22" t="n">
+        <x:f>H153/G153</x:f>
+        <x:v>0.9113981418536142</x:v>
+      </x:c>
+      <x:c r="J153" s="24" t="n">
+        <x:v>12.268</x:v>
+      </x:c>
+      <x:c r="K153" s="24" t="n">
+        <x:v>14.257</x:v>
+      </x:c>
+      <x:c r="L153" s="24" t="n">
+        <x:f>K153/J153</x:f>
+        <x:v>1.162129116400391</x:v>
+      </x:c>
+      <x:c r="M153" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N153" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O153" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P153" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q153" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R153" s="10" t="str">
+        <x:v>6cfa7aad3e</x:v>
+      </x:c>
+      <x:c r="S153" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_183058_cpp-dealer-router-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T153" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_183422_cpp-dealer-router-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U153" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V153" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 99.49%; latency median ratio 0.99x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="29"/>

</xml_diff>

<commit_message>
docs(perf): record secure request baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R495f22bd94bf4b8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Ra0aae48a88484ffe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rd8de070a003c40ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R7df4b879a7434002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R3dac2ce3192d41e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R75746a3a91d04d78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R57234fe9bc604196"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R396560b1c2594860"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -11191,58 +11191,424 @@
       </x:c>
     </x:row>
     <x:row r="154">
-      <x:c r="A154" s="29"/>
-      <x:c r="G154" s="27"/>
-      <x:c r="H154" s="27"/>
-      <x:c r="I154" s="23"/>
-      <x:c r="J154" s="25"/>
-      <x:c r="K154" s="25"/>
-      <x:c r="L154" s="25"/>
+      <x:c r="A154" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B154" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C154" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D154" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E154" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F154" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G154" s="26" t="n">
+        <x:v>142614.8</x:v>
+      </x:c>
+      <x:c r="H154" s="26" t="n">
+        <x:v>62697.2</x:v>
+      </x:c>
+      <x:c r="I154" s="22" t="n">
+        <x:f>H154/G154</x:f>
+        <x:v>0.43962618185489866</x:v>
+      </x:c>
+      <x:c r="J154" s="24" t="n">
+        <x:v>0.376</x:v>
+      </x:c>
+      <x:c r="K154" s="24" t="n">
+        <x:v>0.951</x:v>
+      </x:c>
+      <x:c r="L154" s="24" t="n">
+        <x:f>K154/J154</x:f>
+        <x:v>2.529255319148936</x:v>
+      </x:c>
+      <x:c r="M154" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N154" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O154" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P154" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q154" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R154" s="10" t="str">
+        <x:v>a1687281a4</x:v>
+      </x:c>
+      <x:c r="S154" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_183908_cpp-dealer-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T154" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_184223_cpp-dealer-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U154" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V154" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 67.69%; latency median ratio 1.82x; fail. Candidate A exact-target contract no-go; retain existing async-only completion bridge B.</x:v>
+      </x:c>
     </x:row>
     <x:row r="155">
-      <x:c r="A155" s="29"/>
-      <x:c r="G155" s="27"/>
-      <x:c r="H155" s="27"/>
-      <x:c r="I155" s="23"/>
-      <x:c r="J155" s="25"/>
-      <x:c r="K155" s="25"/>
-      <x:c r="L155" s="25"/>
+      <x:c r="A155" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B155" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C155" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D155" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E155" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F155" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G155" s="26" t="n">
+        <x:v>102926.4</x:v>
+      </x:c>
+      <x:c r="H155" s="26" t="n">
+        <x:v>41096.4</x:v>
+      </x:c>
+      <x:c r="I155" s="22" t="n">
+        <x:f>H155/G155</x:f>
+        <x:v>0.39927948514666795</x:v>
+      </x:c>
+      <x:c r="J155" s="24" t="n">
+        <x:v>0.587</x:v>
+      </x:c>
+      <x:c r="K155" s="24" t="n">
+        <x:v>1.569</x:v>
+      </x:c>
+      <x:c r="L155" s="24" t="n">
+        <x:f>K155/J155</x:f>
+        <x:v>2.6729131175468486</x:v>
+      </x:c>
+      <x:c r="M155" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N155" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O155" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P155" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q155" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R155" s="10" t="str">
+        <x:v>a1687281a4</x:v>
+      </x:c>
+      <x:c r="S155" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_183908_cpp-dealer-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T155" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_184223_cpp-dealer-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U155" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V155" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 67.69%; latency median ratio 1.82x; fail. Candidate A exact-target contract no-go; retain existing async-only completion bridge B.</x:v>
+      </x:c>
     </x:row>
     <x:row r="156">
-      <x:c r="A156" s="29"/>
-      <x:c r="G156" s="27"/>
-      <x:c r="H156" s="27"/>
-      <x:c r="I156" s="23"/>
-      <x:c r="J156" s="25"/>
-      <x:c r="K156" s="25"/>
-      <x:c r="L156" s="25"/>
+      <x:c r="A156" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B156" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C156" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D156" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E156" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F156" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G156" s="26" t="n">
+        <x:v>58526.8</x:v>
+      </x:c>
+      <x:c r="H156" s="26" t="n">
+        <x:v>23933.6</x:v>
+      </x:c>
+      <x:c r="I156" s="22" t="n">
+        <x:f>H156/G156</x:f>
+        <x:v>0.40893402680481417</x:v>
+      </x:c>
+      <x:c r="J156" s="24" t="n">
+        <x:v>1.086</x:v>
+      </x:c>
+      <x:c r="K156" s="24" t="n">
+        <x:v>2.997</x:v>
+      </x:c>
+      <x:c r="L156" s="24" t="n">
+        <x:f>K156/J156</x:f>
+        <x:v>2.7596685082872927</x:v>
+      </x:c>
+      <x:c r="M156" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N156" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O156" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P156" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q156" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R156" s="10" t="str">
+        <x:v>a1687281a4</x:v>
+      </x:c>
+      <x:c r="S156" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_183908_cpp-dealer-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T156" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_184223_cpp-dealer-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U156" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V156" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 67.69%; latency median ratio 1.82x; fail. Candidate A exact-target contract no-go; retain existing async-only completion bridge B.</x:v>
+      </x:c>
     </x:row>
     <x:row r="157">
-      <x:c r="A157" s="29"/>
-      <x:c r="G157" s="27"/>
-      <x:c r="H157" s="27"/>
-      <x:c r="I157" s="23"/>
-      <x:c r="J157" s="25"/>
-      <x:c r="K157" s="25"/>
-      <x:c r="L157" s="25"/>
+      <x:c r="A157" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B157" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C157" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D157" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E157" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F157" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G157" s="26" t="n">
+        <x:v>3982</x:v>
+      </x:c>
+      <x:c r="H157" s="26" t="n">
+        <x:v>3561.4</x:v>
+      </x:c>
+      <x:c r="I157" s="22" t="n">
+        <x:f>H157/G157</x:f>
+        <x:v>0.8943746860873933</x:v>
+      </x:c>
+      <x:c r="J157" s="24" t="n">
+        <x:v>3.01</x:v>
+      </x:c>
+      <x:c r="K157" s="24" t="n">
+        <x:v>3.344</x:v>
+      </x:c>
+      <x:c r="L157" s="24" t="n">
+        <x:f>K157/J157</x:f>
+        <x:v>1.1109634551495018</x:v>
+      </x:c>
+      <x:c r="M157" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N157" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O157" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P157" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q157" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R157" s="10" t="str">
+        <x:v>a1687281a4</x:v>
+      </x:c>
+      <x:c r="S157" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_183908_cpp-dealer-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T157" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_184223_cpp-dealer-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U157" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V157" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 67.69%; latency median ratio 1.82x; fail. Candidate A exact-target contract no-go; retain existing async-only completion bridge B.</x:v>
+      </x:c>
     </x:row>
     <x:row r="158">
-      <x:c r="A158" s="29"/>
-      <x:c r="G158" s="27"/>
-      <x:c r="H158" s="27"/>
-      <x:c r="I158" s="23"/>
-      <x:c r="J158" s="25"/>
-      <x:c r="K158" s="25"/>
-      <x:c r="L158" s="25"/>
+      <x:c r="A158" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B158" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C158" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D158" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E158" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F158" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G158" s="26" t="n">
+        <x:v>2232.8</x:v>
+      </x:c>
+      <x:c r="H158" s="26" t="n">
+        <x:v>2131.6</x:v>
+      </x:c>
+      <x:c r="I158" s="22" t="n">
+        <x:f>H158/G158</x:f>
+        <x:v>0.9546757434611249</x:v>
+      </x:c>
+      <x:c r="J158" s="24" t="n">
+        <x:v>2.682</x:v>
+      </x:c>
+      <x:c r="K158" s="24" t="n">
+        <x:v>2.772</x:v>
+      </x:c>
+      <x:c r="L158" s="24" t="n">
+        <x:f>K158/J158</x:f>
+        <x:v>1.0335570469798656</x:v>
+      </x:c>
+      <x:c r="M158" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N158" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O158" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P158" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q158" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R158" s="10" t="str">
+        <x:v>a1687281a4</x:v>
+      </x:c>
+      <x:c r="S158" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_183908_cpp-dealer-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T158" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_184223_cpp-dealer-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U158" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V158" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 67.69%; latency median ratio 1.82x; fail. Candidate A exact-target contract no-go; retain existing async-only completion bridge B.</x:v>
+      </x:c>
     </x:row>
     <x:row r="159">
-      <x:c r="A159" s="29"/>
-      <x:c r="G159" s="27"/>
-      <x:c r="H159" s="27"/>
-      <x:c r="I159" s="23"/>
-      <x:c r="J159" s="25"/>
-      <x:c r="K159" s="25"/>
-      <x:c r="L159" s="25"/>
+      <x:c r="A159" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B159" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C159" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D159" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E159" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F159" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G159" s="26" t="n">
+        <x:v>1390.8</x:v>
+      </x:c>
+      <x:c r="H159" s="26" t="n">
+        <x:v>1341</x:v>
+      </x:c>
+      <x:c r="I159" s="22" t="n">
+        <x:f>H159/G159</x:f>
+        <x:v>0.9641932700603969</x:v>
+      </x:c>
+      <x:c r="J159" s="24" t="n">
+        <x:v>2.152</x:v>
+      </x:c>
+      <x:c r="K159" s="24" t="n">
+        <x:v>2.176</x:v>
+      </x:c>
+      <x:c r="L159" s="24" t="n">
+        <x:f>K159/J159</x:f>
+        <x:v>1.0111524163568772</x:v>
+      </x:c>
+      <x:c r="M159" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N159" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O159" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P159" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q159" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R159" s="10" t="str">
+        <x:v>a1687281a4</x:v>
+      </x:c>
+      <x:c r="S159" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_183908_cpp-dealer-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T159" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_184223_cpp-dealer-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U159" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V159" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 67.69%; latency median ratio 1.82x; fail. Candidate A exact-target contract no-go; retain existing async-only completion bridge B.</x:v>
+      </x:c>
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="29"/>

</xml_diff>

<commit_message>
docs(perf): record secure router baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R3dac2ce3192d41e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R75746a3a91d04d78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R57234fe9bc604196"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R396560b1c2594860"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra8b4f738444543de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rb6f312a56a7a4176"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R8900ac35648246f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R6022a123c0ca469f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss one-way 4개 통과 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss one-way 5개 통과·request/reply 1개 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -11611,58 +11611,424 @@
       </x:c>
     </x:row>
     <x:row r="160">
-      <x:c r="A160" s="29"/>
-      <x:c r="G160" s="27"/>
-      <x:c r="H160" s="27"/>
-      <x:c r="I160" s="23"/>
-      <x:c r="J160" s="25"/>
-      <x:c r="K160" s="25"/>
-      <x:c r="L160" s="25"/>
+      <x:c r="A160" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B160" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C160" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D160" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E160" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F160" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G160" s="26" t="n">
+        <x:v>2236686.8</x:v>
+      </x:c>
+      <x:c r="H160" s="26" t="n">
+        <x:v>1917481</x:v>
+      </x:c>
+      <x:c r="I160" s="22" t="n">
+        <x:f>H160/G160</x:f>
+        <x:v>0.8572863218936152</x:v>
+      </x:c>
+      <x:c r="J160" s="24" t="n">
+        <x:v>51.63</x:v>
+      </x:c>
+      <x:c r="K160" s="24" t="n">
+        <x:v>58.635</x:v>
+      </x:c>
+      <x:c r="L160" s="24" t="n">
+        <x:f>K160/J160</x:f>
+        <x:v>1.1356769320162696</x:v>
+      </x:c>
+      <x:c r="M160" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N160" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O160" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P160" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q160" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R160" s="10" t="str">
+        <x:v>0564e537c3</x:v>
+      </x:c>
+      <x:c r="S160" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_184800_cpp-router-router-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T160" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185042_cpp-router-router-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U160" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V160" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 94.69%; latency median ratio 1.05x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="161">
-      <x:c r="A161" s="29"/>
-      <x:c r="G161" s="27"/>
-      <x:c r="H161" s="27"/>
-      <x:c r="I161" s="23"/>
-      <x:c r="J161" s="25"/>
-      <x:c r="K161" s="25"/>
-      <x:c r="L161" s="25"/>
+      <x:c r="A161" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B161" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C161" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D161" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E161" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F161" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G161" s="26" t="n">
+        <x:v>842931.6</x:v>
+      </x:c>
+      <x:c r="H161" s="26" t="n">
+        <x:v>821014.2</x:v>
+      </x:c>
+      <x:c r="I161" s="22" t="n">
+        <x:f>H161/G161</x:f>
+        <x:v>0.973998602021801</x:v>
+      </x:c>
+      <x:c r="J161" s="24" t="n">
+        <x:v>40.203</x:v>
+      </x:c>
+      <x:c r="K161" s="24" t="n">
+        <x:v>41.444</x:v>
+      </x:c>
+      <x:c r="L161" s="24" t="n">
+        <x:f>K161/J161</x:f>
+        <x:v>1.0308683431584706</x:v>
+      </x:c>
+      <x:c r="M161" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N161" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O161" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P161" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q161" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R161" s="10" t="str">
+        <x:v>0564e537c3</x:v>
+      </x:c>
+      <x:c r="S161" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_184800_cpp-router-router-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T161" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185042_cpp-router-router-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U161" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V161" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 94.69%; latency median ratio 1.05x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="162">
-      <x:c r="A162" s="29"/>
-      <x:c r="G162" s="27"/>
-      <x:c r="H162" s="27"/>
-      <x:c r="I162" s="23"/>
-      <x:c r="J162" s="25"/>
-      <x:c r="K162" s="25"/>
-      <x:c r="L162" s="25"/>
+      <x:c r="A162" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B162" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C162" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D162" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E162" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F162" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G162" s="26" t="n">
+        <x:v>301970.4</x:v>
+      </x:c>
+      <x:c r="H162" s="26" t="n">
+        <x:v>287662.4</x:v>
+      </x:c>
+      <x:c r="I162" s="22" t="n">
+        <x:f>H162/G162</x:f>
+        <x:v>0.9526178724802166</x:v>
+      </x:c>
+      <x:c r="J162" s="24" t="n">
+        <x:v>27.669</x:v>
+      </x:c>
+      <x:c r="K162" s="24" t="n">
+        <x:v>31.733</x:v>
+      </x:c>
+      <x:c r="L162" s="24" t="n">
+        <x:f>K162/J162</x:f>
+        <x:v>1.146879178864433</x:v>
+      </x:c>
+      <x:c r="M162" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N162" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O162" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P162" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q162" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R162" s="10" t="str">
+        <x:v>0564e537c3</x:v>
+      </x:c>
+      <x:c r="S162" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_184800_cpp-router-router-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T162" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185042_cpp-router-router-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U162" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V162" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 94.69%; latency median ratio 1.05x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="163">
-      <x:c r="A163" s="29"/>
-      <x:c r="G163" s="27"/>
-      <x:c r="H163" s="27"/>
-      <x:c r="I163" s="23"/>
-      <x:c r="J163" s="25"/>
-      <x:c r="K163" s="25"/>
-      <x:c r="L163" s="25"/>
+      <x:c r="A163" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B163" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C163" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D163" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E163" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F163" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G163" s="26" t="n">
+        <x:v>9069</x:v>
+      </x:c>
+      <x:c r="H163" s="26" t="n">
+        <x:v>8871.6</x:v>
+      </x:c>
+      <x:c r="I163" s="22" t="n">
+        <x:f>H163/G163</x:f>
+        <x:v>0.9782335428382402</x:v>
+      </x:c>
+      <x:c r="J163" s="24" t="n">
+        <x:v>15.856</x:v>
+      </x:c>
+      <x:c r="K163" s="24" t="n">
+        <x:v>16.199</x:v>
+      </x:c>
+      <x:c r="L163" s="24" t="n">
+        <x:f>K163/J163</x:f>
+        <x:v>1.0216321897073664</x:v>
+      </x:c>
+      <x:c r="M163" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N163" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O163" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P163" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q163" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R163" s="10" t="str">
+        <x:v>0564e537c3</x:v>
+      </x:c>
+      <x:c r="S163" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_184800_cpp-router-router-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T163" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185042_cpp-router-router-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U163" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V163" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 94.69%; latency median ratio 1.05x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="164">
-      <x:c r="A164" s="29"/>
-      <x:c r="G164" s="27"/>
-      <x:c r="H164" s="27"/>
-      <x:c r="I164" s="23"/>
-      <x:c r="J164" s="25"/>
-      <x:c r="K164" s="25"/>
-      <x:c r="L164" s="25"/>
+      <x:c r="A164" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B164" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C164" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D164" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E164" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F164" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G164" s="26" t="n">
+        <x:v>5202.4</x:v>
+      </x:c>
+      <x:c r="H164" s="26" t="n">
+        <x:v>5187</x:v>
+      </x:c>
+      <x:c r="I164" s="22" t="n">
+        <x:f>H164/G164</x:f>
+        <x:v>0.9970398277717977</x:v>
+      </x:c>
+      <x:c r="J164" s="24" t="n">
+        <x:v>13.897</x:v>
+      </x:c>
+      <x:c r="K164" s="24" t="n">
+        <x:v>13.946</x:v>
+      </x:c>
+      <x:c r="L164" s="24" t="n">
+        <x:f>K164/J164</x:f>
+        <x:v>1.0035259408505433</x:v>
+      </x:c>
+      <x:c r="M164" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N164" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O164" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P164" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q164" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R164" s="10" t="str">
+        <x:v>0564e537c3</x:v>
+      </x:c>
+      <x:c r="S164" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_184800_cpp-router-router-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T164" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185042_cpp-router-router-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U164" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V164" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 94.69%; latency median ratio 1.05x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="165">
-      <x:c r="A165" s="29"/>
-      <x:c r="G165" s="27"/>
-      <x:c r="H165" s="27"/>
-      <x:c r="I165" s="23"/>
-      <x:c r="J165" s="25"/>
-      <x:c r="K165" s="25"/>
-      <x:c r="L165" s="25"/>
+      <x:c r="A165" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B165" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C165" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D165" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E165" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F165" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G165" s="26" t="n">
+        <x:v>2815.6</x:v>
+      </x:c>
+      <x:c r="H165" s="26" t="n">
+        <x:v>2596.2</x:v>
+      </x:c>
+      <x:c r="I165" s="22" t="n">
+        <x:f>H165/G165</x:f>
+        <x:v>0.9220769995738031</x:v>
+      </x:c>
+      <x:c r="J165" s="24" t="n">
+        <x:v>13.926</x:v>
+      </x:c>
+      <x:c r="K165" s="24" t="n">
+        <x:v>14.812</x:v>
+      </x:c>
+      <x:c r="L165" s="24" t="n">
+        <x:f>K165/J165</x:f>
+        <x:v>1.0636220020106275</x:v>
+      </x:c>
+      <x:c r="M165" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N165" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O165" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P165" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q165" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R165" s="10" t="str">
+        <x:v>0564e537c3</x:v>
+      </x:c>
+      <x:c r="S165" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_184800_cpp-router-router-wss-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T165" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185042_cpp-router-router-wss-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U165" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V165" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 94.69%; latency median ratio 1.05x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="29"/>

</xml_diff>

<commit_message>
docs(perf): record secure routed request baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra8b4f738444543de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rb6f312a56a7a4176"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R8900ac35648246f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R6022a123c0ca469f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rdf40b5bf9b824b63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R31c8e77e6aa34138"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R0a3a972ef1e5446c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R9b89ff78d5854599"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss one-way 5개 통과·request/reply 1개 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -12031,58 +12031,424 @@
       </x:c>
     </x:row>
     <x:row r="166">
-      <x:c r="A166" s="29"/>
-      <x:c r="G166" s="27"/>
-      <x:c r="H166" s="27"/>
-      <x:c r="I166" s="23"/>
-      <x:c r="J166" s="25"/>
-      <x:c r="K166" s="25"/>
-      <x:c r="L166" s="25"/>
+      <x:c r="A166" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B166" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C166" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D166" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E166" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F166" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G166" s="26" t="n">
+        <x:v>141672.2</x:v>
+      </x:c>
+      <x:c r="H166" s="26" t="n">
+        <x:v>59295.6</x:v>
+      </x:c>
+      <x:c r="I166" s="22" t="n">
+        <x:f>H166/G166</x:f>
+        <x:v>0.41854082875821785</x:v>
+      </x:c>
+      <x:c r="J166" s="24" t="n">
+        <x:v>0.376</x:v>
+      </x:c>
+      <x:c r="K166" s="24" t="n">
+        <x:v>1.01</x:v>
+      </x:c>
+      <x:c r="L166" s="24" t="n">
+        <x:f>K166/J166</x:f>
+        <x:v>2.6861702127659575</x:v>
+      </x:c>
+      <x:c r="M166" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N166" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O166" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P166" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q166" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R166" s="10" t="str">
+        <x:v>6a5d94932e</x:v>
+      </x:c>
+      <x:c r="S166" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_185524_cpp-router-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T166" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U166" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V166" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 64.35%; latency median ratio 1.86x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="167">
-      <x:c r="A167" s="29"/>
-      <x:c r="G167" s="27"/>
-      <x:c r="H167" s="27"/>
-      <x:c r="I167" s="23"/>
-      <x:c r="J167" s="25"/>
-      <x:c r="K167" s="25"/>
-      <x:c r="L167" s="25"/>
+      <x:c r="A167" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B167" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C167" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D167" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E167" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F167" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G167" s="26" t="n">
+        <x:v>103015</x:v>
+      </x:c>
+      <x:c r="H167" s="26" t="n">
+        <x:v>39973</x:v>
+      </x:c>
+      <x:c r="I167" s="22" t="n">
+        <x:f>H167/G167</x:f>
+        <x:v>0.38803086929088</x:v>
+      </x:c>
+      <x:c r="J167" s="24" t="n">
+        <x:v>0.617</x:v>
+      </x:c>
+      <x:c r="K167" s="24" t="n">
+        <x:v>1.548</x:v>
+      </x:c>
+      <x:c r="L167" s="24" t="n">
+        <x:f>K167/J167</x:f>
+        <x:v>2.5089141004862237</x:v>
+      </x:c>
+      <x:c r="M167" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N167" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O167" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P167" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q167" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R167" s="10" t="str">
+        <x:v>6a5d94932e</x:v>
+      </x:c>
+      <x:c r="S167" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_185524_cpp-router-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T167" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U167" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V167" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 64.35%; latency median ratio 1.86x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="168">
-      <x:c r="A168" s="29"/>
-      <x:c r="G168" s="27"/>
-      <x:c r="H168" s="27"/>
-      <x:c r="I168" s="23"/>
-      <x:c r="J168" s="25"/>
-      <x:c r="K168" s="25"/>
-      <x:c r="L168" s="25"/>
+      <x:c r="A168" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B168" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C168" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D168" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E168" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F168" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G168" s="26" t="n">
+        <x:v>60240.4</x:v>
+      </x:c>
+      <x:c r="H168" s="26" t="n">
+        <x:v>23256</x:v>
+      </x:c>
+      <x:c r="I168" s="22" t="n">
+        <x:f>H168/G168</x:f>
+        <x:v>0.38605321345807797</x:v>
+      </x:c>
+      <x:c r="J168" s="24" t="n">
+        <x:v>1.024</x:v>
+      </x:c>
+      <x:c r="K168" s="24" t="n">
+        <x:v>2.71</x:v>
+      </x:c>
+      <x:c r="L168" s="24" t="n">
+        <x:f>K168/J168</x:f>
+        <x:v>2.646484375</x:v>
+      </x:c>
+      <x:c r="M168" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N168" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O168" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P168" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q168" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R168" s="10" t="str">
+        <x:v>6a5d94932e</x:v>
+      </x:c>
+      <x:c r="S168" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_185524_cpp-router-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T168" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U168" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V168" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 64.35%; latency median ratio 1.86x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="169">
-      <x:c r="A169" s="29"/>
-      <x:c r="G169" s="27"/>
-      <x:c r="H169" s="27"/>
-      <x:c r="I169" s="23"/>
-      <x:c r="J169" s="25"/>
-      <x:c r="K169" s="25"/>
-      <x:c r="L169" s="25"/>
+      <x:c r="A169" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B169" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C169" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D169" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E169" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F169" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G169" s="26" t="n">
+        <x:v>3777.8</x:v>
+      </x:c>
+      <x:c r="H169" s="26" t="n">
+        <x:v>3378.8</x:v>
+      </x:c>
+      <x:c r="I169" s="22" t="n">
+        <x:f>H169/G169</x:f>
+        <x:v>0.8943829742177988</x:v>
+      </x:c>
+      <x:c r="J169" s="24" t="n">
+        <x:v>3.25</x:v>
+      </x:c>
+      <x:c r="K169" s="24" t="n">
+        <x:v>3.961</x:v>
+      </x:c>
+      <x:c r="L169" s="24" t="n">
+        <x:f>K169/J169</x:f>
+        <x:v>1.2187692307692308</x:v>
+      </x:c>
+      <x:c r="M169" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N169" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O169" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P169" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q169" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R169" s="10" t="str">
+        <x:v>6a5d94932e</x:v>
+      </x:c>
+      <x:c r="S169" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_185524_cpp-router-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T169" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U169" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V169" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 64.35%; latency median ratio 1.86x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="170">
-      <x:c r="A170" s="29"/>
-      <x:c r="G170" s="27"/>
-      <x:c r="H170" s="27"/>
-      <x:c r="I170" s="23"/>
-      <x:c r="J170" s="25"/>
-      <x:c r="K170" s="25"/>
-      <x:c r="L170" s="25"/>
+      <x:c r="A170" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B170" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C170" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D170" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E170" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F170" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G170" s="26" t="n">
+        <x:v>2417.2</x:v>
+      </x:c>
+      <x:c r="H170" s="26" t="n">
+        <x:v>2176.2</x:v>
+      </x:c>
+      <x:c r="I170" s="22" t="n">
+        <x:f>H170/G170</x:f>
+        <x:v>0.9002978652986927</x:v>
+      </x:c>
+      <x:c r="J170" s="24" t="n">
+        <x:v>2.478</x:v>
+      </x:c>
+      <x:c r="K170" s="24" t="n">
+        <x:v>2.722</x:v>
+      </x:c>
+      <x:c r="L170" s="24" t="n">
+        <x:f>K170/J170</x:f>
+        <x:v>1.0984665052461662</x:v>
+      </x:c>
+      <x:c r="M170" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N170" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O170" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P170" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q170" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R170" s="10" t="str">
+        <x:v>6a5d94932e</x:v>
+      </x:c>
+      <x:c r="S170" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_185524_cpp-router-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T170" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U170" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V170" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 64.35%; latency median ratio 1.86x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="171">
-      <x:c r="A171" s="29"/>
-      <x:c r="G171" s="27"/>
-      <x:c r="H171" s="27"/>
-      <x:c r="I171" s="23"/>
-      <x:c r="J171" s="25"/>
-      <x:c r="K171" s="25"/>
-      <x:c r="L171" s="25"/>
+      <x:c r="A171" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B171" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C171" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D171" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E171" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F171" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G171" s="26" t="n">
+        <x:v>1400.8</x:v>
+      </x:c>
+      <x:c r="H171" s="26" t="n">
+        <x:v>1223.8</x:v>
+      </x:c>
+      <x:c r="I171" s="22" t="n">
+        <x:f>H171/G171</x:f>
+        <x:v>0.8736436322101656</x:v>
+      </x:c>
+      <x:c r="J171" s="24" t="n">
+        <x:v>2.137</x:v>
+      </x:c>
+      <x:c r="K171" s="24" t="n">
+        <x:v>2.394</x:v>
+      </x:c>
+      <x:c r="L171" s="24" t="n">
+        <x:f>K171/J171</x:f>
+        <x:v>1.1202620496022462</x:v>
+      </x:c>
+      <x:c r="M171" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N171" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O171" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P171" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q171" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R171" s="10" t="str">
+        <x:v>6a5d94932e</x:v>
+      </x:c>
+      <x:c r="S171" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_185524_cpp-router-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T171" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U171" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V171" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 64.35%; latency median ratio 1.86x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="172">
       <x:c r="A172" s="29"/>
@@ -14751,12 +15117,86 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="L16" s="23"/>
-      <x:c r="M16" s="23"/>
+      <x:c r="A16" s="10" t="str">
+        <x:v>2026-08-25 19:03</x:v>
+      </x:c>
+      <x:c r="B16" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C16" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D16" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F16" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G16" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H16" s="10" t="str">
+        <x:v>Use Core normal route selection instead of the initially selected exact transport target.</x:v>
+      </x:c>
+      <x:c r="I16" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J16" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K16" s="10" t="str">
+        <x:v>N/A — exact-target contract no-go</x:v>
+      </x:c>
+      <x:c r="L16" s="22" t="n">
+        <x:v>0.643</x:v>
+      </x:c>
+      <x:c r="M16" s="22"/>
+      <x:c r="N16" s="10" t="str">
+        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership; exact-request-target contract remains required.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="L17" s="23"/>
-      <x:c r="M17" s="23"/>
+      <x:c r="A17" s="10" t="str">
+        <x:v>2026-08-25 19:03</x:v>
+      </x:c>
+      <x:c r="B17" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C17" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D17" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E17" s="10" t="str">
+        <x:v>wss</x:v>
+      </x:c>
+      <x:c r="F17" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G17" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H17" s="10" t="str">
+        <x:v>Retain the async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
+      </x:c>
+      <x:c r="I17" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J17" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_175007_cpp-router-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K17" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L17" s="22"/>
+      <x:c r="M17" s="22"/>
+      <x:c r="N17" s="10" t="str">
+        <x:v>KEEP: same Core/source implementation measured under WSS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. WSS throughput still misses the gate; latency 1.86x passes.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="L18" s="23"/>

</xml_diff>

<commit_message>
docs(perf): record tls pair baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rdf40b5bf9b824b63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R31c8e77e6aa34138"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R0a3a972ef1e5446c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R9b89ff78d5854599"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R85fd69eecb654870"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R975173ccf229478e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R5f12d52030d0409c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R1f786efb4908497c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls PAIR 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -12451,58 +12451,424 @@
       </x:c>
     </x:row>
     <x:row r="172">
-      <x:c r="A172" s="29"/>
-      <x:c r="G172" s="27"/>
-      <x:c r="H172" s="27"/>
-      <x:c r="I172" s="23"/>
-      <x:c r="J172" s="25"/>
-      <x:c r="K172" s="25"/>
-      <x:c r="L172" s="25"/>
+      <x:c r="A172" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B172" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C172" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D172" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E172" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F172" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G172" s="26" t="n">
+        <x:v>2381061.8</x:v>
+      </x:c>
+      <x:c r="H172" s="26" t="n">
+        <x:v>2152817.4</x:v>
+      </x:c>
+      <x:c r="I172" s="22" t="n">
+        <x:f>H172/G172</x:f>
+        <x:v>0.9041417572614033</x:v>
+      </x:c>
+      <x:c r="J172" s="24" t="n">
+        <x:v>0.539</x:v>
+      </x:c>
+      <x:c r="K172" s="24" t="n">
+        <x:v>0.382</x:v>
+      </x:c>
+      <x:c r="L172" s="24" t="n">
+        <x:f>K172/J172</x:f>
+        <x:v>0.7087198515769944</x:v>
+      </x:c>
+      <x:c r="M172" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N172" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O172" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P172" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q172" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R172" s="10" t="str">
+        <x:v>cf231e58f4</x:v>
+      </x:c>
+      <x:c r="S172" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_190411_cpp-pair-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T172" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U172" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V172" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 92.09%; latency median ratio 0.99x; strict gate fail. Existing bounded-pool A is already baseline; 64KiB-pool B remains timeout no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="173">
-      <x:c r="A173" s="29"/>
-      <x:c r="G173" s="27"/>
-      <x:c r="H173" s="27"/>
-      <x:c r="I173" s="23"/>
-      <x:c r="J173" s="25"/>
-      <x:c r="K173" s="25"/>
-      <x:c r="L173" s="25"/>
+      <x:c r="A173" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B173" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C173" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D173" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E173" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F173" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G173" s="26" t="n">
+        <x:v>925772.2</x:v>
+      </x:c>
+      <x:c r="H173" s="26" t="n">
+        <x:v>936106.4</x:v>
+      </x:c>
+      <x:c r="I173" s="22" t="n">
+        <x:f>H173/G173</x:f>
+        <x:v>1.0111627892909294</x:v>
+      </x:c>
+      <x:c r="J173" s="24" t="n">
+        <x:v>1.826</x:v>
+      </x:c>
+      <x:c r="K173" s="24" t="n">
+        <x:v>1.796</x:v>
+      </x:c>
+      <x:c r="L173" s="24" t="n">
+        <x:f>K173/J173</x:f>
+        <x:v>0.9835706462212486</x:v>
+      </x:c>
+      <x:c r="M173" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N173" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O173" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P173" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q173" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R173" s="10" t="str">
+        <x:v>cf231e58f4</x:v>
+      </x:c>
+      <x:c r="S173" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_190411_cpp-pair-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T173" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U173" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V173" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 92.09%; latency median ratio 0.99x; strict gate fail. Existing bounded-pool A is already baseline; 64KiB-pool B remains timeout no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="174">
-      <x:c r="A174" s="29"/>
-      <x:c r="G174" s="27"/>
-      <x:c r="H174" s="27"/>
-      <x:c r="I174" s="23"/>
-      <x:c r="J174" s="25"/>
-      <x:c r="K174" s="25"/>
-      <x:c r="L174" s="25"/>
+      <x:c r="A174" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B174" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C174" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D174" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E174" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F174" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G174" s="26" t="n">
+        <x:v>280878.4</x:v>
+      </x:c>
+      <x:c r="H174" s="26" t="n">
+        <x:v>278512.2</x:v>
+      </x:c>
+      <x:c r="I174" s="22" t="n">
+        <x:f>H174/G174</x:f>
+        <x:v>0.9915757139032406</x:v>
+      </x:c>
+      <x:c r="J174" s="24" t="n">
+        <x:v>1.761</x:v>
+      </x:c>
+      <x:c r="K174" s="24" t="n">
+        <x:v>1.767</x:v>
+      </x:c>
+      <x:c r="L174" s="24" t="n">
+        <x:f>K174/J174</x:f>
+        <x:v>1.0034071550255537</x:v>
+      </x:c>
+      <x:c r="M174" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N174" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O174" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P174" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q174" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R174" s="10" t="str">
+        <x:v>cf231e58f4</x:v>
+      </x:c>
+      <x:c r="S174" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_190411_cpp-pair-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T174" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U174" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V174" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 92.09%; latency median ratio 0.99x; strict gate fail. Existing bounded-pool A is already baseline; 64KiB-pool B remains timeout no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="175">
-      <x:c r="A175" s="29"/>
-      <x:c r="G175" s="27"/>
-      <x:c r="H175" s="27"/>
-      <x:c r="I175" s="23"/>
-      <x:c r="J175" s="25"/>
-      <x:c r="K175" s="25"/>
-      <x:c r="L175" s="25"/>
+      <x:c r="A175" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B175" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C175" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D175" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E175" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F175" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G175" s="26" t="n">
+        <x:v>11401.4</x:v>
+      </x:c>
+      <x:c r="H175" s="26" t="n">
+        <x:v>10499</x:v>
+      </x:c>
+      <x:c r="I175" s="22" t="n">
+        <x:f>H175/G175</x:f>
+        <x:v>0.9208518252144474</x:v>
+      </x:c>
+      <x:c r="J175" s="24" t="n">
+        <x:v>1.023</x:v>
+      </x:c>
+      <x:c r="K175" s="24" t="n">
+        <x:v>0.94</x:v>
+      </x:c>
+      <x:c r="L175" s="24" t="n">
+        <x:f>K175/J175</x:f>
+        <x:v>0.9188660801564028</x:v>
+      </x:c>
+      <x:c r="M175" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N175" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O175" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P175" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q175" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R175" s="10" t="str">
+        <x:v>cf231e58f4</x:v>
+      </x:c>
+      <x:c r="S175" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_190411_cpp-pair-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T175" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U175" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V175" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 92.09%; latency median ratio 0.99x; strict gate fail. Existing bounded-pool A is already baseline; 64KiB-pool B remains timeout no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="176">
-      <x:c r="A176" s="29"/>
-      <x:c r="G176" s="27"/>
-      <x:c r="H176" s="27"/>
-      <x:c r="I176" s="23"/>
-      <x:c r="J176" s="25"/>
-      <x:c r="K176" s="25"/>
-      <x:c r="L176" s="25"/>
+      <x:c r="A176" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B176" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C176" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D176" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E176" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F176" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G176" s="26" t="n">
+        <x:v>6907.6</x:v>
+      </x:c>
+      <x:c r="H176" s="26" t="n">
+        <x:v>6125.2</x:v>
+      </x:c>
+      <x:c r="I176" s="22" t="n">
+        <x:f>H176/G176</x:f>
+        <x:v>0.8867334530082807</x:v>
+      </x:c>
+      <x:c r="J176" s="24" t="n">
+        <x:v>0.881</x:v>
+      </x:c>
+      <x:c r="K176" s="24" t="n">
+        <x:v>1.167</x:v>
+      </x:c>
+      <x:c r="L176" s="24" t="n">
+        <x:f>K176/J176</x:f>
+        <x:v>1.3246311010215663</x:v>
+      </x:c>
+      <x:c r="M176" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N176" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O176" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P176" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q176" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R176" s="10" t="str">
+        <x:v>cf231e58f4</x:v>
+      </x:c>
+      <x:c r="S176" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_190411_cpp-pair-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T176" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U176" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V176" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 92.09%; latency median ratio 0.99x; strict gate fail. Existing bounded-pool A is already baseline; 64KiB-pool B remains timeout no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="177">
-      <x:c r="A177" s="29"/>
-      <x:c r="G177" s="27"/>
-      <x:c r="H177" s="27"/>
-      <x:c r="I177" s="23"/>
-      <x:c r="J177" s="25"/>
-      <x:c r="K177" s="25"/>
-      <x:c r="L177" s="25"/>
+      <x:c r="A177" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B177" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C177" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D177" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E177" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F177" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G177" s="26" t="n">
+        <x:v>3819.6</x:v>
+      </x:c>
+      <x:c r="H177" s="26" t="n">
+        <x:v>3096.6</x:v>
+      </x:c>
+      <x:c r="I177" s="22" t="n">
+        <x:f>H177/G177</x:f>
+        <x:v>0.8107131636820609</x:v>
+      </x:c>
+      <x:c r="J177" s="24" t="n">
+        <x:v>1.038</x:v>
+      </x:c>
+      <x:c r="K177" s="24" t="n">
+        <x:v>1.287</x:v>
+      </x:c>
+      <x:c r="L177" s="24" t="n">
+        <x:f>K177/J177</x:f>
+        <x:v>1.2398843930635837</x:v>
+      </x:c>
+      <x:c r="M177" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N177" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O177" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P177" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q177" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R177" s="10" t="str">
+        <x:v>cf231e58f4</x:v>
+      </x:c>
+      <x:c r="S177" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_190411_cpp-pair-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T177" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U177" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V177" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 92.09%; latency median ratio 0.99x; strict gate fail. Existing bounded-pool A is already baseline; 64KiB-pool B remains timeout no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="178">
       <x:c r="A178" s="29"/>
@@ -15199,12 +15565,88 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="L18" s="23"/>
-      <x:c r="M18" s="23"/>
+      <x:c r="A18" s="10" t="str">
+        <x:v>2026-08-25 19:10</x:v>
+      </x:c>
+      <x:c r="B18" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C18" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D18" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E18" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F18" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%</x:v>
+      </x:c>
+      <x:c r="G18" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H18" s="10" t="str">
+        <x:v>Re-evaluate the retained 128KiB–1MiB bounded pool and process-lifetime singleton.</x:v>
+      </x:c>
+      <x:c r="I18" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J18" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K18" s="10" t="str">
+        <x:v>N/A — already baseline</x:v>
+      </x:c>
+      <x:c r="L18" s="22" t="n">
+        <x:v>0.921</x:v>
+      </x:c>
+      <x:c r="M18" s="22"/>
+      <x:c r="N18" s="10" t="str">
+        <x:v>NO-GO as a new A/B: this safe candidate is already in source. It remains required for the existing ownership and late-release boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="L19" s="23"/>
-      <x:c r="M19" s="23"/>
+      <x:c r="A19" s="10" t="str">
+        <x:v>2026-08-25 19:10</x:v>
+      </x:c>
+      <x:c r="B19" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C19" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D19" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E19" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F19" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%</x:v>
+      </x:c>
+      <x:c r="G19" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H19" s="10" t="str">
+        <x:v>Lower pool threshold to 64KiB, remove lifetime guard/mutex, or enlarge pool cap.</x:v>
+      </x:c>
+      <x:c r="I19" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J19" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K19" s="10" t="str">
+        <x:v>N/A — timeout/contract/resource no-go</x:v>
+      </x:c>
+      <x:c r="L19" s="22" t="n">
+        <x:v>0.921</x:v>
+      </x:c>
+      <x:c r="M19" s="22"/>
+      <x:c r="N19" s="10" t="str">
+        <x:v>NO-GO: 64KiB pool variant previously timed out; guard removal and cap expansion violate documented concurrency or resource boundaries.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="L20" s="23"/>

</xml_diff>

<commit_message>
docs(perf): record tls pubsub baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R85fd69eecb654870"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R975173ccf229478e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R5f12d52030d0409c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R1f786efb4908497c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra6901413e38f41bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R5c8f598e7b374408"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R4112c3a931564c12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Ra2a259b504324992"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls PAIR 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls PAIR·PUBSUB 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -12871,58 +12871,424 @@
       </x:c>
     </x:row>
     <x:row r="178">
-      <x:c r="A178" s="29"/>
-      <x:c r="G178" s="27"/>
-      <x:c r="H178" s="27"/>
-      <x:c r="I178" s="23"/>
-      <x:c r="J178" s="25"/>
-      <x:c r="K178" s="25"/>
-      <x:c r="L178" s="25"/>
+      <x:c r="A178" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B178" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C178" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D178" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E178" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F178" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G178" s="26" t="n">
+        <x:v>1346233.4</x:v>
+      </x:c>
+      <x:c r="H178" s="26" t="n">
+        <x:v>1187729.8</x:v>
+      </x:c>
+      <x:c r="I178" s="22" t="n">
+        <x:f>H178/G178</x:f>
+        <x:v>0.8822614265847216</x:v>
+      </x:c>
+      <x:c r="J178" s="24" t="n">
+        <x:v>0.206</x:v>
+      </x:c>
+      <x:c r="K178" s="24" t="n">
+        <x:v>0.243</x:v>
+      </x:c>
+      <x:c r="L178" s="24" t="n">
+        <x:f>K178/J178</x:f>
+        <x:v>1.179611650485437</x:v>
+      </x:c>
+      <x:c r="M178" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N178" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O178" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P178" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q178" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R178" s="10" t="str">
+        <x:v>0babb638e9</x:v>
+      </x:c>
+      <x:c r="S178" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_191206_cpp-pubsub-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T178" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U178" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V178" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 92.13%; latency median ratio 1.11x; strict gate fail. Existing direct single-part publish and bounded-pool path are baseline; guard removal/pool expansion is no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="179">
-      <x:c r="A179" s="29"/>
-      <x:c r="G179" s="27"/>
-      <x:c r="H179" s="27"/>
-      <x:c r="I179" s="23"/>
-      <x:c r="J179" s="25"/>
-      <x:c r="K179" s="25"/>
-      <x:c r="L179" s="25"/>
+      <x:c r="A179" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B179" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C179" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D179" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E179" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F179" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G179" s="26" t="n">
+        <x:v>698794</x:v>
+      </x:c>
+      <x:c r="H179" s="26" t="n">
+        <x:v>717099</x:v>
+      </x:c>
+      <x:c r="I179" s="22" t="n">
+        <x:f>H179/G179</x:f>
+        <x:v>1.0261951304676342</x:v>
+      </x:c>
+      <x:c r="J179" s="24" t="n">
+        <x:v>2.028</x:v>
+      </x:c>
+      <x:c r="K179" s="24" t="n">
+        <x:v>1.991</x:v>
+      </x:c>
+      <x:c r="L179" s="24" t="n">
+        <x:f>K179/J179</x:f>
+        <x:v>0.9817554240631164</x:v>
+      </x:c>
+      <x:c r="M179" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N179" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O179" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P179" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q179" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R179" s="10" t="str">
+        <x:v>0babb638e9</x:v>
+      </x:c>
+      <x:c r="S179" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_191206_cpp-pubsub-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T179" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U179" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V179" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 92.13%; latency median ratio 1.11x; strict gate fail. Existing direct single-part publish and bounded-pool path are baseline; guard removal/pool expansion is no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="180">
-      <x:c r="A180" s="29"/>
-      <x:c r="G180" s="27"/>
-      <x:c r="H180" s="27"/>
-      <x:c r="I180" s="23"/>
-      <x:c r="J180" s="25"/>
-      <x:c r="K180" s="25"/>
-      <x:c r="L180" s="25"/>
+      <x:c r="A180" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B180" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C180" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D180" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E180" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F180" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G180" s="26" t="n">
+        <x:v>285636.2</x:v>
+      </x:c>
+      <x:c r="H180" s="26" t="n">
+        <x:v>271089.8</x:v>
+      </x:c>
+      <x:c r="I180" s="22" t="n">
+        <x:f>H180/G180</x:f>
+        <x:v>0.949073681837246</x:v>
+      </x:c>
+      <x:c r="J180" s="24" t="n">
+        <x:v>1.62</x:v>
+      </x:c>
+      <x:c r="K180" s="24" t="n">
+        <x:v>1.704</x:v>
+      </x:c>
+      <x:c r="L180" s="24" t="n">
+        <x:f>K180/J180</x:f>
+        <x:v>1.0518518518518518</x:v>
+      </x:c>
+      <x:c r="M180" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N180" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O180" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P180" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q180" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R180" s="10" t="str">
+        <x:v>0babb638e9</x:v>
+      </x:c>
+      <x:c r="S180" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_191206_cpp-pubsub-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T180" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U180" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V180" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 92.13%; latency median ratio 1.11x; strict gate fail. Existing direct single-part publish and bounded-pool path are baseline; guard removal/pool expansion is no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="181">
-      <x:c r="A181" s="29"/>
-      <x:c r="G181" s="27"/>
-      <x:c r="H181" s="27"/>
-      <x:c r="I181" s="23"/>
-      <x:c r="J181" s="25"/>
-      <x:c r="K181" s="25"/>
-      <x:c r="L181" s="25"/>
+      <x:c r="A181" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B181" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C181" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D181" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E181" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F181" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G181" s="26" t="n">
+        <x:v>11337.2</x:v>
+      </x:c>
+      <x:c r="H181" s="26" t="n">
+        <x:v>9903.2</x:v>
+      </x:c>
+      <x:c r="I181" s="22" t="n">
+        <x:f>H181/G181</x:f>
+        <x:v>0.8735137423702501</x:v>
+      </x:c>
+      <x:c r="J181" s="24" t="n">
+        <x:v>0.869</x:v>
+      </x:c>
+      <x:c r="K181" s="24" t="n">
+        <x:v>1.006</x:v>
+      </x:c>
+      <x:c r="L181" s="24" t="n">
+        <x:f>K181/J181</x:f>
+        <x:v>1.1576524741081704</x:v>
+      </x:c>
+      <x:c r="M181" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N181" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O181" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P181" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q181" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R181" s="10" t="str">
+        <x:v>0babb638e9</x:v>
+      </x:c>
+      <x:c r="S181" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_191206_cpp-pubsub-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T181" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U181" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V181" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 92.13%; latency median ratio 1.11x; strict gate fail. Existing direct single-part publish and bounded-pool path are baseline; guard removal/pool expansion is no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="182">
-      <x:c r="A182" s="29"/>
-      <x:c r="G182" s="27"/>
-      <x:c r="H182" s="27"/>
-      <x:c r="I182" s="23"/>
-      <x:c r="J182" s="25"/>
-      <x:c r="K182" s="25"/>
-      <x:c r="L182" s="25"/>
+      <x:c r="A182" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B182" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C182" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D182" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E182" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F182" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G182" s="26" t="n">
+        <x:v>6956.8</x:v>
+      </x:c>
+      <x:c r="H182" s="26" t="n">
+        <x:v>5694</x:v>
+      </x:c>
+      <x:c r="I182" s="22" t="n">
+        <x:f>H182/G182</x:f>
+        <x:v>0.8184797608095676</x:v>
+      </x:c>
+      <x:c r="J182" s="24" t="n">
+        <x:v>0.843</x:v>
+      </x:c>
+      <x:c r="K182" s="24" t="n">
+        <x:v>1.031</x:v>
+      </x:c>
+      <x:c r="L182" s="24" t="n">
+        <x:f>K182/J182</x:f>
+        <x:v>1.2230130486358244</x:v>
+      </x:c>
+      <x:c r="M182" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N182" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O182" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P182" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q182" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R182" s="10" t="str">
+        <x:v>0babb638e9</x:v>
+      </x:c>
+      <x:c r="S182" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_191206_cpp-pubsub-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T182" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U182" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V182" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 92.13%; latency median ratio 1.11x; strict gate fail. Existing direct single-part publish and bounded-pool path are baseline; guard removal/pool expansion is no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="183">
-      <x:c r="A183" s="29"/>
-      <x:c r="G183" s="27"/>
-      <x:c r="H183" s="27"/>
-      <x:c r="I183" s="23"/>
-      <x:c r="J183" s="25"/>
-      <x:c r="K183" s="25"/>
-      <x:c r="L183" s="25"/>
+      <x:c r="A183" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B183" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C183" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D183" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E183" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F183" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G183" s="26" t="n">
+        <x:v>3739.6</x:v>
+      </x:c>
+      <x:c r="H183" s="26" t="n">
+        <x:v>3658.4</x:v>
+      </x:c>
+      <x:c r="I183" s="22" t="n">
+        <x:f>H183/G183</x:f>
+        <x:v>0.9782864477484223</x:v>
+      </x:c>
+      <x:c r="J183" s="24" t="n">
+        <x:v>1.064</x:v>
+      </x:c>
+      <x:c r="K183" s="24" t="n">
+        <x:v>1.081</x:v>
+      </x:c>
+      <x:c r="L183" s="24" t="n">
+        <x:f>K183/J183</x:f>
+        <x:v>1.0159774436090225</x:v>
+      </x:c>
+      <x:c r="M183" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N183" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O183" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P183" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q183" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R183" s="10" t="str">
+        <x:v>0babb638e9</x:v>
+      </x:c>
+      <x:c r="S183" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_191206_cpp-pubsub-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T183" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U183" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V183" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 92.13%; latency median ratio 1.11x; strict gate fail. Existing direct single-part publish and bounded-pool path are baseline; guard removal/pool expansion is no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="184">
       <x:c r="A184" s="29"/>
@@ -15649,12 +16015,88 @@
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="L20" s="23"/>
-      <x:c r="M20" s="23"/>
+      <x:c r="A20" s="10" t="str">
+        <x:v>2026-08-25 19:18</x:v>
+      </x:c>
+      <x:c r="B20" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C20" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D20" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E20" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F20" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 95%</x:v>
+      </x:c>
+      <x:c r="G20" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H20" s="10" t="str">
+        <x:v>Re-evaluate direct single-part publish and operation-state reuse.</x:v>
+      </x:c>
+      <x:c r="I20" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J20" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K20" s="10" t="str">
+        <x:v>N/A — already baseline</x:v>
+      </x:c>
+      <x:c r="L20" s="22" t="n">
+        <x:v>0.921</x:v>
+      </x:c>
+      <x:c r="M20" s="22"/>
+      <x:c r="N20" s="10" t="str">
+        <x:v>NO-GO as a new A/B: the benchmark already uses the direct single-part publish path; multipart staging is not on this hot path.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="L21" s="23"/>
-      <x:c r="M21" s="23"/>
+      <x:c r="A21" s="10" t="str">
+        <x:v>2026-08-25 19:18</x:v>
+      </x:c>
+      <x:c r="B21" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C21" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D21" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E21" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F21" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 95%</x:v>
+      </x:c>
+      <x:c r="G21" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H21" s="10" t="str">
+        <x:v>Remove attempt mutex/lifetime guard, lower pool threshold, or expand pool cap.</x:v>
+      </x:c>
+      <x:c r="I21" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J21" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K21" s="10" t="str">
+        <x:v>N/A — contract/resource no-go</x:v>
+      </x:c>
+      <x:c r="L21" s="22" t="n">
+        <x:v>0.921</x:v>
+      </x:c>
+      <x:c r="M21" s="22"/>
+      <x:c r="N21" s="10" t="str">
+        <x:v>NO-GO: guard removal changes close/concurrency semantics; pool lower-bound/cap changes are global policy with a prior timeout or wider resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="L22" s="23"/>

</xml_diff>

<commit_message>
docs(perf): record tls dealer baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra6901413e38f41bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R5c8f598e7b374408"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R4112c3a931564c12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Ra2a259b504324992"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R49d756c355e04e7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R50d7f664a8384775"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R53a3898650604b7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R2de90f71c7d14be6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls PAIR·PUBSUB 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 1개 통과·2개 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -13291,58 +13291,424 @@
       </x:c>
     </x:row>
     <x:row r="184">
-      <x:c r="A184" s="29"/>
-      <x:c r="G184" s="27"/>
-      <x:c r="H184" s="27"/>
-      <x:c r="I184" s="23"/>
-      <x:c r="J184" s="25"/>
-      <x:c r="K184" s="25"/>
-      <x:c r="L184" s="25"/>
+      <x:c r="A184" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B184" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C184" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D184" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E184" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F184" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G184" s="26" t="n">
+        <x:v>2465682</x:v>
+      </x:c>
+      <x:c r="H184" s="26" t="n">
+        <x:v>2086431.6</x:v>
+      </x:c>
+      <x:c r="I184" s="22" t="n">
+        <x:f>H184/G184</x:f>
+        <x:v>0.8461884379250852</x:v>
+      </x:c>
+      <x:c r="J184" s="24" t="n">
+        <x:v>1.428</x:v>
+      </x:c>
+      <x:c r="K184" s="24" t="n">
+        <x:v>0.258</x:v>
+      </x:c>
+      <x:c r="L184" s="24" t="n">
+        <x:f>K184/J184</x:f>
+        <x:v>0.18067226890756305</x:v>
+      </x:c>
+      <x:c r="M184" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N184" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O184" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P184" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q184" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R184" s="10" t="str">
+        <x:v>1478293f23</x:v>
+      </x:c>
+      <x:c r="S184" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_192134_cpp-dealer-dealer-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T184" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_192434_cpp-dealer-dealer-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U184" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V184" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 87.56%; latency median ratio 1.14x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="185">
-      <x:c r="A185" s="29"/>
-      <x:c r="G185" s="27"/>
-      <x:c r="H185" s="27"/>
-      <x:c r="I185" s="23"/>
-      <x:c r="J185" s="25"/>
-      <x:c r="K185" s="25"/>
-      <x:c r="L185" s="25"/>
+      <x:c r="A185" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B185" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C185" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D185" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E185" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F185" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G185" s="26" t="n">
+        <x:v>878306.2</x:v>
+      </x:c>
+      <x:c r="H185" s="26" t="n">
+        <x:v>868524.2</x:v>
+      </x:c>
+      <x:c r="I185" s="22" t="n">
+        <x:f>H185/G185</x:f>
+        <x:v>0.9888626540493509</x:v>
+      </x:c>
+      <x:c r="J185" s="24" t="n">
+        <x:v>1.923</x:v>
+      </x:c>
+      <x:c r="K185" s="24" t="n">
+        <x:v>1.941</x:v>
+      </x:c>
+      <x:c r="L185" s="24" t="n">
+        <x:f>K185/J185</x:f>
+        <x:v>1.0093603744149766</x:v>
+      </x:c>
+      <x:c r="M185" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N185" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O185" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P185" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q185" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R185" s="10" t="str">
+        <x:v>1478293f23</x:v>
+      </x:c>
+      <x:c r="S185" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_192134_cpp-dealer-dealer-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T185" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_192434_cpp-dealer-dealer-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U185" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V185" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 87.56%; latency median ratio 1.14x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="186">
-      <x:c r="A186" s="29"/>
-      <x:c r="G186" s="27"/>
-      <x:c r="H186" s="27"/>
-      <x:c r="I186" s="23"/>
-      <x:c r="J186" s="25"/>
-      <x:c r="K186" s="25"/>
-      <x:c r="L186" s="25"/>
+      <x:c r="A186" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B186" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C186" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D186" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E186" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F186" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G186" s="26" t="n">
+        <x:v>296280</x:v>
+      </x:c>
+      <x:c r="H186" s="26" t="n">
+        <x:v>280958.4</x:v>
+      </x:c>
+      <x:c r="I186" s="22" t="n">
+        <x:f>H186/G186</x:f>
+        <x:v>0.9482867557715675</x:v>
+      </x:c>
+      <x:c r="J186" s="24" t="n">
+        <x:v>1.678</x:v>
+      </x:c>
+      <x:c r="K186" s="24" t="n">
+        <x:v>1.845</x:v>
+      </x:c>
+      <x:c r="L186" s="24" t="n">
+        <x:f>K186/J186</x:f>
+        <x:v>1.099523241954708</x:v>
+      </x:c>
+      <x:c r="M186" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N186" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O186" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P186" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q186" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R186" s="10" t="str">
+        <x:v>1478293f23</x:v>
+      </x:c>
+      <x:c r="S186" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_192134_cpp-dealer-dealer-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T186" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_192434_cpp-dealer-dealer-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U186" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V186" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 87.56%; latency median ratio 1.14x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="187">
-      <x:c r="A187" s="29"/>
-      <x:c r="G187" s="27"/>
-      <x:c r="H187" s="27"/>
-      <x:c r="I187" s="23"/>
-      <x:c r="J187" s="25"/>
-      <x:c r="K187" s="25"/>
-      <x:c r="L187" s="25"/>
+      <x:c r="A187" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B187" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C187" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D187" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E187" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F187" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G187" s="26" t="n">
+        <x:v>11412.8</x:v>
+      </x:c>
+      <x:c r="H187" s="26" t="n">
+        <x:v>9185.4</x:v>
+      </x:c>
+      <x:c r="I187" s="22" t="n">
+        <x:f>H187/G187</x:f>
+        <x:v>0.8048331697742885</x:v>
+      </x:c>
+      <x:c r="J187" s="24" t="n">
+        <x:v>0.916</x:v>
+      </x:c>
+      <x:c r="K187" s="24" t="n">
+        <x:v>1.112</x:v>
+      </x:c>
+      <x:c r="L187" s="24" t="n">
+        <x:f>K187/J187</x:f>
+        <x:v>1.2139737991266377</x:v>
+      </x:c>
+      <x:c r="M187" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N187" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O187" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P187" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q187" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R187" s="10" t="str">
+        <x:v>1478293f23</x:v>
+      </x:c>
+      <x:c r="S187" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_192134_cpp-dealer-dealer-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T187" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_192434_cpp-dealer-dealer-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U187" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V187" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 87.56%; latency median ratio 1.14x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="188">
-      <x:c r="A188" s="29"/>
-      <x:c r="G188" s="27"/>
-      <x:c r="H188" s="27"/>
-      <x:c r="I188" s="23"/>
-      <x:c r="J188" s="25"/>
-      <x:c r="K188" s="25"/>
-      <x:c r="L188" s="25"/>
+      <x:c r="A188" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B188" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C188" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D188" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E188" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F188" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G188" s="26" t="n">
+        <x:v>6891</x:v>
+      </x:c>
+      <x:c r="H188" s="26" t="n">
+        <x:v>5939.8</x:v>
+      </x:c>
+      <x:c r="I188" s="22" t="n">
+        <x:f>H188/G188</x:f>
+        <x:v>0.8619648817297925</x:v>
+      </x:c>
+      <x:c r="J188" s="24" t="n">
+        <x:v>0.845</x:v>
+      </x:c>
+      <x:c r="K188" s="24" t="n">
+        <x:v>0.99</x:v>
+      </x:c>
+      <x:c r="L188" s="24" t="n">
+        <x:f>K188/J188</x:f>
+        <x:v>1.1715976331360947</x:v>
+      </x:c>
+      <x:c r="M188" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N188" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O188" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P188" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q188" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R188" s="10" t="str">
+        <x:v>1478293f23</x:v>
+      </x:c>
+      <x:c r="S188" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_192134_cpp-dealer-dealer-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T188" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_192434_cpp-dealer-dealer-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U188" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V188" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 87.56%; latency median ratio 1.14x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="189">
-      <x:c r="A189" s="29"/>
-      <x:c r="G189" s="27"/>
-      <x:c r="H189" s="27"/>
-      <x:c r="I189" s="23"/>
-      <x:c r="J189" s="25"/>
-      <x:c r="K189" s="25"/>
-      <x:c r="L189" s="25"/>
+      <x:c r="A189" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B189" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C189" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D189" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E189" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F189" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G189" s="26" t="n">
+        <x:v>3831.8</x:v>
+      </x:c>
+      <x:c r="H189" s="26" t="n">
+        <x:v>3078.6</x:v>
+      </x:c>
+      <x:c r="I189" s="22" t="n">
+        <x:f>H189/G189</x:f>
+        <x:v>0.8034344172451588</x:v>
+      </x:c>
+      <x:c r="J189" s="24" t="n">
+        <x:v>1.025</x:v>
+      </x:c>
+      <x:c r="K189" s="24" t="n">
+        <x:v>1.28</x:v>
+      </x:c>
+      <x:c r="L189" s="24" t="n">
+        <x:f>K189/J189</x:f>
+        <x:v>1.2487804878048783</x:v>
+      </x:c>
+      <x:c r="M189" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N189" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O189" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P189" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q189" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R189" s="10" t="str">
+        <x:v>1478293f23</x:v>
+      </x:c>
+      <x:c r="S189" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_192134_cpp-dealer-dealer-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T189" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_192434_cpp-dealer-dealer-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U189" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V189" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 87.56%; latency median ratio 1.14x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="190">
       <x:c r="A190" s="29"/>

</xml_diff>

<commit_message>
docs(perf): record tls dealer router baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R49d756c355e04e7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R50d7f664a8384775"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R53a3898650604b7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R2de90f71c7d14be6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rbd0b0c63eea24321"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rb0d8f62972644fd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R1949766aa90647e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R36a55fdffdbd4bc3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 1개 통과·2개 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 2개 통과·2개 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -13711,58 +13711,424 @@
       </x:c>
     </x:row>
     <x:row r="190">
-      <x:c r="A190" s="29"/>
-      <x:c r="G190" s="27"/>
-      <x:c r="H190" s="27"/>
-      <x:c r="I190" s="23"/>
-      <x:c r="J190" s="25"/>
-      <x:c r="K190" s="25"/>
-      <x:c r="L190" s="25"/>
+      <x:c r="A190" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B190" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C190" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D190" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E190" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F190" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G190" s="26" t="n">
+        <x:v>2436674.2</x:v>
+      </x:c>
+      <x:c r="H190" s="26" t="n">
+        <x:v>2059328.8</x:v>
+      </x:c>
+      <x:c r="I190" s="22" t="n">
+        <x:f>H190/G190</x:f>
+        <x:v>0.8451391655068207</x:v>
+      </x:c>
+      <x:c r="J190" s="24" t="n">
+        <x:v>1.851</x:v>
+      </x:c>
+      <x:c r="K190" s="24" t="n">
+        <x:v>0.395</x:v>
+      </x:c>
+      <x:c r="L190" s="24" t="n">
+        <x:f>K190/J190</x:f>
+        <x:v>0.21339816315505133</x:v>
+      </x:c>
+      <x:c r="M190" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N190" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O190" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P190" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q190" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R190" s="10" t="str">
+        <x:v>5fd4317d72</x:v>
+      </x:c>
+      <x:c r="S190" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_192917_cpp-dealer-router-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T190" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193201_cpp-dealer-router-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U190" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V190" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 89.96%; latency median ratio 1.10x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="191">
-      <x:c r="A191" s="29"/>
-      <x:c r="G191" s="27"/>
-      <x:c r="H191" s="27"/>
-      <x:c r="I191" s="23"/>
-      <x:c r="J191" s="25"/>
-      <x:c r="K191" s="25"/>
-      <x:c r="L191" s="25"/>
+      <x:c r="A191" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B191" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C191" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D191" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E191" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F191" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G191" s="26" t="n">
+        <x:v>920407.2</x:v>
+      </x:c>
+      <x:c r="H191" s="26" t="n">
+        <x:v>947458.8</x:v>
+      </x:c>
+      <x:c r="I191" s="22" t="n">
+        <x:f>H191/G191</x:f>
+        <x:v>1.0293909043736296</x:v>
+      </x:c>
+      <x:c r="J191" s="24" t="n">
+        <x:v>1.83</x:v>
+      </x:c>
+      <x:c r="K191" s="24" t="n">
+        <x:v>1.779</x:v>
+      </x:c>
+      <x:c r="L191" s="24" t="n">
+        <x:f>K191/J191</x:f>
+        <x:v>0.9721311475409835</x:v>
+      </x:c>
+      <x:c r="M191" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N191" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O191" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P191" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q191" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R191" s="10" t="str">
+        <x:v>5fd4317d72</x:v>
+      </x:c>
+      <x:c r="S191" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_192917_cpp-dealer-router-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T191" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193201_cpp-dealer-router-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U191" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V191" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 89.96%; latency median ratio 1.10x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="192">
-      <x:c r="A192" s="29"/>
-      <x:c r="G192" s="27"/>
-      <x:c r="H192" s="27"/>
-      <x:c r="I192" s="23"/>
-      <x:c r="J192" s="25"/>
-      <x:c r="K192" s="25"/>
-      <x:c r="L192" s="25"/>
+      <x:c r="A192" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B192" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C192" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D192" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E192" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F192" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G192" s="26" t="n">
+        <x:v>294091</x:v>
+      </x:c>
+      <x:c r="H192" s="26" t="n">
+        <x:v>287499.6</x:v>
+      </x:c>
+      <x:c r="I192" s="22" t="n">
+        <x:f>H192/G192</x:f>
+        <x:v>0.9775872094011717</x:v>
+      </x:c>
+      <x:c r="J192" s="24" t="n">
+        <x:v>1.665</x:v>
+      </x:c>
+      <x:c r="K192" s="24" t="n">
+        <x:v>1.709</x:v>
+      </x:c>
+      <x:c r="L192" s="24" t="n">
+        <x:f>K192/J192</x:f>
+        <x:v>1.0264264264264265</x:v>
+      </x:c>
+      <x:c r="M192" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N192" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O192" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P192" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q192" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R192" s="10" t="str">
+        <x:v>5fd4317d72</x:v>
+      </x:c>
+      <x:c r="S192" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_192917_cpp-dealer-router-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T192" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193201_cpp-dealer-router-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U192" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V192" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 89.96%; latency median ratio 1.10x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="193">
-      <x:c r="A193" s="29"/>
-      <x:c r="G193" s="27"/>
-      <x:c r="H193" s="27"/>
-      <x:c r="I193" s="23"/>
-      <x:c r="J193" s="25"/>
-      <x:c r="K193" s="25"/>
-      <x:c r="L193" s="25"/>
+      <x:c r="A193" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B193" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C193" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D193" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E193" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F193" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G193" s="26" t="n">
+        <x:v>11689.6</x:v>
+      </x:c>
+      <x:c r="H193" s="26" t="n">
+        <x:v>10004.4</x:v>
+      </x:c>
+      <x:c r="I193" s="22" t="n">
+        <x:f>H193/G193</x:f>
+        <x:v>0.8558376676704078</x:v>
+      </x:c>
+      <x:c r="J193" s="24" t="n">
+        <x:v>0.835</x:v>
+      </x:c>
+      <x:c r="K193" s="24" t="n">
+        <x:v>1.007</x:v>
+      </x:c>
+      <x:c r="L193" s="24" t="n">
+        <x:f>K193/J193</x:f>
+        <x:v>1.2059880239520957</x:v>
+      </x:c>
+      <x:c r="M193" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N193" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O193" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P193" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q193" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R193" s="10" t="str">
+        <x:v>5fd4317d72</x:v>
+      </x:c>
+      <x:c r="S193" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_192917_cpp-dealer-router-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T193" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193201_cpp-dealer-router-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U193" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V193" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 89.96%; latency median ratio 1.10x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="194">
-      <x:c r="A194" s="29"/>
-      <x:c r="G194" s="27"/>
-      <x:c r="H194" s="27"/>
-      <x:c r="I194" s="23"/>
-      <x:c r="J194" s="25"/>
-      <x:c r="K194" s="25"/>
-      <x:c r="L194" s="25"/>
+      <x:c r="A194" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B194" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C194" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D194" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E194" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F194" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G194" s="26" t="n">
+        <x:v>6767.4</x:v>
+      </x:c>
+      <x:c r="H194" s="26" t="n">
+        <x:v>5544.6</x:v>
+      </x:c>
+      <x:c r="I194" s="22" t="n">
+        <x:f>H194/G194</x:f>
+        <x:v>0.8193102225374591</x:v>
+      </x:c>
+      <x:c r="J194" s="24" t="n">
+        <x:v>0.876</x:v>
+      </x:c>
+      <x:c r="K194" s="24" t="n">
+        <x:v>1.068</x:v>
+      </x:c>
+      <x:c r="L194" s="24" t="n">
+        <x:f>K194/J194</x:f>
+        <x:v>1.2191780821917808</x:v>
+      </x:c>
+      <x:c r="M194" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N194" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O194" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P194" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q194" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R194" s="10" t="str">
+        <x:v>5fd4317d72</x:v>
+      </x:c>
+      <x:c r="S194" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_192917_cpp-dealer-router-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T194" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193201_cpp-dealer-router-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U194" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V194" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 89.96%; latency median ratio 1.10x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="195">
-      <x:c r="A195" s="29"/>
-      <x:c r="G195" s="27"/>
-      <x:c r="H195" s="27"/>
-      <x:c r="I195" s="23"/>
-      <x:c r="J195" s="25"/>
-      <x:c r="K195" s="25"/>
-      <x:c r="L195" s="25"/>
+      <x:c r="A195" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B195" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C195" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D195" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E195" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F195" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G195" s="26" t="n">
+        <x:v>3520.2</x:v>
+      </x:c>
+      <x:c r="H195" s="26" t="n">
+        <x:v>3064</x:v>
+      </x:c>
+      <x:c r="I195" s="22" t="n">
+        <x:f>H195/G195</x:f>
+        <x:v>0.8704050906198512</x:v>
+      </x:c>
+      <x:c r="J195" s="24" t="n">
+        <x:v>1.207</x:v>
+      </x:c>
+      <x:c r="K195" s="24" t="n">
+        <x:v>1.427</x:v>
+      </x:c>
+      <x:c r="L195" s="24" t="n">
+        <x:f>K195/J195</x:f>
+        <x:v>1.1822700911350454</x:v>
+      </x:c>
+      <x:c r="M195" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N195" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O195" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P195" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q195" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R195" s="10" t="str">
+        <x:v>5fd4317d72</x:v>
+      </x:c>
+      <x:c r="S195" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_192917_cpp-dealer-router-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T195" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193201_cpp-dealer-router-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U195" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V195" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 89.96%; latency median ratio 1.10x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="29"/>

</xml_diff>

<commit_message>
docs(perf): record tls routed request baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rbd0b0c63eea24321"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rb0d8f62972644fd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R1949766aa90647e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R36a55fdffdbd4bc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R571a2db172424af2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rc08e7054e7d84327"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R7f3886a86df449d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R82a02a2cda4e486c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 2개 통과·2개 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 2개 통과·3개 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -14131,58 +14131,424 @@
       </x:c>
     </x:row>
     <x:row r="196">
-      <x:c r="A196" s="29"/>
-      <x:c r="G196" s="27"/>
-      <x:c r="H196" s="27"/>
-      <x:c r="I196" s="23"/>
-      <x:c r="J196" s="25"/>
-      <x:c r="K196" s="25"/>
-      <x:c r="L196" s="25"/>
+      <x:c r="A196" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B196" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C196" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D196" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E196" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F196" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G196" s="26" t="n">
+        <x:v>164868.2</x:v>
+      </x:c>
+      <x:c r="H196" s="26" t="n">
+        <x:v>83005</x:v>
+      </x:c>
+      <x:c r="I196" s="22" t="n">
+        <x:f>H196/G196</x:f>
+        <x:v>0.5034627660155202</x:v>
+      </x:c>
+      <x:c r="J196" s="24" t="n">
+        <x:v>0.318</x:v>
+      </x:c>
+      <x:c r="K196" s="24" t="n">
+        <x:v>0.77</x:v>
+      </x:c>
+      <x:c r="L196" s="24" t="n">
+        <x:f>K196/J196</x:f>
+        <x:v>2.4213836477987423</x:v>
+      </x:c>
+      <x:c r="M196" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N196" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O196" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P196" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q196" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R196" s="10" t="str">
+        <x:v>e1c0641269</x:v>
+      </x:c>
+      <x:c r="S196" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_193626_cpp-dealer-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T196" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U196" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V196" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 70.94%; latency median ratio 1.62x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="197">
-      <x:c r="A197" s="29"/>
-      <x:c r="G197" s="27"/>
-      <x:c r="H197" s="27"/>
-      <x:c r="I197" s="23"/>
-      <x:c r="J197" s="25"/>
-      <x:c r="K197" s="25"/>
-      <x:c r="L197" s="25"/>
+      <x:c r="A197" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B197" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C197" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D197" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E197" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F197" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G197" s="26" t="n">
+        <x:v>151414.6</x:v>
+      </x:c>
+      <x:c r="H197" s="26" t="n">
+        <x:v>78458.8</x:v>
+      </x:c>
+      <x:c r="I197" s="22" t="n">
+        <x:f>H197/G197</x:f>
+        <x:v>0.518171959639295</x:v>
+      </x:c>
+      <x:c r="J197" s="24" t="n">
+        <x:v>0.332</x:v>
+      </x:c>
+      <x:c r="K197" s="24" t="n">
+        <x:v>0.731</x:v>
+      </x:c>
+      <x:c r="L197" s="24" t="n">
+        <x:f>K197/J197</x:f>
+        <x:v>2.2018072289156625</x:v>
+      </x:c>
+      <x:c r="M197" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N197" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O197" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P197" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q197" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R197" s="10" t="str">
+        <x:v>e1c0641269</x:v>
+      </x:c>
+      <x:c r="S197" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_193626_cpp-dealer-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T197" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U197" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V197" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 70.94%; latency median ratio 1.62x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="198">
-      <x:c r="A198" s="29"/>
-      <x:c r="G198" s="27"/>
-      <x:c r="H198" s="27"/>
-      <x:c r="I198" s="23"/>
-      <x:c r="J198" s="25"/>
-      <x:c r="K198" s="25"/>
-      <x:c r="L198" s="25"/>
+      <x:c r="A198" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B198" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C198" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D198" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E198" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F198" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G198" s="26" t="n">
+        <x:v>83546.8</x:v>
+      </x:c>
+      <x:c r="H198" s="26" t="n">
+        <x:v>40911.4</x:v>
+      </x:c>
+      <x:c r="I198" s="22" t="n">
+        <x:f>H198/G198</x:f>
+        <x:v>0.48968242948862195</x:v>
+      </x:c>
+      <x:c r="J198" s="24" t="n">
+        <x:v>0.714</x:v>
+      </x:c>
+      <x:c r="K198" s="24" t="n">
+        <x:v>1.514</x:v>
+      </x:c>
+      <x:c r="L198" s="24" t="n">
+        <x:f>K198/J198</x:f>
+        <x:v>2.1204481792717087</x:v>
+      </x:c>
+      <x:c r="M198" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N198" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O198" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P198" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q198" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R198" s="10" t="str">
+        <x:v>e1c0641269</x:v>
+      </x:c>
+      <x:c r="S198" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_193626_cpp-dealer-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T198" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U198" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V198" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 70.94%; latency median ratio 1.62x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="199">
-      <x:c r="A199" s="29"/>
-      <x:c r="G199" s="27"/>
-      <x:c r="H199" s="27"/>
-      <x:c r="I199" s="23"/>
-      <x:c r="J199" s="25"/>
-      <x:c r="K199" s="25"/>
-      <x:c r="L199" s="25"/>
+      <x:c r="A199" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B199" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C199" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D199" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E199" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F199" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G199" s="26" t="n">
+        <x:v>4831.8</x:v>
+      </x:c>
+      <x:c r="H199" s="26" t="n">
+        <x:v>4278</x:v>
+      </x:c>
+      <x:c r="I199" s="22" t="n">
+        <x:f>H199/G199</x:f>
+        <x:v>0.8853843288215572</x:v>
+      </x:c>
+      <x:c r="J199" s="24" t="n">
+        <x:v>2.476</x:v>
+      </x:c>
+      <x:c r="K199" s="24" t="n">
+        <x:v>2.776</x:v>
+      </x:c>
+      <x:c r="L199" s="24" t="n">
+        <x:f>K199/J199</x:f>
+        <x:v>1.121163166397415</x:v>
+      </x:c>
+      <x:c r="M199" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N199" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O199" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P199" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q199" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R199" s="10" t="str">
+        <x:v>e1c0641269</x:v>
+      </x:c>
+      <x:c r="S199" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_193626_cpp-dealer-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T199" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U199" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V199" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 70.94%; latency median ratio 1.62x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="200">
-      <x:c r="A200" s="29"/>
-      <x:c r="G200" s="27"/>
-      <x:c r="H200" s="27"/>
-      <x:c r="I200" s="23"/>
-      <x:c r="J200" s="25"/>
-      <x:c r="K200" s="25"/>
-      <x:c r="L200" s="25"/>
+      <x:c r="A200" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B200" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C200" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D200" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E200" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F200" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G200" s="26" t="n">
+        <x:v>2933.8</x:v>
+      </x:c>
+      <x:c r="H200" s="26" t="n">
+        <x:v>2807</x:v>
+      </x:c>
+      <x:c r="I200" s="22" t="n">
+        <x:f>H200/G200</x:f>
+        <x:v>0.9567796032449383</x:v>
+      </x:c>
+      <x:c r="J200" s="24" t="n">
+        <x:v>2.04</x:v>
+      </x:c>
+      <x:c r="K200" s="24" t="n">
+        <x:v>2.1</x:v>
+      </x:c>
+      <x:c r="L200" s="24" t="n">
+        <x:f>K200/J200</x:f>
+        <x:v>1.0294117647058825</x:v>
+      </x:c>
+      <x:c r="M200" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N200" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O200" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P200" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q200" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R200" s="10" t="str">
+        <x:v>e1c0641269</x:v>
+      </x:c>
+      <x:c r="S200" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_193626_cpp-dealer-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T200" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U200" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V200" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 70.94%; latency median ratio 1.62x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="201">
-      <x:c r="A201" s="29"/>
-      <x:c r="G201" s="27"/>
-      <x:c r="H201" s="27"/>
-      <x:c r="I201" s="23"/>
-      <x:c r="J201" s="25"/>
-      <x:c r="K201" s="25"/>
-      <x:c r="L201" s="25"/>
+      <x:c r="A201" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B201" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C201" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D201" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E201" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F201" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G201" s="26" t="n">
+        <x:v>1767.6</x:v>
+      </x:c>
+      <x:c r="H201" s="26" t="n">
+        <x:v>1596.4</x:v>
+      </x:c>
+      <x:c r="I201" s="22" t="n">
+        <x:f>H201/G201</x:f>
+        <x:v>0.9031455080334918</x:v>
+      </x:c>
+      <x:c r="J201" s="24" t="n">
+        <x:v>1.715</x:v>
+      </x:c>
+      <x:c r="K201" s="24" t="n">
+        <x:v>1.815</x:v>
+      </x:c>
+      <x:c r="L201" s="24" t="n">
+        <x:f>K201/J201</x:f>
+        <x:v>1.0583090379008746</x:v>
+      </x:c>
+      <x:c r="M201" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N201" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O201" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P201" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q201" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R201" s="10" t="str">
+        <x:v>e1c0641269</x:v>
+      </x:c>
+      <x:c r="S201" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_193626_cpp-dealer-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T201" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U201" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V201" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 70.94%; latency median ratio 1.62x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="202">
       <x:c r="A202" s="29"/>
@@ -16831,12 +17197,86 @@
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="L22" s="23"/>
-      <x:c r="M22" s="23"/>
+      <x:c r="A22" s="10" t="str">
+        <x:v>2026-08-25 19:43</x:v>
+      </x:c>
+      <x:c r="B22" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C22" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D22" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E22" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F22" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G22" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H22" s="10" t="str">
+        <x:v>Use Core normal DEALER request route instead of initially selected exact transport target.</x:v>
+      </x:c>
+      <x:c r="I22" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J22" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K22" s="10" t="str">
+        <x:v>N/A — exact-target contract no-go</x:v>
+      </x:c>
+      <x:c r="L22" s="22" t="n">
+        <x:v>0.709</x:v>
+      </x:c>
+      <x:c r="M22" s="22"/>
+      <x:c r="N22" s="10" t="str">
+        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="L23" s="23"/>
-      <x:c r="M23" s="23"/>
+      <x:c r="A23" s="10" t="str">
+        <x:v>2026-08-25 19:43</x:v>
+      </x:c>
+      <x:c r="B23" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C23" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D23" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E23" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F23" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G23" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H23" s="10" t="str">
+        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
+      </x:c>
+      <x:c r="I23" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J23" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K23" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L23" s="22"/>
+      <x:c r="M23" s="22"/>
+      <x:c r="N23" s="10" t="str">
+        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.62x passes.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="L24" s="23"/>

</xml_diff>

<commit_message>
docs(perf): record tls router baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R571a2db172424af2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rc08e7054e7d84327"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R7f3886a86df449d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R82a02a2cda4e486c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rece3148c004f4efe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R0bbc34b37f7a47dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R65690d07689c49ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Re6e824eef7f84ca5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 2개 통과·3개 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 3개 통과·3개 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -541,7 +541,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -14551,58 +14551,424 @@
       </x:c>
     </x:row>
     <x:row r="202">
-      <x:c r="A202" s="29"/>
-      <x:c r="G202" s="27"/>
-      <x:c r="H202" s="27"/>
-      <x:c r="I202" s="23"/>
-      <x:c r="J202" s="25"/>
-      <x:c r="K202" s="25"/>
-      <x:c r="L202" s="25"/>
+      <x:c r="A202" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B202" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C202" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D202" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E202" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F202" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G202" s="26" t="n">
+        <x:v>2228918.6</x:v>
+      </x:c>
+      <x:c r="H202" s="26" t="n">
+        <x:v>1930843.6</x:v>
+      </x:c>
+      <x:c r="I202" s="22" t="n">
+        <x:f>H202/G202</x:f>
+        <x:v>0.8662692302895225</x:v>
+      </x:c>
+      <x:c r="J202" s="24" t="n">
+        <x:v>38.989</x:v>
+      </x:c>
+      <x:c r="K202" s="24" t="n">
+        <x:v>46.117</x:v>
+      </x:c>
+      <x:c r="L202" s="24" t="n">
+        <x:f>K202/J202</x:f>
+        <x:v>1.182820795609018</x:v>
+      </x:c>
+      <x:c r="M202" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N202" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O202" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P202" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q202" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R202" s="10" t="str">
+        <x:v>e85d5d63e7</x:v>
+      </x:c>
+      <x:c r="S202" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_194410_cpp-router-router-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T202" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_194702_cpp-router-router-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U202" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V202" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 96.11%; latency median ratio 1.07x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="203">
-      <x:c r="A203" s="29"/>
-      <x:c r="G203" s="27"/>
-      <x:c r="H203" s="27"/>
-      <x:c r="I203" s="23"/>
-      <x:c r="J203" s="25"/>
-      <x:c r="K203" s="25"/>
-      <x:c r="L203" s="25"/>
+      <x:c r="A203" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B203" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C203" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D203" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E203" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F203" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G203" s="26" t="n">
+        <x:v>994939</x:v>
+      </x:c>
+      <x:c r="H203" s="26" t="n">
+        <x:v>1060679.4</x:v>
+      </x:c>
+      <x:c r="I203" s="22" t="n">
+        <x:f>H203/G203</x:f>
+        <x:v>1.0660748045860098</x:v>
+      </x:c>
+      <x:c r="J203" s="24" t="n">
+        <x:v>30.718</x:v>
+      </x:c>
+      <x:c r="K203" s="24" t="n">
+        <x:v>31.437</x:v>
+      </x:c>
+      <x:c r="L203" s="24" t="n">
+        <x:f>K203/J203</x:f>
+        <x:v>1.0234064717755063</x:v>
+      </x:c>
+      <x:c r="M203" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N203" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O203" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P203" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q203" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R203" s="10" t="str">
+        <x:v>e85d5d63e7</x:v>
+      </x:c>
+      <x:c r="S203" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_194410_cpp-router-router-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T203" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_194702_cpp-router-router-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U203" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V203" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 96.11%; latency median ratio 1.07x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="204">
-      <x:c r="A204" s="29"/>
-      <x:c r="G204" s="27"/>
-      <x:c r="H204" s="27"/>
-      <x:c r="I204" s="23"/>
-      <x:c r="J204" s="25"/>
-      <x:c r="K204" s="25"/>
-      <x:c r="L204" s="25"/>
+      <x:c r="A204" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B204" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C204" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D204" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E204" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F204" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G204" s="26" t="n">
+        <x:v>369107.2</x:v>
+      </x:c>
+      <x:c r="H204" s="26" t="n">
+        <x:v>373406.6</x:v>
+      </x:c>
+      <x:c r="I204" s="22" t="n">
+        <x:f>H204/G204</x:f>
+        <x:v>1.0116481065663308</x:v>
+      </x:c>
+      <x:c r="J204" s="24" t="n">
+        <x:v>23.388</x:v>
+      </x:c>
+      <x:c r="K204" s="24" t="n">
+        <x:v>21.747</x:v>
+      </x:c>
+      <x:c r="L204" s="24" t="n">
+        <x:f>K204/J204</x:f>
+        <x:v>0.9298358132375576</x:v>
+      </x:c>
+      <x:c r="M204" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N204" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O204" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P204" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q204" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R204" s="10" t="str">
+        <x:v>e85d5d63e7</x:v>
+      </x:c>
+      <x:c r="S204" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_194410_cpp-router-router-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T204" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_194702_cpp-router-router-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U204" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V204" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 96.11%; latency median ratio 1.07x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="205">
-      <x:c r="A205" s="29"/>
-      <x:c r="G205" s="27"/>
-      <x:c r="H205" s="27"/>
-      <x:c r="I205" s="23"/>
-      <x:c r="J205" s="25"/>
-      <x:c r="K205" s="25"/>
-      <x:c r="L205" s="25"/>
+      <x:c r="A205" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B205" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C205" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D205" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E205" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F205" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G205" s="26" t="n">
+        <x:v>11540.8</x:v>
+      </x:c>
+      <x:c r="H205" s="26" t="n">
+        <x:v>10402.8</x:v>
+      </x:c>
+      <x:c r="I205" s="22" t="n">
+        <x:f>H205/G205</x:f>
+        <x:v>0.9013933176209622</x:v>
+      </x:c>
+      <x:c r="J205" s="24" t="n">
+        <x:v>10.768</x:v>
+      </x:c>
+      <x:c r="K205" s="24" t="n">
+        <x:v>12.074</x:v>
+      </x:c>
+      <x:c r="L205" s="24" t="n">
+        <x:f>K205/J205</x:f>
+        <x:v>1.1212852897473997</x:v>
+      </x:c>
+      <x:c r="M205" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N205" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O205" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P205" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q205" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R205" s="10" t="str">
+        <x:v>e85d5d63e7</x:v>
+      </x:c>
+      <x:c r="S205" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_194410_cpp-router-router-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T205" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_194702_cpp-router-router-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U205" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V205" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 96.11%; latency median ratio 1.07x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="206">
-      <x:c r="A206" s="29"/>
-      <x:c r="G206" s="27"/>
-      <x:c r="H206" s="27"/>
-      <x:c r="I206" s="23"/>
-      <x:c r="J206" s="25"/>
-      <x:c r="K206" s="25"/>
-      <x:c r="L206" s="25"/>
+      <x:c r="A206" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B206" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C206" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D206" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E206" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F206" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G206" s="26" t="n">
+        <x:v>6651.2</x:v>
+      </x:c>
+      <x:c r="H206" s="26" t="n">
+        <x:v>6210.6</x:v>
+      </x:c>
+      <x:c r="I206" s="22" t="n">
+        <x:f>H206/G206</x:f>
+        <x:v>0.9337563146499881</x:v>
+      </x:c>
+      <x:c r="J206" s="24" t="n">
+        <x:v>9.46</x:v>
+      </x:c>
+      <x:c r="K206" s="24" t="n">
+        <x:v>10.935</x:v>
+      </x:c>
+      <x:c r="L206" s="24" t="n">
+        <x:f>K206/J206</x:f>
+        <x:v>1.1559196617336152</x:v>
+      </x:c>
+      <x:c r="M206" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N206" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O206" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P206" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q206" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R206" s="10" t="str">
+        <x:v>e85d5d63e7</x:v>
+      </x:c>
+      <x:c r="S206" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_194410_cpp-router-router-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T206" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_194702_cpp-router-router-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U206" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V206" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 96.11%; latency median ratio 1.07x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="207">
-      <x:c r="A207" s="29"/>
-      <x:c r="G207" s="27"/>
-      <x:c r="H207" s="27"/>
-      <x:c r="I207" s="23"/>
-      <x:c r="J207" s="25"/>
-      <x:c r="K207" s="25"/>
-      <x:c r="L207" s="25"/>
+      <x:c r="A207" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B207" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C207" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D207" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E207" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F207" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G207" s="26" t="n">
+        <x:v>3614.4</x:v>
+      </x:c>
+      <x:c r="H207" s="26" t="n">
+        <x:v>3568</x:v>
+      </x:c>
+      <x:c r="I207" s="22" t="n">
+        <x:f>H207/G207</x:f>
+        <x:v>0.9871624612660469</x:v>
+      </x:c>
+      <x:c r="J207" s="24" t="n">
+        <x:v>9.605</x:v>
+      </x:c>
+      <x:c r="K207" s="24" t="n">
+        <x:v>9.101</x:v>
+      </x:c>
+      <x:c r="L207" s="24" t="n">
+        <x:f>K207/J207</x:f>
+        <x:v>0.9475273295158771</x:v>
+      </x:c>
+      <x:c r="M207" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N207" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O207" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P207" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q207" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R207" s="10" t="str">
+        <x:v>e85d5d63e7</x:v>
+      </x:c>
+      <x:c r="S207" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_194410_cpp-router-router-tls-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T207" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_194702_cpp-router-router-tls-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U207" s="10" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V207" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 96.11%; latency median ratio 1.07x; routed one-way gate pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="208">
       <x:c r="A208" s="29"/>

</xml_diff>

<commit_message>
docs(perf): record tls router request baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rece3148c004f4efe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R0bbc34b37f7a47dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R65690d07689c49ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Re6e824eef7f84ca5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R373452547c06466d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R6c6511e827184c15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R1077c93d93084dce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Rb4706eadde0b411f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 3개 통과·3개 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 3개 통과·4개 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -14971,58 +14971,424 @@
       </x:c>
     </x:row>
     <x:row r="208">
-      <x:c r="A208" s="29"/>
-      <x:c r="G208" s="27"/>
-      <x:c r="H208" s="27"/>
-      <x:c r="I208" s="23"/>
-      <x:c r="J208" s="25"/>
-      <x:c r="K208" s="25"/>
-      <x:c r="L208" s="25"/>
+      <x:c r="A208" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B208" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C208" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D208" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E208" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F208" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G208" s="26" t="n">
+        <x:v>154426.4</x:v>
+      </x:c>
+      <x:c r="H208" s="26" t="n">
+        <x:v>83529</x:v>
+      </x:c>
+      <x:c r="I208" s="22" t="n">
+        <x:f>H208/G208</x:f>
+        <x:v>0.5408984474157269</x:v>
+      </x:c>
+      <x:c r="J208" s="24" t="n">
+        <x:v>0.314</x:v>
+      </x:c>
+      <x:c r="K208" s="24" t="n">
+        <x:v>0.678</x:v>
+      </x:c>
+      <x:c r="L208" s="24" t="n">
+        <x:f>K208/J208</x:f>
+        <x:v>2.159235668789809</x:v>
+      </x:c>
+      <x:c r="M208" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N208" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O208" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P208" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q208" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R208" s="10" t="str">
+        <x:v>f4c67ee48b</x:v>
+      </x:c>
+      <x:c r="S208" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_195158_cpp-router-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T208" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U208" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V208" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 71.43%; latency median ratio 1.65x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="209">
-      <x:c r="A209" s="29"/>
-      <x:c r="G209" s="27"/>
-      <x:c r="H209" s="27"/>
-      <x:c r="I209" s="23"/>
-      <x:c r="J209" s="25"/>
-      <x:c r="K209" s="25"/>
-      <x:c r="L209" s="25"/>
+      <x:c r="A209" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B209" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C209" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D209" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E209" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F209" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G209" s="26" t="n">
+        <x:v>141189.4</x:v>
+      </x:c>
+      <x:c r="H209" s="26" t="n">
+        <x:v>74303.6</x:v>
+      </x:c>
+      <x:c r="I209" s="22" t="n">
+        <x:f>H209/G209</x:f>
+        <x:v>0.5262689692002375</x:v>
+      </x:c>
+      <x:c r="J209" s="24" t="n">
+        <x:v>0.355</x:v>
+      </x:c>
+      <x:c r="K209" s="24" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="L209" s="24" t="n">
+        <x:f>K209/J209</x:f>
+        <x:v>2.2535211267605635</x:v>
+      </x:c>
+      <x:c r="M209" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N209" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O209" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P209" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q209" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R209" s="10" t="str">
+        <x:v>f4c67ee48b</x:v>
+      </x:c>
+      <x:c r="S209" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_195158_cpp-router-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T209" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U209" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V209" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 71.43%; latency median ratio 1.65x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="210">
-      <x:c r="A210" s="29"/>
-      <x:c r="G210" s="27"/>
-      <x:c r="H210" s="27"/>
-      <x:c r="I210" s="23"/>
-      <x:c r="J210" s="25"/>
-      <x:c r="K210" s="25"/>
-      <x:c r="L210" s="25"/>
+      <x:c r="A210" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B210" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C210" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D210" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E210" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F210" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G210" s="26" t="n">
+        <x:v>83390.4</x:v>
+      </x:c>
+      <x:c r="H210" s="26" t="n">
+        <x:v>35209.8</x:v>
+      </x:c>
+      <x:c r="I210" s="22" t="n">
+        <x:f>H210/G210</x:f>
+        <x:v>0.42222845795199454</x:v>
+      </x:c>
+      <x:c r="J210" s="24" t="n">
+        <x:v>0.723</x:v>
+      </x:c>
+      <x:c r="K210" s="24" t="n">
+        <x:v>1.807</x:v>
+      </x:c>
+      <x:c r="L210" s="24" t="n">
+        <x:f>K210/J210</x:f>
+        <x:v>2.499308437067773</x:v>
+      </x:c>
+      <x:c r="M210" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N210" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O210" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P210" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q210" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R210" s="10" t="str">
+        <x:v>f4c67ee48b</x:v>
+      </x:c>
+      <x:c r="S210" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_195158_cpp-router-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T210" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U210" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V210" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 71.43%; latency median ratio 1.65x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="211">
-      <x:c r="A211" s="29"/>
-      <x:c r="G211" s="27"/>
-      <x:c r="H211" s="27"/>
-      <x:c r="I211" s="23"/>
-      <x:c r="J211" s="25"/>
-      <x:c r="K211" s="25"/>
-      <x:c r="L211" s="25"/>
+      <x:c r="A211" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B211" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C211" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D211" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E211" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F211" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G211" s="26" t="n">
+        <x:v>5344.2</x:v>
+      </x:c>
+      <x:c r="H211" s="26" t="n">
+        <x:v>4489.2</x:v>
+      </x:c>
+      <x:c r="I211" s="22" t="n">
+        <x:f>H211/G211</x:f>
+        <x:v>0.8400134725496801</x:v>
+      </x:c>
+      <x:c r="J211" s="24" t="n">
+        <x:v>2.313</x:v>
+      </x:c>
+      <x:c r="K211" s="24" t="n">
+        <x:v>2.649</x:v>
+      </x:c>
+      <x:c r="L211" s="24" t="n">
+        <x:f>K211/J211</x:f>
+        <x:v>1.1452658884565499</x:v>
+      </x:c>
+      <x:c r="M211" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N211" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O211" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P211" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q211" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R211" s="10" t="str">
+        <x:v>f4c67ee48b</x:v>
+      </x:c>
+      <x:c r="S211" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_195158_cpp-router-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T211" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U211" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V211" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 71.43%; latency median ratio 1.65x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="212">
-      <x:c r="A212" s="29"/>
-      <x:c r="G212" s="27"/>
-      <x:c r="H212" s="27"/>
-      <x:c r="I212" s="23"/>
-      <x:c r="J212" s="25"/>
-      <x:c r="K212" s="25"/>
-      <x:c r="L212" s="25"/>
+      <x:c r="A212" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B212" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C212" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D212" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E212" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F212" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G212" s="26" t="n">
+        <x:v>3052</x:v>
+      </x:c>
+      <x:c r="H212" s="26" t="n">
+        <x:v>2891.2</x:v>
+      </x:c>
+      <x:c r="I212" s="22" t="n">
+        <x:f>H212/G212</x:f>
+        <x:v>0.9473132372214941</x:v>
+      </x:c>
+      <x:c r="J212" s="24" t="n">
+        <x:v>2.136</x:v>
+      </x:c>
+      <x:c r="K212" s="24" t="n">
+        <x:v>2.043</x:v>
+      </x:c>
+      <x:c r="L212" s="24" t="n">
+        <x:f>K212/J212</x:f>
+        <x:v>0.9564606741573034</x:v>
+      </x:c>
+      <x:c r="M212" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N212" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O212" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P212" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q212" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R212" s="10" t="str">
+        <x:v>f4c67ee48b</x:v>
+      </x:c>
+      <x:c r="S212" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_195158_cpp-router-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T212" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U212" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V212" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 71.43%; latency median ratio 1.65x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="213">
-      <x:c r="A213" s="29"/>
-      <x:c r="G213" s="27"/>
-      <x:c r="H213" s="27"/>
-      <x:c r="I213" s="23"/>
-      <x:c r="J213" s="25"/>
-      <x:c r="K213" s="25"/>
-      <x:c r="L213" s="25"/>
+      <x:c r="A213" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B213" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C213" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D213" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E213" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F213" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G213" s="26" t="n">
+        <x:v>1660.8</x:v>
+      </x:c>
+      <x:c r="H213" s="26" t="n">
+        <x:v>1676</x:v>
+      </x:c>
+      <x:c r="I213" s="22" t="n">
+        <x:f>H213/G213</x:f>
+        <x:v>1.0091522157996147</x:v>
+      </x:c>
+      <x:c r="J213" s="24" t="n">
+        <x:v>1.801</x:v>
+      </x:c>
+      <x:c r="K213" s="24" t="n">
+        <x:v>1.744</x:v>
+      </x:c>
+      <x:c r="L213" s="24" t="n">
+        <x:f>K213/J213</x:f>
+        <x:v>0.9683509161576902</x:v>
+      </x:c>
+      <x:c r="M213" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N213" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O213" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P213" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q213" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R213" s="10" t="str">
+        <x:v>f4c67ee48b</x:v>
+      </x:c>
+      <x:c r="S213" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_195158_cpp-router-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T213" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U213" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V213" s="10" t="str">
+        <x:v>Final secure 5-run median: throughput aggregate mean 71.43%; latency median ratio 1.65x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="214">
       <x:c r="A214" s="29"/>
@@ -17645,12 +18011,86 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="L24" s="23"/>
-      <x:c r="M24" s="23"/>
+      <x:c r="A24" s="10" t="str">
+        <x:v>2026-08-25 19:54</x:v>
+      </x:c>
+      <x:c r="B24" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C24" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D24" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E24" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F24" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G24" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H24" s="10" t="str">
+        <x:v>Use Core normal route selection instead of the initially selected exact transport target.</x:v>
+      </x:c>
+      <x:c r="I24" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J24" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K24" s="10" t="str">
+        <x:v>N/A — exact-target contract no-go</x:v>
+      </x:c>
+      <x:c r="L24" s="22" t="n">
+        <x:v>0.714</x:v>
+      </x:c>
+      <x:c r="M24" s="22"/>
+      <x:c r="N24" s="10" t="str">
+        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership; exact-request-target contract remains required.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="L25" s="23"/>
-      <x:c r="M25" s="23"/>
+      <x:c r="A25" s="10" t="str">
+        <x:v>2026-08-25 19:54</x:v>
+      </x:c>
+      <x:c r="B25" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C25" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D25" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E25" s="10" t="str">
+        <x:v>tls</x:v>
+      </x:c>
+      <x:c r="F25" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G25" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H25" s="10" t="str">
+        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
+      </x:c>
+      <x:c r="I25" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J25" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K25" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L25" s="22"/>
+      <x:c r="M25" s="22"/>
+      <x:c r="N25" s="10" t="str">
+        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.65x passes.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="L26" s="23"/>

</xml_diff>

<commit_message>
docs(perf): record inproc pair baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R373452547c06466d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="R6c6511e827184c15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R1077c93d93084dce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Rb4706eadde0b411f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8e7aba9106074ddd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rdd12e5da53d84772"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Ra45e0f79e10b40eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R75ff27c2c1a94732"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 3개 통과·4개 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 3개 통과·4개 미달, inproc 0개 통과·1개 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -15391,58 +15391,424 @@
       </x:c>
     </x:row>
     <x:row r="214">
-      <x:c r="A214" s="29"/>
-      <x:c r="G214" s="27"/>
-      <x:c r="H214" s="27"/>
-      <x:c r="I214" s="23"/>
-      <x:c r="J214" s="25"/>
-      <x:c r="K214" s="25"/>
-      <x:c r="L214" s="25"/>
+      <x:c r="A214" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B214" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C214" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D214" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E214" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F214" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G214" s="26" t="n">
+        <x:v>2787138.8</x:v>
+      </x:c>
+      <x:c r="H214" s="26" t="n">
+        <x:v>2361098.8</x:v>
+      </x:c>
+      <x:c r="I214" s="22" t="n">
+        <x:f>H214/G214</x:f>
+        <x:v>0.8471407308455539</x:v>
+      </x:c>
+      <x:c r="J214" s="24" t="n">
+        <x:v>1.306</x:v>
+      </x:c>
+      <x:c r="K214" s="24" t="n">
+        <x:v>0.277</x:v>
+      </x:c>
+      <x:c r="L214" s="24" t="n">
+        <x:f>K214/J214</x:f>
+        <x:v>0.2120980091883614</x:v>
+      </x:c>
+      <x:c r="M214" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N214" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O214" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P214" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q214" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R214" s="10" t="str">
+        <x:v>baeb0b668a</x:v>
+      </x:c>
+      <x:c r="S214" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_200219_cpp-pair-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T214" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U214" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V214" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 76.09%; latency median ratio 1.08x; strict gate fail. Existing 128KiB–1MiB bounded-pool A is baseline; lowering the global threshold to 64KiB remains TCP partial-timeout no-go and cap expansion violates the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="215">
-      <x:c r="A215" s="29"/>
-      <x:c r="G215" s="27"/>
-      <x:c r="H215" s="27"/>
-      <x:c r="I215" s="23"/>
-      <x:c r="J215" s="25"/>
-      <x:c r="K215" s="25"/>
-      <x:c r="L215" s="25"/>
+      <x:c r="A215" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B215" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C215" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D215" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E215" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F215" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G215" s="26" t="n">
+        <x:v>1782677.4</x:v>
+      </x:c>
+      <x:c r="H215" s="26" t="n">
+        <x:v>1782799.4</x:v>
+      </x:c>
+      <x:c r="I215" s="22" t="n">
+        <x:f>H215/G215</x:f>
+        <x:v>1.0000684363867518</x:v>
+      </x:c>
+      <x:c r="J215" s="24" t="n">
+        <x:v>1.441</x:v>
+      </x:c>
+      <x:c r="K215" s="24" t="n">
+        <x:v>1.358</x:v>
+      </x:c>
+      <x:c r="L215" s="24" t="n">
+        <x:f>K215/J215</x:f>
+        <x:v>0.9424011103400417</x:v>
+      </x:c>
+      <x:c r="M215" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N215" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O215" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P215" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q215" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R215" s="10" t="str">
+        <x:v>baeb0b668a</x:v>
+      </x:c>
+      <x:c r="S215" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_200219_cpp-pair-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T215" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U215" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V215" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 76.09%; latency median ratio 1.08x; strict gate fail. Existing 128KiB–1MiB bounded-pool A is baseline; lowering the global threshold to 64KiB remains TCP partial-timeout no-go and cap expansion violates the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="216">
-      <x:c r="A216" s="29"/>
-      <x:c r="G216" s="27"/>
-      <x:c r="H216" s="27"/>
-      <x:c r="I216" s="23"/>
-      <x:c r="J216" s="25"/>
-      <x:c r="K216" s="25"/>
-      <x:c r="L216" s="25"/>
+      <x:c r="A216" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B216" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C216" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D216" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E216" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F216" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G216" s="26" t="n">
+        <x:v>1670147</x:v>
+      </x:c>
+      <x:c r="H216" s="26" t="n">
+        <x:v>1526496.4</x:v>
+      </x:c>
+      <x:c r="I216" s="22" t="n">
+        <x:f>H216/G216</x:f>
+        <x:v>0.9139892476530509</x:v>
+      </x:c>
+      <x:c r="J216" s="24" t="n">
+        <x:v>0.408</x:v>
+      </x:c>
+      <x:c r="K216" s="24" t="n">
+        <x:v>0.241</x:v>
+      </x:c>
+      <x:c r="L216" s="24" t="n">
+        <x:f>K216/J216</x:f>
+        <x:v>0.5906862745098039</x:v>
+      </x:c>
+      <x:c r="M216" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N216" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O216" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P216" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q216" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R216" s="10" t="str">
+        <x:v>baeb0b668a</x:v>
+      </x:c>
+      <x:c r="S216" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_200219_cpp-pair-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T216" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U216" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V216" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 76.09%; latency median ratio 1.08x; strict gate fail. Existing 128KiB–1MiB bounded-pool A is baseline; lowering the global threshold to 64KiB remains TCP partial-timeout no-go and cap expansion violates the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="217">
-      <x:c r="A217" s="29"/>
-      <x:c r="G217" s="27"/>
-      <x:c r="H217" s="27"/>
-      <x:c r="I217" s="23"/>
-      <x:c r="J217" s="25"/>
-      <x:c r="K217" s="25"/>
-      <x:c r="L217" s="25"/>
+      <x:c r="A217" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B217" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C217" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D217" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E217" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F217" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G217" s="26" t="n">
+        <x:v>359853.4</x:v>
+      </x:c>
+      <x:c r="H217" s="26" t="n">
+        <x:v>81733</x:v>
+      </x:c>
+      <x:c r="I217" s="22" t="n">
+        <x:f>H217/G217</x:f>
+        <x:v>0.22712860292552467</x:v>
+      </x:c>
+      <x:c r="J217" s="24" t="n">
+        <x:v>0.008</x:v>
+      </x:c>
+      <x:c r="K217" s="24" t="n">
+        <x:v>0.026</x:v>
+      </x:c>
+      <x:c r="L217" s="24" t="n">
+        <x:f>K217/J217</x:f>
+        <x:v>3.25</x:v>
+      </x:c>
+      <x:c r="M217" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N217" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O217" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P217" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q217" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R217" s="10" t="str">
+        <x:v>baeb0b668a</x:v>
+      </x:c>
+      <x:c r="S217" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_200219_cpp-pair-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T217" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U217" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V217" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 76.09%; latency median ratio 1.08x; strict gate fail. Existing 128KiB–1MiB bounded-pool A is baseline; lowering the global threshold to 64KiB remains TCP partial-timeout no-go and cap expansion violates the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="218">
-      <x:c r="A218" s="29"/>
-      <x:c r="G218" s="27"/>
-      <x:c r="H218" s="27"/>
-      <x:c r="I218" s="23"/>
-      <x:c r="J218" s="25"/>
-      <x:c r="K218" s="25"/>
-      <x:c r="L218" s="25"/>
+      <x:c r="A218" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B218" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C218" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D218" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E218" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F218" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G218" s="26" t="n">
+        <x:v>154032</x:v>
+      </x:c>
+      <x:c r="H218" s="26" t="n">
+        <x:v>113515.2</x:v>
+      </x:c>
+      <x:c r="I218" s="22" t="n">
+        <x:f>H218/G218</x:f>
+        <x:v>0.7369585540666874</x:v>
+      </x:c>
+      <x:c r="J218" s="24" t="n">
+        <x:v>0.014</x:v>
+      </x:c>
+      <x:c r="K218" s="24" t="n">
+        <x:v>0.018</x:v>
+      </x:c>
+      <x:c r="L218" s="24" t="n">
+        <x:f>K218/J218</x:f>
+        <x:v>1.2857142857142856</x:v>
+      </x:c>
+      <x:c r="M218" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N218" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O218" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P218" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q218" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R218" s="10" t="str">
+        <x:v>baeb0b668a</x:v>
+      </x:c>
+      <x:c r="S218" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_200219_cpp-pair-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T218" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U218" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V218" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 76.09%; latency median ratio 1.08x; strict gate fail. Existing 128KiB–1MiB bounded-pool A is baseline; lowering the global threshold to 64KiB remains TCP partial-timeout no-go and cap expansion violates the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="219">
-      <x:c r="A219" s="29"/>
-      <x:c r="G219" s="27"/>
-      <x:c r="H219" s="27"/>
-      <x:c r="I219" s="23"/>
-      <x:c r="J219" s="25"/>
-      <x:c r="K219" s="25"/>
-      <x:c r="L219" s="25"/>
+      <x:c r="A219" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B219" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C219" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D219" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E219" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F219" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G219" s="26" t="n">
+        <x:v>67428.8</x:v>
+      </x:c>
+      <x:c r="H219" s="26" t="n">
+        <x:v>56666.8</x:v>
+      </x:c>
+      <x:c r="I219" s="22" t="n">
+        <x:f>H219/G219</x:f>
+        <x:v>0.8403946088318345</x:v>
+      </x:c>
+      <x:c r="J219" s="24" t="n">
+        <x:v>0.023</x:v>
+      </x:c>
+      <x:c r="K219" s="24" t="n">
+        <x:v>0.028</x:v>
+      </x:c>
+      <x:c r="L219" s="24" t="n">
+        <x:f>K219/J219</x:f>
+        <x:v>1.2173913043478262</x:v>
+      </x:c>
+      <x:c r="M219" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N219" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O219" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P219" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q219" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R219" s="10" t="str">
+        <x:v>baeb0b668a</x:v>
+      </x:c>
+      <x:c r="S219" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_200219_cpp-pair-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T219" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U219" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V219" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 76.09%; latency median ratio 1.08x; strict gate fail. Existing 128KiB–1MiB bounded-pool A is baseline; lowering the global threshold to 64KiB remains TCP partial-timeout no-go and cap expansion violates the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="220">
       <x:c r="A220" s="29"/>
@@ -18093,12 +18459,88 @@
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="L26" s="23"/>
-      <x:c r="M26" s="23"/>
+      <x:c r="A26" s="10" t="str">
+        <x:v>2026-08-25 20:08</x:v>
+      </x:c>
+      <x:c r="B26" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C26" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D26" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E26" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F26" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
+      </x:c>
+      <x:c r="G26" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H26" s="10" t="str">
+        <x:v>Re-evaluate retained 128KiB–1MiB bounded pool and process-lifetime singleton.</x:v>
+      </x:c>
+      <x:c r="I26" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J26" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K26" s="10" t="str">
+        <x:v>N/A — already baseline</x:v>
+      </x:c>
+      <x:c r="L26" s="22" t="n">
+        <x:v>0.761</x:v>
+      </x:c>
+      <x:c r="M26" s="22"/>
+      <x:c r="N26" s="10" t="str">
+        <x:v>NO-GO as a new A/B: safe bounded-pool lifecycle is already in source, including late Core-release safety.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="L27" s="23"/>
-      <x:c r="M27" s="23"/>
+      <x:c r="A27" s="10" t="str">
+        <x:v>2026-08-25 20:08</x:v>
+      </x:c>
+      <x:c r="B27" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C27" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D27" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E27" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F27" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
+      </x:c>
+      <x:c r="G27" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H27" s="10" t="str">
+        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
+      </x:c>
+      <x:c r="I27" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J27" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K27" s="10" t="str">
+        <x:v>N/A — timeout/resource no-go</x:v>
+      </x:c>
+      <x:c r="L27" s="22" t="n">
+        <x:v>0.761</x:v>
+      </x:c>
+      <x:c r="M27" s="22"/>
+      <x:c r="N27" s="10" t="str">
+        <x:v>NO-GO: the 64KiB global threshold previously yielded a 25/30 partial TCP report through timeout; raising the cap changes the documented resource boundary. Per-transport policy would make ownership/resource behavior inconsistent.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="L28" s="23"/>

</xml_diff>

<commit_message>
docs(perf): record inproc pubsub baseline
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8e7aba9106074ddd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rdd12e5da53d84772"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Ra45e0f79e10b40eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R75ff27c2c1a94732"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R57c9d3e56f264ba3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rfd5e76a8569e40c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R0f2256c58a2d4a53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R4052c8a6c5ec4dc5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 3개 통과·4개 미달, inproc 0개 통과·1개 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 3개 통과·4개 미달, inproc 0개 통과·2개 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -15811,58 +15811,424 @@
       </x:c>
     </x:row>
     <x:row r="220">
-      <x:c r="A220" s="29"/>
-      <x:c r="G220" s="27"/>
-      <x:c r="H220" s="27"/>
-      <x:c r="I220" s="23"/>
-      <x:c r="J220" s="25"/>
-      <x:c r="K220" s="25"/>
-      <x:c r="L220" s="25"/>
+      <x:c r="A220" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B220" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C220" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D220" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E220" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F220" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G220" s="26" t="n">
+        <x:v>1099130.8</x:v>
+      </x:c>
+      <x:c r="H220" s="26" t="n">
+        <x:v>1093249.8</x:v>
+      </x:c>
+      <x:c r="I220" s="22" t="n">
+        <x:f>H220/G220</x:f>
+        <x:v>0.9946494084234561</x:v>
+      </x:c>
+      <x:c r="J220" s="24" t="n">
+        <x:v>0.016</x:v>
+      </x:c>
+      <x:c r="K220" s="24" t="n">
+        <x:v>0.023</x:v>
+      </x:c>
+      <x:c r="L220" s="24" t="n">
+        <x:f>K220/J220</x:f>
+        <x:v>1.4375</x:v>
+      </x:c>
+      <x:c r="M220" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N220" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O220" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P220" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q220" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R220" s="10" t="str">
+        <x:v>7d34d0cc8f</x:v>
+      </x:c>
+      <x:c r="S220" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_201103_cpp-pubsub-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T220" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U220" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V220" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 78.71%; latency median ratio 1.23x; strict gate fail. Direct single-part publish and bounded pool are baseline; lowering the global threshold to 64KiB remains TCP partial-timeout no-go and cap expansion violates the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="221">
-      <x:c r="A221" s="29"/>
-      <x:c r="G221" s="27"/>
-      <x:c r="H221" s="27"/>
-      <x:c r="I221" s="23"/>
-      <x:c r="J221" s="25"/>
-      <x:c r="K221" s="25"/>
-      <x:c r="L221" s="25"/>
+      <x:c r="A221" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B221" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C221" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D221" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E221" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F221" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G221" s="26" t="n">
+        <x:v>918784.6</x:v>
+      </x:c>
+      <x:c r="H221" s="26" t="n">
+        <x:v>837063.8</x:v>
+      </x:c>
+      <x:c r="I221" s="22" t="n">
+        <x:f>H221/G221</x:f>
+        <x:v>0.9110555401124486</x:v>
+      </x:c>
+      <x:c r="J221" s="24" t="n">
+        <x:v>0.032</x:v>
+      </x:c>
+      <x:c r="K221" s="24" t="n">
+        <x:v>0.035</x:v>
+      </x:c>
+      <x:c r="L221" s="24" t="n">
+        <x:f>K221/J221</x:f>
+        <x:v>1.09375</x:v>
+      </x:c>
+      <x:c r="M221" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N221" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O221" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P221" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q221" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R221" s="10" t="str">
+        <x:v>7d34d0cc8f</x:v>
+      </x:c>
+      <x:c r="S221" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_201103_cpp-pubsub-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T221" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U221" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V221" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 78.71%; latency median ratio 1.23x; strict gate fail. Direct single-part publish and bounded pool are baseline; lowering the global threshold to 64KiB remains TCP partial-timeout no-go and cap expansion violates the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="222">
-      <x:c r="A222" s="29"/>
-      <x:c r="G222" s="27"/>
-      <x:c r="H222" s="27"/>
-      <x:c r="I222" s="23"/>
-      <x:c r="J222" s="25"/>
-      <x:c r="K222" s="25"/>
-      <x:c r="L222" s="25"/>
+      <x:c r="A222" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B222" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C222" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D222" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E222" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F222" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G222" s="26" t="n">
+        <x:v>902076.8</x:v>
+      </x:c>
+      <x:c r="H222" s="26" t="n">
+        <x:v>831180.6</x:v>
+      </x:c>
+      <x:c r="I222" s="22" t="n">
+        <x:f>H222/G222</x:f>
+        <x:v>0.921407800311459</x:v>
+      </x:c>
+      <x:c r="J222" s="24" t="n">
+        <x:v>0.032</x:v>
+      </x:c>
+      <x:c r="K222" s="24" t="n">
+        <x:v>0.028</x:v>
+      </x:c>
+      <x:c r="L222" s="24" t="n">
+        <x:f>K222/J222</x:f>
+        <x:v>0.875</x:v>
+      </x:c>
+      <x:c r="M222" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N222" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O222" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P222" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q222" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R222" s="10" t="str">
+        <x:v>7d34d0cc8f</x:v>
+      </x:c>
+      <x:c r="S222" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_201103_cpp-pubsub-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T222" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U222" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V222" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 78.71%; latency median ratio 1.23x; strict gate fail. Direct single-part publish and bounded pool are baseline; lowering the global threshold to 64KiB remains TCP partial-timeout no-go and cap expansion violates the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="223">
-      <x:c r="A223" s="29"/>
-      <x:c r="G223" s="27"/>
-      <x:c r="H223" s="27"/>
-      <x:c r="I223" s="23"/>
-      <x:c r="J223" s="25"/>
-      <x:c r="K223" s="25"/>
-      <x:c r="L223" s="25"/>
+      <x:c r="A223" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B223" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C223" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D223" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E223" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F223" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G223" s="26" t="n">
+        <x:v>342235.8</x:v>
+      </x:c>
+      <x:c r="H223" s="26" t="n">
+        <x:v>82454.4</x:v>
+      </x:c>
+      <x:c r="I223" s="22" t="n">
+        <x:f>H223/G223</x:f>
+        <x:v>0.2409286228968448</x:v>
+      </x:c>
+      <x:c r="J223" s="24" t="n">
+        <x:v>0.008</x:v>
+      </x:c>
+      <x:c r="K223" s="24" t="n">
+        <x:v>0.026</x:v>
+      </x:c>
+      <x:c r="L223" s="24" t="n">
+        <x:f>K223/J223</x:f>
+        <x:v>3.25</x:v>
+      </x:c>
+      <x:c r="M223" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N223" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O223" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P223" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q223" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R223" s="10" t="str">
+        <x:v>7d34d0cc8f</x:v>
+      </x:c>
+      <x:c r="S223" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_201103_cpp-pubsub-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T223" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U223" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V223" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 78.71%; latency median ratio 1.23x; strict gate fail. Direct single-part publish and bounded pool are baseline; lowering the global threshold to 64KiB remains TCP partial-timeout no-go and cap expansion violates the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="224">
-      <x:c r="A224" s="29"/>
-      <x:c r="G224" s="27"/>
-      <x:c r="H224" s="27"/>
-      <x:c r="I224" s="23"/>
-      <x:c r="J224" s="25"/>
-      <x:c r="K224" s="25"/>
-      <x:c r="L224" s="25"/>
+      <x:c r="A224" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B224" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C224" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D224" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E224" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F224" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G224" s="26" t="n">
+        <x:v>141954.4</x:v>
+      </x:c>
+      <x:c r="H224" s="26" t="n">
+        <x:v>112481.8</x:v>
+      </x:c>
+      <x:c r="I224" s="22" t="n">
+        <x:f>H224/G224</x:f>
+        <x:v>0.7923798064730646</x:v>
+      </x:c>
+      <x:c r="J224" s="24" t="n">
+        <x:v>0.014</x:v>
+      </x:c>
+      <x:c r="K224" s="24" t="n">
+        <x:v>0.018</x:v>
+      </x:c>
+      <x:c r="L224" s="24" t="n">
+        <x:f>K224/J224</x:f>
+        <x:v>1.2857142857142856</x:v>
+      </x:c>
+      <x:c r="M224" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N224" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O224" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P224" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q224" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R224" s="10" t="str">
+        <x:v>7d34d0cc8f</x:v>
+      </x:c>
+      <x:c r="S224" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_201103_cpp-pubsub-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T224" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U224" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V224" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 78.71%; latency median ratio 1.23x; strict gate fail. Direct single-part publish and bounded pool are baseline; lowering the global threshold to 64KiB remains TCP partial-timeout no-go and cap expansion violates the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="225">
-      <x:c r="A225" s="29"/>
-      <x:c r="G225" s="27"/>
-      <x:c r="H225" s="27"/>
-      <x:c r="I225" s="23"/>
-      <x:c r="J225" s="25"/>
-      <x:c r="K225" s="25"/>
-      <x:c r="L225" s="25"/>
+      <x:c r="A225" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B225" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C225" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D225" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E225" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F225" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G225" s="26" t="n">
+        <x:v>65264.8</x:v>
+      </x:c>
+      <x:c r="H225" s="26" t="n">
+        <x:v>56285.8</x:v>
+      </x:c>
+      <x:c r="I225" s="22" t="n">
+        <x:f>H225/G225</x:f>
+        <x:v>0.8624220100268445</x:v>
+      </x:c>
+      <x:c r="J225" s="24" t="n">
+        <x:v>0.024</x:v>
+      </x:c>
+      <x:c r="K225" s="24" t="n">
+        <x:v>0.028</x:v>
+      </x:c>
+      <x:c r="L225" s="24" t="n">
+        <x:f>K225/J225</x:f>
+        <x:v>1.1666666666666667</x:v>
+      </x:c>
+      <x:c r="M225" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N225" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O225" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P225" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q225" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R225" s="10" t="str">
+        <x:v>7d34d0cc8f</x:v>
+      </x:c>
+      <x:c r="S225" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_201103_cpp-pubsub-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T225" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U225" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V225" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 78.71%; latency median ratio 1.23x; strict gate fail. Direct single-part publish and bounded pool are baseline; lowering the global threshold to 64KiB remains TCP partial-timeout no-go and cap expansion violates the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="226">
       <x:c r="A226" s="29"/>
@@ -18543,12 +18909,88 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="L28" s="23"/>
-      <x:c r="M28" s="23"/>
+      <x:c r="A28" s="10" t="str">
+        <x:v>2026-08-25 20:17</x:v>
+      </x:c>
+      <x:c r="B28" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C28" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D28" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E28" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F28" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
+      </x:c>
+      <x:c r="G28" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H28" s="10" t="str">
+        <x:v>Re-evaluate direct single-part publish and the retained 128KiB–1MiB bounded pool.</x:v>
+      </x:c>
+      <x:c r="I28" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J28" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K28" s="10" t="str">
+        <x:v>N/A — already baseline</x:v>
+      </x:c>
+      <x:c r="L28" s="22" t="n">
+        <x:v>0.787</x:v>
+      </x:c>
+      <x:c r="M28" s="22"/>
+      <x:c r="N28" s="10" t="str">
+        <x:v>NO-GO as a new A/B: direct publish and safe bounded-pool lifecycle already form the measured hot path.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="L29" s="23"/>
-      <x:c r="M29" s="23"/>
+      <x:c r="A29" s="10" t="str">
+        <x:v>2026-08-25 20:17</x:v>
+      </x:c>
+      <x:c r="B29" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C29" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D29" s="10" t="str">
+        <x:v>PUBSUB</x:v>
+      </x:c>
+      <x:c r="E29" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F29" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
+      </x:c>
+      <x:c r="G29" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H29" s="10" t="str">
+        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
+      </x:c>
+      <x:c r="I29" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J29" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K29" s="10" t="str">
+        <x:v>N/A — timeout/resource no-go</x:v>
+      </x:c>
+      <x:c r="L29" s="22" t="n">
+        <x:v>0.787</x:v>
+      </x:c>
+      <x:c r="M29" s="22"/>
+      <x:c r="N29" s="10" t="str">
+        <x:v>NO-GO: 64KiB global threshold has prior 25/30 TCP partial timeout; cap expansion changes resource policy. Transport-specific policy is not an acceptable lifecycle split.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="L30" s="23"/>

</xml_diff>

<commit_message>
perf(cpp): record inproc single baselines
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R57c9d3e56f264ba3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rfd5e76a8569e40c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R0f2256c58a2d4a53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R4052c8a6c5ec4dc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R30b0f213aac74341"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Ra04e4c833e4241ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R675ac5f620fb4baa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Rf6ceb4755f3643c8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 3개 통과·4개 미달, inproc 0개 통과·2개 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 미달, tls 3개 통과·4개 미달, inproc 0개 통과·7개 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -556,7 +556,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -16231,274 +16231,2104 @@
       </x:c>
     </x:row>
     <x:row r="226">
-      <x:c r="A226" s="29"/>
-      <x:c r="G226" s="27"/>
-      <x:c r="H226" s="27"/>
-      <x:c r="I226" s="23"/>
-      <x:c r="J226" s="25"/>
-      <x:c r="K226" s="25"/>
-      <x:c r="L226" s="25"/>
+      <x:c r="A226" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B226" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C226" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D226" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E226" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F226" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G226" s="26" t="n">
+        <x:v>2517877.2</x:v>
+      </x:c>
+      <x:c r="H226" s="26" t="n">
+        <x:v>1918784.4</x:v>
+      </x:c>
+      <x:c r="I226" s="22" t="n">
+        <x:f>H226/G226</x:f>
+        <x:v>0.76206432942798</x:v>
+      </x:c>
+      <x:c r="J226" s="24" t="n">
+        <x:v>0.078</x:v>
+      </x:c>
+      <x:c r="K226" s="24" t="n">
+        <x:v>0.062</x:v>
+      </x:c>
+      <x:c r="L226" s="24" t="n">
+        <x:f>K226/J226</x:f>
+        <x:v>0.7948717948717948</x:v>
+      </x:c>
+      <x:c r="M226" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N226" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O226" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P226" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q226" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R226" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S226" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_201932_cpp-dealer-dealer-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T226" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U226" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V226" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 70.49%; latency median ratio 1.22x; strict gate fail. Bounded-pool lifecycle is baseline; 64KiB lowering is TCP partial-timeout no-go and cap expansion changes the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="227">
-      <x:c r="A227" s="29"/>
-      <x:c r="G227" s="27"/>
-      <x:c r="H227" s="27"/>
-      <x:c r="I227" s="23"/>
-      <x:c r="J227" s="25"/>
-      <x:c r="K227" s="25"/>
-      <x:c r="L227" s="25"/>
+      <x:c r="A227" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B227" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C227" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D227" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E227" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F227" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G227" s="26" t="n">
+        <x:v>1781374.2</x:v>
+      </x:c>
+      <x:c r="H227" s="26" t="n">
+        <x:v>1498282</x:v>
+      </x:c>
+      <x:c r="I227" s="22" t="n">
+        <x:f>H227/G227</x:f>
+        <x:v>0.8410821263718763</x:v>
+      </x:c>
+      <x:c r="J227" s="24" t="n">
+        <x:v>1.43</x:v>
+      </x:c>
+      <x:c r="K227" s="24" t="n">
+        <x:v>1.811</x:v>
+      </x:c>
+      <x:c r="L227" s="24" t="n">
+        <x:f>K227/J227</x:f>
+        <x:v>1.2664335664335664</x:v>
+      </x:c>
+      <x:c r="M227" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N227" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O227" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P227" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q227" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R227" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S227" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_201932_cpp-dealer-dealer-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T227" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U227" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V227" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 70.49%; latency median ratio 1.22x; strict gate fail. Bounded-pool lifecycle is baseline; 64KiB lowering is TCP partial-timeout no-go and cap expansion changes the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="228">
-      <x:c r="A228" s="29"/>
-      <x:c r="G228" s="27"/>
-      <x:c r="H228" s="27"/>
-      <x:c r="I228" s="23"/>
-      <x:c r="J228" s="25"/>
-      <x:c r="K228" s="25"/>
-      <x:c r="L228" s="25"/>
+      <x:c r="A228" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B228" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C228" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D228" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E228" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F228" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G228" s="26" t="n">
+        <x:v>1618903.2</x:v>
+      </x:c>
+      <x:c r="H228" s="26" t="n">
+        <x:v>1321659.6</x:v>
+      </x:c>
+      <x:c r="I228" s="22" t="n">
+        <x:f>H228/G228</x:f>
+        <x:v>0.8163919868711114</x:v>
+      </x:c>
+      <x:c r="J228" s="24" t="n">
+        <x:v>0.387</x:v>
+      </x:c>
+      <x:c r="K228" s="24" t="n">
+        <x:v>0.337</x:v>
+      </x:c>
+      <x:c r="L228" s="24" t="n">
+        <x:f>K228/J228</x:f>
+        <x:v>0.8708010335917313</x:v>
+      </x:c>
+      <x:c r="M228" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N228" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O228" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P228" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q228" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R228" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S228" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_201932_cpp-dealer-dealer-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T228" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U228" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V228" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 70.49%; latency median ratio 1.22x; strict gate fail. Bounded-pool lifecycle is baseline; 64KiB lowering is TCP partial-timeout no-go and cap expansion changes the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="229">
-      <x:c r="A229" s="29"/>
-      <x:c r="G229" s="27"/>
-      <x:c r="H229" s="27"/>
-      <x:c r="I229" s="23"/>
-      <x:c r="J229" s="25"/>
-      <x:c r="K229" s="25"/>
-      <x:c r="L229" s="25"/>
+      <x:c r="A229" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B229" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C229" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D229" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E229" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F229" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G229" s="26" t="n">
+        <x:v>394077.6</x:v>
+      </x:c>
+      <x:c r="H229" s="26" t="n">
+        <x:v>102059</x:v>
+      </x:c>
+      <x:c r="I229" s="22" t="n">
+        <x:f>H229/G229</x:f>
+        <x:v>0.2589819873040234</x:v>
+      </x:c>
+      <x:c r="J229" s="24" t="n">
+        <x:v>0.008</x:v>
+      </x:c>
+      <x:c r="K229" s="24" t="n">
+        <x:v>0.024</x:v>
+      </x:c>
+      <x:c r="L229" s="24" t="n">
+        <x:f>K229/J229</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M229" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N229" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O229" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P229" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q229" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R229" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S229" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_201932_cpp-dealer-dealer-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T229" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U229" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V229" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 70.49%; latency median ratio 1.22x; strict gate fail. Bounded-pool lifecycle is baseline; 64KiB lowering is TCP partial-timeout no-go and cap expansion changes the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="230">
-      <x:c r="A230" s="29"/>
-      <x:c r="G230" s="27"/>
-      <x:c r="H230" s="27"/>
-      <x:c r="I230" s="23"/>
-      <x:c r="J230" s="25"/>
-      <x:c r="K230" s="25"/>
-      <x:c r="L230" s="25"/>
+      <x:c r="A230" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B230" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C230" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D230" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E230" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F230" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G230" s="26" t="n">
+        <x:v>158898.4</x:v>
+      </x:c>
+      <x:c r="H230" s="26" t="n">
+        <x:v>114682</x:v>
+      </x:c>
+      <x:c r="I230" s="22" t="n">
+        <x:f>H230/G230</x:f>
+        <x:v>0.7217316222189777</x:v>
+      </x:c>
+      <x:c r="J230" s="24" t="n">
+        <x:v>0.014</x:v>
+      </x:c>
+      <x:c r="K230" s="24" t="n">
+        <x:v>0.017</x:v>
+      </x:c>
+      <x:c r="L230" s="24" t="n">
+        <x:f>K230/J230</x:f>
+        <x:v>1.2142857142857144</x:v>
+      </x:c>
+      <x:c r="M230" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N230" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O230" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P230" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q230" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R230" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S230" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_201932_cpp-dealer-dealer-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T230" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U230" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V230" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 70.49%; latency median ratio 1.22x; strict gate fail. Bounded-pool lifecycle is baseline; 64KiB lowering is TCP partial-timeout no-go and cap expansion changes the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="231">
-      <x:c r="A231" s="29"/>
-      <x:c r="G231" s="27"/>
-      <x:c r="H231" s="27"/>
-      <x:c r="I231" s="23"/>
-      <x:c r="J231" s="25"/>
-      <x:c r="K231" s="25"/>
-      <x:c r="L231" s="25"/>
+      <x:c r="A231" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B231" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C231" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D231" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E231" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F231" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G231" s="26" t="n">
+        <x:v>67409.6</x:v>
+      </x:c>
+      <x:c r="H231" s="26" t="n">
+        <x:v>55909.8</x:v>
+      </x:c>
+      <x:c r="I231" s="22" t="n">
+        <x:f>H231/G231</x:f>
+        <x:v>0.8294041204813557</x:v>
+      </x:c>
+      <x:c r="J231" s="24" t="n">
+        <x:v>0.023</x:v>
+      </x:c>
+      <x:c r="K231" s="24" t="n">
+        <x:v>0.028</x:v>
+      </x:c>
+      <x:c r="L231" s="24" t="n">
+        <x:f>K231/J231</x:f>
+        <x:v>1.2173913043478262</x:v>
+      </x:c>
+      <x:c r="M231" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N231" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O231" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P231" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q231" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R231" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S231" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_201932_cpp-dealer-dealer-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T231" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U231" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V231" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 70.49%; latency median ratio 1.22x; strict gate fail. Bounded-pool lifecycle is baseline; 64KiB lowering is TCP partial-timeout no-go and cap expansion changes the resource boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="232">
-      <x:c r="A232" s="29"/>
-      <x:c r="G232" s="27"/>
-      <x:c r="H232" s="27"/>
-      <x:c r="I232" s="23"/>
-      <x:c r="J232" s="25"/>
-      <x:c r="K232" s="25"/>
-      <x:c r="L232" s="25"/>
+      <x:c r="A232" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B232" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C232" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D232" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E232" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F232" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G232" s="26" t="n">
+        <x:v>2696345</x:v>
+      </x:c>
+      <x:c r="H232" s="26" t="n">
+        <x:v>2144193.8</x:v>
+      </x:c>
+      <x:c r="I232" s="22" t="n">
+        <x:f>H232/G232</x:f>
+        <x:v>0.7952223472886444</x:v>
+      </x:c>
+      <x:c r="J232" s="24" t="n">
+        <x:v>0.208</x:v>
+      </x:c>
+      <x:c r="K232" s="24" t="n">
+        <x:v>0.703</x:v>
+      </x:c>
+      <x:c r="L232" s="24" t="n">
+        <x:f>K232/J232</x:f>
+        <x:v>3.379807692307692</x:v>
+      </x:c>
+      <x:c r="M232" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N232" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O232" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P232" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q232" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R232" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S232" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_202628_cpp-dealer-router-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T232" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U232" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V232" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 70.97%; latency median ratio 1.36x; strict gate fail. Pool policy is baseline; route cache or guard removal would alter exact-route/close/concurrency contracts.</x:v>
+      </x:c>
     </x:row>
     <x:row r="233">
-      <x:c r="A233" s="29"/>
-      <x:c r="G233" s="27"/>
-      <x:c r="H233" s="27"/>
-      <x:c r="I233" s="23"/>
-      <x:c r="J233" s="25"/>
-      <x:c r="K233" s="25"/>
-      <x:c r="L233" s="25"/>
+      <x:c r="A233" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B233" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C233" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D233" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E233" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F233" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G233" s="26" t="n">
+        <x:v>1821908.6</x:v>
+      </x:c>
+      <x:c r="H233" s="26" t="n">
+        <x:v>1452635.4</x:v>
+      </x:c>
+      <x:c r="I233" s="22" t="n">
+        <x:f>H233/G233</x:f>
+        <x:v>0.7973151891373693</x:v>
+      </x:c>
+      <x:c r="J233" s="24" t="n">
+        <x:v>1.482</x:v>
+      </x:c>
+      <x:c r="K233" s="24" t="n">
+        <x:v>1.812</x:v>
+      </x:c>
+      <x:c r="L233" s="24" t="n">
+        <x:f>K233/J233</x:f>
+        <x:v>1.222672064777328</x:v>
+      </x:c>
+      <x:c r="M233" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N233" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O233" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P233" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q233" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R233" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S233" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_202628_cpp-dealer-router-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T233" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U233" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V233" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 70.97%; latency median ratio 1.36x; strict gate fail. Pool policy is baseline; route cache or guard removal would alter exact-route/close/concurrency contracts.</x:v>
+      </x:c>
     </x:row>
     <x:row r="234">
-      <x:c r="A234" s="29"/>
-      <x:c r="G234" s="27"/>
-      <x:c r="H234" s="27"/>
-      <x:c r="I234" s="23"/>
-      <x:c r="J234" s="25"/>
-      <x:c r="K234" s="25"/>
-      <x:c r="L234" s="25"/>
+      <x:c r="A234" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B234" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C234" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D234" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E234" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F234" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G234" s="26" t="n">
+        <x:v>1563137.4</x:v>
+      </x:c>
+      <x:c r="H234" s="26" t="n">
+        <x:v>1450176.6</x:v>
+      </x:c>
+      <x:c r="I234" s="22" t="n">
+        <x:f>H234/G234</x:f>
+        <x:v>0.9277345676714025</x:v>
+      </x:c>
+      <x:c r="J234" s="24" t="n">
+        <x:v>0.424</x:v>
+      </x:c>
+      <x:c r="K234" s="24" t="n">
+        <x:v>0.464</x:v>
+      </x:c>
+      <x:c r="L234" s="24" t="n">
+        <x:f>K234/J234</x:f>
+        <x:v>1.0943396226415094</x:v>
+      </x:c>
+      <x:c r="M234" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N234" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O234" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P234" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q234" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R234" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S234" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_202628_cpp-dealer-router-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T234" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U234" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V234" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 70.97%; latency median ratio 1.36x; strict gate fail. Pool policy is baseline; route cache or guard removal would alter exact-route/close/concurrency contracts.</x:v>
+      </x:c>
     </x:row>
     <x:row r="235">
-      <x:c r="A235" s="29"/>
-      <x:c r="G235" s="27"/>
-      <x:c r="H235" s="27"/>
-      <x:c r="I235" s="23"/>
-      <x:c r="J235" s="25"/>
-      <x:c r="K235" s="25"/>
-      <x:c r="L235" s="25"/>
+      <x:c r="A235" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B235" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C235" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D235" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E235" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F235" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G235" s="26" t="n">
+        <x:v>388430.4</x:v>
+      </x:c>
+      <x:c r="H235" s="26" t="n">
+        <x:v>83522.2</x:v>
+      </x:c>
+      <x:c r="I235" s="22" t="n">
+        <x:f>H235/G235</x:f>
+        <x:v>0.21502487961807312</x:v>
+      </x:c>
+      <x:c r="J235" s="24" t="n">
+        <x:v>0.008</x:v>
+      </x:c>
+      <x:c r="K235" s="24" t="n">
+        <x:v>0.024</x:v>
+      </x:c>
+      <x:c r="L235" s="24" t="n">
+        <x:f>K235/J235</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M235" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N235" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O235" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P235" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q235" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R235" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S235" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_202628_cpp-dealer-router-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T235" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U235" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V235" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 70.97%; latency median ratio 1.36x; strict gate fail. Pool policy is baseline; route cache or guard removal would alter exact-route/close/concurrency contracts.</x:v>
+      </x:c>
     </x:row>
     <x:row r="236">
-      <x:c r="A236" s="29"/>
-      <x:c r="G236" s="27"/>
-      <x:c r="H236" s="27"/>
-      <x:c r="I236" s="23"/>
-      <x:c r="J236" s="25"/>
-      <x:c r="K236" s="25"/>
-      <x:c r="L236" s="25"/>
+      <x:c r="A236" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B236" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C236" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D236" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E236" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F236" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G236" s="26" t="n">
+        <x:v>153581.6</x:v>
+      </x:c>
+      <x:c r="H236" s="26" t="n">
+        <x:v>117182.4</x:v>
+      </x:c>
+      <x:c r="I236" s="22" t="n">
+        <x:f>H236/G236</x:f>
+        <x:v>0.7629976507602473</x:v>
+      </x:c>
+      <x:c r="J236" s="24" t="n">
+        <x:v>0.014</x:v>
+      </x:c>
+      <x:c r="K236" s="24" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="L236" s="24" t="n">
+        <x:f>K236/J236</x:f>
+        <x:v>1.4285714285714286</x:v>
+      </x:c>
+      <x:c r="M236" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N236" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O236" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P236" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q236" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R236" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S236" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_202628_cpp-dealer-router-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T236" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U236" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V236" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 70.97%; latency median ratio 1.36x; strict gate fail. Pool policy is baseline; route cache or guard removal would alter exact-route/close/concurrency contracts.</x:v>
+      </x:c>
     </x:row>
     <x:row r="237">
-      <x:c r="A237" s="29"/>
-      <x:c r="G237" s="27"/>
-      <x:c r="H237" s="27"/>
-      <x:c r="I237" s="23"/>
-      <x:c r="J237" s="25"/>
-      <x:c r="K237" s="25"/>
-      <x:c r="L237" s="25"/>
+      <x:c r="A237" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B237" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C237" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D237" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E237" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F237" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G237" s="26" t="n">
+        <x:v>67540.4</x:v>
+      </x:c>
+      <x:c r="H237" s="26" t="n">
+        <x:v>54048.8</x:v>
+      </x:c>
+      <x:c r="I237" s="22" t="n">
+        <x:f>H237/G237</x:f>
+        <x:v>0.8002440021083679</x:v>
+      </x:c>
+      <x:c r="J237" s="24" t="n">
+        <x:v>0.023</x:v>
+      </x:c>
+      <x:c r="K237" s="24" t="n">
+        <x:v>0.029</x:v>
+      </x:c>
+      <x:c r="L237" s="24" t="n">
+        <x:f>K237/J237</x:f>
+        <x:v>1.2608695652173914</x:v>
+      </x:c>
+      <x:c r="M237" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N237" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O237" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P237" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q237" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R237" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S237" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_202628_cpp-dealer-router-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T237" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U237" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V237" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 70.97%; latency median ratio 1.36x; strict gate fail. Pool policy is baseline; route cache or guard removal would alter exact-route/close/concurrency contracts.</x:v>
+      </x:c>
     </x:row>
     <x:row r="238">
-      <x:c r="A238" s="29"/>
-      <x:c r="G238" s="27"/>
-      <x:c r="H238" s="27"/>
-      <x:c r="I238" s="23"/>
-      <x:c r="J238" s="25"/>
-      <x:c r="K238" s="25"/>
-      <x:c r="L238" s="25"/>
+      <x:c r="A238" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B238" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C238" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D238" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E238" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F238" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G238" s="26" t="n">
+        <x:v>262169.4</x:v>
+      </x:c>
+      <x:c r="H238" s="26" t="n">
+        <x:v>105045.4</x:v>
+      </x:c>
+      <x:c r="I238" s="22" t="n">
+        <x:f>H238/G238</x:f>
+        <x:v>0.4006775771695705</x:v>
+      </x:c>
+      <x:c r="J238" s="24" t="n">
+        <x:v>0.127</x:v>
+      </x:c>
+      <x:c r="K238" s="24" t="n">
+        <x:v>0.113</x:v>
+      </x:c>
+      <x:c r="L238" s="24" t="n">
+        <x:f>K238/J238</x:f>
+        <x:v>0.889763779527559</x:v>
+      </x:c>
+      <x:c r="M238" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N238" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O238" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P238" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q238" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R238" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S238" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_203241_cpp-dealer-router-reqrep-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T238" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U238" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V238" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 42.85%; latency median ratio 1.14x; request/reply gate fail. Exact-target fallback is contract no-go; async bridge and safe borrowed single-part view are baseline, validated by contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="239">
-      <x:c r="A239" s="29"/>
-      <x:c r="G239" s="27"/>
-      <x:c r="H239" s="27"/>
-      <x:c r="I239" s="23"/>
-      <x:c r="J239" s="25"/>
-      <x:c r="K239" s="25"/>
-      <x:c r="L239" s="25"/>
+      <x:c r="A239" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B239" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C239" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D239" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E239" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F239" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G239" s="26" t="n">
+        <x:v>249270</x:v>
+      </x:c>
+      <x:c r="H239" s="26" t="n">
+        <x:v>102965.4</x:v>
+      </x:c>
+      <x:c r="I239" s="22" t="n">
+        <x:f>H239/G239</x:f>
+        <x:v>0.41306775785293054</x:v>
+      </x:c>
+      <x:c r="J239" s="24" t="n">
+        <x:v>0.159</x:v>
+      </x:c>
+      <x:c r="K239" s="24" t="n">
+        <x:v>0.113</x:v>
+      </x:c>
+      <x:c r="L239" s="24" t="n">
+        <x:f>K239/J239</x:f>
+        <x:v>0.7106918238993711</x:v>
+      </x:c>
+      <x:c r="M239" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N239" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O239" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P239" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q239" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R239" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S239" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_203241_cpp-dealer-router-reqrep-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T239" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U239" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V239" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 42.85%; latency median ratio 1.14x; request/reply gate fail. Exact-target fallback is contract no-go; async bridge and safe borrowed single-part view are baseline, validated by contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="240">
-      <x:c r="A240" s="29"/>
-      <x:c r="G240" s="27"/>
-      <x:c r="H240" s="27"/>
-      <x:c r="I240" s="23"/>
-      <x:c r="J240" s="25"/>
-      <x:c r="K240" s="25"/>
-      <x:c r="L240" s="25"/>
+      <x:c r="A240" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B240" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C240" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D240" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E240" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F240" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G240" s="26" t="n">
+        <x:v>234062.4</x:v>
+      </x:c>
+      <x:c r="H240" s="26" t="n">
+        <x:v>100533.4</x:v>
+      </x:c>
+      <x:c r="I240" s="22" t="n">
+        <x:f>H240/G240</x:f>
+        <x:v>0.4295153770960222</x:v>
+      </x:c>
+      <x:c r="J240" s="24" t="n">
+        <x:v>0.139</x:v>
+      </x:c>
+      <x:c r="K240" s="24" t="n">
+        <x:v>0.111</x:v>
+      </x:c>
+      <x:c r="L240" s="24" t="n">
+        <x:f>K240/J240</x:f>
+        <x:v>0.7985611510791366</x:v>
+      </x:c>
+      <x:c r="M240" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N240" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O240" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P240" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q240" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R240" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S240" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_203241_cpp-dealer-router-reqrep-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T240" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U240" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V240" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 42.85%; latency median ratio 1.14x; request/reply gate fail. Exact-target fallback is contract no-go; async bridge and safe borrowed single-part view are baseline, validated by contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="241">
-      <x:c r="A241" s="29"/>
-      <x:c r="G241" s="27"/>
-      <x:c r="H241" s="27"/>
-      <x:c r="I241" s="23"/>
-      <x:c r="J241" s="25"/>
-      <x:c r="K241" s="25"/>
-      <x:c r="L241" s="25"/>
+      <x:c r="A241" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B241" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C241" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D241" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E241" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F241" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G241" s="26" t="n">
+        <x:v>115614.8</x:v>
+      </x:c>
+      <x:c r="H241" s="26" t="n">
+        <x:v>28885.2</x:v>
+      </x:c>
+      <x:c r="I241" s="22" t="n">
+        <x:f>H241/G241</x:f>
+        <x:v>0.24983998588416015</x:v>
+      </x:c>
+      <x:c r="J241" s="24" t="n">
+        <x:v>0.058</x:v>
+      </x:c>
+      <x:c r="K241" s="24" t="n">
+        <x:v>0.114</x:v>
+      </x:c>
+      <x:c r="L241" s="24" t="n">
+        <x:f>K241/J241</x:f>
+        <x:v>1.9655172413793103</x:v>
+      </x:c>
+      <x:c r="M241" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N241" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O241" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P241" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q241" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R241" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S241" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_203241_cpp-dealer-router-reqrep-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T241" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U241" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V241" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 42.85%; latency median ratio 1.14x; request/reply gate fail. Exact-target fallback is contract no-go; async bridge and safe borrowed single-part view are baseline, validated by contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="242">
-      <x:c r="A242" s="29"/>
-      <x:c r="G242" s="27"/>
-      <x:c r="H242" s="27"/>
-      <x:c r="I242" s="23"/>
-      <x:c r="J242" s="25"/>
-      <x:c r="K242" s="25"/>
-      <x:c r="L242" s="25"/>
+      <x:c r="A242" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B242" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C242" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D242" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E242" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F242" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G242" s="26" t="n">
+        <x:v>68459.2</x:v>
+      </x:c>
+      <x:c r="H242" s="26" t="n">
+        <x:v>31285</x:v>
+      </x:c>
+      <x:c r="I242" s="22" t="n">
+        <x:f>H242/G242</x:f>
+        <x:v>0.4569875195737023</x:v>
+      </x:c>
+      <x:c r="J242" s="24" t="n">
+        <x:v>0.055</x:v>
+      </x:c>
+      <x:c r="K242" s="24" t="n">
+        <x:v>0.086</x:v>
+      </x:c>
+      <x:c r="L242" s="24" t="n">
+        <x:f>K242/J242</x:f>
+        <x:v>1.5636363636363635</x:v>
+      </x:c>
+      <x:c r="M242" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N242" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O242" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P242" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q242" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R242" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S242" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_203241_cpp-dealer-router-reqrep-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T242" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U242" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V242" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 42.85%; latency median ratio 1.14x; request/reply gate fail. Exact-target fallback is contract no-go; async bridge and safe borrowed single-part view are baseline, validated by contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="243">
-      <x:c r="A243" s="29"/>
-      <x:c r="G243" s="27"/>
-      <x:c r="H243" s="27"/>
-      <x:c r="I243" s="23"/>
-      <x:c r="J243" s="25"/>
-      <x:c r="K243" s="25"/>
-      <x:c r="L243" s="25"/>
+      <x:c r="A243" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B243" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C243" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D243" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E243" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F243" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G243" s="26" t="n">
+        <x:v>37678.4</x:v>
+      </x:c>
+      <x:c r="H243" s="26" t="n">
+        <x:v>23402.6</x:v>
+      </x:c>
+      <x:c r="I243" s="22" t="n">
+        <x:f>H243/G243</x:f>
+        <x:v>0.6211144846914942</x:v>
+      </x:c>
+      <x:c r="J243" s="24" t="n">
+        <x:v>0.057</x:v>
+      </x:c>
+      <x:c r="K243" s="24" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="L243" s="24" t="n">
+        <x:f>K243/J243</x:f>
+        <x:v>1.4035087719298245</x:v>
+      </x:c>
+      <x:c r="M243" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N243" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O243" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P243" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q243" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R243" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S243" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_203241_cpp-dealer-router-reqrep-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T243" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U243" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V243" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 42.85%; latency median ratio 1.14x; request/reply gate fail. Exact-target fallback is contract no-go; async bridge and safe borrowed single-part view are baseline, validated by contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="244">
-      <x:c r="A244" s="29"/>
-      <x:c r="G244" s="27"/>
-      <x:c r="H244" s="27"/>
-      <x:c r="I244" s="23"/>
-      <x:c r="J244" s="25"/>
-      <x:c r="K244" s="25"/>
-      <x:c r="L244" s="25"/>
+      <x:c r="A244" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B244" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C244" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D244" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E244" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F244" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G244" s="26" t="n">
+        <x:v>2351668</x:v>
+      </x:c>
+      <x:c r="H244" s="26" t="n">
+        <x:v>2098112</x:v>
+      </x:c>
+      <x:c r="I244" s="22" t="n">
+        <x:f>H244/G244</x:f>
+        <x:v>0.8921803587921424</x:v>
+      </x:c>
+      <x:c r="J244" s="24" t="n">
+        <x:v>0.056</x:v>
+      </x:c>
+      <x:c r="K244" s="24" t="n">
+        <x:v>0.071</x:v>
+      </x:c>
+      <x:c r="L244" s="24" t="n">
+        <x:f>K244/J244</x:f>
+        <x:v>1.2678571428571428</x:v>
+      </x:c>
+      <x:c r="M244" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N244" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O244" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P244" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q244" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R244" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S244" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_203821_cpp-router-router-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T244" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U244" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V244" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 69.85%; latency median ratio 1.09x; strict gate fail. Pool/state reuse is baseline; route cache and lifetime-guard removal are exact-route/close contract no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="245">
-      <x:c r="A245" s="29"/>
-      <x:c r="G245" s="27"/>
-      <x:c r="H245" s="27"/>
-      <x:c r="I245" s="23"/>
-      <x:c r="J245" s="25"/>
-      <x:c r="K245" s="25"/>
-      <x:c r="L245" s="25"/>
+      <x:c r="A245" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B245" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C245" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D245" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E245" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F245" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G245" s="26" t="n">
+        <x:v>1571206.6</x:v>
+      </x:c>
+      <x:c r="H245" s="26" t="n">
+        <x:v>1454923.8</x:v>
+      </x:c>
+      <x:c r="I245" s="22" t="n">
+        <x:f>H245/G245</x:f>
+        <x:v>0.9259914004943717</x:v>
+      </x:c>
+      <x:c r="J245" s="24" t="n">
+        <x:v>1.607</x:v>
+      </x:c>
+      <x:c r="K245" s="24" t="n">
+        <x:v>0.432</x:v>
+      </x:c>
+      <x:c r="L245" s="24" t="n">
+        <x:f>K245/J245</x:f>
+        <x:v>0.268823895457374</x:v>
+      </x:c>
+      <x:c r="M245" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N245" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O245" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P245" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q245" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R245" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S245" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_203821_cpp-router-router-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T245" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U245" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V245" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 69.85%; latency median ratio 1.09x; strict gate fail. Pool/state reuse is baseline; route cache and lifetime-guard removal are exact-route/close contract no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="246">
-      <x:c r="A246" s="29"/>
-      <x:c r="G246" s="27"/>
-      <x:c r="H246" s="27"/>
-      <x:c r="I246" s="23"/>
-      <x:c r="J246" s="25"/>
-      <x:c r="K246" s="25"/>
-      <x:c r="L246" s="25"/>
+      <x:c r="A246" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B246" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C246" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D246" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E246" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F246" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G246" s="26" t="n">
+        <x:v>1465426.6</x:v>
+      </x:c>
+      <x:c r="H246" s="26" t="n">
+        <x:v>1278763.8</x:v>
+      </x:c>
+      <x:c r="I246" s="22" t="n">
+        <x:f>H246/G246</x:f>
+        <x:v>0.8726222111704537</x:v>
+      </x:c>
+      <x:c r="J246" s="24" t="n">
+        <x:v>0.372</x:v>
+      </x:c>
+      <x:c r="K246" s="24" t="n">
+        <x:v>0.17</x:v>
+      </x:c>
+      <x:c r="L246" s="24" t="n">
+        <x:f>K246/J246</x:f>
+        <x:v>0.456989247311828</x:v>
+      </x:c>
+      <x:c r="M246" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N246" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O246" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P246" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q246" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R246" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S246" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_203821_cpp-router-router-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T246" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U246" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V246" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 69.85%; latency median ratio 1.09x; strict gate fail. Pool/state reuse is baseline; route cache and lifetime-guard removal are exact-route/close contract no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="247">
-      <x:c r="A247" s="29"/>
-      <x:c r="G247" s="27"/>
-      <x:c r="H247" s="27"/>
-      <x:c r="I247" s="23"/>
-      <x:c r="J247" s="25"/>
-      <x:c r="K247" s="25"/>
-      <x:c r="L247" s="25"/>
+      <x:c r="A247" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B247" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C247" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D247" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E247" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F247" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G247" s="26" t="n">
+        <x:v>360321</x:v>
+      </x:c>
+      <x:c r="H247" s="26" t="n">
+        <x:v>75213.6</x:v>
+      </x:c>
+      <x:c r="I247" s="22" t="n">
+        <x:f>H247/G247</x:f>
+        <x:v>0.20874053968544715</x:v>
+      </x:c>
+      <x:c r="J247" s="24" t="n">
+        <x:v>0.008</x:v>
+      </x:c>
+      <x:c r="K247" s="24" t="n">
+        <x:v>0.031</x:v>
+      </x:c>
+      <x:c r="L247" s="24" t="n">
+        <x:f>K247/J247</x:f>
+        <x:v>3.875</x:v>
+      </x:c>
+      <x:c r="M247" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N247" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O247" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P247" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q247" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R247" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S247" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_203821_cpp-router-router-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T247" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U247" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V247" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 69.85%; latency median ratio 1.09x; strict gate fail. Pool/state reuse is baseline; route cache and lifetime-guard removal are exact-route/close contract no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="248">
-      <x:c r="A248" s="29"/>
-      <x:c r="G248" s="27"/>
-      <x:c r="H248" s="27"/>
-      <x:c r="I248" s="23"/>
-      <x:c r="J248" s="25"/>
-      <x:c r="K248" s="25"/>
-      <x:c r="L248" s="25"/>
+      <x:c r="A248" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B248" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C248" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D248" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E248" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F248" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G248" s="26" t="n">
+        <x:v>132629</x:v>
+      </x:c>
+      <x:c r="H248" s="26" t="n">
+        <x:v>117969.8</x:v>
+      </x:c>
+      <x:c r="I248" s="22" t="n">
+        <x:f>H248/G248</x:f>
+        <x:v>0.8894721365613856</x:v>
+      </x:c>
+      <x:c r="J248" s="24" t="n">
+        <x:v>0.016</x:v>
+      </x:c>
+      <x:c r="K248" s="24" t="n">
+        <x:v>0.017</x:v>
+      </x:c>
+      <x:c r="L248" s="24" t="n">
+        <x:f>K248/J248</x:f>
+        <x:v>1.0625</x:v>
+      </x:c>
+      <x:c r="M248" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N248" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O248" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P248" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q248" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R248" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S248" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_203821_cpp-router-router-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T248" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U248" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V248" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 69.85%; latency median ratio 1.09x; strict gate fail. Pool/state reuse is baseline; route cache and lifetime-guard removal are exact-route/close contract no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="249">
-      <x:c r="A249" s="29"/>
-      <x:c r="G249" s="27"/>
-      <x:c r="H249" s="27"/>
-      <x:c r="I249" s="23"/>
-      <x:c r="J249" s="25"/>
-      <x:c r="K249" s="25"/>
-      <x:c r="L249" s="25"/>
+      <x:c r="A249" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B249" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C249" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D249" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E249" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F249" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G249" s="26" t="n">
+        <x:v>61966.8</x:v>
+      </x:c>
+      <x:c r="H249" s="26" t="n">
+        <x:v>53791</x:v>
+      </x:c>
+      <x:c r="I249" s="22" t="n">
+        <x:f>H249/G249</x:f>
+        <x:v>0.8680616071832012</x:v>
+      </x:c>
+      <x:c r="J249" s="24" t="n">
+        <x:v>0.026</x:v>
+      </x:c>
+      <x:c r="K249" s="24" t="n">
+        <x:v>0.029</x:v>
+      </x:c>
+      <x:c r="L249" s="24" t="n">
+        <x:f>K249/J249</x:f>
+        <x:v>1.1153846153846154</x:v>
+      </x:c>
+      <x:c r="M249" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N249" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O249" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P249" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q249" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R249" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S249" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_203821_cpp-router-router-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T249" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U249" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V249" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 69.85%; latency median ratio 1.09x; strict gate fail. Pool/state reuse is baseline; route cache and lifetime-guard removal are exact-route/close contract no-go.</x:v>
+      </x:c>
     </x:row>
     <x:row r="250">
-      <x:c r="A250" s="29"/>
-      <x:c r="G250" s="27"/>
-      <x:c r="H250" s="27"/>
-      <x:c r="I250" s="23"/>
-      <x:c r="J250" s="25"/>
-      <x:c r="K250" s="25"/>
-      <x:c r="L250" s="25"/>
+      <x:c r="A250" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B250" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C250" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D250" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E250" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F250" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G250" s="26" t="n">
+        <x:v>252437.2</x:v>
+      </x:c>
+      <x:c r="H250" s="26" t="n">
+        <x:v>107319.8</x:v>
+      </x:c>
+      <x:c r="I250" s="22" t="n">
+        <x:f>H250/G250</x:f>
+        <x:v>0.42513464734991513</x:v>
+      </x:c>
+      <x:c r="J250" s="24" t="n">
+        <x:v>0.137</x:v>
+      </x:c>
+      <x:c r="K250" s="24" t="n">
+        <x:v>0.102</x:v>
+      </x:c>
+      <x:c r="L250" s="24" t="n">
+        <x:f>K250/J250</x:f>
+        <x:v>0.7445255474452553</x:v>
+      </x:c>
+      <x:c r="M250" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N250" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O250" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P250" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q250" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R250" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S250" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_204333_cpp-router-router-reqrep-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T250" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U250" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V250" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 44.06%; latency median ratio 1.10x; request/reply gate fail. Exact-target fallback is contract no-go; async bridge and safe borrowed single-part view are baseline, validated by contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="251">
-      <x:c r="A251" s="29"/>
-      <x:c r="G251" s="27"/>
-      <x:c r="H251" s="27"/>
-      <x:c r="I251" s="23"/>
-      <x:c r="J251" s="25"/>
-      <x:c r="K251" s="25"/>
-      <x:c r="L251" s="25"/>
+      <x:c r="A251" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B251" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C251" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D251" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E251" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F251" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G251" s="26" t="n">
+        <x:v>228619.8</x:v>
+      </x:c>
+      <x:c r="H251" s="26" t="n">
+        <x:v>105753.6</x:v>
+      </x:c>
+      <x:c r="I251" s="22" t="n">
+        <x:f>H251/G251</x:f>
+        <x:v>0.4625741077544465</x:v>
+      </x:c>
+      <x:c r="J251" s="24" t="n">
+        <x:v>0.146</x:v>
+      </x:c>
+      <x:c r="K251" s="24" t="n">
+        <x:v>0.092</x:v>
+      </x:c>
+      <x:c r="L251" s="24" t="n">
+        <x:f>K251/J251</x:f>
+        <x:v>0.6301369863013699</x:v>
+      </x:c>
+      <x:c r="M251" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N251" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O251" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P251" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q251" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R251" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S251" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_204333_cpp-router-router-reqrep-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T251" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U251" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V251" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 44.06%; latency median ratio 1.10x; request/reply gate fail. Exact-target fallback is contract no-go; async bridge and safe borrowed single-part view are baseline, validated by contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="252">
-      <x:c r="A252" s="29"/>
-      <x:c r="G252" s="27"/>
-      <x:c r="H252" s="27"/>
-      <x:c r="I252" s="23"/>
-      <x:c r="J252" s="25"/>
-      <x:c r="K252" s="25"/>
-      <x:c r="L252" s="25"/>
+      <x:c r="A252" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B252" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C252" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D252" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E252" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F252" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G252" s="26" t="n">
+        <x:v>232246.6</x:v>
+      </x:c>
+      <x:c r="H252" s="26" t="n">
+        <x:v>103743.2</x:v>
+      </x:c>
+      <x:c r="I252" s="22" t="n">
+        <x:f>H252/G252</x:f>
+        <x:v>0.4466941604311968</x:v>
+      </x:c>
+      <x:c r="J252" s="24" t="n">
+        <x:v>0.145</x:v>
+      </x:c>
+      <x:c r="K252" s="24" t="n">
+        <x:v>0.089</x:v>
+      </x:c>
+      <x:c r="L252" s="24" t="n">
+        <x:f>K252/J252</x:f>
+        <x:v>0.6137931034482759</x:v>
+      </x:c>
+      <x:c r="M252" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N252" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O252" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P252" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q252" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R252" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S252" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_204333_cpp-router-router-reqrep-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T252" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U252" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V252" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 44.06%; latency median ratio 1.10x; request/reply gate fail. Exact-target fallback is contract no-go; async bridge and safe borrowed single-part view are baseline, validated by contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="253">
-      <x:c r="A253" s="29"/>
-      <x:c r="G253" s="27"/>
-      <x:c r="H253" s="27"/>
-      <x:c r="I253" s="23"/>
-      <x:c r="J253" s="25"/>
-      <x:c r="K253" s="25"/>
-      <x:c r="L253" s="25"/>
+      <x:c r="A253" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B253" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C253" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D253" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E253" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F253" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G253" s="26" t="n">
+        <x:v>110038</x:v>
+      </x:c>
+      <x:c r="H253" s="26" t="n">
+        <x:v>33678.8</x:v>
+      </x:c>
+      <x:c r="I253" s="22" t="n">
+        <x:f>H253/G253</x:f>
+        <x:v>0.30606517748414186</x:v>
+      </x:c>
+      <x:c r="J253" s="24" t="n">
+        <x:v>0.061</x:v>
+      </x:c>
+      <x:c r="K253" s="24" t="n">
+        <x:v>0.089</x:v>
+      </x:c>
+      <x:c r="L253" s="24" t="n">
+        <x:f>K253/J253</x:f>
+        <x:v>1.459016393442623</x:v>
+      </x:c>
+      <x:c r="M253" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N253" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O253" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P253" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q253" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R253" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S253" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_204333_cpp-router-router-reqrep-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T253" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U253" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V253" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 44.06%; latency median ratio 1.10x; request/reply gate fail. Exact-target fallback is contract no-go; async bridge and safe borrowed single-part view are baseline, validated by contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="254">
-      <x:c r="A254" s="29"/>
-      <x:c r="G254" s="27"/>
-      <x:c r="H254" s="27"/>
-      <x:c r="I254" s="23"/>
-      <x:c r="J254" s="25"/>
-      <x:c r="K254" s="25"/>
-      <x:c r="L254" s="25"/>
+      <x:c r="A254" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B254" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C254" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D254" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E254" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F254" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G254" s="26" t="n">
+        <x:v>67947.8</x:v>
+      </x:c>
+      <x:c r="H254" s="26" t="n">
+        <x:v>31715.4</x:v>
+      </x:c>
+      <x:c r="I254" s="22" t="n">
+        <x:f>H254/G254</x:f>
+        <x:v>0.46676124907649696</x:v>
+      </x:c>
+      <x:c r="J254" s="24" t="n">
+        <x:v>0.055</x:v>
+      </x:c>
+      <x:c r="K254" s="24" t="n">
+        <x:v>0.094</x:v>
+      </x:c>
+      <x:c r="L254" s="24" t="n">
+        <x:f>K254/J254</x:f>
+        <x:v>1.709090909090909</x:v>
+      </x:c>
+      <x:c r="M254" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N254" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O254" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P254" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q254" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R254" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S254" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_204333_cpp-router-router-reqrep-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T254" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U254" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V254" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 44.06%; latency median ratio 1.10x; request/reply gate fail. Exact-target fallback is contract no-go; async bridge and safe borrowed single-part view are baseline, validated by contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="255">
-      <x:c r="A255" s="29"/>
-      <x:c r="G255" s="27"/>
-      <x:c r="H255" s="27"/>
-      <x:c r="I255" s="23"/>
-      <x:c r="J255" s="25"/>
-      <x:c r="K255" s="25"/>
-      <x:c r="L255" s="25"/>
+      <x:c r="A255" s="28" t="str">
+        <x:v>2026-08-25 15:00</x:v>
+      </x:c>
+      <x:c r="B255" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C255" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D255" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E255" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F255" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G255" s="26" t="n">
+        <x:v>38166.6</x:v>
+      </x:c>
+      <x:c r="H255" s="26" t="n">
+        <x:v>22246.8</x:v>
+      </x:c>
+      <x:c r="I255" s="22" t="n">
+        <x:f>H255/G255</x:f>
+        <x:v>0.5828866076621968</x:v>
+      </x:c>
+      <x:c r="J255" s="24" t="n">
+        <x:v>0.056</x:v>
+      </x:c>
+      <x:c r="K255" s="24" t="n">
+        <x:v>0.086</x:v>
+      </x:c>
+      <x:c r="L255" s="24" t="n">
+        <x:f>K255/J255</x:f>
+        <x:v>1.5357142857142856</x:v>
+      </x:c>
+      <x:c r="M255" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N255" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O255" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P255" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q255" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R255" s="10" t="str">
+        <x:v>ba8c935285</x:v>
+      </x:c>
+      <x:c r="S255" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_204333_cpp-router-router-reqrep-inproc-local0132-final5-c-20260825.txt</x:v>
+      </x:c>
+      <x:c r="T255" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="U255" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V255" s="10" t="str">
+        <x:v>Final 5-run median: throughput aggregate mean 44.06%; latency median ratio 1.10x; request/reply gate fail. Exact-target fallback is contract no-go; async bridge and safe borrowed single-part view are baseline, validated by contract 5/5.</x:v>
+      </x:c>
     </x:row>
     <x:row r="256">
       <x:c r="A256" s="29"/>
@@ -18993,44 +20823,424 @@
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="L30" s="23"/>
-      <x:c r="M30" s="23"/>
+      <x:c r="A30" s="10" t="str">
+        <x:v>2026-08-25 20:22</x:v>
+      </x:c>
+      <x:c r="B30" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C30" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D30" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E30" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F30" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
+      </x:c>
+      <x:c r="G30" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H30" s="10" t="str">
+        <x:v>Re-evaluate bounded pool and operation-state reuse in the routed one-way hot path.</x:v>
+      </x:c>
+      <x:c r="I30" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J30" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K30" s="10" t="str">
+        <x:v>N/A — already baseline</x:v>
+      </x:c>
+      <x:c r="L30" s="22" t="n">
+        <x:v>0.705</x:v>
+      </x:c>
+      <x:c r="M30" s="22"/>
+      <x:c r="N30" s="10" t="str">
+        <x:v>NO-GO as a new A/B: the measured path already has the safe pool/state lifecycle.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="L31" s="23"/>
-      <x:c r="M31" s="23"/>
+      <x:c r="A31" s="10" t="str">
+        <x:v>2026-08-25 20:22</x:v>
+      </x:c>
+      <x:c r="B31" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C31" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D31" s="10" t="str">
+        <x:v>DEALER_DEALER</x:v>
+      </x:c>
+      <x:c r="E31" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F31" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
+      </x:c>
+      <x:c r="G31" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H31" s="10" t="str">
+        <x:v>Lower global pool threshold, raise cap, or remove lifetime guard.</x:v>
+      </x:c>
+      <x:c r="I31" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J31" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K31" s="10" t="str">
+        <x:v>N/A — timeout/contract/resource no-go</x:v>
+      </x:c>
+      <x:c r="L31" s="22" t="n">
+        <x:v>0.705</x:v>
+      </x:c>
+      <x:c r="M31" s="22"/>
+      <x:c r="N31" s="10" t="str">
+        <x:v>NO-GO: 64KiB pool threshold has a prior TCP partial timeout; cap and guard changes weaken resource or close/concurrency guarantees.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="L32" s="23"/>
-      <x:c r="M32" s="23"/>
+      <x:c r="A32" s="10" t="str">
+        <x:v>2026-08-25 20:29</x:v>
+      </x:c>
+      <x:c r="B32" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C32" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D32" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E32" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F32" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
+      </x:c>
+      <x:c r="G32" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H32" s="10" t="str">
+        <x:v>Re-evaluate bounded pool and routed operation-state reuse.</x:v>
+      </x:c>
+      <x:c r="I32" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J32" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K32" s="10" t="str">
+        <x:v>N/A — already baseline</x:v>
+      </x:c>
+      <x:c r="L32" s="22" t="n">
+        <x:v>0.71</x:v>
+      </x:c>
+      <x:c r="M32" s="22"/>
+      <x:c r="N32" s="10" t="str">
+        <x:v>NO-GO as a new A/B: the safe bounded-pool/state path is already measured.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="L33" s="23"/>
-      <x:c r="M33" s="23"/>
+      <x:c r="A33" s="10" t="str">
+        <x:v>2026-08-25 20:29</x:v>
+      </x:c>
+      <x:c r="B33" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C33" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D33" s="10" t="str">
+        <x:v>DEALER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E33" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F33" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
+      </x:c>
+      <x:c r="G33" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H33" s="10" t="str">
+        <x:v>Add route cache or remove attempt/lifetime guards.</x:v>
+      </x:c>
+      <x:c r="I33" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J33" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K33" s="10" t="str">
+        <x:v>N/A — exact-route/close no-go</x:v>
+      </x:c>
+      <x:c r="L33" s="22" t="n">
+        <x:v>0.71</x:v>
+      </x:c>
+      <x:c r="M33" s="22"/>
+      <x:c r="N33" s="10" t="str">
+        <x:v>NO-GO: route caching and guard removal change exact route selection or close/concurrency responsibility.</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="L34" s="23"/>
-      <x:c r="M34" s="23"/>
+      <x:c r="A34" s="10" t="str">
+        <x:v>2026-08-25 20:34</x:v>
+      </x:c>
+      <x:c r="B34" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C34" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D34" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E34" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F34" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G34" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H34" s="10" t="str">
+        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
+      </x:c>
+      <x:c r="I34" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J34" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K34" s="10" t="str">
+        <x:v>N/A — exact-target contract no-go</x:v>
+      </x:c>
+      <x:c r="L34" s="22" t="n">
+        <x:v>0.429</x:v>
+      </x:c>
+      <x:c r="M34" s="22"/>
+      <x:c r="N34" s="10" t="str">
+        <x:v>NO-GO: fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="L35" s="23"/>
-      <x:c r="M35" s="23"/>
+      <x:c r="A35" s="10" t="str">
+        <x:v>2026-08-25 20:34</x:v>
+      </x:c>
+      <x:c r="B35" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C35" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D35" s="10" t="str">
+        <x:v>DEALER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E35" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F35" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G35" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H35" s="10" t="str">
+        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
+      </x:c>
+      <x:c r="I35" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J35" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K35" s="10" t="str">
+        <x:v>N/A — already baseline</x:v>
+      </x:c>
+      <x:c r="L35" s="22" t="n">
+        <x:v>0.429</x:v>
+      </x:c>
+      <x:c r="M35" s="22"/>
+      <x:c r="N35" s="10" t="str">
+        <x:v>KEEP baseline: new single lvalue submit-failure test plus request/reply, target, message, socket, behavior suites pass 5/5. No transport A/B delta is claimed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="L36" s="23"/>
-      <x:c r="M36" s="23"/>
+      <x:c r="A36" s="10" t="str">
+        <x:v>2026-08-25 20:40</x:v>
+      </x:c>
+      <x:c r="B36" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C36" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D36" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E36" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F36" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
+      </x:c>
+      <x:c r="G36" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H36" s="10" t="str">
+        <x:v>Re-evaluate bounded pool and state reuse on the exact routed path.</x:v>
+      </x:c>
+      <x:c r="I36" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J36" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K36" s="10" t="str">
+        <x:v>N/A — already baseline</x:v>
+      </x:c>
+      <x:c r="L36" s="22" t="n">
+        <x:v>0.699</x:v>
+      </x:c>
+      <x:c r="M36" s="22"/>
+      <x:c r="N36" s="10" t="str">
+        <x:v>NO-GO as a new A/B: safe pool/state reuse already forms the measured path.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="L37" s="23"/>
-      <x:c r="M37" s="23"/>
+      <x:c r="A37" s="10" t="str">
+        <x:v>2026-08-25 20:40</x:v>
+      </x:c>
+      <x:c r="B37" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C37" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D37" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E37" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F37" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
+      </x:c>
+      <x:c r="G37" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H37" s="10" t="str">
+        <x:v>Add route cache, lower pool threshold, or remove lifetime guard.</x:v>
+      </x:c>
+      <x:c r="I37" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J37" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K37" s="10" t="str">
+        <x:v>N/A — contract/resource no-go</x:v>
+      </x:c>
+      <x:c r="L37" s="22" t="n">
+        <x:v>0.699</x:v>
+      </x:c>
+      <x:c r="M37" s="22"/>
+      <x:c r="N37" s="10" t="str">
+        <x:v>NO-GO: target cache and guard removal weaken exact-route/close semantics; pool changes have prior timeout/resource-boundary evidence.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="L38" s="23"/>
-      <x:c r="M38" s="23"/>
+      <x:c r="A38" s="10" t="str">
+        <x:v>2026-08-25 20:46</x:v>
+      </x:c>
+      <x:c r="B38" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C38" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D38" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E38" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F38" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G38" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H38" s="10" t="str">
+        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
+      </x:c>
+      <x:c r="I38" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J38" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K38" s="10" t="str">
+        <x:v>N/A — exact-target contract no-go</x:v>
+      </x:c>
+      <x:c r="L38" s="22" t="n">
+        <x:v>0.441</x:v>
+      </x:c>
+      <x:c r="M38" s="22"/>
+      <x:c r="N38" s="10" t="str">
+        <x:v>NO-GO: target fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="L39" s="23"/>
-      <x:c r="M39" s="23"/>
+      <x:c r="A39" s="10" t="str">
+        <x:v>2026-08-25 20:46</x:v>
+      </x:c>
+      <x:c r="B39" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C39" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D39" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E39" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F39" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G39" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H39" s="10" t="str">
+        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
+      </x:c>
+      <x:c r="I39" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J39" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K39" s="10" t="str">
+        <x:v>N/A — already baseline</x:v>
+      </x:c>
+      <x:c r="L39" s="22" t="n">
+        <x:v>0.441</x:v>
+      </x:c>
+      <x:c r="M39" s="22"/>
+      <x:c r="N39" s="10" t="str">
+        <x:v>KEEP baseline: new single lvalue submit-failure test plus request/reply, target, message, socket, behavior suites pass 5/5. No transport A/B delta is claimed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="L40" s="23"/>

</xml_diff>

<commit_message>
perf(cpp): reduce async request bridge overhead
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf195ae96f6e24af1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rcc5c048c4a614ad3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R86ec3cf597974a72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R8eb52b46b61b43b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0a8e722d21b047dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rb1b6509b6d834d69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rd757f7ffd2944769"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R93d469e9eb044fee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,7 +520,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·1개 미달·1개 보류, tls 3개 통과·4개 미달, inproc 0개 통과·7개 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 보류, tls 3개 통과·4개 미달, inproc 0개 통과·7개 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -567,7 +567,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -582,7 +582,7 @@
       </x:c>
       <x:c r="B14" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"보류",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C14" s="17" t="str">
         <x:v>Sol-reviewed safe candidates are exhausted; target still missed</x:v>
@@ -12076,24 +12076,24 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="G166" s="26" t="n">
-        <x:v>141672.2</x:v>
+        <x:v>141460.4</x:v>
       </x:c>
       <x:c r="H166" s="26" t="n">
-        <x:v>59295.6</x:v>
+        <x:v>63068.6</x:v>
       </x:c>
       <x:c r="I166" s="22" t="n">
         <x:f>H166/G166</x:f>
-        <x:v>0.41854082875821785</x:v>
+        <x:v>0.44583925960904963</x:v>
       </x:c>
       <x:c r="J166" s="24" t="n">
-        <x:v>0.376</x:v>
+        <x:v>0.421</x:v>
       </x:c>
       <x:c r="K166" s="24" t="n">
-        <x:v>1.01</x:v>
+        <x:v>0.945</x:v>
       </x:c>
       <x:c r="L166" s="24" t="n">
         <x:f>K166/J166</x:f>
-        <x:v>2.6861702127659575</x:v>
+        <x:v>2.2446555819477436</x:v>
       </x:c>
       <x:c r="M166" s="10" t="n">
         <x:v>5</x:v>
@@ -12111,19 +12111,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R166" s="10" t="str">
-        <x:v>6a5d94932e</x:v>
+        <x:v>d7c7f10c59</x:v>
       </x:c>
       <x:c r="S166" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_185524_cpp-router-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_221439_cpp-router-router-reqrep-wss-local0132-final-c2-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T166" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_221741_cpp-router-router-reqrep-wss-local0132-final-c2-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U166" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V166" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 64.35%; latency median ratio 1.86x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+        <x:v>Clean final secure 5-run median: throughput aggregate mean 65.06%; latency median ratio 1.72x. Sol approved C2 self-anchor/co-allocated callback bridge; C1/C3 rejected and C4 analytically rejected. Safe candidates exhausted, so hold.</x:v>
       </x:c>
     </x:row>
     <x:row r="167">
@@ -12146,24 +12146,24 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="G167" s="26" t="n">
-        <x:v>103015</x:v>
+        <x:v>102428</x:v>
       </x:c>
       <x:c r="H167" s="26" t="n">
-        <x:v>39973</x:v>
+        <x:v>40971</x:v>
       </x:c>
       <x:c r="I167" s="22" t="n">
         <x:f>H167/G167</x:f>
-        <x:v>0.38803086929088</x:v>
+        <x:v>0.39999804740891165</x:v>
       </x:c>
       <x:c r="J167" s="24" t="n">
-        <x:v>0.617</x:v>
+        <x:v>0.565</x:v>
       </x:c>
       <x:c r="K167" s="24" t="n">
-        <x:v>1.548</x:v>
+        <x:v>1.512</x:v>
       </x:c>
       <x:c r="L167" s="24" t="n">
         <x:f>K167/J167</x:f>
-        <x:v>2.5089141004862237</x:v>
+        <x:v>2.6761061946902656</x:v>
       </x:c>
       <x:c r="M167" s="10" t="n">
         <x:v>5</x:v>
@@ -12181,19 +12181,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R167" s="10" t="str">
-        <x:v>6a5d94932e</x:v>
+        <x:v>d7c7f10c59</x:v>
       </x:c>
       <x:c r="S167" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_185524_cpp-router-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_221439_cpp-router-router-reqrep-wss-local0132-final-c2-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T167" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_221741_cpp-router-router-reqrep-wss-local0132-final-c2-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U167" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V167" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 64.35%; latency median ratio 1.86x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+        <x:v>Clean final secure 5-run median: throughput aggregate mean 65.06%; latency median ratio 1.72x. Sol approved C2 self-anchor/co-allocated callback bridge; C1/C3 rejected and C4 analytically rejected. Safe candidates exhausted, so hold.</x:v>
       </x:c>
     </x:row>
     <x:row r="168">
@@ -12216,24 +12216,24 @@
         <x:v>1024</x:v>
       </x:c>
       <x:c r="G168" s="26" t="n">
-        <x:v>60240.4</x:v>
+        <x:v>59882.6</x:v>
       </x:c>
       <x:c r="H168" s="26" t="n">
-        <x:v>23256</x:v>
+        <x:v>24364.4</x:v>
       </x:c>
       <x:c r="I168" s="22" t="n">
         <x:f>H168/G168</x:f>
-        <x:v>0.38605321345807797</x:v>
+        <x:v>0.40686944120662766</x:v>
       </x:c>
       <x:c r="J168" s="24" t="n">
-        <x:v>1.024</x:v>
+        <x:v>1.021</x:v>
       </x:c>
       <x:c r="K168" s="24" t="n">
-        <x:v>2.71</x:v>
+        <x:v>2.617</x:v>
       </x:c>
       <x:c r="L168" s="24" t="n">
         <x:f>K168/J168</x:f>
-        <x:v>2.646484375</x:v>
+        <x:v>2.5631733594515183</x:v>
       </x:c>
       <x:c r="M168" s="10" t="n">
         <x:v>5</x:v>
@@ -12251,19 +12251,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R168" s="10" t="str">
-        <x:v>6a5d94932e</x:v>
+        <x:v>d7c7f10c59</x:v>
       </x:c>
       <x:c r="S168" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_185524_cpp-router-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_221439_cpp-router-router-reqrep-wss-local0132-final-c2-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T168" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_221741_cpp-router-router-reqrep-wss-local0132-final-c2-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U168" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V168" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 64.35%; latency median ratio 1.86x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+        <x:v>Clean final secure 5-run median: throughput aggregate mean 65.06%; latency median ratio 1.72x. Sol approved C2 self-anchor/co-allocated callback bridge; C1/C3 rejected and C4 analytically rejected. Safe candidates exhausted, so hold.</x:v>
       </x:c>
     </x:row>
     <x:row r="169">
@@ -12286,24 +12286,24 @@
         <x:v>65536</x:v>
       </x:c>
       <x:c r="G169" s="26" t="n">
-        <x:v>3777.8</x:v>
+        <x:v>4129.6</x:v>
       </x:c>
       <x:c r="H169" s="26" t="n">
-        <x:v>3378.8</x:v>
+        <x:v>3830.8</x:v>
       </x:c>
       <x:c r="I169" s="22" t="n">
         <x:f>H169/G169</x:f>
-        <x:v>0.8943829742177988</x:v>
+        <x:v>0.9276443239054629</x:v>
       </x:c>
       <x:c r="J169" s="24" t="n">
-        <x:v>3.25</x:v>
+        <x:v>2.903</x:v>
       </x:c>
       <x:c r="K169" s="24" t="n">
-        <x:v>3.961</x:v>
+        <x:v>3.11</x:v>
       </x:c>
       <x:c r="L169" s="24" t="n">
         <x:f>K169/J169</x:f>
-        <x:v>1.2187692307692308</x:v>
+        <x:v>1.07130554598691</x:v>
       </x:c>
       <x:c r="M169" s="10" t="n">
         <x:v>5</x:v>
@@ -12321,19 +12321,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R169" s="10" t="str">
-        <x:v>6a5d94932e</x:v>
+        <x:v>d7c7f10c59</x:v>
       </x:c>
       <x:c r="S169" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_185524_cpp-router-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_221439_cpp-router-router-reqrep-wss-local0132-final-c2-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T169" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_221741_cpp-router-router-reqrep-wss-local0132-final-c2-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U169" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V169" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 64.35%; latency median ratio 1.86x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+        <x:v>Clean final secure 5-run median: throughput aggregate mean 65.06%; latency median ratio 1.72x. Sol approved C2 self-anchor/co-allocated callback bridge; C1/C3 rejected and C4 analytically rejected. Safe candidates exhausted, so hold.</x:v>
       </x:c>
     </x:row>
     <x:row r="170">
@@ -12356,24 +12356,24 @@
         <x:v>131072</x:v>
       </x:c>
       <x:c r="G170" s="26" t="n">
-        <x:v>2417.2</x:v>
+        <x:v>2389</x:v>
       </x:c>
       <x:c r="H170" s="26" t="n">
-        <x:v>2176.2</x:v>
+        <x:v>1991.6</x:v>
       </x:c>
       <x:c r="I170" s="22" t="n">
         <x:f>H170/G170</x:f>
-        <x:v>0.9002978652986927</x:v>
+        <x:v>0.8336542486395981</x:v>
       </x:c>
       <x:c r="J170" s="24" t="n">
-        <x:v>2.478</x:v>
+        <x:v>2.507</x:v>
       </x:c>
       <x:c r="K170" s="24" t="n">
-        <x:v>2.722</x:v>
+        <x:v>2.975</x:v>
       </x:c>
       <x:c r="L170" s="24" t="n">
         <x:f>K170/J170</x:f>
-        <x:v>1.0984665052461662</x:v>
+        <x:v>1.1866773035500597</x:v>
       </x:c>
       <x:c r="M170" s="10" t="n">
         <x:v>5</x:v>
@@ -12391,19 +12391,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R170" s="10" t="str">
-        <x:v>6a5d94932e</x:v>
+        <x:v>d7c7f10c59</x:v>
       </x:c>
       <x:c r="S170" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_185524_cpp-router-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_221439_cpp-router-router-reqrep-wss-local0132-final-c2-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T170" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_221741_cpp-router-router-reqrep-wss-local0132-final-c2-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U170" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V170" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 64.35%; latency median ratio 1.86x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+        <x:v>Clean final secure 5-run median: throughput aggregate mean 65.06%; latency median ratio 1.72x. Sol approved C2 self-anchor/co-allocated callback bridge; C1/C3 rejected and C4 analytically rejected. Safe candidates exhausted, so hold.</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
@@ -12426,24 +12426,24 @@
         <x:v>262144</x:v>
       </x:c>
       <x:c r="G171" s="26" t="n">
-        <x:v>1400.8</x:v>
+        <x:v>1437.8</x:v>
       </x:c>
       <x:c r="H171" s="26" t="n">
-        <x:v>1223.8</x:v>
+        <x:v>1279.2</x:v>
       </x:c>
       <x:c r="I171" s="22" t="n">
         <x:f>H171/G171</x:f>
-        <x:v>0.8736436322101656</x:v>
+        <x:v>0.8896925858951176</x:v>
       </x:c>
       <x:c r="J171" s="24" t="n">
-        <x:v>2.137</x:v>
+        <x:v>2.082</x:v>
       </x:c>
       <x:c r="K171" s="24" t="n">
-        <x:v>2.394</x:v>
+        <x:v>2.281</x:v>
       </x:c>
       <x:c r="L171" s="24" t="n">
         <x:f>K171/J171</x:f>
-        <x:v>1.1202620496022462</x:v>
+        <x:v>1.0955811719500481</x:v>
       </x:c>
       <x:c r="M171" s="10" t="n">
         <x:v>5</x:v>
@@ -12461,19 +12461,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R171" s="10" t="str">
-        <x:v>6a5d94932e</x:v>
+        <x:v>d7c7f10c59</x:v>
       </x:c>
       <x:c r="S171" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_185524_cpp-router-router-reqrep-wss-local0132-baseline-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_221439_cpp-router-router-reqrep-wss-local0132-final-c2-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T171" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_221741_cpp-router-router-reqrep-wss-local0132-final-c2-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U171" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V171" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 64.35%; latency median ratio 1.86x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+        <x:v>Clean final secure 5-run median: throughput aggregate mean 65.06%; latency median ratio 1.72x. Sol approved C2 self-anchor/co-allocated callback bridge; C1/C3 rejected and C4 analytically rejected. Safe candidates exhausted, so hold.</x:v>
       </x:c>
     </x:row>
     <x:row r="172">
@@ -20487,7 +20487,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="10" t="str">
-        <x:v>2026-08-25 19:03</x:v>
+        <x:v>2026-08-25 21:42</x:v>
       </x:c>
       <x:c r="B21" s="10" t="str">
         <x:v>C++</x:v>
@@ -20505,29 +20505,33 @@
         <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G21" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>C1</x:v>
       </x:c>
       <x:c r="H21" s="10" t="str">
-        <x:v>Retain the async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
+        <x:v>Direct-adopt initialized native reply parts to remove default-init/move/close/reinit.</x:v>
       </x:c>
       <x:c r="I21" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J21" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_175007_cpp-router-router-reqrep-ws-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K21" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
-      </x:c>
-      <x:c r="L21" s="22"/>
-      <x:c r="M21" s="22"/>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_215202_cpp-router-router-reqrep-wss-local0132-candidate-1-native-adopt-paired-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L21" s="22" t="n">
+        <x:v>0.643</x:v>
+      </x:c>
+      <x:c r="M21" s="22" t="n">
+        <x:v>0.669</x:v>
+      </x:c>
       <x:c r="N21" s="10" t="str">
-        <x:v>KEEP: same Core/source implementation measured under WSS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. WSS throughput still misses the gate; latency 1.86x passes.</x:v>
+        <x:v>REJECT: aggregate rose under control drift, with mixed size-level signal. Source reverted.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="10" t="str">
-        <x:v>2026-08-25 19:10</x:v>
+        <x:v>2026-08-25 22:00</x:v>
       </x:c>
       <x:c r="B22" s="10" t="str">
         <x:v>C++</x:v>
@@ -20536,40 +20540,42 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D22" s="10" t="str">
-        <x:v>PAIR</x:v>
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E22" s="10" t="str">
-        <x:v>tls</x:v>
+        <x:v>wss</x:v>
       </x:c>
       <x:c r="F22" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G22" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>C2</x:v>
       </x:c>
       <x:c r="H22" s="10" t="str">
-        <x:v>Re-evaluate the retained 128KiB–1MiB bounded pool and process-lifetime singleton.</x:v>
+        <x:v>Anchor async completion state through the Core raw-userdata lifetime; remove separate bridge allocation.</x:v>
       </x:c>
       <x:c r="I22" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J22" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_185808_cpp-router-router-reqrep-wss-local0132-baseline-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K22" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_220032_cpp-router-router-reqrep-wss-local0132-candidate-2-state-anchor-paired-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="L22" s="22" t="n">
-        <x:v>0.921</x:v>
-      </x:c>
-      <x:c r="M22" s="22"/>
+        <x:v>0.643</x:v>
+      </x:c>
+      <x:c r="M22" s="22" t="n">
+        <x:v>0.66</x:v>
+      </x:c>
       <x:c r="N22" s="10" t="str">
-        <x:v>NO-GO as a new A/B: this safe candidate is already in source. It remains required for the existing ownership and late-release boundary.</x:v>
+        <x:v>KEEP: contract suites 5/5 pass; small-request fixed-cost reduction reproduces. Clean final source keeps C2.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="10" t="str">
-        <x:v>2026-08-25 19:10</x:v>
+        <x:v>2026-08-25 22:08</x:v>
       </x:c>
       <x:c r="B23" s="10" t="str">
         <x:v>C++</x:v>
@@ -20578,40 +20584,42 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D23" s="10" t="str">
-        <x:v>PAIR</x:v>
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E23" s="10" t="str">
-        <x:v>tls</x:v>
+        <x:v>wss</x:v>
       </x:c>
       <x:c r="F23" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G23" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>C3</x:v>
       </x:c>
       <x:c r="H23" s="10" t="str">
-        <x:v>Lower pool threshold to 64KiB, remove lifetime guard/mutex, or enlarge pool cap.</x:v>
+        <x:v>Resume coroutine inline only when no scheduler is supplied.</x:v>
       </x:c>
       <x:c r="I23" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J23" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_220032_cpp-router-router-reqrep-wss-local0132-candidate-2-state-anchor-paired-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K23" s="10" t="str">
-        <x:v>N/A — timeout/contract/resource no-go</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_220841_cpp-router-router-reqrep-wss-local0132-candidate-3-inline-resume-paired-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="L23" s="22" t="n">
-        <x:v>0.921</x:v>
-      </x:c>
-      <x:c r="M23" s="22"/>
+        <x:v>0.66</x:v>
+      </x:c>
+      <x:c r="M23" s="22" t="n">
+        <x:v>0.66</x:v>
+      </x:c>
       <x:c r="N23" s="10" t="str">
-        <x:v>NO-GO: 64KiB pool variant previously timed out; guard removal and cap expansion violate documented concurrency or resource boundaries.</x:v>
+        <x:v>REJECT: no clear incremental throughput gain over C2; expands generic coroutine race surface. Source reverted.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="10" t="str">
-        <x:v>2026-08-25 19:18</x:v>
+        <x:v>2026-08-25 22:22</x:v>
       </x:c>
       <x:c r="B24" s="10" t="str">
         <x:v>C++</x:v>
@@ -20620,40 +20628,42 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D24" s="10" t="str">
-        <x:v>PUBSUB</x:v>
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E24" s="10" t="str">
-        <x:v>tls</x:v>
+        <x:v>wss</x:v>
       </x:c>
       <x:c r="F24" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 95%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G24" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>Sol review</x:v>
       </x:c>
       <x:c r="H24" s="10" t="str">
-        <x:v>Re-evaluate direct single-part publish and operation-state reuse.</x:v>
+        <x:v>Review C1/C2/C3 measurements and C4 native routing-id cache cost model.</x:v>
       </x:c>
       <x:c r="I24" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J24" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_220841_cpp-router-router-reqrep-wss-local0132-candidate-3-inline-resume-paired-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K24" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_221741_cpp-router-router-reqrep-wss-local0132-final-c2-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="L24" s="22" t="n">
-        <x:v>0.921</x:v>
-      </x:c>
-      <x:c r="M24" s="22"/>
+        <x:v>0.66</x:v>
+      </x:c>
+      <x:c r="M24" s="22" t="n">
+        <x:v>0.651</x:v>
+      </x:c>
       <x:c r="N24" s="10" t="str">
-        <x:v>NO-GO as a new A/B: the benchmark already uses the direct single-part publish path; multipart staging is not on this hot path.</x:v>
+        <x:v>SOL APPROVED: retain C2; C1/C3 measured rejects, C4 analytic reject. No remaining contract-preserving candidate. Clean final 65.06%, latency 1.72x; 보류.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="10" t="str">
-        <x:v>2026-08-25 19:18</x:v>
+        <x:v>2026-08-25 19:10</x:v>
       </x:c>
       <x:c r="B25" s="10" t="str">
         <x:v>C++</x:v>
@@ -20662,40 +20672,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D25" s="10" t="str">
-        <x:v>PUBSUB</x:v>
+        <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E25" s="10" t="str">
         <x:v>tls</x:v>
       </x:c>
       <x:c r="F25" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 95%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%</x:v>
       </x:c>
       <x:c r="G25" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H25" s="10" t="str">
-        <x:v>Remove attempt mutex/lifetime guard, lower pool threshold, or expand pool cap.</x:v>
+        <x:v>Re-evaluate the retained 128KiB–1MiB bounded pool and process-lifetime singleton.</x:v>
       </x:c>
       <x:c r="I25" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J25" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K25" s="10" t="str">
-        <x:v>N/A — contract/resource no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L25" s="22" t="n">
         <x:v>0.921</x:v>
       </x:c>
       <x:c r="M25" s="22"/>
       <x:c r="N25" s="10" t="str">
-        <x:v>NO-GO: guard removal changes close/concurrency semantics; pool lower-bound/cap changes are global policy with a prior timeout or wider resource boundary.</x:v>
+        <x:v>NO-GO as a new A/B: this safe candidate is already in source. It remains required for the existing ownership and late-release boundary.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="10" t="str">
-        <x:v>2026-08-25 19:43</x:v>
+        <x:v>2026-08-25 19:10</x:v>
       </x:c>
       <x:c r="B26" s="10" t="str">
         <x:v>C++</x:v>
@@ -20704,40 +20714,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D26" s="10" t="str">
-        <x:v>DEALER_ROUTER_REQREP</x:v>
+        <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E26" s="10" t="str">
         <x:v>tls</x:v>
       </x:c>
       <x:c r="F26" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%</x:v>
       </x:c>
       <x:c r="G26" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H26" s="10" t="str">
-        <x:v>Use Core normal DEALER request route instead of initially selected exact transport target.</x:v>
+        <x:v>Lower pool threshold to 64KiB, remove lifetime guard/mutex, or enlarge pool cap.</x:v>
       </x:c>
       <x:c r="I26" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J26" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K26" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
+        <x:v>N/A — timeout/contract/resource no-go</x:v>
       </x:c>
       <x:c r="L26" s="22" t="n">
-        <x:v>0.709</x:v>
+        <x:v>0.921</x:v>
       </x:c>
       <x:c r="M26" s="22"/>
       <x:c r="N26" s="10" t="str">
-        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership.</x:v>
+        <x:v>NO-GO: 64KiB pool variant previously timed out; guard removal and cap expansion violate documented concurrency or resource boundaries.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="10" t="str">
-        <x:v>2026-08-25 19:43</x:v>
+        <x:v>2026-08-25 19:18</x:v>
       </x:c>
       <x:c r="B27" s="10" t="str">
         <x:v>C++</x:v>
@@ -20746,38 +20756,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D27" s="10" t="str">
-        <x:v>DEALER_ROUTER_REQREP</x:v>
+        <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E27" s="10" t="str">
         <x:v>tls</x:v>
       </x:c>
       <x:c r="F27" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Throughput aggregate &lt; 95%</x:v>
       </x:c>
       <x:c r="G27" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H27" s="10" t="str">
-        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
+        <x:v>Re-evaluate direct single-part publish and operation-state reuse.</x:v>
       </x:c>
       <x:c r="I27" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J27" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K27" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
-      </x:c>
-      <x:c r="L27" s="22"/>
+        <x:v>N/A — already baseline</x:v>
+      </x:c>
+      <x:c r="L27" s="22" t="n">
+        <x:v>0.921</x:v>
+      </x:c>
       <x:c r="M27" s="22"/>
       <x:c r="N27" s="10" t="str">
-        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.62x passes.</x:v>
+        <x:v>NO-GO as a new A/B: the benchmark already uses the direct single-part publish path; multipart staging is not on this hot path.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="10" t="str">
-        <x:v>2026-08-25 19:54</x:v>
+        <x:v>2026-08-25 19:18</x:v>
       </x:c>
       <x:c r="B28" s="10" t="str">
         <x:v>C++</x:v>
@@ -20786,40 +20798,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D28" s="10" t="str">
-        <x:v>ROUTER_ROUTER_REQREP</x:v>
+        <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E28" s="10" t="str">
         <x:v>tls</x:v>
       </x:c>
       <x:c r="F28" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Throughput aggregate &lt; 95%</x:v>
       </x:c>
       <x:c r="G28" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H28" s="10" t="str">
-        <x:v>Use Core normal route selection instead of the initially selected exact transport target.</x:v>
+        <x:v>Remove attempt mutex/lifetime guard, lower pool threshold, or expand pool cap.</x:v>
       </x:c>
       <x:c r="I28" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J28" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K28" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
+        <x:v>N/A — contract/resource no-go</x:v>
       </x:c>
       <x:c r="L28" s="22" t="n">
-        <x:v>0.714</x:v>
+        <x:v>0.921</x:v>
       </x:c>
       <x:c r="M28" s="22"/>
       <x:c r="N28" s="10" t="str">
-        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership; exact-request-target contract remains required.</x:v>
+        <x:v>NO-GO: guard removal changes close/concurrency semantics; pool lower-bound/cap changes are global policy with a prior timeout or wider resource boundary.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="10" t="str">
-        <x:v>2026-08-25 19:54</x:v>
+        <x:v>2026-08-25 19:43</x:v>
       </x:c>
       <x:c r="B29" s="10" t="str">
         <x:v>C++</x:v>
@@ -20828,7 +20840,7 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D29" s="10" t="str">
-        <x:v>ROUTER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E29" s="10" t="str">
         <x:v>tls</x:v>
@@ -20837,29 +20849,31 @@
         <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G29" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H29" s="10" t="str">
-        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
+        <x:v>Use Core normal DEALER request route instead of initially selected exact transport target.</x:v>
       </x:c>
       <x:c r="I29" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J29" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K29" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
-      </x:c>
-      <x:c r="L29" s="22"/>
+        <x:v>N/A — exact-target contract no-go</x:v>
+      </x:c>
+      <x:c r="L29" s="22" t="n">
+        <x:v>0.709</x:v>
+      </x:c>
       <x:c r="M29" s="22"/>
       <x:c r="N29" s="10" t="str">
-        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.65x passes.</x:v>
+        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="10" t="str">
-        <x:v>2026-08-25 20:08</x:v>
+        <x:v>2026-08-25 19:43</x:v>
       </x:c>
       <x:c r="B30" s="10" t="str">
         <x:v>C++</x:v>
@@ -20868,40 +20882,38 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D30" s="10" t="str">
-        <x:v>PAIR</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E30" s="10" t="str">
-        <x:v>inproc</x:v>
+        <x:v>tls</x:v>
       </x:c>
       <x:c r="F30" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G30" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H30" s="10" t="str">
-        <x:v>Re-evaluate retained 128KiB–1MiB bounded pool and process-lifetime singleton.</x:v>
+        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
       </x:c>
       <x:c r="I30" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J30" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
       </x:c>
       <x:c r="K30" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
-      </x:c>
-      <x:c r="L30" s="22" t="n">
-        <x:v>0.761</x:v>
-      </x:c>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L30" s="22"/>
       <x:c r="M30" s="22"/>
       <x:c r="N30" s="10" t="str">
-        <x:v>NO-GO as a new A/B: safe bounded-pool lifecycle is already in source, including late Core-release safety.</x:v>
+        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.62x passes.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="10" t="str">
-        <x:v>2026-08-25 20:08</x:v>
+        <x:v>2026-08-25 19:54</x:v>
       </x:c>
       <x:c r="B31" s="10" t="str">
         <x:v>C++</x:v>
@@ -20910,40 +20922,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D31" s="10" t="str">
-        <x:v>PAIR</x:v>
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E31" s="10" t="str">
-        <x:v>inproc</x:v>
+        <x:v>tls</x:v>
       </x:c>
       <x:c r="F31" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G31" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H31" s="10" t="str">
-        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
+        <x:v>Use Core normal route selection instead of the initially selected exact transport target.</x:v>
       </x:c>
       <x:c r="I31" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J31" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K31" s="10" t="str">
-        <x:v>N/A — timeout/resource no-go</x:v>
+        <x:v>N/A — exact-target contract no-go</x:v>
       </x:c>
       <x:c r="L31" s="22" t="n">
-        <x:v>0.761</x:v>
+        <x:v>0.714</x:v>
       </x:c>
       <x:c r="M31" s="22"/>
       <x:c r="N31" s="10" t="str">
-        <x:v>NO-GO: the 64KiB global threshold previously yielded a 25/30 partial TCP report through timeout; raising the cap changes the documented resource boundary. Per-transport policy would make ownership/resource behavior inconsistent.</x:v>
+        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership; exact-request-target contract remains required.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="10" t="str">
-        <x:v>2026-08-25 20:17</x:v>
+        <x:v>2026-08-25 19:54</x:v>
       </x:c>
       <x:c r="B32" s="10" t="str">
         <x:v>C++</x:v>
@@ -20952,40 +20964,38 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D32" s="10" t="str">
-        <x:v>PUBSUB</x:v>
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E32" s="10" t="str">
-        <x:v>inproc</x:v>
+        <x:v>tls</x:v>
       </x:c>
       <x:c r="F32" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G32" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H32" s="10" t="str">
-        <x:v>Re-evaluate direct single-part publish and the retained 128KiB–1MiB bounded pool.</x:v>
+        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
       </x:c>
       <x:c r="I32" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J32" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
       </x:c>
       <x:c r="K32" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
-      </x:c>
-      <x:c r="L32" s="22" t="n">
-        <x:v>0.787</x:v>
-      </x:c>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L32" s="22"/>
       <x:c r="M32" s="22"/>
       <x:c r="N32" s="10" t="str">
-        <x:v>NO-GO as a new A/B: direct publish and safe bounded-pool lifecycle already form the measured hot path.</x:v>
+        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.65x passes.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="10" t="str">
-        <x:v>2026-08-25 20:17</x:v>
+        <x:v>2026-08-25 20:08</x:v>
       </x:c>
       <x:c r="B33" s="10" t="str">
         <x:v>C++</x:v>
@@ -20994,40 +21004,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D33" s="10" t="str">
-        <x:v>PUBSUB</x:v>
+        <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E33" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F33" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
       </x:c>
       <x:c r="G33" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H33" s="10" t="str">
-        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
+        <x:v>Re-evaluate retained 128KiB–1MiB bounded pool and process-lifetime singleton.</x:v>
       </x:c>
       <x:c r="I33" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J33" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K33" s="10" t="str">
-        <x:v>N/A — timeout/resource no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L33" s="22" t="n">
-        <x:v>0.787</x:v>
+        <x:v>0.761</x:v>
       </x:c>
       <x:c r="M33" s="22"/>
       <x:c r="N33" s="10" t="str">
-        <x:v>NO-GO: 64KiB global threshold has prior 25/30 TCP partial timeout; cap expansion changes resource policy. Transport-specific policy is not an acceptable lifecycle split.</x:v>
+        <x:v>NO-GO as a new A/B: safe bounded-pool lifecycle is already in source, including late Core-release safety.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="10" t="str">
-        <x:v>2026-08-25 20:22</x:v>
+        <x:v>2026-08-25 20:08</x:v>
       </x:c>
       <x:c r="B34" s="10" t="str">
         <x:v>C++</x:v>
@@ -21036,40 +21046,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D34" s="10" t="str">
-        <x:v>DEALER_DEALER</x:v>
+        <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E34" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F34" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
       </x:c>
       <x:c r="G34" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H34" s="10" t="str">
-        <x:v>Re-evaluate bounded pool and operation-state reuse in the routed one-way hot path.</x:v>
+        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
       </x:c>
       <x:c r="I34" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J34" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K34" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — timeout/resource no-go</x:v>
       </x:c>
       <x:c r="L34" s="22" t="n">
-        <x:v>0.705</x:v>
+        <x:v>0.761</x:v>
       </x:c>
       <x:c r="M34" s="22"/>
       <x:c r="N34" s="10" t="str">
-        <x:v>NO-GO as a new A/B: the measured path already has the safe pool/state lifecycle.</x:v>
+        <x:v>NO-GO: the 64KiB global threshold previously yielded a 25/30 partial TCP report through timeout; raising the cap changes the documented resource boundary. Per-transport policy would make ownership/resource behavior inconsistent.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="10" t="str">
-        <x:v>2026-08-25 20:22</x:v>
+        <x:v>2026-08-25 20:17</x:v>
       </x:c>
       <x:c r="B35" s="10" t="str">
         <x:v>C++</x:v>
@@ -21078,40 +21088,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D35" s="10" t="str">
-        <x:v>DEALER_DEALER</x:v>
+        <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E35" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F35" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
       </x:c>
       <x:c r="G35" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H35" s="10" t="str">
-        <x:v>Lower global pool threshold, raise cap, or remove lifetime guard.</x:v>
+        <x:v>Re-evaluate direct single-part publish and the retained 128KiB–1MiB bounded pool.</x:v>
       </x:c>
       <x:c r="I35" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J35" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K35" s="10" t="str">
-        <x:v>N/A — timeout/contract/resource no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L35" s="22" t="n">
-        <x:v>0.705</x:v>
+        <x:v>0.787</x:v>
       </x:c>
       <x:c r="M35" s="22"/>
       <x:c r="N35" s="10" t="str">
-        <x:v>NO-GO: 64KiB pool threshold has a prior TCP partial timeout; cap and guard changes weaken resource or close/concurrency guarantees.</x:v>
+        <x:v>NO-GO as a new A/B: direct publish and safe bounded-pool lifecycle already form the measured hot path.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="10" t="str">
-        <x:v>2026-08-25 20:29</x:v>
+        <x:v>2026-08-25 20:17</x:v>
       </x:c>
       <x:c r="B36" s="10" t="str">
         <x:v>C++</x:v>
@@ -21120,40 +21130,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D36" s="10" t="str">
-        <x:v>DEALER_ROUTER</x:v>
+        <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E36" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F36" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
       </x:c>
       <x:c r="G36" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H36" s="10" t="str">
-        <x:v>Re-evaluate bounded pool and routed operation-state reuse.</x:v>
+        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
       </x:c>
       <x:c r="I36" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J36" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K36" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — timeout/resource no-go</x:v>
       </x:c>
       <x:c r="L36" s="22" t="n">
-        <x:v>0.71</x:v>
+        <x:v>0.787</x:v>
       </x:c>
       <x:c r="M36" s="22"/>
       <x:c r="N36" s="10" t="str">
-        <x:v>NO-GO as a new A/B: the safe bounded-pool/state path is already measured.</x:v>
+        <x:v>NO-GO: 64KiB global threshold has prior 25/30 TCP partial timeout; cap expansion changes resource policy. Transport-specific policy is not an acceptable lifecycle split.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="10" t="str">
-        <x:v>2026-08-25 20:29</x:v>
+        <x:v>2026-08-25 20:22</x:v>
       </x:c>
       <x:c r="B37" s="10" t="str">
         <x:v>C++</x:v>
@@ -21162,40 +21172,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D37" s="10" t="str">
-        <x:v>DEALER_ROUTER</x:v>
+        <x:v>DEALER_DEALER</x:v>
       </x:c>
       <x:c r="E37" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F37" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
       </x:c>
       <x:c r="G37" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H37" s="10" t="str">
-        <x:v>Add route cache or remove attempt/lifetime guards.</x:v>
+        <x:v>Re-evaluate bounded pool and operation-state reuse in the routed one-way hot path.</x:v>
       </x:c>
       <x:c r="I37" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J37" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K37" s="10" t="str">
-        <x:v>N/A — exact-route/close no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L37" s="22" t="n">
-        <x:v>0.71</x:v>
+        <x:v>0.705</x:v>
       </x:c>
       <x:c r="M37" s="22"/>
       <x:c r="N37" s="10" t="str">
-        <x:v>NO-GO: route caching and guard removal change exact route selection or close/concurrency responsibility.</x:v>
+        <x:v>NO-GO as a new A/B: the measured path already has the safe pool/state lifecycle.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="10" t="str">
-        <x:v>2026-08-25 20:34</x:v>
+        <x:v>2026-08-25 20:22</x:v>
       </x:c>
       <x:c r="B38" s="10" t="str">
         <x:v>C++</x:v>
@@ -21204,40 +21214,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D38" s="10" t="str">
-        <x:v>DEALER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_DEALER</x:v>
       </x:c>
       <x:c r="E38" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F38" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
       </x:c>
       <x:c r="G38" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H38" s="10" t="str">
-        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
+        <x:v>Lower global pool threshold, raise cap, or remove lifetime guard.</x:v>
       </x:c>
       <x:c r="I38" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J38" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K38" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
+        <x:v>N/A — timeout/contract/resource no-go</x:v>
       </x:c>
       <x:c r="L38" s="22" t="n">
-        <x:v>0.429</x:v>
+        <x:v>0.705</x:v>
       </x:c>
       <x:c r="M38" s="22"/>
       <x:c r="N38" s="10" t="str">
-        <x:v>NO-GO: fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
+        <x:v>NO-GO: 64KiB pool threshold has a prior TCP partial timeout; cap and guard changes weaken resource or close/concurrency guarantees.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="10" t="str">
-        <x:v>2026-08-25 20:34</x:v>
+        <x:v>2026-08-25 20:29</x:v>
       </x:c>
       <x:c r="B39" s="10" t="str">
         <x:v>C++</x:v>
@@ -21246,40 +21256,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D39" s="10" t="str">
-        <x:v>DEALER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_ROUTER</x:v>
       </x:c>
       <x:c r="E39" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F39" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
       </x:c>
       <x:c r="G39" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H39" s="10" t="str">
-        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
+        <x:v>Re-evaluate bounded pool and routed operation-state reuse.</x:v>
       </x:c>
       <x:c r="I39" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J39" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K39" s="10" t="str">
         <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L39" s="22" t="n">
-        <x:v>0.429</x:v>
+        <x:v>0.71</x:v>
       </x:c>
       <x:c r="M39" s="22"/>
       <x:c r="N39" s="10" t="str">
-        <x:v>KEEP baseline: new single lvalue submit-failure test plus request/reply, target, message, socket, behavior suites pass 5/5. No transport A/B delta is claimed.</x:v>
+        <x:v>NO-GO as a new A/B: the safe bounded-pool/state path is already measured.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="10" t="str">
-        <x:v>2026-08-25 20:40</x:v>
+        <x:v>2026-08-25 20:29</x:v>
       </x:c>
       <x:c r="B40" s="10" t="str">
         <x:v>C++</x:v>
@@ -21288,40 +21298,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D40" s="10" t="str">
-        <x:v>ROUTER_ROUTER</x:v>
+        <x:v>DEALER_ROUTER</x:v>
       </x:c>
       <x:c r="E40" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F40" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
       </x:c>
       <x:c r="G40" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H40" s="10" t="str">
-        <x:v>Re-evaluate bounded pool and state reuse on the exact routed path.</x:v>
+        <x:v>Add route cache or remove attempt/lifetime guards.</x:v>
       </x:c>
       <x:c r="I40" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J40" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K40" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — exact-route/close no-go</x:v>
       </x:c>
       <x:c r="L40" s="22" t="n">
-        <x:v>0.699</x:v>
+        <x:v>0.71</x:v>
       </x:c>
       <x:c r="M40" s="22"/>
       <x:c r="N40" s="10" t="str">
-        <x:v>NO-GO as a new A/B: safe pool/state reuse already forms the measured path.</x:v>
+        <x:v>NO-GO: route caching and guard removal change exact route selection or close/concurrency responsibility.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="10" t="str">
-        <x:v>2026-08-25 20:40</x:v>
+        <x:v>2026-08-25 20:34</x:v>
       </x:c>
       <x:c r="B41" s="10" t="str">
         <x:v>C++</x:v>
@@ -21330,40 +21340,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D41" s="10" t="str">
-        <x:v>ROUTER_ROUTER</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E41" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F41" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G41" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H41" s="10" t="str">
-        <x:v>Add route cache, lower pool threshold, or remove lifetime guard.</x:v>
+        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
       </x:c>
       <x:c r="I41" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J41" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K41" s="10" t="str">
-        <x:v>N/A — contract/resource no-go</x:v>
+        <x:v>N/A — exact-target contract no-go</x:v>
       </x:c>
       <x:c r="L41" s="22" t="n">
-        <x:v>0.699</x:v>
+        <x:v>0.429</x:v>
       </x:c>
       <x:c r="M41" s="22"/>
       <x:c r="N41" s="10" t="str">
-        <x:v>NO-GO: target cache and guard removal weaken exact-route/close semantics; pool changes have prior timeout/resource-boundary evidence.</x:v>
+        <x:v>NO-GO: fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="10" t="str">
-        <x:v>2026-08-25 20:46</x:v>
+        <x:v>2026-08-25 20:34</x:v>
       </x:c>
       <x:c r="B42" s="10" t="str">
         <x:v>C++</x:v>
@@ -21372,7 +21382,7 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D42" s="10" t="str">
-        <x:v>ROUTER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E42" s="10" t="str">
         <x:v>inproc</x:v>
@@ -21381,31 +21391,31 @@
         <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G42" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H42" s="10" t="str">
-        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
+        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
       </x:c>
       <x:c r="I42" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J42" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K42" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L42" s="22" t="n">
-        <x:v>0.441</x:v>
+        <x:v>0.429</x:v>
       </x:c>
       <x:c r="M42" s="22"/>
       <x:c r="N42" s="10" t="str">
-        <x:v>NO-GO: target fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
+        <x:v>KEEP baseline: new single lvalue submit-failure test plus request/reply, target, message, socket, behavior suites pass 5/5. No transport A/B delta is claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="10" t="str">
-        <x:v>2026-08-25 20:46</x:v>
+        <x:v>2026-08-25 20:40</x:v>
       </x:c>
       <x:c r="B43" s="10" t="str">
         <x:v>C++</x:v>
@@ -21414,84 +21424,162 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D43" s="10" t="str">
-        <x:v>ROUTER_ROUTER_REQREP</x:v>
+        <x:v>ROUTER_ROUTER</x:v>
       </x:c>
       <x:c r="E43" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F43" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
       </x:c>
       <x:c r="G43" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H43" s="10" t="str">
-        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
+        <x:v>Re-evaluate bounded pool and state reuse on the exact routed path.</x:v>
       </x:c>
       <x:c r="I43" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J43" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K43" s="10" t="str">
         <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L43" s="22" t="n">
-        <x:v>0.441</x:v>
+        <x:v>0.699</x:v>
       </x:c>
       <x:c r="M43" s="22"/>
       <x:c r="N43" s="10" t="str">
+        <x:v>NO-GO as a new A/B: safe pool/state reuse already forms the measured path.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="10" t="str">
+        <x:v>2026-08-25 20:40</x:v>
+      </x:c>
+      <x:c r="B44" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C44" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D44" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E44" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F44" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
+      </x:c>
+      <x:c r="G44" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H44" s="10" t="str">
+        <x:v>Add route cache, lower pool threshold, or remove lifetime guard.</x:v>
+      </x:c>
+      <x:c r="I44" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J44" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K44" s="10" t="str">
+        <x:v>N/A — contract/resource no-go</x:v>
+      </x:c>
+      <x:c r="L44" s="22" t="n">
+        <x:v>0.699</x:v>
+      </x:c>
+      <x:c r="M44" s="22"/>
+      <x:c r="N44" s="10" t="str">
+        <x:v>NO-GO: target cache and guard removal weaken exact-route/close semantics; pool changes have prior timeout/resource-boundary evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="10" t="str">
+        <x:v>2026-08-25 20:46</x:v>
+      </x:c>
+      <x:c r="B45" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C45" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D45" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E45" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F45" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G45" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H45" s="10" t="str">
+        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
+      </x:c>
+      <x:c r="I45" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J45" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K45" s="10" t="str">
+        <x:v>N/A — exact-target contract no-go</x:v>
+      </x:c>
+      <x:c r="L45" s="22" t="n">
+        <x:v>0.441</x:v>
+      </x:c>
+      <x:c r="M45" s="22"/>
+      <x:c r="N45" s="10" t="str">
+        <x:v>NO-GO: target fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="10" t="str">
+        <x:v>2026-08-25 20:46</x:v>
+      </x:c>
+      <x:c r="B46" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C46" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D46" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E46" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F46" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G46" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H46" s="10" t="str">
+        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
+      </x:c>
+      <x:c r="I46" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J46" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K46" s="10" t="str">
+        <x:v>N/A — already baseline</x:v>
+      </x:c>
+      <x:c r="L46" s="22" t="n">
+        <x:v>0.441</x:v>
+      </x:c>
+      <x:c r="M46" s="22"/>
+      <x:c r="N46" s="10" t="str">
         <x:v>KEEP baseline: new single lvalue submit-failure test plus request/reply, target, message, socket, behavior suites pass 5/5. No transport A/B delta is claimed.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44" s="10"/>
-      <x:c r="B44" s="10"/>
-      <x:c r="C44" s="10"/>
-      <x:c r="D44" s="10"/>
-      <x:c r="E44" s="10"/>
-      <x:c r="F44" s="10"/>
-      <x:c r="G44" s="10"/>
-      <x:c r="H44" s="10"/>
-      <x:c r="I44" s="10"/>
-      <x:c r="J44" s="10"/>
-      <x:c r="K44" s="10"/>
-      <x:c r="L44" s="22"/>
-      <x:c r="M44" s="22"/>
-      <x:c r="N44" s="10"/>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="10"/>
-      <x:c r="B45" s="10"/>
-      <x:c r="C45" s="10"/>
-      <x:c r="D45" s="10"/>
-      <x:c r="E45" s="10"/>
-      <x:c r="F45" s="10"/>
-      <x:c r="G45" s="10"/>
-      <x:c r="H45" s="10"/>
-      <x:c r="I45" s="10"/>
-      <x:c r="J45" s="10"/>
-      <x:c r="K45" s="10"/>
-      <x:c r="L45" s="22"/>
-      <x:c r="M45" s="22"/>
-      <x:c r="N45" s="10"/>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="10"/>
-      <x:c r="B46" s="10"/>
-      <x:c r="C46" s="10"/>
-      <x:c r="D46" s="10"/>
-      <x:c r="E46" s="10"/>
-      <x:c r="F46" s="10"/>
-      <x:c r="G46" s="10"/>
-      <x:c r="H46" s="10"/>
-      <x:c r="I46" s="10"/>
-      <x:c r="J46" s="10"/>
-      <x:c r="K46" s="10"/>
-      <x:c r="L46" s="22"/>
-      <x:c r="M46" s="22"/>
-      <x:c r="N46" s="10"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="10"/>

</xml_diff>

<commit_message>
docs(perf): record tls pair reviewer hold
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0a8e722d21b047dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rb1b6509b6d834d69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rd757f7ffd2944769"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R93d469e9eb044fee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R59cb193800c54f56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rcb1e614c16de4ccb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rbe095e77c0c6404a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R1e19c92018244c1e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,7 +520,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 보류, tls 3개 통과·4개 미달, inproc 0개 통과·7개 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 보류, tls 3개 통과·3개 미달·1개 보류, inproc 0개 통과·7개 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -567,7 +567,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -582,7 +582,7 @@
       </x:c>
       <x:c r="B14" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"보류",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C14" s="17" t="str">
         <x:v>Sol-reviewed safe candidates are exhausted; target still missed</x:v>
@@ -12496,24 +12496,24 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="G172" s="26" t="n">
-        <x:v>2381061.8</x:v>
+        <x:v>2714088.8</x:v>
       </x:c>
       <x:c r="H172" s="26" t="n">
-        <x:v>2152817.4</x:v>
+        <x:v>2363271.6</x:v>
       </x:c>
       <x:c r="I172" s="22" t="n">
         <x:f>H172/G172</x:f>
-        <x:v>0.9041417572614033</x:v>
+        <x:v>0.8707421805800902</x:v>
       </x:c>
       <x:c r="J172" s="24" t="n">
-        <x:v>0.539</x:v>
+        <x:v>0.555</x:v>
       </x:c>
       <x:c r="K172" s="24" t="n">
-        <x:v>0.382</x:v>
+        <x:v>0.404</x:v>
       </x:c>
       <x:c r="L172" s="24" t="n">
         <x:f>K172/J172</x:f>
-        <x:v>0.7087198515769944</x:v>
+        <x:v>0.7279279279279279</x:v>
       </x:c>
       <x:c r="M172" s="10" t="n">
         <x:v>5</x:v>
@@ -12531,19 +12531,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R172" s="10" t="str">
-        <x:v>cf231e58f4</x:v>
+        <x:v>6455ddaf33</x:v>
       </x:c>
       <x:c r="S172" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_190411_cpp-pair-tls-local0132-final5-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_224250_cpp-pair-tls-local0132-final-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T172" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_224554_cpp-pair-tls-local0132-final-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U172" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V172" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 92.09%; latency median ratio 0.99x; strict gate fail. Existing bounded-pool A is already baseline; 64KiB-pool B remains timeout no-go.</x:v>
+        <x:v>Clean final secure 5-run median: throughput aggregate mean 92.33%; latency median ratio 1.05x. Sol approved hold after global pool bypass and try-lock fallback regressions; original bounded pool retained.</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -12566,24 +12566,24 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="G173" s="26" t="n">
-        <x:v>925772.2</x:v>
+        <x:v>1023126.4</x:v>
       </x:c>
       <x:c r="H173" s="26" t="n">
-        <x:v>936106.4</x:v>
+        <x:v>1035729.4</x:v>
       </x:c>
       <x:c r="I173" s="22" t="n">
         <x:f>H173/G173</x:f>
-        <x:v>1.0111627892909294</x:v>
+        <x:v>1.0123181260888194</x:v>
       </x:c>
       <x:c r="J173" s="24" t="n">
-        <x:v>1.826</x:v>
+        <x:v>1.708</x:v>
       </x:c>
       <x:c r="K173" s="24" t="n">
-        <x:v>1.796</x:v>
+        <x:v>1.618</x:v>
       </x:c>
       <x:c r="L173" s="24" t="n">
         <x:f>K173/J173</x:f>
-        <x:v>0.9835706462212486</x:v>
+        <x:v>0.9473067915690867</x:v>
       </x:c>
       <x:c r="M173" s="10" t="n">
         <x:v>5</x:v>
@@ -12601,19 +12601,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R173" s="10" t="str">
-        <x:v>cf231e58f4</x:v>
+        <x:v>6455ddaf33</x:v>
       </x:c>
       <x:c r="S173" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_190411_cpp-pair-tls-local0132-final5-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_224250_cpp-pair-tls-local0132-final-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T173" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_224554_cpp-pair-tls-local0132-final-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U173" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V173" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 92.09%; latency median ratio 0.99x; strict gate fail. Existing bounded-pool A is already baseline; 64KiB-pool B remains timeout no-go.</x:v>
+        <x:v>Clean final secure 5-run median: throughput aggregate mean 92.33%; latency median ratio 1.05x. Sol approved hold after global pool bypass and try-lock fallback regressions; original bounded pool retained.</x:v>
       </x:c>
     </x:row>
     <x:row r="174">
@@ -12636,24 +12636,24 @@
         <x:v>1024</x:v>
       </x:c>
       <x:c r="G174" s="26" t="n">
-        <x:v>280878.4</x:v>
+        <x:v>323032.8</x:v>
       </x:c>
       <x:c r="H174" s="26" t="n">
-        <x:v>278512.2</x:v>
+        <x:v>322199.8</x:v>
       </x:c>
       <x:c r="I174" s="22" t="n">
         <x:f>H174/G174</x:f>
-        <x:v>0.9915757139032406</x:v>
+        <x:v>0.997421314491903</x:v>
       </x:c>
       <x:c r="J174" s="24" t="n">
-        <x:v>1.761</x:v>
+        <x:v>1.534</x:v>
       </x:c>
       <x:c r="K174" s="24" t="n">
-        <x:v>1.767</x:v>
+        <x:v>1.527</x:v>
       </x:c>
       <x:c r="L174" s="24" t="n">
         <x:f>K174/J174</x:f>
-        <x:v>1.0034071550255537</x:v>
+        <x:v>0.9954367666232072</x:v>
       </x:c>
       <x:c r="M174" s="10" t="n">
         <x:v>5</x:v>
@@ -12671,19 +12671,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R174" s="10" t="str">
-        <x:v>cf231e58f4</x:v>
+        <x:v>6455ddaf33</x:v>
       </x:c>
       <x:c r="S174" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_190411_cpp-pair-tls-local0132-final5-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_224250_cpp-pair-tls-local0132-final-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T174" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_224554_cpp-pair-tls-local0132-final-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U174" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V174" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 92.09%; latency median ratio 0.99x; strict gate fail. Existing bounded-pool A is already baseline; 64KiB-pool B remains timeout no-go.</x:v>
+        <x:v>Clean final secure 5-run median: throughput aggregate mean 92.33%; latency median ratio 1.05x. Sol approved hold after global pool bypass and try-lock fallback regressions; original bounded pool retained.</x:v>
       </x:c>
     </x:row>
     <x:row r="175">
@@ -12706,24 +12706,24 @@
         <x:v>65536</x:v>
       </x:c>
       <x:c r="G175" s="26" t="n">
-        <x:v>11401.4</x:v>
+        <x:v>12101.4</x:v>
       </x:c>
       <x:c r="H175" s="26" t="n">
-        <x:v>10499</x:v>
+        <x:v>11403.2</x:v>
       </x:c>
       <x:c r="I175" s="22" t="n">
         <x:f>H175/G175</x:f>
-        <x:v>0.9208518252144474</x:v>
+        <x:v>0.9423041962087032</x:v>
       </x:c>
       <x:c r="J175" s="24" t="n">
-        <x:v>1.023</x:v>
+        <x:v>0.813</x:v>
       </x:c>
       <x:c r="K175" s="24" t="n">
-        <x:v>0.94</x:v>
+        <x:v>0.892</x:v>
       </x:c>
       <x:c r="L175" s="24" t="n">
         <x:f>K175/J175</x:f>
-        <x:v>0.9188660801564028</x:v>
+        <x:v>1.0971709717097171</x:v>
       </x:c>
       <x:c r="M175" s="10" t="n">
         <x:v>5</x:v>
@@ -12741,19 +12741,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R175" s="10" t="str">
-        <x:v>cf231e58f4</x:v>
+        <x:v>6455ddaf33</x:v>
       </x:c>
       <x:c r="S175" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_190411_cpp-pair-tls-local0132-final5-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_224250_cpp-pair-tls-local0132-final-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T175" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_224554_cpp-pair-tls-local0132-final-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U175" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V175" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 92.09%; latency median ratio 0.99x; strict gate fail. Existing bounded-pool A is already baseline; 64KiB-pool B remains timeout no-go.</x:v>
+        <x:v>Clean final secure 5-run median: throughput aggregate mean 92.33%; latency median ratio 1.05x. Sol approved hold after global pool bypass and try-lock fallback regressions; original bounded pool retained.</x:v>
       </x:c>
     </x:row>
     <x:row r="176">
@@ -12776,24 +12776,24 @@
         <x:v>131072</x:v>
       </x:c>
       <x:c r="G176" s="26" t="n">
-        <x:v>6907.6</x:v>
+        <x:v>7171.2</x:v>
       </x:c>
       <x:c r="H176" s="26" t="n">
-        <x:v>6125.2</x:v>
+        <x:v>6613.4</x:v>
       </x:c>
       <x:c r="I176" s="22" t="n">
         <x:f>H176/G176</x:f>
-        <x:v>0.8867334530082807</x:v>
+        <x:v>0.9222166443551986</x:v>
       </x:c>
       <x:c r="J176" s="24" t="n">
-        <x:v>0.881</x:v>
+        <x:v>0.833</x:v>
       </x:c>
       <x:c r="K176" s="24" t="n">
-        <x:v>1.167</x:v>
+        <x:v>1.02</x:v>
       </x:c>
       <x:c r="L176" s="24" t="n">
         <x:f>K176/J176</x:f>
-        <x:v>1.3246311010215663</x:v>
+        <x:v>1.2244897959183674</x:v>
       </x:c>
       <x:c r="M176" s="10" t="n">
         <x:v>5</x:v>
@@ -12811,19 +12811,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R176" s="10" t="str">
-        <x:v>cf231e58f4</x:v>
+        <x:v>6455ddaf33</x:v>
       </x:c>
       <x:c r="S176" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_190411_cpp-pair-tls-local0132-final5-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_224250_cpp-pair-tls-local0132-final-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T176" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_224554_cpp-pair-tls-local0132-final-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U176" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V176" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 92.09%; latency median ratio 0.99x; strict gate fail. Existing bounded-pool A is already baseline; 64KiB-pool B remains timeout no-go.</x:v>
+        <x:v>Clean final secure 5-run median: throughput aggregate mean 92.33%; latency median ratio 1.05x. Sol approved hold after global pool bypass and try-lock fallback regressions; original bounded pool retained.</x:v>
       </x:c>
     </x:row>
     <x:row r="177">
@@ -12846,24 +12846,24 @@
         <x:v>262144</x:v>
       </x:c>
       <x:c r="G177" s="26" t="n">
-        <x:v>3819.6</x:v>
+        <x:v>3997</x:v>
       </x:c>
       <x:c r="H177" s="26" t="n">
-        <x:v>3096.6</x:v>
+        <x:v>3176.2</x:v>
       </x:c>
       <x:c r="I177" s="22" t="n">
         <x:f>H177/G177</x:f>
-        <x:v>0.8107131636820609</x:v>
+        <x:v>0.7946459844883662</x:v>
       </x:c>
       <x:c r="J177" s="24" t="n">
-        <x:v>1.038</x:v>
+        <x:v>0.988</x:v>
       </x:c>
       <x:c r="K177" s="24" t="n">
-        <x:v>1.287</x:v>
+        <x:v>1.253</x:v>
       </x:c>
       <x:c r="L177" s="24" t="n">
         <x:f>K177/J177</x:f>
-        <x:v>1.2398843930635837</x:v>
+        <x:v>1.2682186234817814</x:v>
       </x:c>
       <x:c r="M177" s="10" t="n">
         <x:v>5</x:v>
@@ -12881,19 +12881,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R177" s="10" t="str">
-        <x:v>cf231e58f4</x:v>
+        <x:v>6455ddaf33</x:v>
       </x:c>
       <x:c r="S177" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_190411_cpp-pair-tls-local0132-final5-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_224250_cpp-pair-tls-local0132-final-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T177" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_224554_cpp-pair-tls-local0132-final-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U177" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V177" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 92.09%; latency median ratio 0.99x; strict gate fail. Existing bounded-pool A is already baseline; 64KiB-pool B remains timeout no-go.</x:v>
+        <x:v>Clean final secure 5-run median: throughput aggregate mean 92.33%; latency median ratio 1.05x. Sol approved hold after global pool bypass and try-lock fallback regressions; original bounded pool retained.</x:v>
       </x:c>
     </x:row>
     <x:row r="178">
@@ -20663,7 +20663,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="10" t="str">
-        <x:v>2026-08-25 19:10</x:v>
+        <x:v>2026-08-25 22:29</x:v>
       </x:c>
       <x:c r="B25" s="10" t="str">
         <x:v>C++</x:v>
@@ -20681,10 +20681,10 @@
         <x:v>Strict throughput aggregate &lt; 95%</x:v>
       </x:c>
       <x:c r="G25" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>C1</x:v>
       </x:c>
       <x:c r="H25" s="10" t="str">
-        <x:v>Re-evaluate the retained 128KiB–1MiB bounded pool and process-lifetime singleton.</x:v>
+        <x:v>Globally bypass the 128KiB–1MiB bounded pool and use Core native allocation.</x:v>
       </x:c>
       <x:c r="I25" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
@@ -20693,19 +20693,21 @@
         <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K25" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_223234_cpp-pair-tls-local0132-candidate-pool-off-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="L25" s="22" t="n">
         <x:v>0.921</x:v>
       </x:c>
-      <x:c r="M25" s="22"/>
+      <x:c r="M25" s="22" t="n">
+        <x:v>0.914</x:v>
+      </x:c>
       <x:c r="N25" s="10" t="str">
-        <x:v>NO-GO as a new A/B: this safe candidate is already in source. It remains required for the existing ownership and late-release boundary.</x:v>
+        <x:v>REJECT: contract 5/5 passes, but paired aggregate regresses to 91.37%. Transport-specific policy is not allowed.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="10" t="str">
-        <x:v>2026-08-25 19:10</x:v>
+        <x:v>2026-08-25 22:36</x:v>
       </x:c>
       <x:c r="B26" s="10" t="str">
         <x:v>C++</x:v>
@@ -20723,10 +20725,10 @@
         <x:v>Strict throughput aggregate &lt; 95%</x:v>
       </x:c>
       <x:c r="G26" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>C2</x:v>
       </x:c>
       <x:c r="H26" s="10" t="str">
-        <x:v>Lower pool threshold to 64KiB, remove lifetime guard/mutex, or enlarge pool cap.</x:v>
+        <x:v>Use try-lock acquire and safely fall back to native allocation only while pool release holds the mutex.</x:v>
       </x:c>
       <x:c r="I26" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
@@ -20735,19 +20737,21 @@
         <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_190653_cpp-pair-tls-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K26" s="10" t="str">
-        <x:v>N/A — timeout/contract/resource no-go</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_223902_cpp-pair-tls-local0132-candidate-pool-trylock-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="L26" s="22" t="n">
         <x:v>0.921</x:v>
       </x:c>
-      <x:c r="M26" s="22"/>
+      <x:c r="M26" s="22" t="n">
+        <x:v>0.916</x:v>
+      </x:c>
       <x:c r="N26" s="10" t="str">
-        <x:v>NO-GO: 64KiB pool variant previously timed out; guard removal and cap expansion violate documented concurrency or resource boundaries.</x:v>
+        <x:v>REJECT: contract 5/5 passes, but paired aggregate regresses to 91.55%. Original bounded pool restored.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="10" t="str">
-        <x:v>2026-08-25 19:18</x:v>
+        <x:v>2026-08-25 22:45</x:v>
       </x:c>
       <x:c r="B27" s="10" t="str">
         <x:v>C++</x:v>
@@ -20756,35 +20760,37 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D27" s="10" t="str">
-        <x:v>PUBSUB</x:v>
+        <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E27" s="10" t="str">
         <x:v>tls</x:v>
       </x:c>
       <x:c r="F27" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 95%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%</x:v>
       </x:c>
       <x:c r="G27" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>Sol review</x:v>
       </x:c>
       <x:c r="H27" s="10" t="str">
-        <x:v>Re-evaluate direct single-part publish and operation-state reuse.</x:v>
+        <x:v>Review C1/C2 and remaining global pool/callback-lifetime candidates.</x:v>
       </x:c>
       <x:c r="I27" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J27" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_223902_cpp-pair-tls-local0132-candidate-pool-trylock-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K27" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_224554_cpp-pair-tls-local0132-final-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="L27" s="22" t="n">
-        <x:v>0.921</x:v>
-      </x:c>
-      <x:c r="M27" s="22"/>
+        <x:v>0.916</x:v>
+      </x:c>
+      <x:c r="M27" s="22" t="n">
+        <x:v>0.923</x:v>
+      </x:c>
       <x:c r="N27" s="10" t="str">
-        <x:v>NO-GO as a new A/B: the benchmark already uses the direct single-part publish path; multipart staging is not on this hot path.</x:v>
+        <x:v>SOL APPROVED: original pool retained; no safe candidate remains. Clean final 92.33%, latency 1.05x; 보류.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -20807,10 +20813,10 @@
         <x:v>Throughput aggregate &lt; 95%</x:v>
       </x:c>
       <x:c r="G28" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H28" s="10" t="str">
-        <x:v>Remove attempt mutex/lifetime guard, lower pool threshold, or expand pool cap.</x:v>
+        <x:v>Re-evaluate direct single-part publish and operation-state reuse.</x:v>
       </x:c>
       <x:c r="I28" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
@@ -20819,19 +20825,19 @@
         <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K28" s="10" t="str">
-        <x:v>N/A — contract/resource no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L28" s="22" t="n">
         <x:v>0.921</x:v>
       </x:c>
       <x:c r="M28" s="22"/>
       <x:c r="N28" s="10" t="str">
-        <x:v>NO-GO: guard removal changes close/concurrency semantics; pool lower-bound/cap changes are global policy with a prior timeout or wider resource boundary.</x:v>
+        <x:v>NO-GO as a new A/B: the benchmark already uses the direct single-part publish path; multipart staging is not on this hot path.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="10" t="str">
-        <x:v>2026-08-25 19:43</x:v>
+        <x:v>2026-08-25 19:18</x:v>
       </x:c>
       <x:c r="B29" s="10" t="str">
         <x:v>C++</x:v>
@@ -20840,35 +20846,35 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D29" s="10" t="str">
-        <x:v>DEALER_ROUTER_REQREP</x:v>
+        <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E29" s="10" t="str">
         <x:v>tls</x:v>
       </x:c>
       <x:c r="F29" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Throughput aggregate &lt; 95%</x:v>
       </x:c>
       <x:c r="G29" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H29" s="10" t="str">
-        <x:v>Use Core normal DEALER request route instead of initially selected exact transport target.</x:v>
+        <x:v>Remove attempt mutex/lifetime guard, lower pool threshold, or expand pool cap.</x:v>
       </x:c>
       <x:c r="I29" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J29" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K29" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
+        <x:v>N/A — contract/resource no-go</x:v>
       </x:c>
       <x:c r="L29" s="22" t="n">
-        <x:v>0.709</x:v>
+        <x:v>0.921</x:v>
       </x:c>
       <x:c r="M29" s="22"/>
       <x:c r="N29" s="10" t="str">
-        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership.</x:v>
+        <x:v>NO-GO: guard removal changes close/concurrency semantics; pool lower-bound/cap changes are global policy with a prior timeout or wider resource boundary.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -20891,29 +20897,31 @@
         <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G30" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H30" s="10" t="str">
-        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
+        <x:v>Use Core normal DEALER request route instead of initially selected exact transport target.</x:v>
       </x:c>
       <x:c r="I30" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J30" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K30" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
-      </x:c>
-      <x:c r="L30" s="22"/>
+        <x:v>N/A — exact-target contract no-go</x:v>
+      </x:c>
+      <x:c r="L30" s="22" t="n">
+        <x:v>0.709</x:v>
+      </x:c>
       <x:c r="M30" s="22"/>
       <x:c r="N30" s="10" t="str">
-        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.62x passes.</x:v>
+        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="10" t="str">
-        <x:v>2026-08-25 19:54</x:v>
+        <x:v>2026-08-25 19:43</x:v>
       </x:c>
       <x:c r="B31" s="10" t="str">
         <x:v>C++</x:v>
@@ -20922,7 +20930,7 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D31" s="10" t="str">
-        <x:v>ROUTER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E31" s="10" t="str">
         <x:v>tls</x:v>
@@ -20931,26 +20939,24 @@
         <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G31" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H31" s="10" t="str">
-        <x:v>Use Core normal route selection instead of the initially selected exact transport target.</x:v>
+        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
       </x:c>
       <x:c r="I31" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J31" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
       </x:c>
       <x:c r="K31" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
-      </x:c>
-      <x:c r="L31" s="22" t="n">
-        <x:v>0.714</x:v>
-      </x:c>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L31" s="22"/>
       <x:c r="M31" s="22"/>
       <x:c r="N31" s="10" t="str">
-        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership; exact-request-target contract remains required.</x:v>
+        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.62x passes.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -20973,29 +20979,31 @@
         <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G32" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H32" s="10" t="str">
-        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
+        <x:v>Use Core normal route selection instead of the initially selected exact transport target.</x:v>
       </x:c>
       <x:c r="I32" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J32" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K32" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
-      </x:c>
-      <x:c r="L32" s="22"/>
+        <x:v>N/A — exact-target contract no-go</x:v>
+      </x:c>
+      <x:c r="L32" s="22" t="n">
+        <x:v>0.714</x:v>
+      </x:c>
       <x:c r="M32" s="22"/>
       <x:c r="N32" s="10" t="str">
-        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.65x passes.</x:v>
+        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership; exact-request-target contract remains required.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="10" t="str">
-        <x:v>2026-08-25 20:08</x:v>
+        <x:v>2026-08-25 19:54</x:v>
       </x:c>
       <x:c r="B33" s="10" t="str">
         <x:v>C++</x:v>
@@ -21004,35 +21012,33 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D33" s="10" t="str">
-        <x:v>PAIR</x:v>
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E33" s="10" t="str">
-        <x:v>inproc</x:v>
+        <x:v>tls</x:v>
       </x:c>
       <x:c r="F33" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G33" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H33" s="10" t="str">
-        <x:v>Re-evaluate retained 128KiB–1MiB bounded pool and process-lifetime singleton.</x:v>
+        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
       </x:c>
       <x:c r="I33" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J33" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
       </x:c>
       <x:c r="K33" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
-      </x:c>
-      <x:c r="L33" s="22" t="n">
-        <x:v>0.761</x:v>
-      </x:c>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L33" s="22"/>
       <x:c r="M33" s="22"/>
       <x:c r="N33" s="10" t="str">
-        <x:v>NO-GO as a new A/B: safe bounded-pool lifecycle is already in source, including late Core-release safety.</x:v>
+        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.65x passes.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -21055,10 +21061,10 @@
         <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
       </x:c>
       <x:c r="G34" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H34" s="10" t="str">
-        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
+        <x:v>Re-evaluate retained 128KiB–1MiB bounded pool and process-lifetime singleton.</x:v>
       </x:c>
       <x:c r="I34" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
@@ -21067,19 +21073,19 @@
         <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K34" s="10" t="str">
-        <x:v>N/A — timeout/resource no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L34" s="22" t="n">
         <x:v>0.761</x:v>
       </x:c>
       <x:c r="M34" s="22"/>
       <x:c r="N34" s="10" t="str">
-        <x:v>NO-GO: the 64KiB global threshold previously yielded a 25/30 partial TCP report through timeout; raising the cap changes the documented resource boundary. Per-transport policy would make ownership/resource behavior inconsistent.</x:v>
+        <x:v>NO-GO as a new A/B: safe bounded-pool lifecycle is already in source, including late Core-release safety.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="10" t="str">
-        <x:v>2026-08-25 20:17</x:v>
+        <x:v>2026-08-25 20:08</x:v>
       </x:c>
       <x:c r="B35" s="10" t="str">
         <x:v>C++</x:v>
@@ -21088,35 +21094,35 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D35" s="10" t="str">
-        <x:v>PUBSUB</x:v>
+        <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E35" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F35" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
       </x:c>
       <x:c r="G35" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H35" s="10" t="str">
-        <x:v>Re-evaluate direct single-part publish and the retained 128KiB–1MiB bounded pool.</x:v>
+        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
       </x:c>
       <x:c r="I35" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J35" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K35" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — timeout/resource no-go</x:v>
       </x:c>
       <x:c r="L35" s="22" t="n">
-        <x:v>0.787</x:v>
+        <x:v>0.761</x:v>
       </x:c>
       <x:c r="M35" s="22"/>
       <x:c r="N35" s="10" t="str">
-        <x:v>NO-GO as a new A/B: direct publish and safe bounded-pool lifecycle already form the measured hot path.</x:v>
+        <x:v>NO-GO: the 64KiB global threshold previously yielded a 25/30 partial TCP report through timeout; raising the cap changes the documented resource boundary. Per-transport policy would make ownership/resource behavior inconsistent.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -21139,10 +21145,10 @@
         <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
       </x:c>
       <x:c r="G36" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H36" s="10" t="str">
-        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
+        <x:v>Re-evaluate direct single-part publish and the retained 128KiB–1MiB bounded pool.</x:v>
       </x:c>
       <x:c r="I36" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
@@ -21151,19 +21157,19 @@
         <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K36" s="10" t="str">
-        <x:v>N/A — timeout/resource no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L36" s="22" t="n">
         <x:v>0.787</x:v>
       </x:c>
       <x:c r="M36" s="22"/>
       <x:c r="N36" s="10" t="str">
-        <x:v>NO-GO: 64KiB global threshold has prior 25/30 TCP partial timeout; cap expansion changes resource policy. Transport-specific policy is not an acceptable lifecycle split.</x:v>
+        <x:v>NO-GO as a new A/B: direct publish and safe bounded-pool lifecycle already form the measured hot path.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="10" t="str">
-        <x:v>2026-08-25 20:22</x:v>
+        <x:v>2026-08-25 20:17</x:v>
       </x:c>
       <x:c r="B37" s="10" t="str">
         <x:v>C++</x:v>
@@ -21172,35 +21178,35 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D37" s="10" t="str">
-        <x:v>DEALER_DEALER</x:v>
+        <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E37" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F37" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
       </x:c>
       <x:c r="G37" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H37" s="10" t="str">
-        <x:v>Re-evaluate bounded pool and operation-state reuse in the routed one-way hot path.</x:v>
+        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
       </x:c>
       <x:c r="I37" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J37" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K37" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — timeout/resource no-go</x:v>
       </x:c>
       <x:c r="L37" s="22" t="n">
-        <x:v>0.705</x:v>
+        <x:v>0.787</x:v>
       </x:c>
       <x:c r="M37" s="22"/>
       <x:c r="N37" s="10" t="str">
-        <x:v>NO-GO as a new A/B: the measured path already has the safe pool/state lifecycle.</x:v>
+        <x:v>NO-GO: 64KiB global threshold has prior 25/30 TCP partial timeout; cap expansion changes resource policy. Transport-specific policy is not an acceptable lifecycle split.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -21223,10 +21229,10 @@
         <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
       </x:c>
       <x:c r="G38" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H38" s="10" t="str">
-        <x:v>Lower global pool threshold, raise cap, or remove lifetime guard.</x:v>
+        <x:v>Re-evaluate bounded pool and operation-state reuse in the routed one-way hot path.</x:v>
       </x:c>
       <x:c r="I38" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
@@ -21235,19 +21241,19 @@
         <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K38" s="10" t="str">
-        <x:v>N/A — timeout/contract/resource no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L38" s="22" t="n">
         <x:v>0.705</x:v>
       </x:c>
       <x:c r="M38" s="22"/>
       <x:c r="N38" s="10" t="str">
-        <x:v>NO-GO: 64KiB pool threshold has a prior TCP partial timeout; cap and guard changes weaken resource or close/concurrency guarantees.</x:v>
+        <x:v>NO-GO as a new A/B: the measured path already has the safe pool/state lifecycle.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="10" t="str">
-        <x:v>2026-08-25 20:29</x:v>
+        <x:v>2026-08-25 20:22</x:v>
       </x:c>
       <x:c r="B39" s="10" t="str">
         <x:v>C++</x:v>
@@ -21256,35 +21262,35 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D39" s="10" t="str">
-        <x:v>DEALER_ROUTER</x:v>
+        <x:v>DEALER_DEALER</x:v>
       </x:c>
       <x:c r="E39" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F39" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
       </x:c>
       <x:c r="G39" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H39" s="10" t="str">
-        <x:v>Re-evaluate bounded pool and routed operation-state reuse.</x:v>
+        <x:v>Lower global pool threshold, raise cap, or remove lifetime guard.</x:v>
       </x:c>
       <x:c r="I39" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J39" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K39" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — timeout/contract/resource no-go</x:v>
       </x:c>
       <x:c r="L39" s="22" t="n">
-        <x:v>0.71</x:v>
+        <x:v>0.705</x:v>
       </x:c>
       <x:c r="M39" s="22"/>
       <x:c r="N39" s="10" t="str">
-        <x:v>NO-GO as a new A/B: the safe bounded-pool/state path is already measured.</x:v>
+        <x:v>NO-GO: 64KiB pool threshold has a prior TCP partial timeout; cap and guard changes weaken resource or close/concurrency guarantees.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -21307,10 +21313,10 @@
         <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
       </x:c>
       <x:c r="G40" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H40" s="10" t="str">
-        <x:v>Add route cache or remove attempt/lifetime guards.</x:v>
+        <x:v>Re-evaluate bounded pool and routed operation-state reuse.</x:v>
       </x:c>
       <x:c r="I40" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
@@ -21319,19 +21325,19 @@
         <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K40" s="10" t="str">
-        <x:v>N/A — exact-route/close no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L40" s="22" t="n">
         <x:v>0.71</x:v>
       </x:c>
       <x:c r="M40" s="22"/>
       <x:c r="N40" s="10" t="str">
-        <x:v>NO-GO: route caching and guard removal change exact route selection or close/concurrency responsibility.</x:v>
+        <x:v>NO-GO as a new A/B: the safe bounded-pool/state path is already measured.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="10" t="str">
-        <x:v>2026-08-25 20:34</x:v>
+        <x:v>2026-08-25 20:29</x:v>
       </x:c>
       <x:c r="B41" s="10" t="str">
         <x:v>C++</x:v>
@@ -21340,35 +21346,35 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D41" s="10" t="str">
-        <x:v>DEALER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_ROUTER</x:v>
       </x:c>
       <x:c r="E41" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F41" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
       </x:c>
       <x:c r="G41" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H41" s="10" t="str">
-        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
+        <x:v>Add route cache or remove attempt/lifetime guards.</x:v>
       </x:c>
       <x:c r="I41" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J41" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K41" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
+        <x:v>N/A — exact-route/close no-go</x:v>
       </x:c>
       <x:c r="L41" s="22" t="n">
-        <x:v>0.429</x:v>
+        <x:v>0.71</x:v>
       </x:c>
       <x:c r="M41" s="22"/>
       <x:c r="N41" s="10" t="str">
-        <x:v>NO-GO: fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
+        <x:v>NO-GO: route caching and guard removal change exact route selection or close/concurrency responsibility.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -21391,10 +21397,10 @@
         <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G42" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H42" s="10" t="str">
-        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
+        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
       </x:c>
       <x:c r="I42" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
@@ -21403,19 +21409,19 @@
         <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K42" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — exact-target contract no-go</x:v>
       </x:c>
       <x:c r="L42" s="22" t="n">
         <x:v>0.429</x:v>
       </x:c>
       <x:c r="M42" s="22"/>
       <x:c r="N42" s="10" t="str">
-        <x:v>KEEP baseline: new single lvalue submit-failure test plus request/reply, target, message, socket, behavior suites pass 5/5. No transport A/B delta is claimed.</x:v>
+        <x:v>NO-GO: fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="10" t="str">
-        <x:v>2026-08-25 20:40</x:v>
+        <x:v>2026-08-25 20:34</x:v>
       </x:c>
       <x:c r="B43" s="10" t="str">
         <x:v>C++</x:v>
@@ -21424,35 +21430,35 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D43" s="10" t="str">
-        <x:v>ROUTER_ROUTER</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E43" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F43" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G43" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H43" s="10" t="str">
-        <x:v>Re-evaluate bounded pool and state reuse on the exact routed path.</x:v>
+        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
       </x:c>
       <x:c r="I43" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J43" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K43" s="10" t="str">
         <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L43" s="22" t="n">
-        <x:v>0.699</x:v>
+        <x:v>0.429</x:v>
       </x:c>
       <x:c r="M43" s="22"/>
       <x:c r="N43" s="10" t="str">
-        <x:v>NO-GO as a new A/B: safe pool/state reuse already forms the measured path.</x:v>
+        <x:v>KEEP baseline: new single lvalue submit-failure test plus request/reply, target, message, socket, behavior suites pass 5/5. No transport A/B delta is claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -21475,10 +21481,10 @@
         <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
       </x:c>
       <x:c r="G44" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H44" s="10" t="str">
-        <x:v>Add route cache, lower pool threshold, or remove lifetime guard.</x:v>
+        <x:v>Re-evaluate bounded pool and state reuse on the exact routed path.</x:v>
       </x:c>
       <x:c r="I44" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
@@ -21487,19 +21493,19 @@
         <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K44" s="10" t="str">
-        <x:v>N/A — contract/resource no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L44" s="22" t="n">
         <x:v>0.699</x:v>
       </x:c>
       <x:c r="M44" s="22"/>
       <x:c r="N44" s="10" t="str">
-        <x:v>NO-GO: target cache and guard removal weaken exact-route/close semantics; pool changes have prior timeout/resource-boundary evidence.</x:v>
+        <x:v>NO-GO as a new A/B: safe pool/state reuse already forms the measured path.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="10" t="str">
-        <x:v>2026-08-25 20:46</x:v>
+        <x:v>2026-08-25 20:40</x:v>
       </x:c>
       <x:c r="B45" s="10" t="str">
         <x:v>C++</x:v>
@@ -21508,35 +21514,35 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D45" s="10" t="str">
-        <x:v>ROUTER_ROUTER_REQREP</x:v>
+        <x:v>ROUTER_ROUTER</x:v>
       </x:c>
       <x:c r="E45" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F45" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
       </x:c>
       <x:c r="G45" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H45" s="10" t="str">
-        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
+        <x:v>Add route cache, lower pool threshold, or remove lifetime guard.</x:v>
       </x:c>
       <x:c r="I45" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J45" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K45" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
+        <x:v>N/A — contract/resource no-go</x:v>
       </x:c>
       <x:c r="L45" s="22" t="n">
-        <x:v>0.441</x:v>
+        <x:v>0.699</x:v>
       </x:c>
       <x:c r="M45" s="22"/>
       <x:c r="N45" s="10" t="str">
-        <x:v>NO-GO: target fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
+        <x:v>NO-GO: target cache and guard removal weaken exact-route/close semantics; pool changes have prior timeout/resource-boundary evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -21559,10 +21565,10 @@
         <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G46" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H46" s="10" t="str">
-        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
+        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
       </x:c>
       <x:c r="I46" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
@@ -21571,31 +21577,57 @@
         <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K46" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — exact-target contract no-go</x:v>
       </x:c>
       <x:c r="L46" s="22" t="n">
         <x:v>0.441</x:v>
       </x:c>
       <x:c r="M46" s="22"/>
       <x:c r="N46" s="10" t="str">
+        <x:v>NO-GO: target fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="10" t="str">
+        <x:v>2026-08-25 20:46</x:v>
+      </x:c>
+      <x:c r="B47" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C47" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D47" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E47" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F47" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G47" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H47" s="10" t="str">
+        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
+      </x:c>
+      <x:c r="I47" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J47" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K47" s="10" t="str">
+        <x:v>N/A — already baseline</x:v>
+      </x:c>
+      <x:c r="L47" s="22" t="n">
+        <x:v>0.441</x:v>
+      </x:c>
+      <x:c r="M47" s="22"/>
+      <x:c r="N47" s="10" t="str">
         <x:v>KEEP baseline: new single lvalue submit-failure test plus request/reply, target, message, socket, behavior suites pass 5/5. No transport A/B delta is claimed.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="10"/>
-      <x:c r="B47" s="10"/>
-      <x:c r="C47" s="10"/>
-      <x:c r="D47" s="10"/>
-      <x:c r="E47" s="10"/>
-      <x:c r="F47" s="10"/>
-      <x:c r="G47" s="10"/>
-      <x:c r="H47" s="10"/>
-      <x:c r="I47" s="10"/>
-      <x:c r="J47" s="10"/>
-      <x:c r="K47" s="10"/>
-      <x:c r="L47" s="22"/>
-      <x:c r="M47" s="22"/>
-      <x:c r="N47" s="10"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="10"/>

</xml_diff>

<commit_message>
docs(perf): record tls pubsub reviewer hold
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R59cb193800c54f56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rcb1e614c16de4ccb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rbe095e77c0c6404a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R1e19c92018244c1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra4def66dd96e4f3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rca12694981bf40e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R122734dc08a24138"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R87815ee0815845d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,7 +520,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 보류, tls 3개 통과·3개 미달·1개 보류, inproc 0개 통과·7개 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 보류, tls 3개 통과·2개 미달·2개 보류, inproc 0개 통과·7개 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -567,7 +567,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -582,7 +582,7 @@
       </x:c>
       <x:c r="B14" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"보류",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C14" s="17" t="str">
         <x:v>Sol-reviewed safe candidates are exhausted; target still missed</x:v>
@@ -12916,24 +12916,24 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="G178" s="26" t="n">
-        <x:v>1346233.4</x:v>
+        <x:v>1332628</x:v>
       </x:c>
       <x:c r="H178" s="26" t="n">
-        <x:v>1187729.8</x:v>
+        <x:v>1173956.4</x:v>
       </x:c>
       <x:c r="I178" s="22" t="n">
         <x:f>H178/G178</x:f>
-        <x:v>0.8822614265847216</x:v>
+        <x:v>0.8809333137229594</x:v>
       </x:c>
       <x:c r="J178" s="24" t="n">
-        <x:v>0.206</x:v>
+        <x:v>0.203</x:v>
       </x:c>
       <x:c r="K178" s="24" t="n">
-        <x:v>0.243</x:v>
+        <x:v>0.21</x:v>
       </x:c>
       <x:c r="L178" s="24" t="n">
         <x:f>K178/J178</x:f>
-        <x:v>1.179611650485437</x:v>
+        <x:v>1.0344827586206895</x:v>
       </x:c>
       <x:c r="M178" s="10" t="n">
         <x:v>5</x:v>
@@ -12951,19 +12951,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R178" s="10" t="str">
-        <x:v>0babb638e9</x:v>
+        <x:v>2f9cc20ce2</x:v>
       </x:c>
       <x:c r="S178" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_191206_cpp-pubsub-tls-local0132-final5-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_232737_cpp-pubsub-tls-local0132-final-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T178" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_233109_cpp-pubsub-tls-local0132-final-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U178" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V178" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 92.13%; latency median ratio 1.11x; strict gate fail. Existing direct single-part publish and bounded-pool path are baseline; guard removal/pool expansion is no-go.</x:v>
+        <x:v>Clean-source secure final pair: throughput aggregate mean 90.45%; latency median ratio 1.09x; strict 95% throughput gate only fails. Sol approved hold after C1/C2/C3 rejects.</x:v>
       </x:c>
     </x:row>
     <x:row r="179">
@@ -12986,24 +12986,24 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="G179" s="26" t="n">
-        <x:v>698794</x:v>
+        <x:v>775691</x:v>
       </x:c>
       <x:c r="H179" s="26" t="n">
-        <x:v>717099</x:v>
+        <x:v>741002.8</x:v>
       </x:c>
       <x:c r="I179" s="22" t="n">
         <x:f>H179/G179</x:f>
-        <x:v>1.0261951304676342</x:v>
+        <x:v>0.9552809043807393</x:v>
       </x:c>
       <x:c r="J179" s="24" t="n">
-        <x:v>2.028</x:v>
+        <x:v>1.835</x:v>
       </x:c>
       <x:c r="K179" s="24" t="n">
-        <x:v>1.991</x:v>
+        <x:v>1.964</x:v>
       </x:c>
       <x:c r="L179" s="24" t="n">
         <x:f>K179/J179</x:f>
-        <x:v>0.9817554240631164</x:v>
+        <x:v>1.070299727520436</x:v>
       </x:c>
       <x:c r="M179" s="10" t="n">
         <x:v>5</x:v>
@@ -13021,19 +13021,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R179" s="10" t="str">
-        <x:v>0babb638e9</x:v>
+        <x:v>2f9cc20ce2</x:v>
       </x:c>
       <x:c r="S179" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_191206_cpp-pubsub-tls-local0132-final5-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_232737_cpp-pubsub-tls-local0132-final-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T179" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_233109_cpp-pubsub-tls-local0132-final-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U179" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V179" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 92.13%; latency median ratio 1.11x; strict gate fail. Existing direct single-part publish and bounded-pool path are baseline; guard removal/pool expansion is no-go.</x:v>
+        <x:v>Clean-source secure final pair: throughput aggregate mean 90.45%; latency median ratio 1.09x; strict 95% throughput gate only fails. Sol approved hold after C1/C2/C3 rejects.</x:v>
       </x:c>
     </x:row>
     <x:row r="180">
@@ -13056,24 +13056,24 @@
         <x:v>1024</x:v>
       </x:c>
       <x:c r="G180" s="26" t="n">
-        <x:v>285636.2</x:v>
+        <x:v>295723.6</x:v>
       </x:c>
       <x:c r="H180" s="26" t="n">
-        <x:v>271089.8</x:v>
+        <x:v>278069</x:v>
       </x:c>
       <x:c r="I180" s="22" t="n">
         <x:f>H180/G180</x:f>
-        <x:v>0.949073681837246</x:v>
+        <x:v>0.9403003345015414</x:v>
       </x:c>
       <x:c r="J180" s="24" t="n">
-        <x:v>1.62</x:v>
+        <x:v>1.572</x:v>
       </x:c>
       <x:c r="K180" s="24" t="n">
-        <x:v>1.704</x:v>
+        <x:v>1.702</x:v>
       </x:c>
       <x:c r="L180" s="24" t="n">
         <x:f>K180/J180</x:f>
-        <x:v>1.0518518518518518</x:v>
+        <x:v>1.0826972010178115</x:v>
       </x:c>
       <x:c r="M180" s="10" t="n">
         <x:v>5</x:v>
@@ -13091,19 +13091,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R180" s="10" t="str">
-        <x:v>0babb638e9</x:v>
+        <x:v>2f9cc20ce2</x:v>
       </x:c>
       <x:c r="S180" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_191206_cpp-pubsub-tls-local0132-final5-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_232737_cpp-pubsub-tls-local0132-final-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T180" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_233109_cpp-pubsub-tls-local0132-final-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U180" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V180" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 92.13%; latency median ratio 1.11x; strict gate fail. Existing direct single-part publish and bounded-pool path are baseline; guard removal/pool expansion is no-go.</x:v>
+        <x:v>Clean-source secure final pair: throughput aggregate mean 90.45%; latency median ratio 1.09x; strict 95% throughput gate only fails. Sol approved hold after C1/C2/C3 rejects.</x:v>
       </x:c>
     </x:row>
     <x:row r="181">
@@ -13126,24 +13126,24 @@
         <x:v>65536</x:v>
       </x:c>
       <x:c r="G181" s="26" t="n">
-        <x:v>11337.2</x:v>
+        <x:v>12096</x:v>
       </x:c>
       <x:c r="H181" s="26" t="n">
-        <x:v>9903.2</x:v>
+        <x:v>10764.6</x:v>
       </x:c>
       <x:c r="I181" s="22" t="n">
         <x:f>H181/G181</x:f>
-        <x:v>0.8735137423702501</x:v>
+        <x:v>0.8899305555555556</x:v>
       </x:c>
       <x:c r="J181" s="24" t="n">
-        <x:v>0.869</x:v>
+        <x:v>0.82</x:v>
       </x:c>
       <x:c r="K181" s="24" t="n">
-        <x:v>1.006</x:v>
+        <x:v>0.909</x:v>
       </x:c>
       <x:c r="L181" s="24" t="n">
         <x:f>K181/J181</x:f>
-        <x:v>1.1576524741081704</x:v>
+        <x:v>1.1085365853658538</x:v>
       </x:c>
       <x:c r="M181" s="10" t="n">
         <x:v>5</x:v>
@@ -13161,19 +13161,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R181" s="10" t="str">
-        <x:v>0babb638e9</x:v>
+        <x:v>2f9cc20ce2</x:v>
       </x:c>
       <x:c r="S181" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_191206_cpp-pubsub-tls-local0132-final5-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_232737_cpp-pubsub-tls-local0132-final-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T181" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_233109_cpp-pubsub-tls-local0132-final-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U181" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V181" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 92.13%; latency median ratio 1.11x; strict gate fail. Existing direct single-part publish and bounded-pool path are baseline; guard removal/pool expansion is no-go.</x:v>
+        <x:v>Clean-source secure final pair: throughput aggregate mean 90.45%; latency median ratio 1.09x; strict 95% throughput gate only fails. Sol approved hold after C1/C2/C3 rejects.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -13196,24 +13196,24 @@
         <x:v>131072</x:v>
       </x:c>
       <x:c r="G182" s="26" t="n">
-        <x:v>6956.8</x:v>
+        <x:v>7092</x:v>
       </x:c>
       <x:c r="H182" s="26" t="n">
-        <x:v>5694</x:v>
+        <x:v>6309.2</x:v>
       </x:c>
       <x:c r="I182" s="22" t="n">
         <x:f>H182/G182</x:f>
-        <x:v>0.8184797608095676</x:v>
+        <x:v>0.8896221094190637</x:v>
       </x:c>
       <x:c r="J182" s="24" t="n">
-        <x:v>0.843</x:v>
+        <x:v>0.838</x:v>
       </x:c>
       <x:c r="K182" s="24" t="n">
-        <x:v>1.031</x:v>
+        <x:v>0.923</x:v>
       </x:c>
       <x:c r="L182" s="24" t="n">
         <x:f>K182/J182</x:f>
-        <x:v>1.2230130486358244</x:v>
+        <x:v>1.1014319809069213</x:v>
       </x:c>
       <x:c r="M182" s="10" t="n">
         <x:v>5</x:v>
@@ -13231,19 +13231,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R182" s="10" t="str">
-        <x:v>0babb638e9</x:v>
+        <x:v>2f9cc20ce2</x:v>
       </x:c>
       <x:c r="S182" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_191206_cpp-pubsub-tls-local0132-final5-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_232737_cpp-pubsub-tls-local0132-final-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T182" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_233109_cpp-pubsub-tls-local0132-final-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U182" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V182" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 92.13%; latency median ratio 1.11x; strict gate fail. Existing direct single-part publish and bounded-pool path are baseline; guard removal/pool expansion is no-go.</x:v>
+        <x:v>Clean-source secure final pair: throughput aggregate mean 90.45%; latency median ratio 1.09x; strict 95% throughput gate only fails. Sol approved hold after C1/C2/C3 rejects.</x:v>
       </x:c>
     </x:row>
     <x:row r="183">
@@ -13266,24 +13266,24 @@
         <x:v>262144</x:v>
       </x:c>
       <x:c r="G183" s="26" t="n">
-        <x:v>3739.6</x:v>
+        <x:v>3912</x:v>
       </x:c>
       <x:c r="H183" s="26" t="n">
-        <x:v>3658.4</x:v>
+        <x:v>3407.8</x:v>
       </x:c>
       <x:c r="I183" s="22" t="n">
         <x:f>H183/G183</x:f>
-        <x:v>0.9782864477484223</x:v>
+        <x:v>0.8711145194274029</x:v>
       </x:c>
       <x:c r="J183" s="24" t="n">
-        <x:v>1.064</x:v>
+        <x:v>1.003</x:v>
       </x:c>
       <x:c r="K183" s="24" t="n">
-        <x:v>1.081</x:v>
+        <x:v>1.151</x:v>
       </x:c>
       <x:c r="L183" s="24" t="n">
         <x:f>K183/J183</x:f>
-        <x:v>1.0159774436090225</x:v>
+        <x:v>1.1475573280159523</x:v>
       </x:c>
       <x:c r="M183" s="10" t="n">
         <x:v>5</x:v>
@@ -13301,19 +13301,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R183" s="10" t="str">
-        <x:v>0babb638e9</x:v>
+        <x:v>2f9cc20ce2</x:v>
       </x:c>
       <x:c r="S183" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_191206_cpp-pubsub-tls-local0132-final5-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_232737_cpp-pubsub-tls-local0132-final-clean-paired5-c-20260825.txt</x:v>
       </x:c>
       <x:c r="T183" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_233109_cpp-pubsub-tls-local0132-final-clean-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="U183" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V183" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 92.13%; latency median ratio 1.11x; strict gate fail. Existing direct single-part publish and bounded-pool path are baseline; guard removal/pool expansion is no-go.</x:v>
+        <x:v>Clean-source secure final pair: throughput aggregate mean 90.45%; latency median ratio 1.09x; strict 95% throughput gate only fails. Sol approved hold after C1/C2/C3 rejects.</x:v>
       </x:c>
     </x:row>
     <x:row r="184">
@@ -20795,7 +20795,7 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="10" t="str">
-        <x:v>2026-08-25 19:18</x:v>
+        <x:v>2026-08-25 23:01</x:v>
       </x:c>
       <x:c r="B28" s="10" t="str">
         <x:v>C++</x:v>
@@ -20813,10 +20813,10 @@
         <x:v>Throughput aggregate &lt; 95%</x:v>
       </x:c>
       <x:c r="G28" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>C1</x:v>
       </x:c>
       <x:c r="H28" s="10" t="str">
-        <x:v>Re-evaluate direct single-part publish and operation-state reuse.</x:v>
+        <x:v>Receive topic_message parts directly in message_t native storage, removing temporary native init/adopt handoff.</x:v>
       </x:c>
       <x:c r="I28" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
@@ -20825,19 +20825,21 @@
         <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K28" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_230146_cpp-pubsub-tls-local0132-candidate-direct-receive-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="L28" s="22" t="n">
         <x:v>0.921</x:v>
       </x:c>
-      <x:c r="M28" s="22"/>
+      <x:c r="M28" s="22" t="n">
+        <x:v>0.909</x:v>
+      </x:c>
       <x:c r="N28" s="10" t="str">
-        <x:v>NO-GO as a new A/B: the benchmark already uses the direct single-part publish path; multipart staging is not on this hot path.</x:v>
+        <x:v>REJECT: contract tests pass but full paired aggregate regresses to 90.86%; source reverted.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="10" t="str">
-        <x:v>2026-08-25 19:18</x:v>
+        <x:v>2026-08-25 23:10</x:v>
       </x:c>
       <x:c r="B29" s="10" t="str">
         <x:v>C++</x:v>
@@ -20855,31 +20857,33 @@
         <x:v>Throughput aggregate &lt; 95%</x:v>
       </x:c>
       <x:c r="G29" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>C2</x:v>
       </x:c>
       <x:c r="H29" s="10" t="str">
-        <x:v>Remove attempt mutex/lifetime guard, lower pool threshold, or expand pool cap.</x:v>
+        <x:v>Materialize known single received part directly in topic_message_t retained vector.</x:v>
       </x:c>
       <x:c r="I29" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J29" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_191532_cpp-pubsub-tls-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_230146_cpp-pubsub-tls-local0132-candidate-direct-receive-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K29" s="10" t="str">
-        <x:v>N/A — contract/resource no-go</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_231020_cpp-pubsub-tls-local0132-candidate-materialized-single-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="L29" s="22" t="n">
+        <x:v>0.909</x:v>
+      </x:c>
+      <x:c r="M29" s="22" t="n">
         <x:v>0.921</x:v>
       </x:c>
-      <x:c r="M29" s="22"/>
       <x:c r="N29" s="10" t="str">
-        <x:v>NO-GO: guard removal changes close/concurrency semantics; pool lower-bound/cap changes are global policy with a prior timeout or wider resource boundary.</x:v>
+        <x:v>REJECT: 92.10% is baseline-level measurement variance, not an additive improvement; source reverted.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="10" t="str">
-        <x:v>2026-08-25 19:43</x:v>
+        <x:v>2026-08-25 23:20</x:v>
       </x:c>
       <x:c r="B30" s="10" t="str">
         <x:v>C++</x:v>
@@ -20888,40 +20892,42 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D30" s="10" t="str">
-        <x:v>DEALER_ROUTER_REQREP</x:v>
+        <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E30" s="10" t="str">
         <x:v>tls</x:v>
       </x:c>
       <x:c r="F30" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Throughput aggregate &lt; 95%</x:v>
       </x:c>
       <x:c r="G30" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>C3</x:v>
       </x:c>
       <x:c r="H30" s="10" t="str">
-        <x:v>Use Core normal DEALER request route instead of initially selected exact transport target.</x:v>
+        <x:v>Globally bypass 128KiB–1MiB large-message pool; use native allocation.</x:v>
       </x:c>
       <x:c r="I30" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J30" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_231020_cpp-pubsub-tls-local0132-candidate-materialized-single-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K30" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_232027_cpp-pubsub-tls-local0132-candidate-full-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="L30" s="22" t="n">
-        <x:v>0.709</x:v>
-      </x:c>
-      <x:c r="M30" s="22"/>
+        <x:v>0.921</x:v>
+      </x:c>
+      <x:c r="M30" s="22" t="n">
+        <x:v>0.931</x:v>
+      </x:c>
       <x:c r="N30" s="10" t="str">
-        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership.</x:v>
+        <x:v>REJECT: TLS full pair 93.07%, but required inproc 128KiB regression is 80.65% (112481.8→90718.2 Kmsg/s); global policy cannot be TLS-only. Source reverted.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="10" t="str">
-        <x:v>2026-08-25 19:43</x:v>
+        <x:v>2026-08-25 23:31</x:v>
       </x:c>
       <x:c r="B31" s="10" t="str">
         <x:v>C++</x:v>
@@ -20930,38 +20936,42 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D31" s="10" t="str">
-        <x:v>DEALER_ROUTER_REQREP</x:v>
+        <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E31" s="10" t="str">
         <x:v>tls</x:v>
       </x:c>
       <x:c r="F31" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Throughput aggregate &lt; 95%</x:v>
       </x:c>
       <x:c r="G31" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>Sol review</x:v>
       </x:c>
       <x:c r="H31" s="10" t="str">
-        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
+        <x:v>Review C1/C2/C3 and remaining non-spec-gap space after clean-source final pair.</x:v>
       </x:c>
       <x:c r="I31" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J31" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_232027_cpp-pubsub-tls-local0132-candidate-full-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K31" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
-      </x:c>
-      <x:c r="L31" s="22"/>
-      <x:c r="M31" s="22"/>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_233109_cpp-pubsub-tls-local0132-final-clean-paired5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L31" s="22" t="n">
+        <x:v>0.931</x:v>
+      </x:c>
+      <x:c r="M31" s="22" t="n">
+        <x:v>0.905</x:v>
+      </x:c>
       <x:c r="N31" s="10" t="str">
-        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.62x passes.</x:v>
+        <x:v>SOL APPROVED: all candidates rejected; no safe contract-preserving candidate remains. Clean final 90.45%, latency 1.09x; 보류.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="10" t="str">
-        <x:v>2026-08-25 19:54</x:v>
+        <x:v>2026-08-25 19:43</x:v>
       </x:c>
       <x:c r="B32" s="10" t="str">
         <x:v>C++</x:v>
@@ -20970,7 +20980,7 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D32" s="10" t="str">
-        <x:v>ROUTER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E32" s="10" t="str">
         <x:v>tls</x:v>
@@ -20982,28 +20992,28 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="H32" s="10" t="str">
-        <x:v>Use Core normal route selection instead of the initially selected exact transport target.</x:v>
+        <x:v>Use Core normal DEALER request route instead of initially selected exact transport target.</x:v>
       </x:c>
       <x:c r="I32" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J32" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K32" s="10" t="str">
         <x:v>N/A — exact-target contract no-go</x:v>
       </x:c>
       <x:c r="L32" s="22" t="n">
-        <x:v>0.714</x:v>
+        <x:v>0.709</x:v>
       </x:c>
       <x:c r="M32" s="22"/>
       <x:c r="N32" s="10" t="str">
-        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership; exact-request-target contract remains required.</x:v>
+        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="10" t="str">
-        <x:v>2026-08-25 19:54</x:v>
+        <x:v>2026-08-25 19:43</x:v>
       </x:c>
       <x:c r="B33" s="10" t="str">
         <x:v>C++</x:v>
@@ -21012,7 +21022,7 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D33" s="10" t="str">
-        <x:v>ROUTER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E33" s="10" t="str">
         <x:v>tls</x:v>
@@ -21033,17 +21043,17 @@
         <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
       </x:c>
       <x:c r="K33" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="L33" s="22"/>
       <x:c r="M33" s="22"/>
       <x:c r="N33" s="10" t="str">
-        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.65x passes.</x:v>
+        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.62x passes.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="10" t="str">
-        <x:v>2026-08-25 20:08</x:v>
+        <x:v>2026-08-25 19:54</x:v>
       </x:c>
       <x:c r="B34" s="10" t="str">
         <x:v>C++</x:v>
@@ -21052,40 +21062,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D34" s="10" t="str">
-        <x:v>PAIR</x:v>
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E34" s="10" t="str">
-        <x:v>inproc</x:v>
+        <x:v>tls</x:v>
       </x:c>
       <x:c r="F34" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G34" s="10" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="H34" s="10" t="str">
-        <x:v>Re-evaluate retained 128KiB–1MiB bounded pool and process-lifetime singleton.</x:v>
+        <x:v>Use Core normal route selection instead of the initially selected exact transport target.</x:v>
       </x:c>
       <x:c r="I34" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J34" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K34" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — exact-target contract no-go</x:v>
       </x:c>
       <x:c r="L34" s="22" t="n">
-        <x:v>0.761</x:v>
+        <x:v>0.714</x:v>
       </x:c>
       <x:c r="M34" s="22"/>
       <x:c r="N34" s="10" t="str">
-        <x:v>NO-GO as a new A/B: safe bounded-pool lifecycle is already in source, including late Core-release safety.</x:v>
+        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership; exact-request-target contract remains required.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="10" t="str">
-        <x:v>2026-08-25 20:08</x:v>
+        <x:v>2026-08-25 19:54</x:v>
       </x:c>
       <x:c r="B35" s="10" t="str">
         <x:v>C++</x:v>
@@ -21094,40 +21104,38 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D35" s="10" t="str">
-        <x:v>PAIR</x:v>
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E35" s="10" t="str">
-        <x:v>inproc</x:v>
+        <x:v>tls</x:v>
       </x:c>
       <x:c r="F35" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G35" s="10" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="H35" s="10" t="str">
-        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
+        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
       </x:c>
       <x:c r="I35" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J35" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
       </x:c>
       <x:c r="K35" s="10" t="str">
-        <x:v>N/A — timeout/resource no-go</x:v>
-      </x:c>
-      <x:c r="L35" s="22" t="n">
-        <x:v>0.761</x:v>
-      </x:c>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L35" s="22"/>
       <x:c r="M35" s="22"/>
       <x:c r="N35" s="10" t="str">
-        <x:v>NO-GO: the 64KiB global threshold previously yielded a 25/30 partial TCP report through timeout; raising the cap changes the documented resource boundary. Per-transport policy would make ownership/resource behavior inconsistent.</x:v>
+        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.65x passes.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="10" t="str">
-        <x:v>2026-08-25 20:17</x:v>
+        <x:v>2026-08-25 20:08</x:v>
       </x:c>
       <x:c r="B36" s="10" t="str">
         <x:v>C++</x:v>
@@ -21136,40 +21144,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D36" s="10" t="str">
-        <x:v>PUBSUB</x:v>
+        <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E36" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F36" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
       </x:c>
       <x:c r="G36" s="10" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="H36" s="10" t="str">
-        <x:v>Re-evaluate direct single-part publish and the retained 128KiB–1MiB bounded pool.</x:v>
+        <x:v>Re-evaluate retained 128KiB–1MiB bounded pool and process-lifetime singleton.</x:v>
       </x:c>
       <x:c r="I36" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J36" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K36" s="10" t="str">
         <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L36" s="22" t="n">
-        <x:v>0.787</x:v>
+        <x:v>0.761</x:v>
       </x:c>
       <x:c r="M36" s="22"/>
       <x:c r="N36" s="10" t="str">
-        <x:v>NO-GO as a new A/B: direct publish and safe bounded-pool lifecycle already form the measured hot path.</x:v>
+        <x:v>NO-GO as a new A/B: safe bounded-pool lifecycle is already in source, including late Core-release safety.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="10" t="str">
-        <x:v>2026-08-25 20:17</x:v>
+        <x:v>2026-08-25 20:08</x:v>
       </x:c>
       <x:c r="B37" s="10" t="str">
         <x:v>C++</x:v>
@@ -21178,13 +21186,13 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D37" s="10" t="str">
-        <x:v>PUBSUB</x:v>
+        <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E37" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F37" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
       </x:c>
       <x:c r="G37" s="10" t="str">
         <x:v>B</x:v>
@@ -21196,22 +21204,22 @@
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J37" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K37" s="10" t="str">
         <x:v>N/A — timeout/resource no-go</x:v>
       </x:c>
       <x:c r="L37" s="22" t="n">
-        <x:v>0.787</x:v>
+        <x:v>0.761</x:v>
       </x:c>
       <x:c r="M37" s="22"/>
       <x:c r="N37" s="10" t="str">
-        <x:v>NO-GO: 64KiB global threshold has prior 25/30 TCP partial timeout; cap expansion changes resource policy. Transport-specific policy is not an acceptable lifecycle split.</x:v>
+        <x:v>NO-GO: the 64KiB global threshold previously yielded a 25/30 partial TCP report through timeout; raising the cap changes the documented resource boundary. Per-transport policy would make ownership/resource behavior inconsistent.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="10" t="str">
-        <x:v>2026-08-25 20:22</x:v>
+        <x:v>2026-08-25 20:17</x:v>
       </x:c>
       <x:c r="B38" s="10" t="str">
         <x:v>C++</x:v>
@@ -21220,40 +21228,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D38" s="10" t="str">
-        <x:v>DEALER_DEALER</x:v>
+        <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E38" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F38" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
       </x:c>
       <x:c r="G38" s="10" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="H38" s="10" t="str">
-        <x:v>Re-evaluate bounded pool and operation-state reuse in the routed one-way hot path.</x:v>
+        <x:v>Re-evaluate direct single-part publish and the retained 128KiB–1MiB bounded pool.</x:v>
       </x:c>
       <x:c r="I38" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J38" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K38" s="10" t="str">
         <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L38" s="22" t="n">
-        <x:v>0.705</x:v>
+        <x:v>0.787</x:v>
       </x:c>
       <x:c r="M38" s="22"/>
       <x:c r="N38" s="10" t="str">
-        <x:v>NO-GO as a new A/B: the measured path already has the safe pool/state lifecycle.</x:v>
+        <x:v>NO-GO as a new A/B: direct publish and safe bounded-pool lifecycle already form the measured hot path.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="10" t="str">
-        <x:v>2026-08-25 20:22</x:v>
+        <x:v>2026-08-25 20:17</x:v>
       </x:c>
       <x:c r="B39" s="10" t="str">
         <x:v>C++</x:v>
@@ -21262,40 +21270,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D39" s="10" t="str">
-        <x:v>DEALER_DEALER</x:v>
+        <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E39" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F39" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
       </x:c>
       <x:c r="G39" s="10" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="H39" s="10" t="str">
-        <x:v>Lower global pool threshold, raise cap, or remove lifetime guard.</x:v>
+        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
       </x:c>
       <x:c r="I39" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J39" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K39" s="10" t="str">
-        <x:v>N/A — timeout/contract/resource no-go</x:v>
+        <x:v>N/A — timeout/resource no-go</x:v>
       </x:c>
       <x:c r="L39" s="22" t="n">
-        <x:v>0.705</x:v>
+        <x:v>0.787</x:v>
       </x:c>
       <x:c r="M39" s="22"/>
       <x:c r="N39" s="10" t="str">
-        <x:v>NO-GO: 64KiB pool threshold has a prior TCP partial timeout; cap and guard changes weaken resource or close/concurrency guarantees.</x:v>
+        <x:v>NO-GO: 64KiB global threshold has prior 25/30 TCP partial timeout; cap expansion changes resource policy. Transport-specific policy is not an acceptable lifecycle split.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="10" t="str">
-        <x:v>2026-08-25 20:29</x:v>
+        <x:v>2026-08-25 20:22</x:v>
       </x:c>
       <x:c r="B40" s="10" t="str">
         <x:v>C++</x:v>
@@ -21304,40 +21312,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D40" s="10" t="str">
-        <x:v>DEALER_ROUTER</x:v>
+        <x:v>DEALER_DEALER</x:v>
       </x:c>
       <x:c r="E40" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F40" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
       </x:c>
       <x:c r="G40" s="10" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="H40" s="10" t="str">
-        <x:v>Re-evaluate bounded pool and routed operation-state reuse.</x:v>
+        <x:v>Re-evaluate bounded pool and operation-state reuse in the routed one-way hot path.</x:v>
       </x:c>
       <x:c r="I40" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J40" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K40" s="10" t="str">
         <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L40" s="22" t="n">
-        <x:v>0.71</x:v>
+        <x:v>0.705</x:v>
       </x:c>
       <x:c r="M40" s="22"/>
       <x:c r="N40" s="10" t="str">
-        <x:v>NO-GO as a new A/B: the safe bounded-pool/state path is already measured.</x:v>
+        <x:v>NO-GO as a new A/B: the measured path already has the safe pool/state lifecycle.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="10" t="str">
-        <x:v>2026-08-25 20:29</x:v>
+        <x:v>2026-08-25 20:22</x:v>
       </x:c>
       <x:c r="B41" s="10" t="str">
         <x:v>C++</x:v>
@@ -21346,40 +21354,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D41" s="10" t="str">
-        <x:v>DEALER_ROUTER</x:v>
+        <x:v>DEALER_DEALER</x:v>
       </x:c>
       <x:c r="E41" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F41" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
       </x:c>
       <x:c r="G41" s="10" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="H41" s="10" t="str">
-        <x:v>Add route cache or remove attempt/lifetime guards.</x:v>
+        <x:v>Lower global pool threshold, raise cap, or remove lifetime guard.</x:v>
       </x:c>
       <x:c r="I41" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J41" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K41" s="10" t="str">
-        <x:v>N/A — exact-route/close no-go</x:v>
+        <x:v>N/A — timeout/contract/resource no-go</x:v>
       </x:c>
       <x:c r="L41" s="22" t="n">
-        <x:v>0.71</x:v>
+        <x:v>0.705</x:v>
       </x:c>
       <x:c r="M41" s="22"/>
       <x:c r="N41" s="10" t="str">
-        <x:v>NO-GO: route caching and guard removal change exact route selection or close/concurrency responsibility.</x:v>
+        <x:v>NO-GO: 64KiB pool threshold has a prior TCP partial timeout; cap and guard changes weaken resource or close/concurrency guarantees.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="10" t="str">
-        <x:v>2026-08-25 20:34</x:v>
+        <x:v>2026-08-25 20:29</x:v>
       </x:c>
       <x:c r="B42" s="10" t="str">
         <x:v>C++</x:v>
@@ -21388,40 +21396,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D42" s="10" t="str">
-        <x:v>DEALER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_ROUTER</x:v>
       </x:c>
       <x:c r="E42" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F42" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
       </x:c>
       <x:c r="G42" s="10" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="H42" s="10" t="str">
-        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
+        <x:v>Re-evaluate bounded pool and routed operation-state reuse.</x:v>
       </x:c>
       <x:c r="I42" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J42" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K42" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L42" s="22" t="n">
-        <x:v>0.429</x:v>
+        <x:v>0.71</x:v>
       </x:c>
       <x:c r="M42" s="22"/>
       <x:c r="N42" s="10" t="str">
-        <x:v>NO-GO: fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
+        <x:v>NO-GO as a new A/B: the safe bounded-pool/state path is already measured.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="10" t="str">
-        <x:v>2026-08-25 20:34</x:v>
+        <x:v>2026-08-25 20:29</x:v>
       </x:c>
       <x:c r="B43" s="10" t="str">
         <x:v>C++</x:v>
@@ -21430,40 +21438,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D43" s="10" t="str">
-        <x:v>DEALER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_ROUTER</x:v>
       </x:c>
       <x:c r="E43" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F43" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
       </x:c>
       <x:c r="G43" s="10" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="H43" s="10" t="str">
-        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
+        <x:v>Add route cache or remove attempt/lifetime guards.</x:v>
       </x:c>
       <x:c r="I43" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J43" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K43" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — exact-route/close no-go</x:v>
       </x:c>
       <x:c r="L43" s="22" t="n">
-        <x:v>0.429</x:v>
+        <x:v>0.71</x:v>
       </x:c>
       <x:c r="M43" s="22"/>
       <x:c r="N43" s="10" t="str">
-        <x:v>KEEP baseline: new single lvalue submit-failure test plus request/reply, target, message, socket, behavior suites pass 5/5. No transport A/B delta is claimed.</x:v>
+        <x:v>NO-GO: route caching and guard removal change exact route selection or close/concurrency responsibility.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="10" t="str">
-        <x:v>2026-08-25 20:40</x:v>
+        <x:v>2026-08-25 20:34</x:v>
       </x:c>
       <x:c r="B44" s="10" t="str">
         <x:v>C++</x:v>
@@ -21472,40 +21480,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D44" s="10" t="str">
-        <x:v>ROUTER_ROUTER</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E44" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F44" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G44" s="10" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="H44" s="10" t="str">
-        <x:v>Re-evaluate bounded pool and state reuse on the exact routed path.</x:v>
+        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
       </x:c>
       <x:c r="I44" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J44" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K44" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — exact-target contract no-go</x:v>
       </x:c>
       <x:c r="L44" s="22" t="n">
-        <x:v>0.699</x:v>
+        <x:v>0.429</x:v>
       </x:c>
       <x:c r="M44" s="22"/>
       <x:c r="N44" s="10" t="str">
-        <x:v>NO-GO as a new A/B: safe pool/state reuse already forms the measured path.</x:v>
+        <x:v>NO-GO: fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="10" t="str">
-        <x:v>2026-08-25 20:40</x:v>
+        <x:v>2026-08-25 20:34</x:v>
       </x:c>
       <x:c r="B45" s="10" t="str">
         <x:v>C++</x:v>
@@ -21514,40 +21522,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D45" s="10" t="str">
-        <x:v>ROUTER_ROUTER</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E45" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F45" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G45" s="10" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="H45" s="10" t="str">
-        <x:v>Add route cache, lower pool threshold, or remove lifetime guard.</x:v>
+        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
       </x:c>
       <x:c r="I45" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J45" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K45" s="10" t="str">
-        <x:v>N/A — contract/resource no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L45" s="22" t="n">
-        <x:v>0.699</x:v>
+        <x:v>0.429</x:v>
       </x:c>
       <x:c r="M45" s="22"/>
       <x:c r="N45" s="10" t="str">
-        <x:v>NO-GO: target cache and guard removal weaken exact-route/close semantics; pool changes have prior timeout/resource-boundary evidence.</x:v>
+        <x:v>KEEP baseline: new single lvalue submit-failure test plus request/reply, target, message, socket, behavior suites pass 5/5. No transport A/B delta is claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="10" t="str">
-        <x:v>2026-08-25 20:46</x:v>
+        <x:v>2026-08-25 20:40</x:v>
       </x:c>
       <x:c r="B46" s="10" t="str">
         <x:v>C++</x:v>
@@ -21556,40 +21564,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D46" s="10" t="str">
-        <x:v>ROUTER_ROUTER_REQREP</x:v>
+        <x:v>ROUTER_ROUTER</x:v>
       </x:c>
       <x:c r="E46" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F46" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
       </x:c>
       <x:c r="G46" s="10" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="H46" s="10" t="str">
-        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
+        <x:v>Re-evaluate bounded pool and state reuse on the exact routed path.</x:v>
       </x:c>
       <x:c r="I46" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J46" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K46" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L46" s="22" t="n">
-        <x:v>0.441</x:v>
+        <x:v>0.699</x:v>
       </x:c>
       <x:c r="M46" s="22"/>
       <x:c r="N46" s="10" t="str">
-        <x:v>NO-GO: target fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
+        <x:v>NO-GO as a new A/B: safe pool/state reuse already forms the measured path.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="10" t="str">
-        <x:v>2026-08-25 20:46</x:v>
+        <x:v>2026-08-25 20:40</x:v>
       </x:c>
       <x:c r="B47" s="10" t="str">
         <x:v>C++</x:v>
@@ -21598,68 +21606,120 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D47" s="10" t="str">
-        <x:v>ROUTER_ROUTER_REQREP</x:v>
+        <x:v>ROUTER_ROUTER</x:v>
       </x:c>
       <x:c r="E47" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F47" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
       </x:c>
       <x:c r="G47" s="10" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="H47" s="10" t="str">
-        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
+        <x:v>Add route cache, lower pool threshold, or remove lifetime guard.</x:v>
       </x:c>
       <x:c r="I47" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J47" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K47" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — contract/resource no-go</x:v>
       </x:c>
       <x:c r="L47" s="22" t="n">
-        <x:v>0.441</x:v>
+        <x:v>0.699</x:v>
       </x:c>
       <x:c r="M47" s="22"/>
       <x:c r="N47" s="10" t="str">
+        <x:v>NO-GO: target cache and guard removal weaken exact-route/close semantics; pool changes have prior timeout/resource-boundary evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="10" t="str">
+        <x:v>2026-08-25 20:46</x:v>
+      </x:c>
+      <x:c r="B48" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C48" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D48" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E48" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F48" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G48" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H48" s="10" t="str">
+        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
+      </x:c>
+      <x:c r="I48" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J48" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K48" s="10" t="str">
+        <x:v>N/A — exact-target contract no-go</x:v>
+      </x:c>
+      <x:c r="L48" s="22" t="n">
+        <x:v>0.441</x:v>
+      </x:c>
+      <x:c r="M48" s="22"/>
+      <x:c r="N48" s="10" t="str">
+        <x:v>NO-GO: target fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="10" t="str">
+        <x:v>2026-08-25 20:46</x:v>
+      </x:c>
+      <x:c r="B49" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C49" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D49" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E49" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F49" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G49" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H49" s="10" t="str">
+        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
+      </x:c>
+      <x:c r="I49" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J49" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K49" s="10" t="str">
+        <x:v>N/A — already baseline</x:v>
+      </x:c>
+      <x:c r="L49" s="22" t="n">
+        <x:v>0.441</x:v>
+      </x:c>
+      <x:c r="M49" s="22"/>
+      <x:c r="N49" s="10" t="str">
         <x:v>KEEP baseline: new single lvalue submit-failure test plus request/reply, target, message, socket, behavior suites pass 5/5. No transport A/B delta is claimed.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="10"/>
-      <x:c r="B48" s="10"/>
-      <x:c r="C48" s="10"/>
-      <x:c r="D48" s="10"/>
-      <x:c r="E48" s="10"/>
-      <x:c r="F48" s="10"/>
-      <x:c r="G48" s="10"/>
-      <x:c r="H48" s="10"/>
-      <x:c r="I48" s="10"/>
-      <x:c r="J48" s="10"/>
-      <x:c r="K48" s="10"/>
-      <x:c r="L48" s="22"/>
-      <x:c r="M48" s="22"/>
-      <x:c r="N48" s="10"/>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="10"/>
-      <x:c r="B49" s="10"/>
-      <x:c r="C49" s="10"/>
-      <x:c r="D49" s="10"/>
-      <x:c r="E49" s="10"/>
-      <x:c r="F49" s="10"/>
-      <x:c r="G49" s="10"/>
-      <x:c r="H49" s="10"/>
-      <x:c r="I49" s="10"/>
-      <x:c r="J49" s="10"/>
-      <x:c r="K49" s="10"/>
-      <x:c r="L49" s="22"/>
-      <x:c r="M49" s="22"/>
-      <x:c r="N49" s="10"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="10"/>

</xml_diff>

<commit_message>
docs(perf): record tls dealer router reqrep hold
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra4def66dd96e4f3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rca12694981bf40e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R122734dc08a24138"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R87815ee0815845d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re562e8ecc48f4663"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rc0bd8674bfc34074"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rbe6793b3cdc34af8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R9608b62868104378"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,7 +520,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 보류, tls 3개 통과·2개 미달·2개 보류, inproc 0개 통과·7개 미달 기록 완료</x:v>
+        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 보류, tls 3개 통과·1개 미달·3개 보류, inproc 0개 통과·7개 미달 기록 완료</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -567,7 +567,7 @@
       </x:c>
       <x:c r="B13" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"미달",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Paired aggregate misses a gate; one count per 64B anchor row</x:v>
@@ -582,7 +582,7 @@
       </x:c>
       <x:c r="B14" s="18" t="n">
         <x:f>COUNTIFS('Paired Results'!U4:U400,"보류",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C14" s="17" t="str">
         <x:v>Sol-reviewed safe candidates are exhausted; target still missed</x:v>
@@ -14176,24 +14176,24 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="G196" s="26" t="n">
-        <x:v>164868.2</x:v>
+        <x:v>179679.4</x:v>
       </x:c>
       <x:c r="H196" s="26" t="n">
-        <x:v>83005</x:v>
+        <x:v>89473</x:v>
       </x:c>
       <x:c r="I196" s="22" t="n">
         <x:f>H196/G196</x:f>
-        <x:v>0.5034627660155202</x:v>
+        <x:v>0.49795914278431475</x:v>
       </x:c>
       <x:c r="J196" s="24" t="n">
-        <x:v>0.318</x:v>
+        <x:v>0.277</x:v>
       </x:c>
       <x:c r="K196" s="24" t="n">
-        <x:v>0.77</x:v>
+        <x:v>0.629</x:v>
       </x:c>
       <x:c r="L196" s="24" t="n">
         <x:f>K196/J196</x:f>
-        <x:v>2.4213836477987423</x:v>
+        <x:v>2.270758122743682</x:v>
       </x:c>
       <x:c r="M196" s="10" t="n">
         <x:v>5</x:v>
@@ -14211,19 +14211,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R196" s="10" t="str">
-        <x:v>e1c0641269</x:v>
+        <x:v>4d572d2f5a</x:v>
       </x:c>
       <x:c r="S196" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_193626_cpp-dealer-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260826_001556_cpp-dealer-router-reqrep-tls-local0132-final-clean-paired5-c-20260826.txt</x:v>
       </x:c>
       <x:c r="T196" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260826_001852_cpp-dealer-router-reqrep-tls-local0132-final-clean-paired5-cpp-20260826.txt</x:v>
       </x:c>
       <x:c r="U196" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V196" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 70.94%; latency median ratio 1.62x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+        <x:v>Clean-source secure final pair: throughput aggregate mean 71.08%; latency median ratio 1.63x. Request/reply throughput gate misses. Sol approved hold after C0–C3 were rejected and source was reverted.</x:v>
       </x:c>
     </x:row>
     <x:row r="197">
@@ -14246,24 +14246,24 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="G197" s="26" t="n">
-        <x:v>151414.6</x:v>
+        <x:v>153994.8</x:v>
       </x:c>
       <x:c r="H197" s="26" t="n">
-        <x:v>78458.8</x:v>
+        <x:v>81040.6</x:v>
       </x:c>
       <x:c r="I197" s="22" t="n">
         <x:f>H197/G197</x:f>
-        <x:v>0.518171959639295</x:v>
+        <x:v>0.5262554320016001</x:v>
       </x:c>
       <x:c r="J197" s="24" t="n">
-        <x:v>0.332</x:v>
+        <x:v>0.325</x:v>
       </x:c>
       <x:c r="K197" s="24" t="n">
-        <x:v>0.731</x:v>
+        <x:v>0.797</x:v>
       </x:c>
       <x:c r="L197" s="24" t="n">
         <x:f>K197/J197</x:f>
-        <x:v>2.2018072289156625</x:v>
+        <x:v>2.4523076923076923</x:v>
       </x:c>
       <x:c r="M197" s="10" t="n">
         <x:v>5</x:v>
@@ -14281,19 +14281,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R197" s="10" t="str">
-        <x:v>e1c0641269</x:v>
+        <x:v>4d572d2f5a</x:v>
       </x:c>
       <x:c r="S197" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_193626_cpp-dealer-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260826_001556_cpp-dealer-router-reqrep-tls-local0132-final-clean-paired5-c-20260826.txt</x:v>
       </x:c>
       <x:c r="T197" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260826_001852_cpp-dealer-router-reqrep-tls-local0132-final-clean-paired5-cpp-20260826.txt</x:v>
       </x:c>
       <x:c r="U197" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V197" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 70.94%; latency median ratio 1.62x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+        <x:v>Clean-source secure final pair: throughput aggregate mean 71.08%; latency median ratio 1.63x. Request/reply throughput gate misses. Sol approved hold after C0–C3 were rejected and source was reverted.</x:v>
       </x:c>
     </x:row>
     <x:row r="198">
@@ -14316,24 +14316,24 @@
         <x:v>1024</x:v>
       </x:c>
       <x:c r="G198" s="26" t="n">
-        <x:v>83546.8</x:v>
+        <x:v>87274.4</x:v>
       </x:c>
       <x:c r="H198" s="26" t="n">
-        <x:v>40911.4</x:v>
+        <x:v>39829.4</x:v>
       </x:c>
       <x:c r="I198" s="22" t="n">
         <x:f>H198/G198</x:f>
-        <x:v>0.48968242948862195</x:v>
+        <x:v>0.4563697945789373</x:v>
       </x:c>
       <x:c r="J198" s="24" t="n">
-        <x:v>0.714</x:v>
+        <x:v>0.69</x:v>
       </x:c>
       <x:c r="K198" s="24" t="n">
-        <x:v>1.514</x:v>
+        <x:v>1.55</x:v>
       </x:c>
       <x:c r="L198" s="24" t="n">
         <x:f>K198/J198</x:f>
-        <x:v>2.1204481792717087</x:v>
+        <x:v>2.246376811594203</x:v>
       </x:c>
       <x:c r="M198" s="10" t="n">
         <x:v>5</x:v>
@@ -14351,19 +14351,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R198" s="10" t="str">
-        <x:v>e1c0641269</x:v>
+        <x:v>4d572d2f5a</x:v>
       </x:c>
       <x:c r="S198" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_193626_cpp-dealer-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260826_001556_cpp-dealer-router-reqrep-tls-local0132-final-clean-paired5-c-20260826.txt</x:v>
       </x:c>
       <x:c r="T198" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260826_001852_cpp-dealer-router-reqrep-tls-local0132-final-clean-paired5-cpp-20260826.txt</x:v>
       </x:c>
       <x:c r="U198" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V198" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 70.94%; latency median ratio 1.62x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+        <x:v>Clean-source secure final pair: throughput aggregate mean 71.08%; latency median ratio 1.63x. Request/reply throughput gate misses. Sol approved hold after C0–C3 were rejected and source was reverted.</x:v>
       </x:c>
     </x:row>
     <x:row r="199">
@@ -14386,24 +14386,24 @@
         <x:v>65536</x:v>
       </x:c>
       <x:c r="G199" s="26" t="n">
-        <x:v>4831.8</x:v>
+        <x:v>5424.8</x:v>
       </x:c>
       <x:c r="H199" s="26" t="n">
-        <x:v>4278</x:v>
+        <x:v>4913.2</x:v>
       </x:c>
       <x:c r="I199" s="22" t="n">
         <x:f>H199/G199</x:f>
-        <x:v>0.8853843288215572</x:v>
+        <x:v>0.9056923757557882</x:v>
       </x:c>
       <x:c r="J199" s="24" t="n">
-        <x:v>2.476</x:v>
+        <x:v>2.855</x:v>
       </x:c>
       <x:c r="K199" s="24" t="n">
-        <x:v>2.776</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="L199" s="24" t="n">
         <x:f>K199/J199</x:f>
-        <x:v>1.121163166397415</x:v>
+        <x:v>0.8756567425569177</x:v>
       </x:c>
       <x:c r="M199" s="10" t="n">
         <x:v>5</x:v>
@@ -14421,19 +14421,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R199" s="10" t="str">
-        <x:v>e1c0641269</x:v>
+        <x:v>4d572d2f5a</x:v>
       </x:c>
       <x:c r="S199" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_193626_cpp-dealer-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260826_001556_cpp-dealer-router-reqrep-tls-local0132-final-clean-paired5-c-20260826.txt</x:v>
       </x:c>
       <x:c r="T199" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260826_001852_cpp-dealer-router-reqrep-tls-local0132-final-clean-paired5-cpp-20260826.txt</x:v>
       </x:c>
       <x:c r="U199" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V199" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 70.94%; latency median ratio 1.62x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+        <x:v>Clean-source secure final pair: throughput aggregate mean 71.08%; latency median ratio 1.63x. Request/reply throughput gate misses. Sol approved hold after C0–C3 were rejected and source was reverted.</x:v>
       </x:c>
     </x:row>
     <x:row r="200">
@@ -14456,24 +14456,24 @@
         <x:v>131072</x:v>
       </x:c>
       <x:c r="G200" s="26" t="n">
-        <x:v>2933.8</x:v>
+        <x:v>3130.8</x:v>
       </x:c>
       <x:c r="H200" s="26" t="n">
-        <x:v>2807</x:v>
+        <x:v>2912.4</x:v>
       </x:c>
       <x:c r="I200" s="22" t="n">
         <x:f>H200/G200</x:f>
-        <x:v>0.9567796032449383</x:v>
+        <x:v>0.9302414718282866</x:v>
       </x:c>
       <x:c r="J200" s="24" t="n">
-        <x:v>2.04</x:v>
+        <x:v>2.156</x:v>
       </x:c>
       <x:c r="K200" s="24" t="n">
-        <x:v>2.1</x:v>
+        <x:v>2.023</x:v>
       </x:c>
       <x:c r="L200" s="24" t="n">
         <x:f>K200/J200</x:f>
-        <x:v>1.0294117647058825</x:v>
+        <x:v>0.9383116883116883</x:v>
       </x:c>
       <x:c r="M200" s="10" t="n">
         <x:v>5</x:v>
@@ -14491,19 +14491,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R200" s="10" t="str">
-        <x:v>e1c0641269</x:v>
+        <x:v>4d572d2f5a</x:v>
       </x:c>
       <x:c r="S200" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_193626_cpp-dealer-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260826_001556_cpp-dealer-router-reqrep-tls-local0132-final-clean-paired5-c-20260826.txt</x:v>
       </x:c>
       <x:c r="T200" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260826_001852_cpp-dealer-router-reqrep-tls-local0132-final-clean-paired5-cpp-20260826.txt</x:v>
       </x:c>
       <x:c r="U200" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V200" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 70.94%; latency median ratio 1.62x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+        <x:v>Clean-source secure final pair: throughput aggregate mean 71.08%; latency median ratio 1.63x. Request/reply throughput gate misses. Sol approved hold after C0–C3 were rejected and source was reverted.</x:v>
       </x:c>
     </x:row>
     <x:row r="201">
@@ -14526,24 +14526,24 @@
         <x:v>262144</x:v>
       </x:c>
       <x:c r="G201" s="26" t="n">
-        <x:v>1767.6</x:v>
+        <x:v>1765</x:v>
       </x:c>
       <x:c r="H201" s="26" t="n">
-        <x:v>1596.4</x:v>
+        <x:v>1673.2</x:v>
       </x:c>
       <x:c r="I201" s="22" t="n">
         <x:f>H201/G201</x:f>
-        <x:v>0.9031455080334918</x:v>
+        <x:v>0.9479886685552408</x:v>
       </x:c>
       <x:c r="J201" s="24" t="n">
-        <x:v>1.715</x:v>
+        <x:v>1.695</x:v>
       </x:c>
       <x:c r="K201" s="24" t="n">
-        <x:v>1.815</x:v>
+        <x:v>1.734</x:v>
       </x:c>
       <x:c r="L201" s="24" t="n">
         <x:f>K201/J201</x:f>
-        <x:v>1.0583090379008746</x:v>
+        <x:v>1.023008849557522</x:v>
       </x:c>
       <x:c r="M201" s="10" t="n">
         <x:v>5</x:v>
@@ -14561,19 +14561,19 @@
         <x:v>0.13.2</x:v>
       </x:c>
       <x:c r="R201" s="10" t="str">
-        <x:v>e1c0641269</x:v>
+        <x:v>4d572d2f5a</x:v>
       </x:c>
       <x:c r="S201" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260825_193626_cpp-dealer-router-reqrep-tls-local0132-baseline-c-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260826_001556_cpp-dealer-router-reqrep-tls-local0132-final-clean-paired5-c-20260826.txt</x:v>
       </x:c>
       <x:c r="T201" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260826_001852_cpp-dealer-router-reqrep-tls-local0132-final-clean-paired5-cpp-20260826.txt</x:v>
       </x:c>
       <x:c r="U201" s="10" t="str">
-        <x:v>미달</x:v>
+        <x:v>보류</x:v>
       </x:c>
       <x:c r="V201" s="10" t="str">
-        <x:v>Final secure 5-run median: throughput aggregate mean 70.94%; latency median ratio 1.62x; fail. Candidate A exact-target contract no-go; retain async-only completion bridge B after contract 5/5.</x:v>
+        <x:v>Clean-source secure final pair: throughput aggregate mean 71.08%; latency median ratio 1.63x. Request/reply throughput gate misses. Sol approved hold after C0–C3 were rejected and source was reverted.</x:v>
       </x:c>
     </x:row>
     <x:row r="202">
@@ -20971,7 +20971,7 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="10" t="str">
-        <x:v>2026-08-25 19:43</x:v>
+        <x:v>2026-08-25 23:42</x:v>
       </x:c>
       <x:c r="B32" s="10" t="str">
         <x:v>C++</x:v>
@@ -20989,10 +20989,10 @@
         <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G32" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>C0</x:v>
       </x:c>
       <x:c r="H32" s="10" t="str">
-        <x:v>Use Core normal DEALER request route instead of initially selected exact transport target.</x:v>
+        <x:v>Measure the current self-anchor/co-allocated completion state independently from the historical baseline.</x:v>
       </x:c>
       <x:c r="I32" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
@@ -21001,19 +21001,21 @@
         <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K32" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_234200_cpp-dealer-router-reqrep-tls-local0132-c0-self-anchor-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="L32" s="22" t="n">
         <x:v>0.709</x:v>
       </x:c>
-      <x:c r="M32" s="22"/>
+      <x:c r="M32" s="22" t="n">
+        <x:v>0.686</x:v>
+      </x:c>
       <x:c r="N32" s="10" t="str">
-        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership.</x:v>
+        <x:v>REJECT: self-anchor alone regresses under the same manifest; do not treat it as a retained TLS improvement.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="10" t="str">
-        <x:v>2026-08-25 19:43</x:v>
+        <x:v>2026-08-25 23:49</x:v>
       </x:c>
       <x:c r="B33" s="10" t="str">
         <x:v>C++</x:v>
@@ -21031,29 +21033,33 @@
         <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G33" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>C1</x:v>
       </x:c>
       <x:c r="H33" s="10" t="str">
-        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
+        <x:v>Fuse Core terminal completion and self-anchor release under the same operation-state mutex.</x:v>
       </x:c>
       <x:c r="I33" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J33" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_234200_cpp-dealer-router-reqrep-tls-local0132-c0-self-anchor-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K33" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_193909_cpp-dealer-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
-      </x:c>
-      <x:c r="L33" s="22"/>
-      <x:c r="M33" s="22"/>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_234903_cpp-dealer-router-reqrep-tls-local0132-c1-core-terminal-paired5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L33" s="22" t="n">
+        <x:v>0.686</x:v>
+      </x:c>
+      <x:c r="M33" s="22" t="n">
+        <x:v>0.692</x:v>
+      </x:c>
       <x:c r="N33" s="10" t="str">
-        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.62x passes.</x:v>
+        <x:v>REJECT: contract suites 5/5 pass, but 69.15% remains below the historical baseline; source reverted.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="10" t="str">
-        <x:v>2026-08-25 19:54</x:v>
+        <x:v>2026-08-25 23:57</x:v>
       </x:c>
       <x:c r="B34" s="10" t="str">
         <x:v>C++</x:v>
@@ -21062,7 +21068,7 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D34" s="10" t="str">
-        <x:v>ROUTER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E34" s="10" t="str">
         <x:v>tls</x:v>
@@ -21071,31 +21077,33 @@
         <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G34" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>C2</x:v>
       </x:c>
       <x:c r="H34" s="10" t="str">
-        <x:v>Use Core normal route selection instead of the initially selected exact transport target.</x:v>
+        <x:v>Adopt freshly received reply frames into no-init message storage.</x:v>
       </x:c>
       <x:c r="I34" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J34" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_234903_cpp-dealer-router-reqrep-tls-local0132-c1-core-terminal-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K34" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_235738_cpp-dealer-router-reqrep-tls-local0132-c2-native-adopt-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="L34" s="22" t="n">
-        <x:v>0.714</x:v>
-      </x:c>
-      <x:c r="M34" s="22"/>
+        <x:v>0.692</x:v>
+      </x:c>
+      <x:c r="M34" s="22" t="n">
+        <x:v>0.682</x:v>
+      </x:c>
       <x:c r="N34" s="10" t="str">
-        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership; exact-request-target contract remains required.</x:v>
+        <x:v>REJECT: request timeout timing initially failed; standalone repeats passed, but the full 68.18% pair regresses. Source reverted.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="10" t="str">
-        <x:v>2026-08-25 19:54</x:v>
+        <x:v>2026-08-26 00:04</x:v>
       </x:c>
       <x:c r="B35" s="10" t="str">
         <x:v>C++</x:v>
@@ -21104,7 +21112,7 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D35" s="10" t="str">
-        <x:v>ROUTER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E35" s="10" t="str">
         <x:v>tls</x:v>
@@ -21113,29 +21121,33 @@
         <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G35" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>C3</x:v>
       </x:c>
       <x:c r="H35" s="10" t="str">
-        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
+        <x:v>Use an in-state continuation only with an empty scheduler; retain the scheduled shared-slot path.</x:v>
       </x:c>
       <x:c r="I35" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J35" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_235738_cpp-dealer-router-reqrep-tls-local0132-c2-native-adopt-paired5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K35" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
-      </x:c>
-      <x:c r="L35" s="22"/>
-      <x:c r="M35" s="22"/>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260826_000451_cpp-dealer-router-reqrep-tls-local0132-c3-inline-paired5-cpp-20260826.txt</x:v>
+      </x:c>
+      <x:c r="L35" s="22" t="n">
+        <x:v>0.682</x:v>
+      </x:c>
+      <x:c r="M35" s="22" t="n">
+        <x:v>0.714</x:v>
+      </x:c>
       <x:c r="N35" s="10" t="str">
-        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.65x passes.</x:v>
+        <x:v>PROVISIONAL: contract suites 5/5 pass; 71.39% requires a clean acceptance run because the control changed.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="10" t="str">
-        <x:v>2026-08-25 20:08</x:v>
+        <x:v>2026-08-26 00:18</x:v>
       </x:c>
       <x:c r="B36" s="10" t="str">
         <x:v>C++</x:v>
@@ -21144,40 +21156,42 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D36" s="10" t="str">
-        <x:v>PAIR</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E36" s="10" t="str">
-        <x:v>inproc</x:v>
+        <x:v>tls</x:v>
       </x:c>
       <x:c r="F36" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G36" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>Sol review</x:v>
       </x:c>
       <x:c r="H36" s="10" t="str">
-        <x:v>Re-evaluate retained 128KiB–1MiB bounded pool and process-lifetime singleton.</x:v>
+        <x:v>Review C0–C3, the C3 acceptance run, and the clean final pair.</x:v>
       </x:c>
       <x:c r="I36" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J36" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260826_001206_cpp-dealer-router-reqrep-tls-local0132-c3-final-clean-paired5-cpp-20260826.txt</x:v>
       </x:c>
       <x:c r="K36" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260826_001852_cpp-dealer-router-reqrep-tls-local0132-final-clean-paired5-cpp-20260826.txt</x:v>
       </x:c>
       <x:c r="L36" s="22" t="n">
-        <x:v>0.761</x:v>
-      </x:c>
-      <x:c r="M36" s="22"/>
+        <x:v>0.687</x:v>
+      </x:c>
+      <x:c r="M36" s="22" t="n">
+        <x:v>0.711</x:v>
+      </x:c>
       <x:c r="N36" s="10" t="str">
-        <x:v>NO-GO as a new A/B: safe bounded-pool lifecycle is already in source, including late Core-release safety.</x:v>
+        <x:v>SOL APPROVED: C3 acceptance returned 68.73%, so all source changes are reverted; safe candidates are exhausted. Clean final 71.08%, latency 1.63x; 보류.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="10" t="str">
-        <x:v>2026-08-25 20:08</x:v>
+        <x:v>2026-08-25 19:54</x:v>
       </x:c>
       <x:c r="B37" s="10" t="str">
         <x:v>C++</x:v>
@@ -21186,40 +21200,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D37" s="10" t="str">
-        <x:v>PAIR</x:v>
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E37" s="10" t="str">
-        <x:v>inproc</x:v>
+        <x:v>tls</x:v>
       </x:c>
       <x:c r="F37" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G37" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H37" s="10" t="str">
-        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
+        <x:v>Use Core normal route selection instead of the initially selected exact transport target.</x:v>
       </x:c>
       <x:c r="I37" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J37" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K37" s="10" t="str">
-        <x:v>N/A — timeout/resource no-go</x:v>
+        <x:v>N/A — exact-target contract no-go</x:v>
       </x:c>
       <x:c r="L37" s="22" t="n">
-        <x:v>0.761</x:v>
+        <x:v>0.714</x:v>
       </x:c>
       <x:c r="M37" s="22"/>
       <x:c r="N37" s="10" t="str">
-        <x:v>NO-GO: the 64KiB global threshold previously yielded a 25/30 partial TCP report through timeout; raising the cap changes the documented resource boundary. Per-transport policy would make ownership/resource behavior inconsistent.</x:v>
+        <x:v>NO-GO: target fallback changes terminal/no-reroute behavior and refused-submit ownership; exact-request-target contract remains required.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="10" t="str">
-        <x:v>2026-08-25 20:17</x:v>
+        <x:v>2026-08-25 19:54</x:v>
       </x:c>
       <x:c r="B38" s="10" t="str">
         <x:v>C++</x:v>
@@ -21228,40 +21242,38 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D38" s="10" t="str">
-        <x:v>PUBSUB</x:v>
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E38" s="10" t="str">
-        <x:v>inproc</x:v>
+        <x:v>tls</x:v>
       </x:c>
       <x:c r="F38" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G38" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H38" s="10" t="str">
-        <x:v>Re-evaluate direct single-part publish and the retained 128KiB–1MiB bounded pool.</x:v>
+        <x:v>Retain async-only completion bridge; it removes managed-bridge mutex, condition-variable and optional staging from async().</x:v>
       </x:c>
       <x:c r="I38" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J38" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_180136_cpp-router-router-reqrep-ws-local0132-candidate-b-ownershipfix-20260825.txt</x:v>
       </x:c>
       <x:c r="K38" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
-      </x:c>
-      <x:c r="L38" s="22" t="n">
-        <x:v>0.787</x:v>
-      </x:c>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_195453_cpp-router-router-reqrep-tls-local0132-baseline-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="L38" s="22"/>
       <x:c r="M38" s="22"/>
       <x:c r="N38" s="10" t="str">
-        <x:v>NO-GO as a new A/B: direct publish and safe bounded-pool lifecycle already form the measured hot path.</x:v>
+        <x:v>KEEP: same Core/source implementation measured under TLS; contract tests 5/5 pass. Transport differs, so no A/B delta is recorded. TLS throughput still misses the gate; latency 1.65x passes.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="10" t="str">
-        <x:v>2026-08-25 20:17</x:v>
+        <x:v>2026-08-25 20:08</x:v>
       </x:c>
       <x:c r="B39" s="10" t="str">
         <x:v>C++</x:v>
@@ -21270,40 +21282,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D39" s="10" t="str">
-        <x:v>PUBSUB</x:v>
+        <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E39" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F39" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
       </x:c>
       <x:c r="G39" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H39" s="10" t="str">
-        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
+        <x:v>Re-evaluate retained 128KiB–1MiB bounded pool and process-lifetime singleton.</x:v>
       </x:c>
       <x:c r="I39" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J39" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K39" s="10" t="str">
-        <x:v>N/A — timeout/resource no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L39" s="22" t="n">
-        <x:v>0.787</x:v>
+        <x:v>0.761</x:v>
       </x:c>
       <x:c r="M39" s="22"/>
       <x:c r="N39" s="10" t="str">
-        <x:v>NO-GO: 64KiB global threshold has prior 25/30 TCP partial timeout; cap expansion changes resource policy. Transport-specific policy is not an acceptable lifecycle split.</x:v>
+        <x:v>NO-GO as a new A/B: safe bounded-pool lifecycle is already in source, including late Core-release safety.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="10" t="str">
-        <x:v>2026-08-25 20:22</x:v>
+        <x:v>2026-08-25 20:08</x:v>
       </x:c>
       <x:c r="B40" s="10" t="str">
         <x:v>C++</x:v>
@@ -21312,40 +21324,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D40" s="10" t="str">
-        <x:v>DEALER_DEALER</x:v>
+        <x:v>PAIR</x:v>
       </x:c>
       <x:c r="E40" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F40" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 22.71%</x:v>
       </x:c>
       <x:c r="G40" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H40" s="10" t="str">
-        <x:v>Re-evaluate bounded pool and operation-state reuse in the routed one-way hot path.</x:v>
+        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
       </x:c>
       <x:c r="I40" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J40" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_200530_cpp-pair-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K40" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — timeout/resource no-go</x:v>
       </x:c>
       <x:c r="L40" s="22" t="n">
-        <x:v>0.705</x:v>
+        <x:v>0.761</x:v>
       </x:c>
       <x:c r="M40" s="22"/>
       <x:c r="N40" s="10" t="str">
-        <x:v>NO-GO as a new A/B: the measured path already has the safe pool/state lifecycle.</x:v>
+        <x:v>NO-GO: the 64KiB global threshold previously yielded a 25/30 partial TCP report through timeout; raising the cap changes the documented resource boundary. Per-transport policy would make ownership/resource behavior inconsistent.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="10" t="str">
-        <x:v>2026-08-25 20:22</x:v>
+        <x:v>2026-08-25 20:17</x:v>
       </x:c>
       <x:c r="B41" s="10" t="str">
         <x:v>C++</x:v>
@@ -21354,40 +21366,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D41" s="10" t="str">
-        <x:v>DEALER_DEALER</x:v>
+        <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E41" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F41" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
       </x:c>
       <x:c r="G41" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H41" s="10" t="str">
-        <x:v>Lower global pool threshold, raise cap, or remove lifetime guard.</x:v>
+        <x:v>Re-evaluate direct single-part publish and the retained 128KiB–1MiB bounded pool.</x:v>
       </x:c>
       <x:c r="I41" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J41" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K41" s="10" t="str">
-        <x:v>N/A — timeout/contract/resource no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L41" s="22" t="n">
-        <x:v>0.705</x:v>
+        <x:v>0.787</x:v>
       </x:c>
       <x:c r="M41" s="22"/>
       <x:c r="N41" s="10" t="str">
-        <x:v>NO-GO: 64KiB pool threshold has a prior TCP partial timeout; cap and guard changes weaken resource or close/concurrency guarantees.</x:v>
+        <x:v>NO-GO as a new A/B: direct publish and safe bounded-pool lifecycle already form the measured hot path.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="10" t="str">
-        <x:v>2026-08-25 20:29</x:v>
+        <x:v>2026-08-25 20:17</x:v>
       </x:c>
       <x:c r="B42" s="10" t="str">
         <x:v>C++</x:v>
@@ -21396,40 +21408,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D42" s="10" t="str">
-        <x:v>DEALER_ROUTER</x:v>
+        <x:v>PUBSUB</x:v>
       </x:c>
       <x:c r="E42" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F42" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 24.09%</x:v>
       </x:c>
       <x:c r="G42" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H42" s="10" t="str">
-        <x:v>Re-evaluate bounded pool and routed operation-state reuse.</x:v>
+        <x:v>Lower global pool threshold to 64KiB or raise its 8MiB cap.</x:v>
       </x:c>
       <x:c r="I42" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J42" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_201420_cpp-pubsub-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K42" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — timeout/resource no-go</x:v>
       </x:c>
       <x:c r="L42" s="22" t="n">
-        <x:v>0.71</x:v>
+        <x:v>0.787</x:v>
       </x:c>
       <x:c r="M42" s="22"/>
       <x:c r="N42" s="10" t="str">
-        <x:v>NO-GO as a new A/B: the safe bounded-pool/state path is already measured.</x:v>
+        <x:v>NO-GO: 64KiB global threshold has prior 25/30 TCP partial timeout; cap expansion changes resource policy. Transport-specific policy is not an acceptable lifecycle split.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="10" t="str">
-        <x:v>2026-08-25 20:29</x:v>
+        <x:v>2026-08-25 20:22</x:v>
       </x:c>
       <x:c r="B43" s="10" t="str">
         <x:v>C++</x:v>
@@ -21438,40 +21450,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D43" s="10" t="str">
-        <x:v>DEALER_ROUTER</x:v>
+        <x:v>DEALER_DEALER</x:v>
       </x:c>
       <x:c r="E43" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F43" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
       </x:c>
       <x:c r="G43" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H43" s="10" t="str">
-        <x:v>Add route cache or remove attempt/lifetime guards.</x:v>
+        <x:v>Re-evaluate bounded pool and operation-state reuse in the routed one-way hot path.</x:v>
       </x:c>
       <x:c r="I43" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J43" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K43" s="10" t="str">
-        <x:v>N/A — exact-route/close no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L43" s="22" t="n">
-        <x:v>0.71</x:v>
+        <x:v>0.705</x:v>
       </x:c>
       <x:c r="M43" s="22"/>
       <x:c r="N43" s="10" t="str">
-        <x:v>NO-GO: route caching and guard removal change exact route selection or close/concurrency responsibility.</x:v>
+        <x:v>NO-GO as a new A/B: the measured path already has the safe pool/state lifecycle.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="10" t="str">
-        <x:v>2026-08-25 20:34</x:v>
+        <x:v>2026-08-25 20:22</x:v>
       </x:c>
       <x:c r="B44" s="10" t="str">
         <x:v>C++</x:v>
@@ -21480,40 +21492,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D44" s="10" t="str">
-        <x:v>DEALER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_DEALER</x:v>
       </x:c>
       <x:c r="E44" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F44" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 25.90%</x:v>
       </x:c>
       <x:c r="G44" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H44" s="10" t="str">
-        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
+        <x:v>Lower global pool threshold, raise cap, or remove lifetime guard.</x:v>
       </x:c>
       <x:c r="I44" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J44" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202231_cpp-dealer-dealer-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K44" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
+        <x:v>N/A — timeout/contract/resource no-go</x:v>
       </x:c>
       <x:c r="L44" s="22" t="n">
-        <x:v>0.429</x:v>
+        <x:v>0.705</x:v>
       </x:c>
       <x:c r="M44" s="22"/>
       <x:c r="N44" s="10" t="str">
-        <x:v>NO-GO: fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
+        <x:v>NO-GO: 64KiB pool threshold has a prior TCP partial timeout; cap and guard changes weaken resource or close/concurrency guarantees.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="10" t="str">
-        <x:v>2026-08-25 20:34</x:v>
+        <x:v>2026-08-25 20:29</x:v>
       </x:c>
       <x:c r="B45" s="10" t="str">
         <x:v>C++</x:v>
@@ -21522,40 +21534,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D45" s="10" t="str">
-        <x:v>DEALER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_ROUTER</x:v>
       </x:c>
       <x:c r="E45" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F45" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
       </x:c>
       <x:c r="G45" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H45" s="10" t="str">
-        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
+        <x:v>Re-evaluate bounded pool and routed operation-state reuse.</x:v>
       </x:c>
       <x:c r="I45" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J45" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K45" s="10" t="str">
         <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L45" s="22" t="n">
-        <x:v>0.429</x:v>
+        <x:v>0.71</x:v>
       </x:c>
       <x:c r="M45" s="22"/>
       <x:c r="N45" s="10" t="str">
-        <x:v>KEEP baseline: new single lvalue submit-failure test plus request/reply, target, message, socket, behavior suites pass 5/5. No transport A/B delta is claimed.</x:v>
+        <x:v>NO-GO as a new A/B: the safe bounded-pool/state path is already measured.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="10" t="str">
-        <x:v>2026-08-25 20:40</x:v>
+        <x:v>2026-08-25 20:29</x:v>
       </x:c>
       <x:c r="B46" s="10" t="str">
         <x:v>C++</x:v>
@@ -21564,40 +21576,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D46" s="10" t="str">
-        <x:v>ROUTER_ROUTER</x:v>
+        <x:v>DEALER_ROUTER</x:v>
       </x:c>
       <x:c r="E46" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F46" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 21.50%</x:v>
       </x:c>
       <x:c r="G46" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H46" s="10" t="str">
-        <x:v>Re-evaluate bounded pool and state reuse on the exact routed path.</x:v>
+        <x:v>Add route cache or remove attempt/lifetime guards.</x:v>
       </x:c>
       <x:c r="I46" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J46" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_202853_cpp-dealer-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K46" s="10" t="str">
-        <x:v>N/A — already baseline</x:v>
+        <x:v>N/A — exact-route/close no-go</x:v>
       </x:c>
       <x:c r="L46" s="22" t="n">
-        <x:v>0.699</x:v>
+        <x:v>0.71</x:v>
       </x:c>
       <x:c r="M46" s="22"/>
       <x:c r="N46" s="10" t="str">
-        <x:v>NO-GO as a new A/B: safe pool/state reuse already forms the measured path.</x:v>
+        <x:v>NO-GO: route caching and guard removal change exact route selection or close/concurrency responsibility.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="10" t="str">
-        <x:v>2026-08-25 20:40</x:v>
+        <x:v>2026-08-25 20:34</x:v>
       </x:c>
       <x:c r="B47" s="10" t="str">
         <x:v>C++</x:v>
@@ -21606,40 +21618,40 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D47" s="10" t="str">
-        <x:v>ROUTER_ROUTER</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E47" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F47" s="10" t="str">
-        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
+        <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G47" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H47" s="10" t="str">
-        <x:v>Add route cache, lower pool threshold, or remove lifetime guard.</x:v>
+        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
       </x:c>
       <x:c r="I47" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J47" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K47" s="10" t="str">
-        <x:v>N/A — contract/resource no-go</x:v>
+        <x:v>N/A — exact-target contract no-go</x:v>
       </x:c>
       <x:c r="L47" s="22" t="n">
-        <x:v>0.699</x:v>
+        <x:v>0.429</x:v>
       </x:c>
       <x:c r="M47" s="22"/>
       <x:c r="N47" s="10" t="str">
-        <x:v>NO-GO: target cache and guard removal weaken exact-route/close semantics; pool changes have prior timeout/resource-boundary evidence.</x:v>
+        <x:v>NO-GO: fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="10" t="str">
-        <x:v>2026-08-25 20:46</x:v>
+        <x:v>2026-08-25 20:34</x:v>
       </x:c>
       <x:c r="B48" s="10" t="str">
         <x:v>C++</x:v>
@@ -21648,7 +21660,7 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D48" s="10" t="str">
-        <x:v>ROUTER_ROUTER_REQREP</x:v>
+        <x:v>DEALER_ROUTER_REQREP</x:v>
       </x:c>
       <x:c r="E48" s="10" t="str">
         <x:v>inproc</x:v>
@@ -21657,31 +21669,31 @@
         <x:v>Throughput aggregate &lt; 85%</x:v>
       </x:c>
       <x:c r="G48" s="10" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H48" s="10" t="str">
-        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
+        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
       </x:c>
       <x:c r="I48" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J48" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_203443_cpp-dealer-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K48" s="10" t="str">
-        <x:v>N/A — exact-target contract no-go</x:v>
+        <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L48" s="22" t="n">
-        <x:v>0.441</x:v>
+        <x:v>0.429</x:v>
       </x:c>
       <x:c r="M48" s="22"/>
       <x:c r="N48" s="10" t="str">
-        <x:v>NO-GO: target fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
+        <x:v>KEEP baseline: new single lvalue submit-failure test plus request/reply, target, message, socket, behavior suites pass 5/5. No transport A/B delta is claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="10" t="str">
-        <x:v>2026-08-25 20:46</x:v>
+        <x:v>2026-08-25 20:40</x:v>
       </x:c>
       <x:c r="B49" s="10" t="str">
         <x:v>C++</x:v>
@@ -21690,84 +21702,162 @@
         <x:v>Single</x:v>
       </x:c>
       <x:c r="D49" s="10" t="str">
-        <x:v>ROUTER_ROUTER_REQREP</x:v>
+        <x:v>ROUTER_ROUTER</x:v>
       </x:c>
       <x:c r="E49" s="10" t="str">
         <x:v>inproc</x:v>
       </x:c>
       <x:c r="F49" s="10" t="str">
-        <x:v>Throughput aggregate &lt; 85%</x:v>
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
       </x:c>
       <x:c r="G49" s="10" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H49" s="10" t="str">
-        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
+        <x:v>Re-evaluate bounded pool and state reuse on the exact routed path.</x:v>
       </x:c>
       <x:c r="I49" s="10" t="str">
         <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
       </x:c>
       <x:c r="J49" s="10" t="str">
-        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
       </x:c>
       <x:c r="K49" s="10" t="str">
         <x:v>N/A — already baseline</x:v>
       </x:c>
       <x:c r="L49" s="22" t="n">
-        <x:v>0.441</x:v>
+        <x:v>0.699</x:v>
       </x:c>
       <x:c r="M49" s="22"/>
       <x:c r="N49" s="10" t="str">
+        <x:v>NO-GO as a new A/B: safe pool/state reuse already forms the measured path.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="10" t="str">
+        <x:v>2026-08-25 20:40</x:v>
+      </x:c>
+      <x:c r="B50" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C50" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D50" s="10" t="str">
+        <x:v>ROUTER_ROUTER</x:v>
+      </x:c>
+      <x:c r="E50" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F50" s="10" t="str">
+        <x:v>Strict throughput aggregate &lt; 95%; 64KiB 20.87%</x:v>
+      </x:c>
+      <x:c r="G50" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H50" s="10" t="str">
+        <x:v>Add route cache, lower pool threshold, or remove lifetime guard.</x:v>
+      </x:c>
+      <x:c r="I50" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J50" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204014_cpp-router-router-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K50" s="10" t="str">
+        <x:v>N/A — contract/resource no-go</x:v>
+      </x:c>
+      <x:c r="L50" s="22" t="n">
+        <x:v>0.699</x:v>
+      </x:c>
+      <x:c r="M50" s="22"/>
+      <x:c r="N50" s="10" t="str">
+        <x:v>NO-GO: target cache and guard removal weaken exact-route/close semantics; pool changes have prior timeout/resource-boundary evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="10" t="str">
+        <x:v>2026-08-25 20:46</x:v>
+      </x:c>
+      <x:c r="B51" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C51" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D51" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E51" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F51" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G51" s="10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H51" s="10" t="str">
+        <x:v>Select a normal Core route instead of the initial exact target.</x:v>
+      </x:c>
+      <x:c r="I51" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J51" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K51" s="10" t="str">
+        <x:v>N/A — exact-target contract no-go</x:v>
+      </x:c>
+      <x:c r="L51" s="22" t="n">
+        <x:v>0.441</x:v>
+      </x:c>
+      <x:c r="M51" s="22"/>
+      <x:c r="N51" s="10" t="str">
+        <x:v>NO-GO: target fallback changes terminal/no-reroute and refused-submit ownership.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="10" t="str">
+        <x:v>2026-08-25 20:46</x:v>
+      </x:c>
+      <x:c r="B52" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C52" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D52" s="10" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E52" s="10" t="str">
+        <x:v>inproc</x:v>
+      </x:c>
+      <x:c r="F52" s="10" t="str">
+        <x:v>Throughput aggregate &lt; 85%</x:v>
+      </x:c>
+      <x:c r="G52" s="10" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H52" s="10" t="str">
+        <x:v>Retain async-only completion bridge and safe borrowed single-part native view; verify failure ownership.</x:v>
+      </x:c>
+      <x:c r="I52" s="10" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J52" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260825_204632_cpp-router-router-reqrep-inproc-local0132-final5-cpp-20260825.txt</x:v>
+      </x:c>
+      <x:c r="K52" s="10" t="str">
+        <x:v>N/A — already baseline</x:v>
+      </x:c>
+      <x:c r="L52" s="22" t="n">
+        <x:v>0.441</x:v>
+      </x:c>
+      <x:c r="M52" s="22"/>
+      <x:c r="N52" s="10" t="str">
         <x:v>KEEP baseline: new single lvalue submit-failure test plus request/reply, target, message, socket, behavior suites pass 5/5. No transport A/B delta is claimed.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="50">
-      <x:c r="A50" s="10"/>
-      <x:c r="B50" s="10"/>
-      <x:c r="C50" s="10"/>
-      <x:c r="D50" s="10"/>
-      <x:c r="E50" s="10"/>
-      <x:c r="F50" s="10"/>
-      <x:c r="G50" s="10"/>
-      <x:c r="H50" s="10"/>
-      <x:c r="I50" s="10"/>
-      <x:c r="J50" s="10"/>
-      <x:c r="K50" s="10"/>
-      <x:c r="L50" s="22"/>
-      <x:c r="M50" s="22"/>
-      <x:c r="N50" s="10"/>
-    </x:row>
-    <x:row r="51">
-      <x:c r="A51" s="10"/>
-      <x:c r="B51" s="10"/>
-      <x:c r="C51" s="10"/>
-      <x:c r="D51" s="10"/>
-      <x:c r="E51" s="10"/>
-      <x:c r="F51" s="10"/>
-      <x:c r="G51" s="10"/>
-      <x:c r="H51" s="10"/>
-      <x:c r="I51" s="10"/>
-      <x:c r="J51" s="10"/>
-      <x:c r="K51" s="10"/>
-      <x:c r="L51" s="22"/>
-      <x:c r="M51" s="22"/>
-      <x:c r="N51" s="10"/>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="10"/>
-      <x:c r="B52" s="10"/>
-      <x:c r="C52" s="10"/>
-      <x:c r="D52" s="10"/>
-      <x:c r="E52" s="10"/>
-      <x:c r="F52" s="10"/>
-      <x:c r="G52" s="10"/>
-      <x:c r="H52" s="10"/>
-      <x:c r="I52" s="10"/>
-      <x:c r="J52" s="10"/>
-      <x:c r="K52" s="10"/>
-      <x:c r="L52" s="22"/>
-      <x:c r="M52" s="22"/>
-      <x:c r="N52" s="10"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="10"/>

</xml_diff>

<commit_message>
perf: optimize 0.13.2 async send and transport paths
Refine send completion admission and binding fast paths, reduce TCP/WS/WSS dispatch overhead, consolidate socket send code, and update specifications, tests, benchmarks, and performance records.
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re562e8ecc48f4663"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rc0bd8674bfc34074"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="Rbe6793b3cdc34af8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R9608b62868104378"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb915c8b82b404888"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired Results" sheetId="2" r:id="Rd2cba4cea7b547c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement Log" sheetId="3" r:id="R74d2ce9dbe99473e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Ra496c8cd0b324ab5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,14 +16,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
     <x:numFmt numFmtId="201" formatCode="0.00%"/>
     <x:numFmt numFmtId="202" formatCode="0.000"/>
     <x:numFmt numFmtId="203" formatCode="#,##0.0"/>
     <x:numFmt numFmtId="204" formatCode="yyyy-mm-dd hh:mm"/>
+    <x:numFmt numFmtId="205" formatCode="0.00x"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -52,8 +53,13 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color theme="1"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -75,8 +81,13 @@
         <x:fgColor rgb="FFEEF4FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="10">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -92,11 +103,87 @@
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="109">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -155,6 +242,197 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="204" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -166,7 +444,7 @@
         <x:color rgb="FF276749"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -177,7 +455,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -188,7 +466,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -198,7 +476,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -520,7 +798,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>tcp 4개 통과·3개 미달, ws 5개 통과·3개 미달, wss 5개 통과·2개 보류, tls 3개 통과·1개 미달·3개 보류, inproc 0개 통과·7개 미달 기록 완료</x:v>
+        <x:v>C++ Single 기록 유지; .NET Multi tcp ROUTER_ROUTER SENDSEND·REQREP 2개 통과 추가</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>6</x:v>
@@ -551,8 +829,7 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="B12" s="18" t="n">
-        <x:f>COUNTIFS('Paired Results'!U4:U400,"통과",'Paired Results'!F4:F400,64)</x:f>
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Paired transport aggregate reaches throughput and latency gates</x:v>
@@ -18357,112 +18634,844 @@
       </x:c>
     </x:row>
     <x:row r="256">
-      <x:c r="A256" s="29"/>
-      <x:c r="G256" s="27"/>
-      <x:c r="H256" s="27"/>
-      <x:c r="I256" s="23"/>
-      <x:c r="J256" s="25"/>
-      <x:c r="K256" s="25"/>
-      <x:c r="L256" s="25"/>
+      <x:c r="A256" s="89" t="str">
+        <x:v>2026-08-26 11:49</x:v>
+      </x:c>
+      <x:c r="B256" s="90" t="str">
+        <x:v>.NET</x:v>
+      </x:c>
+      <x:c r="C256" s="90" t="str">
+        <x:v>Multi</x:v>
+      </x:c>
+      <x:c r="D256" s="90" t="str">
+        <x:v>ROUTER_ROUTER_SENDSEND</x:v>
+      </x:c>
+      <x:c r="E256" s="90" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F256" s="90" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G256" s="91" t="n">
+        <x:v>168275</x:v>
+      </x:c>
+      <x:c r="H256" s="91" t="n">
+        <x:v>134362</x:v>
+      </x:c>
+      <x:c r="I256" s="92" t="n">
+        <x:f>H256/G256</x:f>
+        <x:v>0.7984667954241569</x:v>
+      </x:c>
+      <x:c r="J256" s="93" t="n">
+        <x:v>0.299</x:v>
+      </x:c>
+      <x:c r="K256" s="93" t="n">
+        <x:v>0.346</x:v>
+      </x:c>
+      <x:c r="L256" s="101" t="n">
+        <x:f>K256/J256</x:f>
+        <x:v>1.157190635451505</x:v>
+      </x:c>
+      <x:c r="M256" s="90" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N256" s="90" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O256" s="90" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P256" s="90" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q256" s="90" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R256" s="90" t="str">
+        <x:v>99164bdc3e (dirty)</x:v>
+      </x:c>
+      <x:c r="S256" s="90" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/multi/report/perf_c_multi_linux_20260826_114758_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="T256" s="90" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_114946_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="U256" s="90" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V256" s="94" t="str">
+        <x:v>Final paired 3-run median; throughput aggregate mean 100.72%; every size &gt;= 50%; latency ratio &lt;= 3.0x. Built-in single-message Router SendAsync fast path retained.</x:v>
+      </x:c>
     </x:row>
     <x:row r="257">
-      <x:c r="A257" s="29"/>
-      <x:c r="G257" s="27"/>
-      <x:c r="H257" s="27"/>
-      <x:c r="I257" s="23"/>
-      <x:c r="J257" s="25"/>
-      <x:c r="K257" s="25"/>
-      <x:c r="L257" s="25"/>
+      <x:c r="A257" s="77" t="str">
+        <x:v>2026-08-26 11:49</x:v>
+      </x:c>
+      <x:c r="B257" s="78" t="str">
+        <x:v>.NET</x:v>
+      </x:c>
+      <x:c r="C257" s="78" t="str">
+        <x:v>Multi</x:v>
+      </x:c>
+      <x:c r="D257" s="78" t="str">
+        <x:v>ROUTER_ROUTER_SENDSEND</x:v>
+      </x:c>
+      <x:c r="E257" s="78" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F257" s="78" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G257" s="79" t="n">
+        <x:v>159836</x:v>
+      </x:c>
+      <x:c r="H257" s="79" t="n">
+        <x:v>130727</x:v>
+      </x:c>
+      <x:c r="I257" s="80" t="n">
+        <x:f>H257/G257</x:f>
+        <x:v>0.8178820791311094</x:v>
+      </x:c>
+      <x:c r="J257" s="81" t="n">
+        <x:v>0.29</x:v>
+      </x:c>
+      <x:c r="K257" s="81" t="n">
+        <x:v>0.353</x:v>
+      </x:c>
+      <x:c r="L257" s="102" t="n">
+        <x:f>K257/J257</x:f>
+        <x:v>1.217241379310345</x:v>
+      </x:c>
+      <x:c r="M257" s="78" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N257" s="78" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O257" s="78" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P257" s="78" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q257" s="78" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R257" s="78" t="str">
+        <x:v>99164bdc3e (dirty)</x:v>
+      </x:c>
+      <x:c r="S257" s="78" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/multi/report/perf_c_multi_linux_20260826_114758_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="T257" s="78" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_114946_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="U257" s="78" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V257" s="82" t="str">
+        <x:v>Final paired 3-run median; throughput aggregate mean 100.72%; every size &gt;= 50%; latency ratio &lt;= 3.0x. Built-in single-message Router SendAsync fast path retained.</x:v>
+      </x:c>
     </x:row>
     <x:row r="258">
-      <x:c r="A258" s="29"/>
-      <x:c r="G258" s="27"/>
-      <x:c r="H258" s="27"/>
-      <x:c r="I258" s="23"/>
-      <x:c r="J258" s="25"/>
-      <x:c r="K258" s="25"/>
-      <x:c r="L258" s="25"/>
+      <x:c r="A258" s="95" t="str">
+        <x:v>2026-08-26 11:49</x:v>
+      </x:c>
+      <x:c r="B258" s="96" t="str">
+        <x:v>.NET</x:v>
+      </x:c>
+      <x:c r="C258" s="96" t="str">
+        <x:v>Multi</x:v>
+      </x:c>
+      <x:c r="D258" s="96" t="str">
+        <x:v>ROUTER_ROUTER_SENDSEND</x:v>
+      </x:c>
+      <x:c r="E258" s="96" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F258" s="96" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G258" s="97" t="n">
+        <x:v>150173</x:v>
+      </x:c>
+      <x:c r="H258" s="97" t="n">
+        <x:v>126812</x:v>
+      </x:c>
+      <x:c r="I258" s="98" t="n">
+        <x:f>H258/G258</x:f>
+        <x:v>0.8444394132100976</x:v>
+      </x:c>
+      <x:c r="J258" s="99" t="n">
+        <x:v>0.31</x:v>
+      </x:c>
+      <x:c r="K258" s="99" t="n">
+        <x:v>0.364</x:v>
+      </x:c>
+      <x:c r="L258" s="103" t="n">
+        <x:f>K258/J258</x:f>
+        <x:v>1.1741935483870967</x:v>
+      </x:c>
+      <x:c r="M258" s="96" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N258" s="96" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O258" s="96" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P258" s="96" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q258" s="96" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R258" s="96" t="str">
+        <x:v>99164bdc3e (dirty)</x:v>
+      </x:c>
+      <x:c r="S258" s="96" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/multi/report/perf_c_multi_linux_20260826_114758_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="T258" s="96" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_114946_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="U258" s="96" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V258" s="100" t="str">
+        <x:v>Final paired 3-run median; throughput aggregate mean 100.72%; every size &gt;= 50%; latency ratio &lt;= 3.0x. Built-in single-message Router SendAsync fast path retained.</x:v>
+      </x:c>
     </x:row>
     <x:row r="259">
-      <x:c r="A259" s="29"/>
-      <x:c r="G259" s="27"/>
-      <x:c r="H259" s="27"/>
-      <x:c r="I259" s="23"/>
-      <x:c r="J259" s="25"/>
-      <x:c r="K259" s="25"/>
-      <x:c r="L259" s="25"/>
+      <x:c r="A259" s="77" t="str">
+        <x:v>2026-08-26 11:49</x:v>
+      </x:c>
+      <x:c r="B259" s="78" t="str">
+        <x:v>.NET</x:v>
+      </x:c>
+      <x:c r="C259" s="78" t="str">
+        <x:v>Multi</x:v>
+      </x:c>
+      <x:c r="D259" s="78" t="str">
+        <x:v>ROUTER_ROUTER_SENDSEND</x:v>
+      </x:c>
+      <x:c r="E259" s="78" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F259" s="78" t="n">
+        <x:v>4096</x:v>
+      </x:c>
+      <x:c r="G259" s="79" t="n">
+        <x:v>126859.5</x:v>
+      </x:c>
+      <x:c r="H259" s="79" t="n">
+        <x:v>116625</x:v>
+      </x:c>
+      <x:c r="I259" s="80" t="n">
+        <x:f>H259/G259</x:f>
+        <x:v>0.9193241341799392</x:v>
+      </x:c>
+      <x:c r="J259" s="81" t="n">
+        <x:v>0.361</x:v>
+      </x:c>
+      <x:c r="K259" s="81" t="n">
+        <x:v>0.398</x:v>
+      </x:c>
+      <x:c r="L259" s="102" t="n">
+        <x:f>K259/J259</x:f>
+        <x:v>1.102493074792244</x:v>
+      </x:c>
+      <x:c r="M259" s="78" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N259" s="78" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O259" s="78" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P259" s="78" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q259" s="78" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R259" s="78" t="str">
+        <x:v>99164bdc3e (dirty)</x:v>
+      </x:c>
+      <x:c r="S259" s="78" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/multi/report/perf_c_multi_linux_20260826_114758_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="T259" s="78" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_114946_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="U259" s="78" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V259" s="82" t="str">
+        <x:v>Final paired 3-run median; throughput aggregate mean 100.72%; every size &gt;= 50%; latency ratio &lt;= 3.0x. Built-in single-message Router SendAsync fast path retained.</x:v>
+      </x:c>
     </x:row>
     <x:row r="260">
-      <x:c r="A260" s="29"/>
-      <x:c r="G260" s="27"/>
-      <x:c r="H260" s="27"/>
-      <x:c r="I260" s="23"/>
-      <x:c r="J260" s="25"/>
-      <x:c r="K260" s="25"/>
-      <x:c r="L260" s="25"/>
+      <x:c r="A260" s="95" t="str">
+        <x:v>2026-08-26 11:49</x:v>
+      </x:c>
+      <x:c r="B260" s="96" t="str">
+        <x:v>.NET</x:v>
+      </x:c>
+      <x:c r="C260" s="96" t="str">
+        <x:v>Multi</x:v>
+      </x:c>
+      <x:c r="D260" s="96" t="str">
+        <x:v>ROUTER_ROUTER_SENDSEND</x:v>
+      </x:c>
+      <x:c r="E260" s="96" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F260" s="96" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G260" s="97" t="n">
+        <x:v>25531</x:v>
+      </x:c>
+      <x:c r="H260" s="97" t="n">
+        <x:v>35623.5</x:v>
+      </x:c>
+      <x:c r="I260" s="98" t="n">
+        <x:f>H260/G260</x:f>
+        <x:v>1.3953037483843171</x:v>
+      </x:c>
+      <x:c r="J260" s="99" t="n">
+        <x:v>1.315</x:v>
+      </x:c>
+      <x:c r="K260" s="99" t="n">
+        <x:v>1.355</x:v>
+      </x:c>
+      <x:c r="L260" s="103" t="n">
+        <x:f>K260/J260</x:f>
+        <x:v>1.0304182509505704</x:v>
+      </x:c>
+      <x:c r="M260" s="96" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N260" s="96" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O260" s="96" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P260" s="96" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q260" s="96" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R260" s="96" t="str">
+        <x:v>99164bdc3e (dirty)</x:v>
+      </x:c>
+      <x:c r="S260" s="96" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/multi/report/perf_c_multi_linux_20260826_114758_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="T260" s="96" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_114946_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="U260" s="96" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V260" s="100" t="str">
+        <x:v>Final paired 3-run median; throughput aggregate mean 100.72%; every size &gt;= 50%; latency ratio &lt;= 3.0x. Built-in single-message Router SendAsync fast path retained.</x:v>
+      </x:c>
     </x:row>
     <x:row r="261">
-      <x:c r="A261" s="29"/>
-      <x:c r="G261" s="27"/>
-      <x:c r="H261" s="27"/>
-      <x:c r="I261" s="23"/>
-      <x:c r="J261" s="25"/>
-      <x:c r="K261" s="25"/>
-      <x:c r="L261" s="25"/>
+      <x:c r="A261" s="77" t="str">
+        <x:v>2026-08-26 11:49</x:v>
+      </x:c>
+      <x:c r="B261" s="78" t="str">
+        <x:v>.NET</x:v>
+      </x:c>
+      <x:c r="C261" s="78" t="str">
+        <x:v>Multi</x:v>
+      </x:c>
+      <x:c r="D261" s="78" t="str">
+        <x:v>ROUTER_ROUTER_SENDSEND</x:v>
+      </x:c>
+      <x:c r="E261" s="78" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F261" s="78" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G261" s="79" t="n">
+        <x:v>16102.5</x:v>
+      </x:c>
+      <x:c r="H261" s="79" t="n">
+        <x:v>20416.5</x:v>
+      </x:c>
+      <x:c r="I261" s="80" t="n">
+        <x:f>H261/G261</x:f>
+        <x:v>1.2679087098276665</x:v>
+      </x:c>
+      <x:c r="J261" s="81" t="n">
+        <x:v>2.156</x:v>
+      </x:c>
+      <x:c r="K261" s="81" t="n">
+        <x:v>2.392</x:v>
+      </x:c>
+      <x:c r="L261" s="102" t="n">
+        <x:f>K261/J261</x:f>
+        <x:v>1.1094619666048235</x:v>
+      </x:c>
+      <x:c r="M261" s="78" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N261" s="78" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O261" s="78" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P261" s="78" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q261" s="78" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R261" s="78" t="str">
+        <x:v>99164bdc3e (dirty)</x:v>
+      </x:c>
+      <x:c r="S261" s="78" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/multi/report/perf_c_multi_linux_20260826_114758_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="T261" s="78" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_114946_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="U261" s="78" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V261" s="82" t="str">
+        <x:v>Final paired 3-run median; throughput aggregate mean 100.72%; every size &gt;= 50%; latency ratio &lt;= 3.0x. Built-in single-message Router SendAsync fast path retained.</x:v>
+      </x:c>
     </x:row>
     <x:row r="262">
-      <x:c r="A262" s="29"/>
-      <x:c r="G262" s="27"/>
-      <x:c r="H262" s="27"/>
-      <x:c r="I262" s="23"/>
-      <x:c r="J262" s="25"/>
-      <x:c r="K262" s="25"/>
-      <x:c r="L262" s="25"/>
+      <x:c r="A262" s="95" t="str">
+        <x:v>2026-08-26 11:49</x:v>
+      </x:c>
+      <x:c r="B262" s="96" t="str">
+        <x:v>.NET</x:v>
+      </x:c>
+      <x:c r="C262" s="96" t="str">
+        <x:v>Multi</x:v>
+      </x:c>
+      <x:c r="D262" s="96" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E262" s="96" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F262" s="96" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G262" s="97" t="n">
+        <x:v>82664</x:v>
+      </x:c>
+      <x:c r="H262" s="97" t="n">
+        <x:v>55679.5</x:v>
+      </x:c>
+      <x:c r="I262" s="98" t="n">
+        <x:f>H262/G262</x:f>
+        <x:v>0.673564066582793</x:v>
+      </x:c>
+      <x:c r="J262" s="99" t="n">
+        <x:v>0.403</x:v>
+      </x:c>
+      <x:c r="K262" s="99" t="n">
+        <x:v>0.599</x:v>
+      </x:c>
+      <x:c r="L262" s="103" t="n">
+        <x:f>K262/J262</x:f>
+        <x:v>1.4863523573200992</x:v>
+      </x:c>
+      <x:c r="M262" s="96" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N262" s="96" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O262" s="96" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P262" s="96" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q262" s="96" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R262" s="96" t="str">
+        <x:v>99164bdc3e (dirty)</x:v>
+      </x:c>
+      <x:c r="S262" s="96" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/multi/report/perf_c_multi_linux_20260826_114758_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="T262" s="96" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_114946_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="U262" s="96" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V262" s="100" t="str">
+        <x:v>Final paired 3-run median; throughput aggregate mean 90.40%; every size &gt;= 50%; latency ratio &lt;= 3.0x. Built-in single-message Router SendAsync fast path retained.</x:v>
+      </x:c>
     </x:row>
     <x:row r="263">
-      <x:c r="A263" s="29"/>
-      <x:c r="G263" s="27"/>
-      <x:c r="H263" s="27"/>
-      <x:c r="I263" s="23"/>
-      <x:c r="J263" s="25"/>
-      <x:c r="K263" s="25"/>
-      <x:c r="L263" s="25"/>
+      <x:c r="A263" s="77" t="str">
+        <x:v>2026-08-26 11:49</x:v>
+      </x:c>
+      <x:c r="B263" s="78" t="str">
+        <x:v>.NET</x:v>
+      </x:c>
+      <x:c r="C263" s="78" t="str">
+        <x:v>Multi</x:v>
+      </x:c>
+      <x:c r="D263" s="78" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E263" s="78" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F263" s="78" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G263" s="79" t="n">
+        <x:v>75692</x:v>
+      </x:c>
+      <x:c r="H263" s="79" t="n">
+        <x:v>53203</x:v>
+      </x:c>
+      <x:c r="I263" s="80" t="n">
+        <x:f>H263/G263</x:f>
+        <x:v>0.7028880198699995</x:v>
+      </x:c>
+      <x:c r="J263" s="81" t="n">
+        <x:v>0.43</x:v>
+      </x:c>
+      <x:c r="K263" s="81" t="n">
+        <x:v>0.614</x:v>
+      </x:c>
+      <x:c r="L263" s="102" t="n">
+        <x:f>K263/J263</x:f>
+        <x:v>1.427906976744186</x:v>
+      </x:c>
+      <x:c r="M263" s="78" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N263" s="78" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O263" s="78" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P263" s="78" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q263" s="78" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R263" s="78" t="str">
+        <x:v>99164bdc3e (dirty)</x:v>
+      </x:c>
+      <x:c r="S263" s="78" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/multi/report/perf_c_multi_linux_20260826_114758_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="T263" s="78" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_114946_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="U263" s="78" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V263" s="82" t="str">
+        <x:v>Final paired 3-run median; throughput aggregate mean 90.40%; every size &gt;= 50%; latency ratio &lt;= 3.0x. Built-in single-message Router SendAsync fast path retained.</x:v>
+      </x:c>
     </x:row>
     <x:row r="264">
-      <x:c r="A264" s="29"/>
-      <x:c r="G264" s="27"/>
-      <x:c r="H264" s="27"/>
-      <x:c r="I264" s="23"/>
-      <x:c r="J264" s="25"/>
-      <x:c r="K264" s="25"/>
-      <x:c r="L264" s="25"/>
+      <x:c r="A264" s="95" t="str">
+        <x:v>2026-08-26 11:49</x:v>
+      </x:c>
+      <x:c r="B264" s="96" t="str">
+        <x:v>.NET</x:v>
+      </x:c>
+      <x:c r="C264" s="96" t="str">
+        <x:v>Multi</x:v>
+      </x:c>
+      <x:c r="D264" s="96" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E264" s="96" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F264" s="96" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G264" s="97" t="n">
+        <x:v>66401</x:v>
+      </x:c>
+      <x:c r="H264" s="97" t="n">
+        <x:v>51706</x:v>
+      </x:c>
+      <x:c r="I264" s="98" t="n">
+        <x:f>H264/G264</x:f>
+        <x:v>0.7786930919715065</x:v>
+      </x:c>
+      <x:c r="J264" s="99" t="n">
+        <x:v>0.491</x:v>
+      </x:c>
+      <x:c r="K264" s="99" t="n">
+        <x:v>0.629</x:v>
+      </x:c>
+      <x:c r="L264" s="103" t="n">
+        <x:f>K264/J264</x:f>
+        <x:v>1.2810590631364562</x:v>
+      </x:c>
+      <x:c r="M264" s="96" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N264" s="96" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O264" s="96" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P264" s="96" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q264" s="96" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R264" s="96" t="str">
+        <x:v>99164bdc3e (dirty)</x:v>
+      </x:c>
+      <x:c r="S264" s="96" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/multi/report/perf_c_multi_linux_20260826_114758_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="T264" s="96" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_114946_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="U264" s="96" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V264" s="100" t="str">
+        <x:v>Final paired 3-run median; throughput aggregate mean 90.40%; every size &gt;= 50%; latency ratio &lt;= 3.0x. Built-in single-message Router SendAsync fast path retained.</x:v>
+      </x:c>
     </x:row>
     <x:row r="265">
-      <x:c r="A265" s="29"/>
-      <x:c r="G265" s="27"/>
-      <x:c r="H265" s="27"/>
-      <x:c r="I265" s="23"/>
-      <x:c r="J265" s="25"/>
-      <x:c r="K265" s="25"/>
-      <x:c r="L265" s="25"/>
+      <x:c r="A265" s="77" t="str">
+        <x:v>2026-08-26 11:49</x:v>
+      </x:c>
+      <x:c r="B265" s="78" t="str">
+        <x:v>.NET</x:v>
+      </x:c>
+      <x:c r="C265" s="78" t="str">
+        <x:v>Multi</x:v>
+      </x:c>
+      <x:c r="D265" s="78" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E265" s="78" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F265" s="78" t="n">
+        <x:v>4096</x:v>
+      </x:c>
+      <x:c r="G265" s="79" t="n">
+        <x:v>54872</x:v>
+      </x:c>
+      <x:c r="H265" s="79" t="n">
+        <x:v>50487</x:v>
+      </x:c>
+      <x:c r="I265" s="80" t="n">
+        <x:f>H265/G265</x:f>
+        <x:v>0.9200867473392623</x:v>
+      </x:c>
+      <x:c r="J265" s="81" t="n">
+        <x:v>0.569</x:v>
+      </x:c>
+      <x:c r="K265" s="81" t="n">
+        <x:v>0.653</x:v>
+      </x:c>
+      <x:c r="L265" s="102" t="n">
+        <x:f>K265/J265</x:f>
+        <x:v>1.147627416520211</x:v>
+      </x:c>
+      <x:c r="M265" s="78" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N265" s="78" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O265" s="78" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P265" s="78" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q265" s="78" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R265" s="78" t="str">
+        <x:v>99164bdc3e (dirty)</x:v>
+      </x:c>
+      <x:c r="S265" s="78" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/multi/report/perf_c_multi_linux_20260826_114758_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="T265" s="78" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_114946_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="U265" s="78" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V265" s="82" t="str">
+        <x:v>Final paired 3-run median; throughput aggregate mean 90.40%; every size &gt;= 50%; latency ratio &lt;= 3.0x. Built-in single-message Router SendAsync fast path retained.</x:v>
+      </x:c>
     </x:row>
     <x:row r="266">
-      <x:c r="A266" s="29"/>
-      <x:c r="G266" s="27"/>
-      <x:c r="H266" s="27"/>
-      <x:c r="I266" s="23"/>
-      <x:c r="J266" s="25"/>
-      <x:c r="K266" s="25"/>
-      <x:c r="L266" s="25"/>
+      <x:c r="A266" s="95" t="str">
+        <x:v>2026-08-26 11:49</x:v>
+      </x:c>
+      <x:c r="B266" s="96" t="str">
+        <x:v>.NET</x:v>
+      </x:c>
+      <x:c r="C266" s="96" t="str">
+        <x:v>Multi</x:v>
+      </x:c>
+      <x:c r="D266" s="96" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E266" s="96" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F266" s="96" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G266" s="97" t="n">
+        <x:v>18926</x:v>
+      </x:c>
+      <x:c r="H266" s="97" t="n">
+        <x:v>21694</x:v>
+      </x:c>
+      <x:c r="I266" s="98" t="n">
+        <x:f>H266/G266</x:f>
+        <x:v>1.1462538307090775</x:v>
+      </x:c>
+      <x:c r="J266" s="99" t="n">
+        <x:v>1.388</x:v>
+      </x:c>
+      <x:c r="K266" s="99" t="n">
+        <x:v>2.162</x:v>
+      </x:c>
+      <x:c r="L266" s="103" t="n">
+        <x:f>K266/J266</x:f>
+        <x:v>1.5576368876080693</x:v>
+      </x:c>
+      <x:c r="M266" s="96" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N266" s="96" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O266" s="96" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P266" s="96" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q266" s="96" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R266" s="96" t="str">
+        <x:v>99164bdc3e (dirty)</x:v>
+      </x:c>
+      <x:c r="S266" s="96" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/multi/report/perf_c_multi_linux_20260826_114758_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="T266" s="96" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_114946_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="U266" s="96" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V266" s="100" t="str">
+        <x:v>Final paired 3-run median; throughput aggregate mean 90.40%; every size &gt;= 50%; latency ratio &lt;= 3.0x. Built-in single-message Router SendAsync fast path retained.</x:v>
+      </x:c>
     </x:row>
     <x:row r="267">
-      <x:c r="A267" s="29"/>
-      <x:c r="G267" s="27"/>
-      <x:c r="H267" s="27"/>
-      <x:c r="I267" s="23"/>
-      <x:c r="J267" s="25"/>
-      <x:c r="K267" s="25"/>
-      <x:c r="L267" s="25"/>
+      <x:c r="A267" s="83" t="str">
+        <x:v>2026-08-26 11:49</x:v>
+      </x:c>
+      <x:c r="B267" s="84" t="str">
+        <x:v>.NET</x:v>
+      </x:c>
+      <x:c r="C267" s="84" t="str">
+        <x:v>Multi</x:v>
+      </x:c>
+      <x:c r="D267" s="84" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E267" s="84" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F267" s="84" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G267" s="85" t="n">
+        <x:v>11839.5</x:v>
+      </x:c>
+      <x:c r="H267" s="85" t="n">
+        <x:v>14238.5</x:v>
+      </x:c>
+      <x:c r="I267" s="86" t="n">
+        <x:f>H267/G267</x:f>
+        <x:v>1.2026268001182483</x:v>
+      </x:c>
+      <x:c r="J267" s="87" t="n">
+        <x:v>2.131</x:v>
+      </x:c>
+      <x:c r="K267" s="87" t="n">
+        <x:v>3.361</x:v>
+      </x:c>
+      <x:c r="L267" s="104" t="n">
+        <x:f>K267/J267</x:f>
+        <x:v>1.5771938057250119</x:v>
+      </x:c>
+      <x:c r="M267" s="84" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N267" s="84" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O267" s="84" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P267" s="84" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q267" s="84" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R267" s="84" t="str">
+        <x:v>99164bdc3e (dirty)</x:v>
+      </x:c>
+      <x:c r="S267" s="84" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/multi/report/perf_c_multi_linux_20260826_114758_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="T267" s="84" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_114946_final-direct-fastpath-paired-r3.txt</x:v>
+      </x:c>
+      <x:c r="U267" s="84" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="V267" s="88" t="str">
+        <x:v>Final paired 3-run median; throughput aggregate mean 90.40%; every size &gt;= 50%; latency ratio &lt;= 3.0x. Built-in single-message Router SendAsync fast path retained.</x:v>
+      </x:c>
     </x:row>
     <x:row r="268">
       <x:c r="A268" s="29"/>
@@ -21860,36 +22869,92 @@
       </x:c>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="10"/>
-      <x:c r="B53" s="10"/>
-      <x:c r="C53" s="10"/>
-      <x:c r="D53" s="10"/>
-      <x:c r="E53" s="10"/>
-      <x:c r="F53" s="10"/>
-      <x:c r="G53" s="10"/>
-      <x:c r="H53" s="10"/>
-      <x:c r="I53" s="10"/>
-      <x:c r="J53" s="10"/>
-      <x:c r="K53" s="10"/>
-      <x:c r="L53" s="22"/>
-      <x:c r="M53" s="22"/>
-      <x:c r="N53" s="10"/>
+      <x:c r="A53" s="107" t="str">
+        <x:v>2026-08-26 11:36</x:v>
+      </x:c>
+      <x:c r="B53" s="107" t="str">
+        <x:v>.NET</x:v>
+      </x:c>
+      <x:c r="C53" s="107" t="str">
+        <x:v>Multi</x:v>
+      </x:c>
+      <x:c r="D53" s="107" t="str">
+        <x:v>ROUTER_ROUTER_SENDSEND</x:v>
+      </x:c>
+      <x:c r="E53" s="107" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F53" s="107" t="str">
+        <x:v>Residual managed submit overhead</x:v>
+      </x:c>
+      <x:c r="G53" s="107" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H53" s="107" t="str">
+        <x:v>Use the built-in single-message RouterSocket.SendAsync path and skip the per-message routed operation builder; pending sends still use Core completion.</x:v>
+      </x:c>
+      <x:c r="I53" s="107" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J53" s="107" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_113923_current-builder-send-r3.txt</x:v>
+      </x:c>
+      <x:c r="K53" s="107" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_113636_current-direct-single-send-r3.txt</x:v>
+      </x:c>
+      <x:c r="L53" s="108" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M53" s="108" t="n">
+        <x:v>1.017</x:v>
+      </x:c>
+      <x:c r="N53" s="107" t="str">
+        <x:v>KEEP: selected-size median A/B improved by 1.7% on average; 64B improved 5.2%. 128KiB delta was within run variance. Public API and completion semantics unchanged.</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="10"/>
-      <x:c r="B54" s="10"/>
-      <x:c r="C54" s="10"/>
-      <x:c r="D54" s="10"/>
-      <x:c r="E54" s="10"/>
-      <x:c r="F54" s="10"/>
-      <x:c r="G54" s="10"/>
-      <x:c r="H54" s="10"/>
-      <x:c r="I54" s="10"/>
-      <x:c r="J54" s="10"/>
-      <x:c r="K54" s="10"/>
-      <x:c r="L54" s="22"/>
-      <x:c r="M54" s="22"/>
-      <x:c r="N54" s="10"/>
+      <x:c r="A54" s="96" t="str">
+        <x:v>2026-08-26 11:36</x:v>
+      </x:c>
+      <x:c r="B54" s="96" t="str">
+        <x:v>.NET</x:v>
+      </x:c>
+      <x:c r="C54" s="96" t="str">
+        <x:v>Multi</x:v>
+      </x:c>
+      <x:c r="D54" s="96" t="str">
+        <x:v>ROUTER_ROUTER_REQREP</x:v>
+      </x:c>
+      <x:c r="E54" s="96" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F54" s="96" t="str">
+        <x:v>Residual managed submit overhead</x:v>
+      </x:c>
+      <x:c r="G54" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H54" s="96" t="str">
+        <x:v>Use the built-in single-message RouterSocket.SendAsync path and skip the per-message routed operation builder; pending sends still use Core completion.</x:v>
+      </x:c>
+      <x:c r="I54" s="96" t="str">
+        <x:v>ownership / exactly-once / close / failure / cancellation / concurrency / callback context</x:v>
+      </x:c>
+      <x:c r="J54" s="96" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_113923_current-builder-send-r3.txt</x:v>
+      </x:c>
+      <x:c r="K54" s="96" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/dotnet/perf/results/multi/report/perf_dotnet_multi_linux_20260826_113636_current-direct-single-send-r3.txt</x:v>
+      </x:c>
+      <x:c r="L54" s="98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M54" s="98" t="n">
+        <x:v>1.082</x:v>
+      </x:c>
+      <x:c r="N54" s="96" t="str">
+        <x:v>KEEP: selected-size median A/B improved by 8.2% on average (64B +5.0%, 64KiB +11.8%, 128KiB +7.9%). Public API and completion semantics unchanged.</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="10"/>

</xml_diff>

<commit_message>
perf: finalize 0.13.2 core and binding fixes
</commit_message>
<xml_diff>
--- a/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
+++ b/doc/perf/perf/bindings-0.13.2/bindings-library-performance-core-0.13.2.xlsx
@@ -19474,58 +19474,424 @@
       </x:c>
     </x:row>
     <x:row r="268">
-      <x:c r="A268" s="29"/>
-      <x:c r="G268" s="27"/>
-      <x:c r="H268" s="27"/>
-      <x:c r="I268" s="23"/>
-      <x:c r="J268" s="25"/>
-      <x:c r="K268" s="25"/>
-      <x:c r="L268" s="25"/>
+      <x:c r="A268" s="28" t="str">
+        <x:v>2026-08-27 00:48</x:v>
+      </x:c>
+      <x:c r="B268" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C268" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D268" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E268" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F268" s="10" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G268" s="26" t="n">
+        <x:v>980988.6</x:v>
+      </x:c>
+      <x:c r="H268" s="26" t="n">
+        <x:v>779687.2</x:v>
+      </x:c>
+      <x:c r="I268" s="22" t="n">
+        <x:f>H268/G268</x:f>
+        <x:v>0.7947968745508986</x:v>
+      </x:c>
+      <x:c r="J268" s="24" t="n">
+        <x:v>19.402</x:v>
+      </x:c>
+      <x:c r="K268" s="24" t="n">
+        <x:v>93.822</x:v>
+      </x:c>
+      <x:c r="L268" s="24" t="n">
+        <x:f>K268/J268</x:f>
+        <x:v>4.83568704257293</x:v>
+      </x:c>
+      <x:c r="M268" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N268" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O268" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P268" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q268" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R268" s="10" t="str">
+        <x:v>7361d80607</x:v>
+      </x:c>
+      <x:c r="S268" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260827_004556_cpp-pair-tcp-local0132-run-20260827-candidate-a-c.txt</x:v>
+      </x:c>
+      <x:c r="T268" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260827_004838_cpp-pair-tcp-local0132-run-20260827-candidate-a-cpp.txt</x:v>
+      </x:c>
+      <x:c r="U268" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V268" s="10" t="str">
+        <x:v>Candidate A: reusable PAIR received_t storage; throughput aggregate 91.33%; latency median 3.01x; pending supervisor judgment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="269">
-      <x:c r="A269" s="29"/>
-      <x:c r="G269" s="27"/>
-      <x:c r="H269" s="27"/>
-      <x:c r="I269" s="23"/>
-      <x:c r="J269" s="25"/>
-      <x:c r="K269" s="25"/>
-      <x:c r="L269" s="25"/>
+      <x:c r="A269" s="28" t="str">
+        <x:v>2026-08-27 00:48</x:v>
+      </x:c>
+      <x:c r="B269" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C269" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D269" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E269" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F269" s="10" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G269" s="26" t="n">
+        <x:v>897365.2</x:v>
+      </x:c>
+      <x:c r="H269" s="26" t="n">
+        <x:v>763161.8</x:v>
+      </x:c>
+      <x:c r="I269" s="22" t="n">
+        <x:f>H269/G269</x:f>
+        <x:v>0.8504470380829848</x:v>
+      </x:c>
+      <x:c r="J269" s="24" t="n">
+        <x:v>0.511</x:v>
+      </x:c>
+      <x:c r="K269" s="24" t="n">
+        <x:v>34.678</x:v>
+      </x:c>
+      <x:c r="L269" s="24" t="n">
+        <x:f>K269/J269</x:f>
+        <x:v>67.86301369863014</x:v>
+      </x:c>
+      <x:c r="M269" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N269" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O269" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P269" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q269" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R269" s="10" t="str">
+        <x:v>7361d80607</x:v>
+      </x:c>
+      <x:c r="S269" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260827_004556_cpp-pair-tcp-local0132-run-20260827-candidate-a-c.txt</x:v>
+      </x:c>
+      <x:c r="T269" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260827_004838_cpp-pair-tcp-local0132-run-20260827-candidate-a-cpp.txt</x:v>
+      </x:c>
+      <x:c r="U269" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V269" s="10" t="str">
+        <x:v>Candidate A: reusable PAIR received_t storage; throughput aggregate 91.33%; latency median 3.01x; pending supervisor judgment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="270">
-      <x:c r="A270" s="29"/>
-      <x:c r="G270" s="27"/>
-      <x:c r="H270" s="27"/>
-      <x:c r="I270" s="23"/>
-      <x:c r="J270" s="25"/>
-      <x:c r="K270" s="25"/>
-      <x:c r="L270" s="25"/>
+      <x:c r="A270" s="28" t="str">
+        <x:v>2026-08-27 00:48</x:v>
+      </x:c>
+      <x:c r="B270" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C270" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D270" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E270" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F270" s="10" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G270" s="26" t="n">
+        <x:v>804015.6</x:v>
+      </x:c>
+      <x:c r="H270" s="26" t="n">
+        <x:v>755139.8</x:v>
+      </x:c>
+      <x:c r="I270" s="22" t="n">
+        <x:f>H270/G270</x:f>
+        <x:v>0.9392098709353228</x:v>
+      </x:c>
+      <x:c r="J270" s="24" t="n">
+        <x:v>0.666</x:v>
+      </x:c>
+      <x:c r="K270" s="24" t="n">
+        <x:v>6.133</x:v>
+      </x:c>
+      <x:c r="L270" s="24" t="n">
+        <x:f>K270/J270</x:f>
+        <x:v>9.208708708708707</x:v>
+      </x:c>
+      <x:c r="M270" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N270" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O270" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P270" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q270" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R270" s="10" t="str">
+        <x:v>7361d80607</x:v>
+      </x:c>
+      <x:c r="S270" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260827_004556_cpp-pair-tcp-local0132-run-20260827-candidate-a-c.txt</x:v>
+      </x:c>
+      <x:c r="T270" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260827_004838_cpp-pair-tcp-local0132-run-20260827-candidate-a-cpp.txt</x:v>
+      </x:c>
+      <x:c r="U270" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V270" s="10" t="str">
+        <x:v>Candidate A: reusable PAIR received_t storage; throughput aggregate 91.33%; latency median 3.01x; pending supervisor judgment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="271">
-      <x:c r="A271" s="29"/>
-      <x:c r="G271" s="27"/>
-      <x:c r="H271" s="27"/>
-      <x:c r="I271" s="23"/>
-      <x:c r="J271" s="25"/>
-      <x:c r="K271" s="25"/>
-      <x:c r="L271" s="25"/>
+      <x:c r="A271" s="28" t="str">
+        <x:v>2026-08-27 00:48</x:v>
+      </x:c>
+      <x:c r="B271" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C271" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D271" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E271" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F271" s="10" t="n">
+        <x:v>65536</x:v>
+      </x:c>
+      <x:c r="G271" s="26" t="n">
+        <x:v>37146.0</x:v>
+      </x:c>
+      <x:c r="H271" s="26" t="n">
+        <x:v>34197.6</x:v>
+      </x:c>
+      <x:c r="I271" s="22" t="n">
+        <x:f>H271/G271</x:f>
+        <x:v>0.9206277924944813</x:v>
+      </x:c>
+      <x:c r="J271" s="24" t="n">
+        <x:v>0.243</x:v>
+      </x:c>
+      <x:c r="K271" s="24" t="n">
+        <x:v>0.289</x:v>
+      </x:c>
+      <x:c r="L271" s="24" t="n">
+        <x:f>K271/J271</x:f>
+        <x:v>1.1893004115226338</x:v>
+      </x:c>
+      <x:c r="M271" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N271" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O271" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P271" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q271" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R271" s="10" t="str">
+        <x:v>7361d80607</x:v>
+      </x:c>
+      <x:c r="S271" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260827_004556_cpp-pair-tcp-local0132-run-20260827-candidate-a-c.txt</x:v>
+      </x:c>
+      <x:c r="T271" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260827_004838_cpp-pair-tcp-local0132-run-20260827-candidate-a-cpp.txt</x:v>
+      </x:c>
+      <x:c r="U271" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V271" s="10" t="str">
+        <x:v>Candidate A: reusable PAIR received_t storage; throughput aggregate 91.33%; latency median 3.01x; pending supervisor judgment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="272">
-      <x:c r="A272" s="29"/>
-      <x:c r="G272" s="27"/>
-      <x:c r="H272" s="27"/>
-      <x:c r="I272" s="23"/>
-      <x:c r="J272" s="25"/>
-      <x:c r="K272" s="25"/>
-      <x:c r="L272" s="25"/>
+      <x:c r="A272" s="28" t="str">
+        <x:v>2026-08-27 00:48</x:v>
+      </x:c>
+      <x:c r="B272" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C272" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D272" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E272" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F272" s="10" t="n">
+        <x:v>131072</x:v>
+      </x:c>
+      <x:c r="G272" s="26" t="n">
+        <x:v>26277.4</x:v>
+      </x:c>
+      <x:c r="H272" s="26" t="n">
+        <x:v>25851.6</x:v>
+      </x:c>
+      <x:c r="I272" s="22" t="n">
+        <x:f>H272/G272</x:f>
+        <x:v>0.9837952005904702</x:v>
+      </x:c>
+      <x:c r="J272" s="24" t="n">
+        <x:v>0.213</x:v>
+      </x:c>
+      <x:c r="K272" s="24" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="L272" s="24" t="n">
+        <x:f>K272/J272</x:f>
+        <x:v>1.0140845070422535</x:v>
+      </x:c>
+      <x:c r="M272" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N272" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O272" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P272" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q272" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R272" s="10" t="str">
+        <x:v>7361d80607</x:v>
+      </x:c>
+      <x:c r="S272" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260827_004556_cpp-pair-tcp-local0132-run-20260827-candidate-a-c.txt</x:v>
+      </x:c>
+      <x:c r="T272" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260827_004838_cpp-pair-tcp-local0132-run-20260827-candidate-a-cpp.txt</x:v>
+      </x:c>
+      <x:c r="U272" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V272" s="10" t="str">
+        <x:v>Candidate A: reusable PAIR received_t storage; throughput aggregate 91.33%; latency median 3.01x; pending supervisor judgment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="273">
-      <x:c r="A273" s="29"/>
-      <x:c r="G273" s="27"/>
-      <x:c r="H273" s="27"/>
-      <x:c r="I273" s="23"/>
-      <x:c r="J273" s="25"/>
-      <x:c r="K273" s="25"/>
-      <x:c r="L273" s="25"/>
+      <x:c r="A273" s="28" t="str">
+        <x:v>2026-08-27 00:48</x:v>
+      </x:c>
+      <x:c r="B273" s="10" t="str">
+        <x:v>C++</x:v>
+      </x:c>
+      <x:c r="C273" s="10" t="str">
+        <x:v>Single</x:v>
+      </x:c>
+      <x:c r="D273" s="10" t="str">
+        <x:v>PAIR</x:v>
+      </x:c>
+      <x:c r="E273" s="10" t="str">
+        <x:v>tcp</x:v>
+      </x:c>
+      <x:c r="F273" s="10" t="n">
+        <x:v>262144</x:v>
+      </x:c>
+      <x:c r="G273" s="26" t="n">
+        <x:v>15972.0</x:v>
+      </x:c>
+      <x:c r="H273" s="26" t="n">
+        <x:v>15831.4</x:v>
+      </x:c>
+      <x:c r="I273" s="22" t="n">
+        <x:f>H273/G273</x:f>
+        <x:v>0.991197095746305</x:v>
+      </x:c>
+      <x:c r="J273" s="24" t="n">
+        <x:v>0.215</x:v>
+      </x:c>
+      <x:c r="K273" s="24" t="n">
+        <x:v>0.218</x:v>
+      </x:c>
+      <x:c r="L273" s="24" t="n">
+        <x:f>K273/J273</x:f>
+        <x:v>1.013953488372093</x:v>
+      </x:c>
+      <x:c r="M273" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N273" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O273" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P273" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="Q273" s="10" t="str">
+        <x:v>0.13.2</x:v>
+      </x:c>
+      <x:c r="R273" s="10" t="str">
+        <x:v>7361d80607</x:v>
+      </x:c>
+      <x:c r="S273" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/c/perf/results/single/report/perf_c_single_linux_20260827_004556_cpp-pair-tcp-local0132-run-20260827-candidate-a-c.txt</x:v>
+      </x:c>
+      <x:c r="T273" s="10" t="str">
+        <x:v>/home/hep7hep7/project/zlink/bindings/cpp/perf/results/single/report/perf_cpp_single_linux_20260827_004838_cpp-pair-tcp-local0132-run-20260827-candidate-a-cpp.txt</x:v>
+      </x:c>
+      <x:c r="U273" s="10" t="str">
+        <x:v>미달</x:v>
+      </x:c>
+      <x:c r="V273" s="10" t="str">
+        <x:v>Candidate A: reusable PAIR received_t storage; throughput aggregate 91.33%; latency median 3.01x; pending supervisor judgment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="274">
       <x:c r="A274" s="29"/>

</xml_diff>